<commit_message>
Adapting latest PCHA uncertainty to MCS-LC.
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Back-up\Drive_74_Backup\STORMSIM_DELIVERABLES\GitLab\For_Rusty\StormSim_Unified\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{229F551E-EBEB-48A7-BE69-46DDDA01B6B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{19B7A384-E454-4BD3-9EBD-FD87126F1025}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="161">
   <si>
     <t>StormSim Project General Inputs</t>
   </si>
@@ -314,9 +314,6 @@
     <t>Mean Value</t>
   </si>
   <si>
-    <t>Standard Deviation</t>
-  </si>
-  <si>
     <t>crest_elevation</t>
   </si>
   <si>
@@ -461,18 +458,6 @@
     <t>Roughness Coefficient, 2 for grass; 1 for concrete, asphalt, or closed blocks; 0.9 for basalt or placed revetment blocks; 0.8 for stepped structure; (rubble mound here! )</t>
   </si>
   <si>
-    <t>E:\Back-up\Drive_74_Backup\STORMSIM_DELIVERABLES\GitLab\For_Rusty\StormSim_Unified\CHS_Dataset_That_Failed.zip</t>
-  </si>
-  <si>
-    <t>pros_mode</t>
-  </si>
-  <si>
-    <t>StormSim: PROS Tier (RB1 Only)</t>
-  </si>
-  <si>
-    <t>RB1</t>
-  </si>
-  <si>
     <t>SWL Absolute Uncertainty, U_a</t>
   </si>
   <si>
@@ -524,13 +509,16 @@
     <t>CHS Region Bias File</t>
   </si>
   <si>
-    <t>E:\Back-up\Drive_74_Backup\STORMSIM_DELIVERABLES\GitLab\For_Rusty\StormSim_Unified\StormSim_Library\CHS\Bias_Correction_Files\NACCS_Comb_BiasUncertainty_perVG_rta.mat</t>
-  </si>
-  <si>
     <t>chs_bias_file</t>
   </si>
   <si>
     <t>StormSim workflow to call for project. (1 - StormSim:PROS, 2- StormSim:MCS, 3- StormSim: MCS/CSR, 4- StormSim: EVA (SST + JPM)</t>
+  </si>
+  <si>
+    <t>C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\StormSim_Library\CHS\Bias_Correction_Files\NACCS_Comb_BiasUncertainty_perVG_rta.mat</t>
+  </si>
+  <si>
+    <t>C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\CHS_Dataset_That_Failed.zip</t>
   </si>
 </sst>
 </file>
@@ -1269,34 +1257,33 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51D29750-2AFD-4BF7-A911-1DC4ADC0FD7A}">
-  <dimension ref="A1:J66"/>
+  <dimension ref="A1:I66"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="79" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="92.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="171.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="25.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="28.42578125" customWidth="1"/>
-    <col min="8" max="8" width="50" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="46.140625" customWidth="1"/>
+    <col min="6" max="6" width="28.42578125" customWidth="1"/>
+    <col min="7" max="7" width="50" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="46.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
       <c r="D1" s="6"/>
-      <c r="G1" s="32" t="s">
+      <c r="F1" s="32" t="s">
         <v>88</v>
       </c>
+      <c r="G1" s="33"/>
       <c r="H1" s="33"/>
       <c r="I1" s="33"/>
-      <c r="J1" s="33"/>
-    </row>
-    <row r="2" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>3</v>
       </c>
@@ -1309,20 +1296,20 @@
       <c r="D2" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="F2" s="9" t="s">
         <v>3</v>
       </c>
+      <c r="G2" s="10" t="s">
+        <v>7</v>
+      </c>
       <c r="H2" s="10" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I2" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="J2" s="10" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
         <v>8</v>
       </c>
@@ -1335,20 +1322,20 @@
       <c r="D3" s="1" t="s">
         <v>11</v>
       </c>
+      <c r="F3" s="49" t="s">
+        <v>147</v>
+      </c>
       <c r="G3" s="49" t="s">
-        <v>152</v>
-      </c>
-      <c r="H3" s="49" t="s">
-        <v>145</v>
-      </c>
-      <c r="I3" s="13" t="s">
+        <v>140</v>
+      </c>
+      <c r="H3" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="J3" s="13">
+      <c r="I3" s="13">
         <v>0.33979999999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
         <v>14</v>
       </c>
@@ -1361,20 +1348,20 @@
       <c r="D4" s="2" t="s">
         <v>16</v>
       </c>
+      <c r="F4" s="49" t="s">
+        <v>148</v>
+      </c>
       <c r="G4" s="49" t="s">
-        <v>153</v>
-      </c>
-      <c r="H4" s="49" t="s">
-        <v>146</v>
-      </c>
-      <c r="I4" s="13" t="s">
+        <v>141</v>
+      </c>
+      <c r="H4" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="J4" s="13">
+      <c r="I4" s="13">
         <v>0.38219999999999998</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>20</v>
       </c>
@@ -1387,20 +1374,20 @@
       <c r="D5" s="2">
         <v>3</v>
       </c>
+      <c r="F5" s="49" t="s">
+        <v>150</v>
+      </c>
       <c r="G5" s="49" t="s">
-        <v>155</v>
-      </c>
-      <c r="H5" s="49" t="s">
-        <v>147</v>
-      </c>
-      <c r="I5" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="H5" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="J5" s="13">
+      <c r="I5" s="13">
         <v>0.3</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
         <v>22</v>
       </c>
@@ -1411,22 +1398,22 @@
         <v>10</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
+      </c>
+      <c r="F6" s="49" t="s">
+        <v>149</v>
       </c>
       <c r="G6" s="49" t="s">
-        <v>154</v>
-      </c>
-      <c r="H6" s="49" t="s">
-        <v>148</v>
-      </c>
-      <c r="I6" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="H6" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="J6" s="13">
+      <c r="I6" s="13">
         <v>0.3</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>26</v>
       </c>
@@ -1437,22 +1424,22 @@
         <v>10</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="G7" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="H7" s="15" t="s">
-        <v>150</v>
-      </c>
-      <c r="I7" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="J7" s="2">
+        <v>122</v>
+      </c>
+      <c r="F7" s="14" t="s">
+        <v>151</v>
+      </c>
+      <c r="G7" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="H7" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I7" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="14" t="s">
         <v>30</v>
       </c>
@@ -1465,25 +1452,25 @@
       <c r="D8" s="2">
         <v>0</v>
       </c>
-      <c r="G8" s="17" t="s">
-        <v>151</v>
-      </c>
-      <c r="H8" s="18" t="s">
-        <v>149</v>
-      </c>
-      <c r="I8" s="19" t="s">
+      <c r="F8" s="17" t="s">
+        <v>146</v>
+      </c>
+      <c r="G8" s="18" t="s">
+        <v>144</v>
+      </c>
+      <c r="H8" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="J8" s="3">
+      <c r="I8" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C9" s="16" t="s">
         <v>10</v>
@@ -1491,32 +1478,32 @@
       <c r="D9" s="2">
         <v>1</v>
       </c>
+      <c r="F9" s="33"/>
       <c r="G9" s="33"/>
       <c r="H9" s="33"/>
       <c r="I9" s="33"/>
-      <c r="J9" s="33"/>
-    </row>
-    <row r="10" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="14" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="C10" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D10" s="2">
-        <v>3</v>
-      </c>
-      <c r="G10" s="26" t="s">
-        <v>157</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="F10" s="26" t="s">
+        <v>152</v>
+      </c>
+      <c r="G10" s="27"/>
       <c r="H10" s="27"/>
       <c r="I10" s="27"/>
-      <c r="J10" s="27"/>
-    </row>
-    <row r="11" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="14" t="s">
         <v>33</v>
       </c>
@@ -1529,20 +1516,20 @@
       <c r="D11" s="2">
         <v>0</v>
       </c>
-      <c r="G11" s="9" t="s">
+      <c r="F11" s="9" t="s">
         <v>3</v>
       </c>
+      <c r="G11" s="10" t="s">
+        <v>7</v>
+      </c>
       <c r="H11" s="10" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="J11" s="10" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>35</v>
       </c>
@@ -1555,20 +1542,20 @@
       <c r="D12" s="2">
         <v>1</v>
       </c>
-      <c r="G12" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="H12" s="15" t="s">
+      <c r="F12" s="30" t="s">
+        <v>154</v>
+      </c>
+      <c r="G12" s="15" t="s">
         <v>61</v>
       </c>
-      <c r="I12" s="16" t="s">
+      <c r="H12" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="J12" s="2">
+      <c r="I12" s="2">
         <v>0.5</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="17" t="s">
         <v>39</v>
       </c>
@@ -1581,58 +1568,58 @@
       <c r="D13" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="G13" s="30" t="s">
-        <v>160</v>
-      </c>
-      <c r="H13" s="15" t="s">
+      <c r="F13" s="30" t="s">
+        <v>155</v>
+      </c>
+      <c r="G13" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="I13" s="31" t="s">
+      <c r="H13" s="31" t="s">
         <v>75</v>
       </c>
-      <c r="J13" s="2">
+      <c r="I13" s="2">
         <v>0.43</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="6"/>
       <c r="B14" s="22"/>
       <c r="C14" s="23"/>
       <c r="D14" s="23"/>
-      <c r="G14" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="H14" s="15" t="s">
+      <c r="F14" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="G14" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="I14" s="16" t="s">
+      <c r="H14" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="J14" s="2">
+      <c r="I14" s="2">
         <v>0.78</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="24" t="s">
         <v>47</v>
       </c>
       <c r="B15" s="25"/>
       <c r="C15" s="25"/>
       <c r="D15" s="25"/>
-      <c r="G15" s="17" t="s">
-        <v>132</v>
-      </c>
-      <c r="H15" s="18" t="s">
+      <c r="F15" s="17" t="s">
+        <v>131</v>
+      </c>
+      <c r="G15" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="I15" s="19" t="s">
+      <c r="H15" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="J15" s="3">
+      <c r="I15" s="3">
         <v>0.13</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="9" t="s">
         <v>3</v>
       </c>
@@ -1645,17 +1632,17 @@
       <c r="D16" s="10" t="s">
         <v>6</v>
       </c>
+      <c r="F16" s="27"/>
       <c r="G16" s="27"/>
       <c r="H16" s="27"/>
       <c r="I16" s="27"/>
-      <c r="J16" s="27"/>
-    </row>
-    <row r="17" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="B17" s="15" t="s">
         <v>125</v>
-      </c>
-      <c r="B17" s="15" t="s">
-        <v>126</v>
       </c>
       <c r="C17" s="16" t="s">
         <v>10</v>
@@ -1663,18 +1650,18 @@
       <c r="D17" s="2">
         <v>1</v>
       </c>
-      <c r="G17" s="7" t="s">
+      <c r="F17" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="H17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8" t="s">
+        <v>2</v>
+      </c>
       <c r="I17" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="J17" s="8" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="18" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
         <v>50</v>
       </c>
@@ -1687,46 +1674,46 @@
       <c r="D18" s="1">
         <v>1</v>
       </c>
-      <c r="G18" s="9" t="s">
+      <c r="F18" s="9" t="s">
         <v>3</v>
       </c>
+      <c r="G18" s="10" t="s">
+        <v>7</v>
+      </c>
       <c r="H18" s="10" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="J18" s="10" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="C19" s="28" t="s">
         <v>10</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="G19" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="F19" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="H19" s="12" t="s">
+      <c r="G19" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="I19" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="J19" s="1">
+      <c r="H19" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="I19" s="1">
         <v>9</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
         <v>54</v>
       </c>
@@ -1737,22 +1724,22 @@
         <v>10</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="G20" s="14" t="s">
+        <v>160</v>
+      </c>
+      <c r="F20" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="H20" s="15" t="s">
+      <c r="G20" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="I20" s="16" t="s">
+      <c r="H20" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="J20" s="2">
+      <c r="I20" s="2">
         <v>50</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
         <v>58</v>
       </c>
@@ -1765,20 +1752,20 @@
       <c r="D21" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="G21" s="14" t="s">
+      <c r="F21" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="H21" s="15" t="s">
+      <c r="G21" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="I21" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="J21" s="2">
+      <c r="H21" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I21" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="14" t="s">
         <v>62</v>
       </c>
@@ -1791,20 +1778,20 @@
       <c r="D22" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="G22" s="17" t="s">
+      <c r="F22" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="H22" s="18" t="s">
+      <c r="G22" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="I22" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="J22" s="3">
+      <c r="H22" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="I22" s="3">
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
         <v>67</v>
       </c>
@@ -1817,12 +1804,12 @@
       <c r="D23" s="2" t="s">
         <v>69</v>
       </c>
+      <c r="F23" s="8"/>
       <c r="G23" s="8"/>
       <c r="H23" s="8"/>
       <c r="I23" s="8"/>
-      <c r="J23" s="8"/>
-    </row>
-    <row r="24" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="24" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="14" t="s">
         <v>71</v>
       </c>
@@ -1835,14 +1822,14 @@
       <c r="D24" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="G24" s="20" t="s">
+      <c r="F24" s="20" t="s">
         <v>32</v>
       </c>
+      <c r="G24" s="21"/>
       <c r="H24" s="21"/>
       <c r="I24" s="21"/>
-      <c r="J24" s="21"/>
-    </row>
-    <row r="25" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="25" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="14" t="s">
         <v>76</v>
       </c>
@@ -1855,20 +1842,20 @@
       <c r="D25" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="G25" s="9" t="s">
+      <c r="F25" s="9" t="s">
         <v>3</v>
       </c>
+      <c r="G25" s="10" t="s">
+        <v>7</v>
+      </c>
       <c r="H25" s="10" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I25" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="J25" s="10" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
         <v>79</v>
       </c>
@@ -1881,20 +1868,20 @@
       <c r="D26" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="G26" s="11" t="s">
+      <c r="F26" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="H26" s="12" t="s">
+      <c r="G26" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="I26" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="J26" s="1">
+      <c r="H26" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="I26" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
         <v>82</v>
       </c>
@@ -1907,20 +1894,20 @@
       <c r="D27" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="G27" s="14" t="s">
+      <c r="F27" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="H27" s="15" t="s">
+      <c r="G27" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="I27" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="J27" s="2">
+      <c r="H27" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I27" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="17" t="s">
         <v>85</v>
       </c>
@@ -1933,51 +1920,50 @@
       <c r="D28" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="G28" s="14" t="s">
+      <c r="F28" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="H28" s="15" t="s">
+      <c r="G28" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="I28" s="16" t="s">
+      <c r="H28" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="J28" s="2">
+      <c r="I28" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="25"/>
       <c r="B29" s="25"/>
       <c r="C29" s="25"/>
       <c r="D29" s="25"/>
-      <c r="G29" s="17" t="s">
+      <c r="F29" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="H29" s="18" t="s">
+      <c r="G29" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="I29" s="19" t="s">
+      <c r="H29" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="J29" s="3">
+      <c r="I29" s="3">
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="34" t="s">
         <v>90</v>
       </c>
       <c r="B30" s="35"/>
       <c r="C30" s="35"/>
       <c r="D30" s="35"/>
-      <c r="E30" s="35"/>
+      <c r="F30" s="21"/>
       <c r="G30" s="21"/>
       <c r="H30" s="21"/>
       <c r="I30" s="21"/>
-      <c r="J30" s="21"/>
-    </row>
-    <row r="31" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="31" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="9" t="s">
         <v>3</v>
       </c>
@@ -1990,22 +1976,19 @@
       <c r="D31" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="E31" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="G31" s="26" t="s">
+      <c r="F31" s="26" t="s">
         <v>53</v>
       </c>
+      <c r="G31" s="27"/>
       <c r="H31" s="27"/>
       <c r="I31" s="27"/>
-      <c r="J31" s="27"/>
-    </row>
-    <row r="32" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="32" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C32" s="13" t="s">
         <v>10</v>
@@ -2013,28 +1996,25 @@
       <c r="D32" s="1">
         <v>1.2320122</v>
       </c>
-      <c r="E32" s="1">
-        <v>0</v>
-      </c>
-      <c r="G32" s="9" t="s">
+      <c r="F32" s="9" t="s">
         <v>3</v>
       </c>
+      <c r="G32" s="10" t="s">
+        <v>7</v>
+      </c>
       <c r="H32" s="10" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="J32" s="10" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B33" s="15" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C33" s="16" t="s">
         <v>10</v>
@@ -2042,28 +2022,25 @@
       <c r="D33" s="2">
         <v>1.5243902</v>
       </c>
-      <c r="E33" s="2">
-        <v>0</v>
-      </c>
-      <c r="G33" s="11" t="s">
-        <v>142</v>
-      </c>
-      <c r="H33" s="12" t="s">
-        <v>143</v>
-      </c>
-      <c r="I33" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="J33" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F33" s="29" t="s">
+        <v>56</v>
+      </c>
+      <c r="G33" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="H33" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="I33" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="B34" s="15" t="s">
         <v>95</v>
-      </c>
-      <c r="B34" s="15" t="s">
-        <v>96</v>
       </c>
       <c r="C34" s="16" t="s">
         <v>46</v>
@@ -2071,28 +2048,13 @@
       <c r="D34" s="2">
         <v>-1.5969511999999999</v>
       </c>
-      <c r="E34" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="G34" s="29" t="s">
-        <v>56</v>
-      </c>
-      <c r="H34" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="I34" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="J34" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="B35" s="15" t="s">
         <v>97</v>
-      </c>
-      <c r="B35" s="15" t="s">
-        <v>98</v>
       </c>
       <c r="C35" s="16" t="s">
         <v>10</v>
@@ -2100,16 +2062,13 @@
       <c r="D35" s="2">
         <v>1.5</v>
       </c>
-      <c r="E35" s="16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="B36" s="15" t="s">
         <v>99</v>
-      </c>
-      <c r="B36" s="15" t="s">
-        <v>100</v>
       </c>
       <c r="C36" s="16" t="s">
         <v>10</v>
@@ -2117,16 +2076,13 @@
       <c r="D36" s="2">
         <v>1.5</v>
       </c>
-      <c r="E36" s="16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="39" t="s">
+        <v>133</v>
+      </c>
+      <c r="B37" s="39" t="s">
         <v>134</v>
-      </c>
-      <c r="B37" s="39" t="s">
-        <v>135</v>
       </c>
       <c r="C37" s="45" t="s">
         <v>10</v>
@@ -2134,16 +2090,13 @@
       <c r="D37" s="46">
         <v>0</v>
       </c>
-      <c r="E37" s="45" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C38" s="16" t="s">
         <v>10</v>
@@ -2151,16 +2104,13 @@
       <c r="D38" s="2">
         <v>20</v>
       </c>
-      <c r="E38" s="16" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="39" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="38" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B39" s="38" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C39" s="43" t="s">
         <v>10</v>
@@ -2168,27 +2118,22 @@
       <c r="D39" s="44">
         <v>20</v>
       </c>
-      <c r="E39" s="43" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="34"/>
       <c r="B40" s="34"/>
       <c r="C40" s="34"/>
       <c r="D40" s="34"/>
-      <c r="E40" s="34"/>
-    </row>
-    <row r="41" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="41" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="36" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B41" s="37"/>
       <c r="C41" s="37"/>
       <c r="D41" s="37"/>
-      <c r="E41" s="37"/>
-    </row>
-    <row r="42" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="42" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="9" t="s">
         <v>3</v>
       </c>
@@ -2201,16 +2146,13 @@
       <c r="D42" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="E42" s="10" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="B43" s="12" t="s">
         <v>102</v>
-      </c>
-      <c r="B43" s="12" t="s">
-        <v>103</v>
       </c>
       <c r="C43" s="13" t="s">
         <v>10</v>
@@ -2218,84 +2160,69 @@
       <c r="D43" s="1">
         <v>1.65</v>
       </c>
-      <c r="E43" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="B44" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="B44" s="15" t="s">
+      <c r="C44" s="16" t="s">
         <v>105</v>
-      </c>
-      <c r="C44" s="16" t="s">
-        <v>106</v>
       </c>
       <c r="D44" s="2">
         <v>907.18</v>
       </c>
-      <c r="E44" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="B45" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="B45" s="15" t="s">
-        <v>108</v>
-      </c>
       <c r="C45" s="16" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D45" s="2">
         <v>907.18</v>
       </c>
-      <c r="E45" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="B46" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="B46" s="15" t="s">
+      <c r="C46" s="16" t="s">
         <v>110</v>
-      </c>
-      <c r="C46" s="16" t="s">
-        <v>111</v>
       </c>
       <c r="D46" s="2">
         <v>1027</v>
       </c>
-      <c r="E46" s="16" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="B47" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="B47" s="15" t="s">
+      <c r="C47" s="16" t="s">
         <v>113</v>
-      </c>
-      <c r="C47" s="16" t="s">
-        <v>114</v>
       </c>
       <c r="D47" s="2">
         <v>0.4</v>
       </c>
-      <c r="E47" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="B48" s="15" t="s">
         <v>115</v>
-      </c>
-      <c r="B48" s="15" t="s">
-        <v>116</v>
       </c>
       <c r="C48" s="16" t="s">
         <v>10</v>
@@ -2303,16 +2230,13 @@
       <c r="D48" s="2">
         <v>20</v>
       </c>
-      <c r="E48" s="16" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="B49" s="15" t="s">
         <v>117</v>
-      </c>
-      <c r="B49" s="15" t="s">
-        <v>118</v>
       </c>
       <c r="C49" s="16" t="s">
         <v>10</v>
@@ -2320,16 +2244,13 @@
       <c r="D49" s="2">
         <v>20</v>
       </c>
-      <c r="E49" s="16" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="B50" s="15" t="s">
         <v>119</v>
-      </c>
-      <c r="B50" s="15" t="s">
-        <v>120</v>
       </c>
       <c r="C50" s="16" t="s">
         <v>10</v>
@@ -2337,16 +2258,13 @@
       <c r="D50" s="2">
         <v>5</v>
       </c>
-      <c r="E50" s="16" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="39" t="s">
+        <v>120</v>
+      </c>
+      <c r="B51" s="40" t="s">
         <v>121</v>
-      </c>
-      <c r="B51" s="40" t="s">
-        <v>122</v>
       </c>
       <c r="C51" s="41" t="s">
         <v>10</v>
@@ -2354,16 +2272,13 @@
       <c r="D51" s="42">
         <v>2</v>
       </c>
-      <c r="E51" s="41" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="52" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="18" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B52" s="48" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C52" s="19" t="s">
         <v>10</v>
@@ -2371,16 +2286,12 @@
       <c r="D52" s="4">
         <v>2</v>
       </c>
-      <c r="E52" s="19" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="37"/>
       <c r="B53" s="37"/>
       <c r="C53" s="37"/>
       <c r="D53" s="37"/>
-      <c r="E53" s="37"/>
     </row>
     <row r="66" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B66" s="47"/>
@@ -2388,7 +2299,7 @@
   </sheetData>
   <sheetProtection formatColumns="0" selectLockedCells="1"/>
   <protectedRanges>
-    <protectedRange sqref="D32:D36 E35:E36 E32:E33 D17:D28 E43:E45 E47 J19:J22 D43:D52 E51 J33:J34 J3:J6 J8 J12:J16 J26:J29 D3:D13" name="Range1_1"/>
+    <protectedRange sqref="D32:D36 I3:I6 I8 D17:D28 I12:I16 I26:I29 I19:I22 D43:D52 D3:D13 I33" name="Range1_1"/>
   </protectedRanges>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Uploading random tide function.
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{19B7A384-E454-4BD3-9EBD-FD87126F1025}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63E0B7CD-9E28-474B-9647-4F8640A00382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="164">
   <si>
     <t>StormSim Project General Inputs</t>
   </si>
@@ -515,10 +515,19 @@
     <t>StormSim workflow to call for project. (1 - StormSim:PROS, 2- StormSim:MCS, 3- StormSim: MCS/CSR, 4- StormSim: EVA (SST + JPM)</t>
   </si>
   <si>
-    <t>C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\StormSim_Library\CHS\Bias_Correction_Files\NACCS_Comb_BiasUncertainty_perVG_rta.mat</t>
-  </si>
-  <si>
-    <t>C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\CHS_Dataset_That_Failed.zip</t>
+    <t>tide_file</t>
+  </si>
+  <si>
+    <t>Tidal file used to randomly sample tidal values for storm SWL.</t>
+  </si>
+  <si>
+    <t>C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\</t>
+  </si>
+  <si>
+    <t>CHS_Dataset_That_Failed.zip</t>
+  </si>
+  <si>
+    <t>StormSim_Library\CHS\Bias_Correction_Files\NACCS_Comb_BiasUncertainty_perVG_rta.mat</t>
   </si>
 </sst>
 </file>
@@ -1257,7 +1266,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51D29750-2AFD-4BF7-A911-1DC4ADC0FD7A}">
-  <dimension ref="A1:I66"/>
+  <dimension ref="A1:I67"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="79" bestFit="1" customWidth="1"/>
@@ -1467,16 +1476,16 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>127</v>
+        <v>160</v>
       </c>
       <c r="C9" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="2">
-        <v>1</v>
+      <c r="D9" s="2" t="s">
+        <v>161</v>
       </c>
       <c r="F9" s="33"/>
       <c r="G9" s="33"/>
@@ -1485,10 +1494,10 @@
     </row>
     <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="14" t="s">
-        <v>126</v>
+        <v>153</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>158</v>
+        <v>127</v>
       </c>
       <c r="C10" s="16" t="s">
         <v>10</v>
@@ -1505,16 +1514,16 @@
     </row>
     <row r="11" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="14" t="s">
-        <v>33</v>
+        <v>126</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>34</v>
+        <v>158</v>
       </c>
       <c r="C11" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>3</v>
@@ -1531,16 +1540,16 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C12" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D12" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F12" s="30" t="s">
         <v>154</v>
@@ -1555,18 +1564,18 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="17" t="s">
-        <v>39</v>
-      </c>
-      <c r="B13" s="18" t="s">
-        <v>40</v>
-      </c>
-      <c r="C13" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>41</v>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" s="2">
+        <v>1</v>
       </c>
       <c r="F13" s="30" t="s">
         <v>155</v>
@@ -1581,11 +1590,19 @@
         <v>0.43</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="6"/>
-      <c r="B14" s="22"/>
-      <c r="C14" s="23"/>
-      <c r="D14" s="23"/>
+    <row r="14" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>41</v>
+      </c>
       <c r="F14" s="14" t="s">
         <v>130</v>
       </c>
@@ -1600,12 +1617,10 @@
       </c>
     </row>
     <row r="15" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="24" t="s">
-        <v>47</v>
-      </c>
-      <c r="B15" s="25"/>
-      <c r="C15" s="25"/>
-      <c r="D15" s="25"/>
+      <c r="A15" s="6"/>
+      <c r="B15" s="22"/>
+      <c r="C15" s="23"/>
+      <c r="D15" s="23"/>
       <c r="F15" s="17" t="s">
         <v>131</v>
       </c>
@@ -1620,35 +1635,29 @@
       </c>
     </row>
     <row r="16" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B16" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="D16" s="10" t="s">
-        <v>6</v>
-      </c>
+      <c r="A16" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="B16" s="25"/>
+      <c r="C16" s="25"/>
+      <c r="D16" s="25"/>
       <c r="F16" s="27"/>
       <c r="G16" s="27"/>
       <c r="H16" s="27"/>
       <c r="I16" s="27"/>
     </row>
     <row r="17" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="14" t="s">
-        <v>124</v>
-      </c>
-      <c r="B17" s="15" t="s">
-        <v>125</v>
-      </c>
-      <c r="C17" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D17" s="2">
-        <v>1</v>
+      <c r="A17" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>6</v>
       </c>
       <c r="F17" s="7" t="s">
         <v>1</v>
@@ -1662,16 +1671,16 @@
       </c>
     </row>
     <row r="18" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="B18" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="C18" s="28" t="s">
-        <v>52</v>
-      </c>
-      <c r="D18" s="1">
+      <c r="A18" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="B18" s="15" t="s">
+        <v>125</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18" s="2">
         <v>1</v>
       </c>
       <c r="F18" s="9" t="s">
@@ -1689,16 +1698,16 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
-        <v>157</v>
+        <v>50</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>156</v>
+        <v>51</v>
       </c>
       <c r="C19" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>159</v>
+        <v>52</v>
+      </c>
+      <c r="D19" s="1">
+        <v>1</v>
       </c>
       <c r="F19" s="11" t="s">
         <v>12</v>
@@ -1714,17 +1723,17 @@
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="B20" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="C20" s="16" t="s">
+      <c r="A20" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>156</v>
+      </c>
+      <c r="C20" s="28" t="s">
         <v>10</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="F20" s="14" t="s">
         <v>17</v>
@@ -1741,16 +1750,16 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="C21" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>60</v>
+        <v>162</v>
       </c>
       <c r="F21" s="14" t="s">
         <v>24</v>
@@ -1767,16 +1776,16 @@
     </row>
     <row r="22" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="14" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C22" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="F22" s="17" t="s">
         <v>28</v>
@@ -1793,16 +1802,16 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="C23" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="F23" s="8"/>
       <c r="G23" s="8"/>
@@ -1811,16 +1820,16 @@
     </row>
     <row r="24" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="14" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C24" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="F24" s="20" t="s">
         <v>32</v>
@@ -1831,16 +1840,16 @@
     </row>
     <row r="25" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="14" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C25" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="F25" s="9" t="s">
         <v>3</v>
@@ -1857,16 +1866,16 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C26" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="F26" s="11" t="s">
         <v>37</v>
@@ -1883,16 +1892,16 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C27" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="F27" s="14" t="s">
         <v>42</v>
@@ -1907,18 +1916,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="17" t="s">
-        <v>85</v>
-      </c>
-      <c r="B28" s="18" t="s">
-        <v>86</v>
-      </c>
-      <c r="C28" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>87</v>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="B28" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="C28" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>84</v>
       </c>
       <c r="F28" s="14" t="s">
         <v>44</v>
@@ -1934,10 +1943,18 @@
       </c>
     </row>
     <row r="29" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="25"/>
-      <c r="B29" s="25"/>
-      <c r="C29" s="25"/>
-      <c r="D29" s="25"/>
+      <c r="A29" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="B29" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="C29" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>87</v>
+      </c>
       <c r="F29" s="17" t="s">
         <v>48</v>
       </c>
@@ -1951,31 +1968,23 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="34" t="s">
-        <v>90</v>
-      </c>
-      <c r="B30" s="35"/>
-      <c r="C30" s="35"/>
-      <c r="D30" s="35"/>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" s="25"/>
+      <c r="B30" s="25"/>
+      <c r="C30" s="25"/>
+      <c r="D30" s="25"/>
       <c r="F30" s="21"/>
       <c r="G30" s="21"/>
       <c r="H30" s="21"/>
       <c r="I30" s="21"/>
     </row>
     <row r="31" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B31" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C31" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="D31" s="10" t="s">
-        <v>91</v>
-      </c>
+      <c r="A31" s="34" t="s">
+        <v>90</v>
+      </c>
+      <c r="B31" s="35"/>
+      <c r="C31" s="35"/>
+      <c r="D31" s="35"/>
       <c r="F31" s="26" t="s">
         <v>53</v>
       </c>
@@ -1984,17 +1993,17 @@
       <c r="I31" s="27"/>
     </row>
     <row r="32" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="B32" s="12" t="s">
-        <v>128</v>
-      </c>
-      <c r="C32" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="D32" s="1">
-        <v>1.2320122</v>
+      <c r="A32" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B32" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C32" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D32" s="10" t="s">
+        <v>91</v>
       </c>
       <c r="F32" s="9" t="s">
         <v>3</v>
@@ -2010,17 +2019,17 @@
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="14" t="s">
-        <v>93</v>
-      </c>
-      <c r="B33" s="15" t="s">
-        <v>129</v>
-      </c>
-      <c r="C33" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D33" s="2">
-        <v>1.5243902</v>
+      <c r="A33" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="B33" s="12" t="s">
+        <v>128</v>
+      </c>
+      <c r="C33" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D33" s="1">
+        <v>1.2320122</v>
       </c>
       <c r="F33" s="29" t="s">
         <v>56</v>
@@ -2037,38 +2046,38 @@
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>95</v>
+        <v>129</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>46</v>
+        <v>10</v>
       </c>
       <c r="D34" s="2">
-        <v>-1.5969511999999999</v>
+        <v>1.5243902</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B35" s="15" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C35" s="16" t="s">
-        <v>10</v>
+        <v>46</v>
       </c>
       <c r="D35" s="2">
-        <v>1.5</v>
+        <v>-1.5969511999999999</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B36" s="15" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C36" s="16" t="s">
         <v>10</v>
@@ -2078,109 +2087,109 @@
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A37" s="39" t="s">
+      <c r="A37" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="B37" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="C37" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D37" s="2">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A38" s="39" t="s">
         <v>133</v>
       </c>
-      <c r="B37" s="39" t="s">
+      <c r="B38" s="39" t="s">
         <v>134</v>
       </c>
-      <c r="C37" s="45" t="s">
-        <v>10</v>
-      </c>
-      <c r="D37" s="46">
+      <c r="C38" s="45" t="s">
+        <v>10</v>
+      </c>
+      <c r="D38" s="46">
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A38" s="14" t="s">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A39" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="B38" s="14" t="s">
+      <c r="B39" s="14" t="s">
         <v>137</v>
       </c>
-      <c r="C38" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D38" s="2">
+      <c r="C39" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D39" s="2">
         <v>20</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="38" t="s">
+    <row r="40" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="38" t="s">
         <v>136</v>
       </c>
-      <c r="B39" s="38" t="s">
+      <c r="B40" s="38" t="s">
         <v>138</v>
       </c>
-      <c r="C39" s="43" t="s">
-        <v>10</v>
-      </c>
-      <c r="D39" s="44">
+      <c r="C40" s="43" t="s">
+        <v>10</v>
+      </c>
+      <c r="D40" s="44">
         <v>20</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A40" s="34"/>
-      <c r="B40" s="34"/>
-      <c r="C40" s="34"/>
-      <c r="D40" s="34"/>
-    </row>
-    <row r="41" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="36" t="s">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A41" s="34"/>
+      <c r="B41" s="34"/>
+      <c r="C41" s="34"/>
+      <c r="D41" s="34"/>
+    </row>
+    <row r="42" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="36" t="s">
         <v>100</v>
       </c>
-      <c r="B41" s="37"/>
-      <c r="C41" s="37"/>
-      <c r="D41" s="37"/>
-    </row>
-    <row r="42" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="9" t="s">
+      <c r="B42" s="37"/>
+      <c r="C42" s="37"/>
+      <c r="D42" s="37"/>
+    </row>
+    <row r="43" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="B42" s="10" t="s">
+      <c r="B43" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C42" s="10" t="s">
+      <c r="C43" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="D42" s="10" t="s">
+      <c r="D43" s="10" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A43" s="11" t="s">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A44" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="B43" s="12" t="s">
+      <c r="B44" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="C43" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="D43" s="1">
+      <c r="C44" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D44" s="1">
         <v>1.65</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A44" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="B44" s="15" t="s">
-        <v>104</v>
-      </c>
-      <c r="C44" s="16" t="s">
-        <v>105</v>
-      </c>
-      <c r="D44" s="2">
-        <v>907.18</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B45" s="15" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C45" s="16" t="s">
         <v>105</v>
@@ -2191,52 +2200,52 @@
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B46" s="15" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C46" s="16" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="D46" s="2">
-        <v>1027</v>
+        <v>907.18</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B47" s="15" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C47" s="16" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="D47" s="2">
-        <v>0.4</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B48" s="15" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C48" s="16" t="s">
-        <v>10</v>
+        <v>113</v>
       </c>
       <c r="D48" s="2">
-        <v>20</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B49" s="15" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C49" s="16" t="s">
         <v>10</v>
@@ -2247,59 +2256,73 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="B50" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="C50" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D50" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="B50" s="15" t="s">
+      <c r="B51" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="C50" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D50" s="2">
+      <c r="C51" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D51" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="39" t="s">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" s="39" t="s">
         <v>120</v>
       </c>
-      <c r="B51" s="40" t="s">
+      <c r="B52" s="40" t="s">
         <v>121</v>
       </c>
-      <c r="C51" s="41" t="s">
-        <v>10</v>
-      </c>
-      <c r="D51" s="42">
+      <c r="C52" s="41" t="s">
+        <v>10</v>
+      </c>
+      <c r="D52" s="42">
         <v>2</v>
       </c>
     </row>
-    <row r="52" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="18" t="s">
+    <row r="53" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="B52" s="48" t="s">
+      <c r="B53" s="48" t="s">
         <v>139</v>
       </c>
-      <c r="C52" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D52" s="4">
+      <c r="C53" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D53" s="4">
         <v>2</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="37"/>
-      <c r="B53" s="37"/>
-      <c r="C53" s="37"/>
-      <c r="D53" s="37"/>
-    </row>
-    <row r="66" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B66" s="47"/>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" s="37"/>
+      <c r="B54" s="37"/>
+      <c r="C54" s="37"/>
+      <c r="D54" s="37"/>
+    </row>
+    <row r="67" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B67" s="47"/>
     </row>
   </sheetData>
   <sheetProtection formatColumns="0" selectLockedCells="1"/>
   <protectedRanges>
-    <protectedRange sqref="D32:D36 I3:I6 I8 D17:D28 I12:I16 I26:I29 I19:I22 D43:D52 D3:D13 I33" name="Range1_1"/>
+    <protectedRange sqref="D33:D37 I3:I6 I8 D18:D29 I12:I16 I26:I29 I19:I22 D44:D53 D3:D14 I33" name="Range1_1"/>
   </protectedRanges>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
First staage integration of PROS.
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63E0B7CD-9E28-474B-9647-4F8640A00382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C55D4119-96C3-49C2-A20D-47DE9157BC15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
+    <workbookView xWindow="3480" yWindow="6855" windowWidth="28725" windowHeight="15345" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
   <sheets>
     <sheet name="Full_Inputs" sheetId="1" r:id="rId1"/>
@@ -521,13 +521,13 @@
     <t>Tidal file used to randomly sample tidal values for storm SWL.</t>
   </si>
   <si>
-    <t>C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\</t>
-  </si>
-  <si>
     <t>CHS_Dataset_That_Failed.zip</t>
   </si>
   <si>
     <t>StormSim_Library\CHS\Bias_Correction_Files\NACCS_Comb_BiasUncertainty_perVG_rta.mat</t>
+  </si>
+  <si>
+    <t>C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\CO-OPS_8571421_Bishops_Head_Pred_tide_MSL_ft.csv</t>
   </si>
 </sst>
 </file>
@@ -1485,7 +1485,7 @@
         <v>10</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="F9" s="33"/>
       <c r="G9" s="33"/>
@@ -1733,7 +1733,7 @@
         <v>10</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F20" s="14" t="s">
         <v>17</v>
@@ -1759,7 +1759,7 @@
         <v>10</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F21" s="14" t="s">
         <v>24</v>
@@ -2125,7 +2125,7 @@
         <v>10</v>
       </c>
       <c r="D39" s="2">
-        <v>20</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2139,7 +2139,7 @@
         <v>10</v>
       </c>
       <c r="D40" s="44">
-        <v>20</v>
+        <v>-0.5</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Upload StormSim PROS phase 2 integration.
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C55D4119-96C3-49C2-A20D-47DE9157BC15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C7743C7-5AC0-43AE-A9A6-66E63AED9303}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3480" yWindow="6855" windowWidth="28725" windowHeight="15345" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
   <sheets>
     <sheet name="Full_Inputs" sheetId="1" r:id="rId1"/>
@@ -1523,7 +1523,7 @@
         <v>10</v>
       </c>
       <c r="D11" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>3</v>

</xml_diff>

<commit_message>
Debuggin peaks only run.
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC675CC8-AE5C-4223-9025-D2EF8F352AA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A0FF0F7-2431-400D-AED4-7D16D8E4E27E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="156">
   <si>
     <t>StormSim Project General Inputs</t>
   </si>
@@ -218,9 +218,6 @@
     <t>ADCIRC TC Peaks</t>
   </si>
   <si>
-    <t>CHS-NA_XH_SimB_Post0_SP01972_ADCIRC01_Peaks.h5</t>
-  </si>
-  <si>
     <t>Dn50 Uncertainty</t>
   </si>
   <si>
@@ -230,9 +227,6 @@
     <t>ADCIRC TC Timeseries</t>
   </si>
   <si>
-    <t>CHS-NA_XH_SimB_Post0_SP01972_ADCIRC01_Timeseries.h5</t>
-  </si>
-  <si>
     <t>Overtopping Uncertainty</t>
   </si>
   <si>
@@ -245,9 +239,6 @@
     <t>STWAVE TC Peaks</t>
   </si>
   <si>
-    <t>CHS-NA_XH_SimB_Post0_SP0848_STWAVE04_Peaks.h5</t>
-  </si>
-  <si>
     <t>Runup Uncertainty</t>
   </si>
   <si>
@@ -257,9 +248,6 @@
     <t>STWAVE TC Timeseries</t>
   </si>
   <si>
-    <t>CHS-NA_XH_SimB_Post0_SP0848_STWAVE04_Timeseries.h5</t>
-  </si>
-  <si>
     <t>Surface Pressure (p1) Uncertainty' (Floodwalls Only)</t>
   </si>
   <si>
@@ -272,34 +260,22 @@
     <t>ADCIRC XC Peaks</t>
   </si>
   <si>
-    <t>CHS-NA_TS_SimB_Post0_SP01972_ADCIRC01_Peaks.h5</t>
-  </si>
-  <si>
     <t>chs_xc_swl_timeseries</t>
   </si>
   <si>
     <t>ADCIRC XC Timeseries</t>
   </si>
   <si>
-    <t>CHS-NA_TS_SimB_Post0_SP01972_ADCIRC01_Timeseries.h5</t>
-  </si>
-  <si>
     <t>chs_xc_hm0_peaks</t>
   </si>
   <si>
     <t>STWAVE XC Peaks</t>
   </si>
   <si>
-    <t>CHS-NA_TS_SimB_Post0_SP0848_STWAVE04_Peaks.h5</t>
-  </si>
-  <si>
     <t>chs_xc_hm0_timeseries</t>
   </si>
   <si>
     <t>STWAVE XC Timeseries</t>
-  </si>
-  <si>
-    <t>CHS-NA_TS_SimB_Post0_SP0848_STWAVE04_Timeseries.h5</t>
   </si>
   <si>
     <t xml:space="preserve">StormSim Project Forcing Uncertainty </t>
@@ -1286,7 +1262,7 @@
       <c r="C1" s="6"/>
       <c r="D1" s="6"/>
       <c r="F1" s="32" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="G1" s="33"/>
       <c r="H1" s="33"/>
@@ -1332,10 +1308,10 @@
         <v>11</v>
       </c>
       <c r="F3" s="49" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="G3" s="49" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="H3" s="13" t="s">
         <v>46</v>
@@ -1358,10 +1334,10 @@
         <v>16</v>
       </c>
       <c r="F4" s="49" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="G4" s="49" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="H4" s="13" t="s">
         <v>46</v>
@@ -1384,10 +1360,10 @@
         <v>3</v>
       </c>
       <c r="F5" s="49" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="G5" s="49" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="H5" s="13" t="s">
         <v>46</v>
@@ -1407,13 +1383,13 @@
         <v>10</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="F6" s="49" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="G6" s="49" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="H6" s="13" t="s">
         <v>46</v>
@@ -1433,13 +1409,13 @@
         <v>10</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="G7" s="15" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="H7" s="16" t="s">
         <v>10</v>
@@ -1462,13 +1438,13 @@
         <v>0</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="H8" s="19" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="I8" s="3">
         <v>0</v>
@@ -1476,16 +1452,16 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="C9" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="F9" s="33"/>
       <c r="G9" s="33"/>
@@ -1494,10 +1470,10 @@
     </row>
     <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="14" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="C10" s="16" t="s">
         <v>10</v>
@@ -1506,7 +1482,7 @@
         <v>1</v>
       </c>
       <c r="F10" s="26" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="G10" s="27"/>
       <c r="H10" s="27"/>
@@ -1514,10 +1490,10 @@
     </row>
     <row r="11" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="14" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="C11" s="16" t="s">
         <v>10</v>
@@ -1552,10 +1528,10 @@
         <v>0</v>
       </c>
       <c r="F12" s="30" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="G12" s="15" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="H12" s="16" t="s">
         <v>46</v>
@@ -1578,13 +1554,13 @@
         <v>1</v>
       </c>
       <c r="F13" s="30" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="G13" s="15" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="H13" s="31" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="I13" s="2">
         <v>0.43</v>
@@ -1604,13 +1580,13 @@
         <v>41</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="G14" s="15" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="H14" s="16" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I14" s="2">
         <v>0.78</v>
@@ -1622,10 +1598,10 @@
       <c r="C15" s="23"/>
       <c r="D15" s="23"/>
       <c r="F15" s="17" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="G15" s="18" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="H15" s="19" t="s">
         <v>46</v>
@@ -1672,10 +1648,10 @@
     </row>
     <row r="18" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="14" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="C18" s="16" t="s">
         <v>10</v>
@@ -1724,16 +1700,16 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="C20" s="28" t="s">
         <v>10</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="F20" s="14" t="s">
         <v>17</v>
@@ -1759,7 +1735,7 @@
         <v>10</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="F21" s="14" t="s">
         <v>24</v>
@@ -1784,9 +1760,7 @@
       <c r="C22" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D22" s="2" t="s">
-        <v>60</v>
-      </c>
+      <c r="D22" s="2"/>
       <c r="F22" s="17" t="s">
         <v>28</v>
       </c>
@@ -1802,17 +1776,15 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="B23" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="B23" s="15" t="s">
-        <v>63</v>
-      </c>
       <c r="C23" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D23" s="2" t="s">
-        <v>64</v>
-      </c>
+      <c r="D23" s="2"/>
       <c r="F23" s="8"/>
       <c r="G23" s="8"/>
       <c r="H23" s="8"/>
@@ -1820,17 +1792,15 @@
     </row>
     <row r="24" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="14" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C24" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D24" s="2" t="s">
-        <v>69</v>
-      </c>
+      <c r="D24" s="2"/>
       <c r="F24" s="20" t="s">
         <v>32</v>
       </c>
@@ -1840,17 +1810,15 @@
     </row>
     <row r="25" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="14" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C25" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D25" s="2" t="s">
-        <v>73</v>
-      </c>
+      <c r="D25" s="2"/>
       <c r="F25" s="9" t="s">
         <v>3</v>
       </c>
@@ -1866,17 +1834,15 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C26" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D26" s="2" t="s">
-        <v>78</v>
-      </c>
+      <c r="D26" s="2"/>
       <c r="F26" s="11" t="s">
         <v>37</v>
       </c>
@@ -1892,17 +1858,15 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C27" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D27" s="2" t="s">
-        <v>81</v>
-      </c>
+      <c r="D27" s="2"/>
       <c r="F27" s="14" t="s">
         <v>42</v>
       </c>
@@ -1918,17 +1882,15 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="C28" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D28" s="2" t="s">
-        <v>84</v>
-      </c>
+      <c r="D28" s="2"/>
       <c r="F28" s="14" t="s">
         <v>44</v>
       </c>
@@ -1944,17 +1906,15 @@
     </row>
     <row r="29" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="17" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="B29" s="18" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="C29" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="D29" s="3" t="s">
-        <v>87</v>
-      </c>
+      <c r="D29" s="3"/>
       <c r="F29" s="17" t="s">
         <v>48</v>
       </c>
@@ -1980,7 +1940,7 @@
     </row>
     <row r="31" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="34" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="B31" s="35"/>
       <c r="C31" s="35"/>
@@ -2003,7 +1963,7 @@
         <v>5</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="F32" s="9" t="s">
         <v>3</v>
@@ -2020,10 +1980,10 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="11" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="C33" s="13" t="s">
         <v>10</v>
@@ -2046,10 +2006,10 @@
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="C34" s="16" t="s">
         <v>10</v>
@@ -2060,10 +2020,10 @@
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B35" s="15" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="C35" s="16" t="s">
         <v>46</v>
@@ -2074,10 +2034,10 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="B36" s="15" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="C36" s="16" t="s">
         <v>10</v>
@@ -2088,10 +2048,10 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="C37" s="16" t="s">
         <v>10</v>
@@ -2102,10 +2062,10 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="39" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="B38" s="39" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="C38" s="45" t="s">
         <v>10</v>
@@ -2116,10 +2076,10 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="C39" s="16" t="s">
         <v>10</v>
@@ -2130,10 +2090,10 @@
     </row>
     <row r="40" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="38" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="B40" s="38" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="C40" s="43" t="s">
         <v>10</v>
@@ -2150,7 +2110,7 @@
     </row>
     <row r="42" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="36" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="B42" s="37"/>
       <c r="C42" s="37"/>
@@ -2167,15 +2127,15 @@
         <v>5</v>
       </c>
       <c r="D43" s="10" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="11" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="B44" s="12" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="C44" s="13" t="s">
         <v>10</v>
@@ -2186,13 +2146,13 @@
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="B45" s="15" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="C45" s="16" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="D45" s="2">
         <v>907.18</v>
@@ -2200,13 +2160,13 @@
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="B46" s="15" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C46" s="16" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="D46" s="2">
         <v>907.18</v>
@@ -2214,13 +2174,13 @@
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="B47" s="15" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="C47" s="16" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="D47" s="2">
         <v>1027</v>
@@ -2228,13 +2188,13 @@
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="B48" s="15" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="C48" s="16" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="D48" s="2">
         <v>0.4</v>
@@ -2242,10 +2202,10 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="B49" s="15" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="C49" s="16" t="s">
         <v>10</v>
@@ -2256,10 +2216,10 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="B50" s="15" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="C50" s="16" t="s">
         <v>10</v>
@@ -2270,10 +2230,10 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="14" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="B51" s="15" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="C51" s="16" t="s">
         <v>10</v>
@@ -2284,10 +2244,10 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="39" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="B52" s="40" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="C52" s="41" t="s">
         <v>10</v>
@@ -2298,10 +2258,10 @@
     </row>
     <row r="53" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="18" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="B53" s="48" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="C53" s="19" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
Fixing RB3 related bugs.
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A0FF0F7-2431-400D-AED4-7D16D8E4E27E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD3679FF-7416-4848-B4B2-0669E6BBA02F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
   <sheets>
     <sheet name="Full_Inputs" sheetId="1" r:id="rId1"/>
+    <sheet name="NAE_Structure" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="169">
   <si>
     <t>StormSim Project General Inputs</t>
   </si>
@@ -137,18 +138,6 @@
     <t>StormSim: Coastal Structure Reliability Damage  (CSR) Module</t>
   </si>
   <si>
-    <t>plots_show_figures</t>
-  </si>
-  <si>
-    <t>Show output plots (0/1)</t>
-  </si>
-  <si>
-    <t>plots_show_percentiles</t>
-  </si>
-  <si>
-    <t>Show percentiles (0/1) in output plots (when applicable)</t>
-  </si>
-  <si>
     <t>csr_call_dpa</t>
   </si>
   <si>
@@ -383,9 +372,6 @@
     <t>CC</t>
   </si>
   <si>
-    <t>MSL</t>
-  </si>
-  <si>
     <t>use_timeseries</t>
   </si>
   <si>
@@ -497,13 +483,67 @@
     <t>Tidal file used to randomly sample tidal values for storm SWL.</t>
   </si>
   <si>
-    <t>CHS_Dataset_That_Failed.zip</t>
-  </si>
-  <si>
     <t>StormSim_Library\CHS\Bias_Correction_Files\NACCS_Comb_BiasUncertainty_perVG_rta.mat</t>
   </si>
   <si>
-    <t>C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\CO-OPS_8571421_Bishops_Head_Pred_tide_MSL_ft.csv</t>
+    <t>C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\CO-OPS_88638660_NAVD88_m_Tidal_Pred_1_year.csv</t>
+  </si>
+  <si>
+    <t>NAVD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Given </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Structure Type </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crest Width </t>
+  </si>
+  <si>
+    <t>ft</t>
+  </si>
+  <si>
+    <t>Crest Elevation</t>
+  </si>
+  <si>
+    <t>ft, NAVD88</t>
+  </si>
+  <si>
+    <t>Toe Elevation</t>
+  </si>
+  <si>
+    <t>Side Slope</t>
+  </si>
+  <si>
+    <t>Coverage (RipRap)</t>
+  </si>
+  <si>
+    <t>NAVD88 to MSL</t>
+  </si>
+  <si>
+    <t>Spatially Varying Uncertainty (+/-): 0.298 US_ft</t>
+  </si>
+  <si>
+    <t>How shoud we account for this ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Convert Datums And Units </t>
+  </si>
+  <si>
+    <t>m</t>
+  </si>
+  <si>
+    <t>m, MSL</t>
+  </si>
+  <si>
+    <t>CHSFileDownload_2023-02-23_11-31-35.zip</t>
+  </si>
+  <si>
+    <t>chs_sp_depth</t>
+  </si>
+  <si>
+    <t>CHS savepoint depth (Will be used if not found in h5)</t>
   </si>
 </sst>
 </file>
@@ -816,7 +856,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -927,6 +967,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1242,7 +1285,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51D29750-2AFD-4BF7-A911-1DC4ADC0FD7A}">
-  <dimension ref="A1:I67"/>
+  <dimension ref="A1:I66"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="79" bestFit="1" customWidth="1"/>
@@ -1262,7 +1305,7 @@
       <c r="C1" s="6"/>
       <c r="D1" s="6"/>
       <c r="F1" s="32" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="G1" s="33"/>
       <c r="H1" s="33"/>
@@ -1308,13 +1351,13 @@
         <v>11</v>
       </c>
       <c r="F3" s="49" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="G3" s="49" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="H3" s="13" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="I3" s="13">
         <v>0.33979999999999999</v>
@@ -1334,13 +1377,13 @@
         <v>16</v>
       </c>
       <c r="F4" s="49" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="G4" s="49" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="H4" s="13" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="I4" s="13">
         <v>0.38219999999999998</v>
@@ -1357,16 +1400,16 @@
         <v>10</v>
       </c>
       <c r="D5" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F5" s="49" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="G5" s="49" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="I5" s="13">
         <v>0.3</v>
@@ -1383,16 +1426,16 @@
         <v>10</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>115</v>
+        <v>150</v>
       </c>
       <c r="F6" s="49" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="G6" s="49" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="H6" s="13" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="I6" s="13">
         <v>0.3</v>
@@ -1409,13 +1452,13 @@
         <v>10</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="G7" s="15" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="H7" s="16" t="s">
         <v>10</v>
@@ -1438,13 +1481,13 @@
         <v>0</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="H8" s="19" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="I8" s="3">
         <v>0</v>
@@ -1452,16 +1495,16 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="C9" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="F9" s="33"/>
       <c r="G9" s="33"/>
@@ -1470,10 +1513,10 @@
     </row>
     <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="14" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="C10" s="16" t="s">
         <v>10</v>
@@ -1482,7 +1525,7 @@
         <v>1</v>
       </c>
       <c r="F10" s="26" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="G10" s="27"/>
       <c r="H10" s="27"/>
@@ -1490,10 +1533,10 @@
     </row>
     <row r="11" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="14" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="C11" s="16" t="s">
         <v>10</v>
@@ -1514,126 +1557,126 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="B12" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="C12" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D12" s="2">
-        <v>0</v>
+    <row r="12" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>37</v>
       </c>
       <c r="F12" s="30" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="G12" s="15" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="H12" s="16" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="I12" s="2">
         <v>0.5</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="B13" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="C13" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D13" s="2">
-        <v>1</v>
-      </c>
+      <c r="A13" s="6"/>
+      <c r="B13" s="22"/>
+      <c r="C13" s="23"/>
+      <c r="D13" s="23"/>
       <c r="F13" s="30" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="G13" s="15" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="H13" s="31" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="I13" s="2">
         <v>0.43</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="17" t="s">
-        <v>39</v>
-      </c>
-      <c r="B14" s="18" t="s">
-        <v>40</v>
-      </c>
-      <c r="C14" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>41</v>
-      </c>
+      <c r="A14" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="B14" s="25"/>
+      <c r="C14" s="25"/>
+      <c r="D14" s="25"/>
       <c r="F14" s="14" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="G14" s="15" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="H14" s="16" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I14" s="2">
         <v>0.78</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="6"/>
-      <c r="B15" s="22"/>
-      <c r="C15" s="23"/>
-      <c r="D15" s="23"/>
+      <c r="A15" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>6</v>
+      </c>
       <c r="F15" s="17" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="G15" s="18" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="H15" s="19" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="I15" s="3">
         <v>0.13</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="24" t="s">
-        <v>47</v>
-      </c>
-      <c r="B16" s="25"/>
-      <c r="C16" s="25"/>
-      <c r="D16" s="25"/>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="B16" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" s="2">
+        <v>1</v>
+      </c>
       <c r="F16" s="27"/>
       <c r="G16" s="27"/>
       <c r="H16" s="27"/>
       <c r="I16" s="27"/>
     </row>
     <row r="17" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B17" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="C17" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="D17" s="10" t="s">
-        <v>6</v>
+      <c r="A17" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17" s="28" t="s">
+        <v>48</v>
+      </c>
+      <c r="D17" s="1">
+        <v>1</v>
       </c>
       <c r="F17" s="7" t="s">
         <v>1</v>
@@ -1647,17 +1690,17 @@
       </c>
     </row>
     <row r="18" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="14" t="s">
-        <v>116</v>
-      </c>
-      <c r="B18" s="15" t="s">
-        <v>117</v>
-      </c>
-      <c r="C18" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D18" s="2">
-        <v>1</v>
+      <c r="A18" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="C18" s="28" t="s">
+        <v>164</v>
+      </c>
+      <c r="D18" s="1">
+        <v>5</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>3</v>
@@ -1674,16 +1717,16 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
-        <v>50</v>
+        <v>144</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>51</v>
+        <v>143</v>
       </c>
       <c r="C19" s="28" t="s">
-        <v>52</v>
-      </c>
-      <c r="D19" s="1">
-        <v>1</v>
+        <v>10</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>148</v>
       </c>
       <c r="F19" s="11" t="s">
         <v>12</v>
@@ -1699,17 +1742,17 @@
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="11" t="s">
-        <v>149</v>
-      </c>
-      <c r="B20" s="12" t="s">
-        <v>148</v>
-      </c>
-      <c r="C20" s="28" t="s">
+      <c r="A20" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="B20" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="F20" s="14" t="s">
         <v>17</v>
@@ -1734,9 +1777,7 @@
       <c r="C21" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D21" s="2" t="s">
-        <v>153</v>
-      </c>
+      <c r="D21" s="2"/>
       <c r="F21" s="14" t="s">
         <v>24</v>
       </c>
@@ -1752,10 +1793,10 @@
     </row>
     <row r="22" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="B22" s="15" t="s">
         <v>58</v>
-      </c>
-      <c r="B22" s="15" t="s">
-        <v>59</v>
       </c>
       <c r="C22" s="16" t="s">
         <v>10</v>
@@ -1792,10 +1833,10 @@
     </row>
     <row r="24" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="B24" s="15" t="s">
         <v>65</v>
-      </c>
-      <c r="B24" s="15" t="s">
-        <v>66</v>
       </c>
       <c r="C24" s="16" t="s">
         <v>10</v>
@@ -1834,20 +1875,20 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C26" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D26" s="2"/>
       <c r="F26" s="11" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="G26" s="12" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="H26" s="13" t="s">
         <v>10</v>
@@ -1858,20 +1899,20 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C27" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D27" s="2"/>
       <c r="F27" s="14" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="G27" s="15" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="H27" s="16" t="s">
         <v>10</v>
@@ -1880,90 +1921,93 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="14" t="s">
-        <v>76</v>
-      </c>
-      <c r="B28" s="15" t="s">
-        <v>77</v>
-      </c>
-      <c r="C28" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D28" s="2"/>
+    <row r="28" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="B28" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="C28" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D28" s="3"/>
       <c r="F28" s="14" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="G28" s="15" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H28" s="16" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="I28" s="2">
         <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="17" t="s">
-        <v>78</v>
-      </c>
-      <c r="B29" s="18" t="s">
-        <v>79</v>
-      </c>
-      <c r="C29" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D29" s="3"/>
+      <c r="A29" s="25"/>
+      <c r="B29" s="25"/>
+      <c r="C29" s="25"/>
+      <c r="D29" s="25"/>
       <c r="F29" s="17" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="G29" s="18" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="H29" s="19" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="I29" s="3">
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="25"/>
-      <c r="B30" s="25"/>
-      <c r="C30" s="25"/>
-      <c r="D30" s="25"/>
+    <row r="30" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="34" t="s">
+        <v>78</v>
+      </c>
+      <c r="B30" s="35"/>
+      <c r="C30" s="35"/>
+      <c r="D30" s="35"/>
       <c r="F30" s="21"/>
       <c r="G30" s="21"/>
       <c r="H30" s="21"/>
       <c r="I30" s="21"/>
     </row>
     <row r="31" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="34" t="s">
-        <v>82</v>
-      </c>
-      <c r="B31" s="35"/>
-      <c r="C31" s="35"/>
-      <c r="D31" s="35"/>
+      <c r="A31" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D31" s="10" t="s">
+        <v>79</v>
+      </c>
       <c r="F31" s="26" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="G31" s="27"/>
       <c r="H31" s="27"/>
       <c r="I31" s="27"/>
     </row>
     <row r="32" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B32" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C32" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="D32" s="10" t="s">
-        <v>83</v>
+      <c r="A32" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="B32" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="C32" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D32" s="1">
+        <f>NAE_Structure!B12</f>
+        <v>4.9590959999999997</v>
       </c>
       <c r="F32" s="9" t="s">
         <v>3</v>
@@ -1979,23 +2023,24 @@
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="11" t="s">
-        <v>84</v>
-      </c>
-      <c r="B33" s="12" t="s">
-        <v>120</v>
-      </c>
-      <c r="C33" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="D33" s="1">
-        <v>1.2320122</v>
+      <c r="A33" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="B33" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="C33" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D33" s="2">
+        <f>NAE_Structure!B11</f>
+        <v>3.130296</v>
       </c>
       <c r="F33" s="29" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="G33" s="12" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="H33" s="13" t="s">
         <v>10</v>
@@ -2006,153 +2051,156 @@
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>121</v>
+        <v>83</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="D34" s="2">
-        <v>1.5243902</v>
+        <f>NAE_Structure!B13*-1</f>
+        <v>-2.8254960000000002</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B35" s="15" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C35" s="16" t="s">
-        <v>46</v>
+        <v>10</v>
       </c>
       <c r="D35" s="2">
-        <v>-1.5969511999999999</v>
+        <f>NAE_Structure!B6</f>
+        <v>3</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="B36" s="15" t="s">
+        <v>87</v>
+      </c>
+      <c r="C36" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D36" s="2">
+        <f>NAE_Structure!B6</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37" s="39" t="s">
+        <v>120</v>
+      </c>
+      <c r="B37" s="39" t="s">
+        <v>121</v>
+      </c>
+      <c r="C37" s="45" t="s">
+        <v>10</v>
+      </c>
+      <c r="D37" s="46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A38" s="14" t="s">
+        <v>122</v>
+      </c>
+      <c r="B38" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="C38" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D38" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="38" t="s">
+        <v>123</v>
+      </c>
+      <c r="B39" s="38" t="s">
+        <v>125</v>
+      </c>
+      <c r="C39" s="43" t="s">
+        <v>10</v>
+      </c>
+      <c r="D39" s="44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A40" s="34"/>
+      <c r="B40" s="34"/>
+      <c r="C40" s="34"/>
+      <c r="D40" s="34"/>
+    </row>
+    <row r="41" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="36" t="s">
         <v>88</v>
       </c>
-      <c r="B36" s="15" t="s">
+      <c r="B41" s="37"/>
+      <c r="C41" s="37"/>
+      <c r="D41" s="37"/>
+    </row>
+    <row r="42" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B42" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C42" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D42" s="10" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A43" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="C36" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D36" s="2">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A37" s="14" t="s">
+      <c r="B43" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="B37" s="15" t="s">
+      <c r="C43" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D43" s="1">
+        <v>1.65</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A44" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="C37" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D37" s="2">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A38" s="39" t="s">
-        <v>125</v>
-      </c>
-      <c r="B38" s="39" t="s">
-        <v>126</v>
-      </c>
-      <c r="C38" s="45" t="s">
-        <v>10</v>
-      </c>
-      <c r="D38" s="46">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A39" s="14" t="s">
-        <v>127</v>
-      </c>
-      <c r="B39" s="14" t="s">
-        <v>129</v>
-      </c>
-      <c r="C39" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D39" s="2">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="38" t="s">
-        <v>128</v>
-      </c>
-      <c r="B40" s="38" t="s">
-        <v>130</v>
-      </c>
-      <c r="C40" s="43" t="s">
-        <v>10</v>
-      </c>
-      <c r="D40" s="44">
-        <v>-0.5</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A41" s="34"/>
-      <c r="B41" s="34"/>
-      <c r="C41" s="34"/>
-      <c r="D41" s="34"/>
-    </row>
-    <row r="42" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="36" t="s">
+      <c r="B44" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="B42" s="37"/>
-      <c r="C42" s="37"/>
-      <c r="D42" s="37"/>
-    </row>
-    <row r="43" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B43" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C43" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="D43" s="10" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A44" s="11" t="s">
+      <c r="C44" s="16" t="s">
         <v>93</v>
       </c>
-      <c r="B44" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="C44" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="D44" s="1">
-        <v>1.65</v>
+      <c r="D44" s="2">
+        <v>907.18</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="B45" s="15" t="s">
         <v>95</v>
       </c>
-      <c r="B45" s="15" t="s">
-        <v>96</v>
-      </c>
       <c r="C45" s="16" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D45" s="2">
         <v>907.18</v>
@@ -2160,52 +2208,52 @@
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="B46" s="15" t="s">
+        <v>97</v>
+      </c>
+      <c r="C46" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="B46" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="C46" s="16" t="s">
-        <v>97</v>
-      </c>
       <c r="D46" s="2">
-        <v>907.18</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="B47" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="B47" s="15" t="s">
+      <c r="C47" s="16" t="s">
         <v>101</v>
       </c>
-      <c r="C47" s="16" t="s">
-        <v>102</v>
-      </c>
       <c r="D47" s="2">
-        <v>1027</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="B48" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="B48" s="15" t="s">
-        <v>104</v>
-      </c>
       <c r="C48" s="16" t="s">
-        <v>105</v>
+        <v>10</v>
       </c>
       <c r="D48" s="2">
-        <v>0.4</v>
+        <v>20</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B49" s="15" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C49" s="16" t="s">
         <v>10</v>
@@ -2216,75 +2264,194 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="B50" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="C50" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D50" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="39" t="s">
         <v>108</v>
       </c>
-      <c r="B50" s="15" t="s">
+      <c r="B51" s="40" t="s">
         <v>109</v>
       </c>
-      <c r="C50" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D50" s="2">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="14" t="s">
-        <v>110</v>
-      </c>
-      <c r="B51" s="15" t="s">
-        <v>111</v>
-      </c>
-      <c r="C51" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D51" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="39" t="s">
-        <v>112</v>
-      </c>
-      <c r="B52" s="40" t="s">
-        <v>113</v>
-      </c>
-      <c r="C52" s="41" t="s">
-        <v>10</v>
-      </c>
-      <c r="D52" s="42">
+      <c r="C51" s="41" t="s">
+        <v>10</v>
+      </c>
+      <c r="D51" s="42">
         <v>2</v>
       </c>
     </row>
-    <row r="53" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="18" t="s">
-        <v>124</v>
-      </c>
-      <c r="B53" s="48" t="s">
-        <v>131</v>
-      </c>
-      <c r="C53" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D53" s="4">
+    <row r="52" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="18" t="s">
+        <v>119</v>
+      </c>
+      <c r="B52" s="48" t="s">
+        <v>126</v>
+      </c>
+      <c r="C52" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D52" s="4">
         <v>2</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="37"/>
-      <c r="B54" s="37"/>
-      <c r="C54" s="37"/>
-      <c r="D54" s="37"/>
-    </row>
-    <row r="67" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B67" s="47"/>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" s="37"/>
+      <c r="B53" s="37"/>
+      <c r="C53" s="37"/>
+      <c r="D53" s="37"/>
+    </row>
+    <row r="66" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B66" s="47"/>
     </row>
   </sheetData>
   <sheetProtection formatColumns="0" selectLockedCells="1"/>
   <protectedRanges>
-    <protectedRange sqref="D33:D37 I3:I6 I8 D18:D29 I12:I16 I26:I29 I19:I22 D44:D53 D3:D14 I33" name="Range1_1"/>
+    <protectedRange sqref="D32:D36 I3:I6 I8 D16:D28 I12:I16 I26:I29 I19:I22 D43:D52 I33 D3:D12" name="Range1_1"/>
   </protectedRanges>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF7B9495-7AF2-49CC-975F-069DD3B5C2E2}">
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>153</v>
+      </c>
+      <c r="B3">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B4">
+        <v>16</v>
+      </c>
+      <c r="C4" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>157</v>
+      </c>
+      <c r="B5">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>158</v>
+      </c>
+      <c r="B6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>159</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>160</v>
+      </c>
+      <c r="B8">
+        <f>1.8-1.53</f>
+        <v>0.27</v>
+      </c>
+      <c r="C8" s="50" t="s">
+        <v>161</v>
+      </c>
+      <c r="D8" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>153</v>
+      </c>
+      <c r="B11">
+        <f>(B3+$B$8)*0.3048</f>
+        <v>3.130296</v>
+      </c>
+      <c r="C11" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>155</v>
+      </c>
+      <c r="B12">
+        <f t="shared" ref="B12:B13" si="0">(B4+$B$8)*0.3048</f>
+        <v>4.9590959999999997</v>
+      </c>
+      <c r="C12" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>157</v>
+      </c>
+      <c r="B13">
+        <f t="shared" si="0"/>
+        <v>2.8254960000000002</v>
+      </c>
+      <c r="C13" t="s">
+        <v>165</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Integrated CC outputs for RB workflows. Fixed AEP/AEF bugs
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD3679FF-7416-4848-B4B2-0669E6BBA02F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6727A132-42B0-413D-B539-665E52729C87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
   <sheets>
-    <sheet name="Full_Inputs" sheetId="1" r:id="rId1"/>
+    <sheet name="James_Island_Midbay" sheetId="1" r:id="rId1"/>
     <sheet name="NAE_Structure" sheetId="2" r:id="rId2"/>
+    <sheet name="NAE_Structure_Inputs" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="493" uniqueCount="172">
   <si>
     <t>StormSim Project General Inputs</t>
   </si>
@@ -150,9 +151,6 @@
     <t>Percentiles to compute CLs (max 4, 50 is already being calculated)</t>
   </si>
   <si>
-    <t>[2 16 84 98]</t>
-  </si>
-  <si>
     <t>csr_apply_structure_repair</t>
   </si>
   <si>
@@ -486,9 +484,6 @@
     <t>StormSim_Library\CHS\Bias_Correction_Files\NACCS_Comb_BiasUncertainty_perVG_rta.mat</t>
   </si>
   <si>
-    <t>C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\CO-OPS_88638660_NAVD88_m_Tidal_Pred_1_year.csv</t>
-  </si>
-  <si>
     <t>NAVD</t>
   </si>
   <si>
@@ -544,6 +539,21 @@
   </si>
   <si>
     <t>CHS savepoint depth (Will be used if not found in h5)</t>
+  </si>
+  <si>
+    <t>[16 84]</t>
+  </si>
+  <si>
+    <t>C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\CO-OPS_8571421_Bishops_Head_Pred_tide_MSL_m.csv</t>
+  </si>
+  <si>
+    <t>Midbay_CHS_Data.zip</t>
+  </si>
+  <si>
+    <t>Use AEP or AEF for hazard curves (1 - AEP, 0-AEF)</t>
+  </si>
+  <si>
+    <t>pros_use_aep</t>
   </si>
 </sst>
 </file>
@@ -1305,7 +1315,7 @@
       <c r="C1" s="6"/>
       <c r="D1" s="6"/>
       <c r="F1" s="32" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G1" s="33"/>
       <c r="H1" s="33"/>
@@ -1351,13 +1361,13 @@
         <v>11</v>
       </c>
       <c r="F3" s="49" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G3" s="49" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H3" s="13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I3" s="13">
         <v>0.33979999999999999</v>
@@ -1377,13 +1387,13 @@
         <v>16</v>
       </c>
       <c r="F4" s="49" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G4" s="49" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H4" s="13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I4" s="13">
         <v>0.38219999999999998</v>
@@ -1403,13 +1413,13 @@
         <v>1</v>
       </c>
       <c r="F5" s="49" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G5" s="49" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I5" s="13">
         <v>0.3</v>
@@ -1426,16 +1436,16 @@
         <v>10</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F6" s="49" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G6" s="49" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H6" s="13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I6" s="13">
         <v>0.3</v>
@@ -1452,13 +1462,13 @@
         <v>10</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G7" s="15" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="H7" s="16" t="s">
         <v>10</v>
@@ -1481,13 +1491,13 @@
         <v>0</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H8" s="19" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="I8" s="3">
         <v>0</v>
@@ -1495,16 +1505,16 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="B9" s="15" t="s">
         <v>146</v>
       </c>
-      <c r="B9" s="15" t="s">
-        <v>147</v>
-      </c>
       <c r="C9" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>149</v>
+        <v>168</v>
       </c>
       <c r="F9" s="33"/>
       <c r="G9" s="33"/>
@@ -1513,10 +1523,10 @@
     </row>
     <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C10" s="16" t="s">
         <v>10</v>
@@ -1525,7 +1535,7 @@
         <v>1</v>
       </c>
       <c r="F10" s="26" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G10" s="27"/>
       <c r="H10" s="27"/>
@@ -1533,10 +1543,10 @@
     </row>
     <row r="11" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="14" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C11" s="16" t="s">
         <v>10</v>
@@ -1568,16 +1578,16 @@
         <v>10</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>37</v>
+        <v>167</v>
       </c>
       <c r="F12" s="30" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G12" s="15" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H12" s="16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I12" s="2">
         <v>0.5</v>
@@ -1589,13 +1599,13 @@
       <c r="C13" s="23"/>
       <c r="D13" s="23"/>
       <c r="F13" s="30" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G13" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="H13" s="31" t="s">
         <v>66</v>
-      </c>
-      <c r="H13" s="31" t="s">
-        <v>67</v>
       </c>
       <c r="I13" s="2">
         <v>0.43</v>
@@ -1603,19 +1613,19 @@
     </row>
     <row r="14" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="24" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B14" s="25"/>
       <c r="C14" s="25"/>
       <c r="D14" s="25"/>
       <c r="F14" s="14" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G14" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="H14" s="16" t="s">
         <v>59</v>
-      </c>
-      <c r="H14" s="16" t="s">
-        <v>60</v>
       </c>
       <c r="I14" s="2">
         <v>0.78</v>
@@ -1635,13 +1645,13 @@
         <v>6</v>
       </c>
       <c r="F15" s="17" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G15" s="18" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H15" s="19" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I15" s="3">
         <v>0.13</v>
@@ -1649,10 +1659,10 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="B16" s="15" t="s">
         <v>111</v>
-      </c>
-      <c r="B16" s="15" t="s">
-        <v>112</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>10</v>
@@ -1667,13 +1677,13 @@
     </row>
     <row r="17" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B17" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="B17" s="12" t="s">
+      <c r="C17" s="28" t="s">
         <v>47</v>
-      </c>
-      <c r="C17" s="28" t="s">
-        <v>48</v>
       </c>
       <c r="D17" s="1">
         <v>1</v>
@@ -1691,13 +1701,13 @@
     </row>
     <row r="18" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C18" s="28" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="D18" s="1">
         <v>5</v>
@@ -1717,16 +1727,16 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C19" s="28" t="s">
         <v>10</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F19" s="11" t="s">
         <v>12</v>
@@ -1743,16 +1753,16 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="B20" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="B20" s="15" t="s">
-        <v>51</v>
-      </c>
       <c r="C20" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="F20" s="14" t="s">
         <v>17</v>
@@ -1769,10 +1779,10 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="B21" s="15" t="s">
         <v>54</v>
-      </c>
-      <c r="B21" s="15" t="s">
-        <v>55</v>
       </c>
       <c r="C21" s="16" t="s">
         <v>10</v>
@@ -1793,10 +1803,10 @@
     </row>
     <row r="22" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="B22" s="15" t="s">
         <v>57</v>
-      </c>
-      <c r="B22" s="15" t="s">
-        <v>58</v>
       </c>
       <c r="C22" s="16" t="s">
         <v>10</v>
@@ -1817,10 +1827,10 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="B23" s="15" t="s">
         <v>61</v>
-      </c>
-      <c r="B23" s="15" t="s">
-        <v>62</v>
       </c>
       <c r="C23" s="16" t="s">
         <v>10</v>
@@ -1833,10 +1843,10 @@
     </row>
     <row r="24" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="14" t="s">
+        <v>63</v>
+      </c>
+      <c r="B24" s="15" t="s">
         <v>64</v>
-      </c>
-      <c r="B24" s="15" t="s">
-        <v>65</v>
       </c>
       <c r="C24" s="16" t="s">
         <v>10</v>
@@ -1851,10 +1861,10 @@
     </row>
     <row r="25" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="B25" s="15" t="s">
         <v>68</v>
-      </c>
-      <c r="B25" s="15" t="s">
-        <v>69</v>
       </c>
       <c r="C25" s="16" t="s">
         <v>10</v>
@@ -1875,10 +1885,10 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="B26" s="15" t="s">
         <v>70</v>
-      </c>
-      <c r="B26" s="15" t="s">
-        <v>71</v>
       </c>
       <c r="C26" s="16" t="s">
         <v>10</v>
@@ -1899,20 +1909,20 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="B27" s="15" t="s">
         <v>72</v>
-      </c>
-      <c r="B27" s="15" t="s">
-        <v>73</v>
       </c>
       <c r="C27" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D27" s="2"/>
       <c r="F27" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="G27" s="15" t="s">
         <v>38</v>
-      </c>
-      <c r="G27" s="15" t="s">
-        <v>39</v>
       </c>
       <c r="H27" s="16" t="s">
         <v>10</v>
@@ -1923,23 +1933,23 @@
     </row>
     <row r="28" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="B28" s="18" t="s">
         <v>74</v>
-      </c>
-      <c r="B28" s="18" t="s">
-        <v>75</v>
       </c>
       <c r="C28" s="19" t="s">
         <v>10</v>
       </c>
       <c r="D28" s="3"/>
       <c r="F28" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="G28" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="G28" s="15" t="s">
+      <c r="H28" s="16" t="s">
         <v>41</v>
-      </c>
-      <c r="H28" s="16" t="s">
-        <v>42</v>
       </c>
       <c r="I28" s="2">
         <v>0</v>
@@ -1951,13 +1961,13 @@
       <c r="C29" s="25"/>
       <c r="D29" s="25"/>
       <c r="F29" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="G29" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="G29" s="18" t="s">
-        <v>45</v>
-      </c>
       <c r="H29" s="19" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I29" s="3">
         <v>1</v>
@@ -1965,7 +1975,7 @@
     </row>
     <row r="30" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="34" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B30" s="35"/>
       <c r="C30" s="35"/>
@@ -1986,10 +1996,10 @@
         <v>5</v>
       </c>
       <c r="D31" s="10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F31" s="26" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G31" s="27"/>
       <c r="H31" s="27"/>
@@ -1997,17 +2007,16 @@
     </row>
     <row r="32" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C32" s="13" t="s">
         <v>10</v>
       </c>
       <c r="D32" s="1">
-        <f>NAE_Structure!B12</f>
-        <v>4.9590959999999997</v>
+        <v>1.2320122</v>
       </c>
       <c r="F32" s="9" t="s">
         <v>3</v>
@@ -2024,23 +2033,22 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B33" s="15" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C33" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D33" s="2">
-        <f>NAE_Structure!B11</f>
-        <v>3.130296</v>
+        <v>1.5243902</v>
       </c>
       <c r="F33" s="29" t="s">
+        <v>51</v>
+      </c>
+      <c r="G33" s="12" t="s">
         <v>52</v>
-      </c>
-      <c r="G33" s="12" t="s">
-        <v>53</v>
       </c>
       <c r="H33" s="13" t="s">
         <v>10</v>
@@ -2049,57 +2057,66 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="B34" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="B34" s="15" t="s">
-        <v>83</v>
-      </c>
       <c r="C34" s="16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D34" s="2">
-        <f>NAE_Structure!B13*-1</f>
-        <v>-2.8254960000000002</v>
+        <v>-1.5969511999999999</v>
+      </c>
+      <c r="F34" s="17" t="s">
+        <v>171</v>
+      </c>
+      <c r="G34" s="18" t="s">
+        <v>170</v>
+      </c>
+      <c r="H34" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="I34" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="B35" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="B35" s="15" t="s">
-        <v>85</v>
-      </c>
       <c r="C35" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D35" s="2">
-        <f>NAE_Structure!B6</f>
-        <v>3</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="B36" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="B36" s="15" t="s">
-        <v>87</v>
-      </c>
       <c r="C36" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D36" s="2">
-        <f>NAE_Structure!B6</f>
-        <v>3</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="39" t="s">
+        <v>119</v>
+      </c>
+      <c r="B37" s="39" t="s">
         <v>120</v>
-      </c>
-      <c r="B37" s="39" t="s">
-        <v>121</v>
       </c>
       <c r="C37" s="45" t="s">
         <v>10</v>
@@ -2110,10 +2127,10 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C38" s="16" t="s">
         <v>10</v>
@@ -2124,10 +2141,10 @@
     </row>
     <row r="39" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="38" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B39" s="38" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C39" s="43" t="s">
         <v>10</v>
@@ -2144,7 +2161,7 @@
     </row>
     <row r="41" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="36" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B41" s="37"/>
       <c r="C41" s="37"/>
@@ -2161,15 +2178,15 @@
         <v>5</v>
       </c>
       <c r="D42" s="10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="B43" s="12" t="s">
         <v>89</v>
-      </c>
-      <c r="B43" s="12" t="s">
-        <v>90</v>
       </c>
       <c r="C43" s="13" t="s">
         <v>10</v>
@@ -2180,41 +2197,41 @@
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="B44" s="15" t="s">
         <v>91</v>
       </c>
-      <c r="B44" s="15" t="s">
+      <c r="C44" s="16" t="s">
         <v>92</v>
       </c>
-      <c r="C44" s="16" t="s">
-        <v>93</v>
-      </c>
       <c r="D44" s="2">
-        <v>907.18</v>
+        <v>500</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="B45" s="15" t="s">
         <v>94</v>
       </c>
-      <c r="B45" s="15" t="s">
-        <v>95</v>
-      </c>
       <c r="C45" s="16" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D45" s="2">
-        <v>907.18</v>
+        <v>500</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="B46" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="B46" s="15" t="s">
+      <c r="C46" s="16" t="s">
         <v>97</v>
-      </c>
-      <c r="C46" s="16" t="s">
-        <v>98</v>
       </c>
       <c r="D46" s="2">
         <v>1027</v>
@@ -2222,13 +2239,13 @@
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="B47" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="B47" s="15" t="s">
+      <c r="C47" s="16" t="s">
         <v>100</v>
-      </c>
-      <c r="C47" s="16" t="s">
-        <v>101</v>
       </c>
       <c r="D47" s="2">
         <v>0.4</v>
@@ -2236,10 +2253,10 @@
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="B48" s="15" t="s">
         <v>102</v>
-      </c>
-      <c r="B48" s="15" t="s">
-        <v>103</v>
       </c>
       <c r="C48" s="16" t="s">
         <v>10</v>
@@ -2250,10 +2267,10 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="B49" s="15" t="s">
         <v>104</v>
-      </c>
-      <c r="B49" s="15" t="s">
-        <v>105</v>
       </c>
       <c r="C49" s="16" t="s">
         <v>10</v>
@@ -2264,24 +2281,24 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="B50" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="B50" s="15" t="s">
-        <v>107</v>
-      </c>
       <c r="C50" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D50" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="39" t="s">
+        <v>107</v>
+      </c>
+      <c r="B51" s="40" t="s">
         <v>108</v>
-      </c>
-      <c r="B51" s="40" t="s">
-        <v>109</v>
       </c>
       <c r="C51" s="41" t="s">
         <v>10</v>
@@ -2292,10 +2309,10 @@
     </row>
     <row r="52" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="18" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B52" s="48" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C52" s="19" t="s">
         <v>10</v>
@@ -2316,7 +2333,10 @@
   </sheetData>
   <sheetProtection formatColumns="0" selectLockedCells="1"/>
   <protectedRanges>
-    <protectedRange sqref="D32:D36 I3:I6 I8 D16:D28 I12:I16 I26:I29 I19:I22 D43:D52 I33 D3:D12" name="Range1_1"/>
+    <protectedRange sqref="I3:I6 I8 D16:D28 I12:I16 I26:I29 I19:I22 I33 D3:D11" name="Range1_1"/>
+    <protectedRange sqref="D12" name="Range1_1_1"/>
+    <protectedRange sqref="D32:D36" name="Range1_1_3"/>
+    <protectedRange sqref="D43:D52" name="Range1_1_4"/>
   </protectedRanges>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -2334,12 +2354,12 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -2347,40 +2367,40 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B3">
         <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B4">
         <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B5">
         <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B6">
         <v>3</v>
@@ -2388,7 +2408,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B7">
         <v>1</v>
@@ -2396,62 +2416,1103 @@
     </row>
     <row r="8" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B8">
         <f>1.8-1.53</f>
         <v>0.27</v>
       </c>
       <c r="C8" s="50" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D8" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B11">
         <f>(B3+$B$8)*0.3048</f>
         <v>3.130296</v>
       </c>
       <c r="C11" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B12">
         <f t="shared" ref="B12:B13" si="0">(B4+$B$8)*0.3048</f>
         <v>4.9590959999999997</v>
       </c>
       <c r="C12" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B13">
         <f t="shared" si="0"/>
         <v>2.8254960000000002</v>
       </c>
       <c r="C13" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9768969-90B5-4E8F-92CE-56AC3208C5A3}">
+  <dimension ref="A1:I66"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="79" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="92.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="171.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="28.42578125" customWidth="1"/>
+    <col min="7" max="7" width="50" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="46.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="F1" s="32" t="s">
+        <v>75</v>
+      </c>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
+    </row>
+    <row r="2" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="I2" s="10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="49" t="s">
+        <v>133</v>
+      </c>
+      <c r="G3" s="49" t="s">
+        <v>126</v>
+      </c>
+      <c r="H3" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="I3" s="13">
+        <v>0.33979999999999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" s="49" t="s">
+        <v>134</v>
+      </c>
+      <c r="G4" s="49" t="s">
+        <v>127</v>
+      </c>
+      <c r="H4" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="I4" s="13">
+        <v>0.38219999999999998</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="2">
+        <v>1</v>
+      </c>
+      <c r="F5" s="49" t="s">
+        <v>136</v>
+      </c>
+      <c r="G5" s="49" t="s">
+        <v>128</v>
+      </c>
+      <c r="H5" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="I5" s="13">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="F6" s="49" t="s">
+        <v>135</v>
+      </c>
+      <c r="G6" s="49" t="s">
+        <v>129</v>
+      </c>
+      <c r="H6" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="I6" s="13">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="F7" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="G7" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="H7" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I7" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" s="2">
+        <v>0</v>
+      </c>
+      <c r="F8" s="17" t="s">
+        <v>132</v>
+      </c>
+      <c r="G8" s="18" t="s">
+        <v>130</v>
+      </c>
+      <c r="H8" s="19" t="s">
+        <v>76</v>
+      </c>
+      <c r="I8" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="B9" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="F9" s="33"/>
+      <c r="G9" s="33"/>
+      <c r="H9" s="33"/>
+      <c r="I9" s="33"/>
+    </row>
+    <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>113</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="2">
+        <v>1</v>
+      </c>
+      <c r="F10" s="26" t="s">
+        <v>138</v>
+      </c>
+      <c r="G10" s="27"/>
+      <c r="H10" s="27"/>
+      <c r="I10" s="27"/>
+    </row>
+    <row r="11" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" s="2">
+        <v>1</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="H11" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="I11" s="10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="F12" s="30" t="s">
+        <v>140</v>
+      </c>
+      <c r="G12" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="H12" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="I12" s="2">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="6"/>
+      <c r="B13" s="22"/>
+      <c r="C13" s="23"/>
+      <c r="D13" s="23"/>
+      <c r="F13" s="30" t="s">
+        <v>141</v>
+      </c>
+      <c r="G13" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="H13" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="I13" s="2">
+        <v>0.43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="B14" s="25"/>
+      <c r="C14" s="25"/>
+      <c r="D14" s="25"/>
+      <c r="F14" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="G14" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="H14" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="I14" s="2">
+        <v>0.78</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="F15" s="17" t="s">
+        <v>117</v>
+      </c>
+      <c r="G15" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="H15" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="I15" s="3">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="B16" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" s="2">
+        <v>1</v>
+      </c>
+      <c r="F16" s="27"/>
+      <c r="G16" s="27"/>
+      <c r="H16" s="27"/>
+      <c r="I16" s="27"/>
+    </row>
+    <row r="17" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="C17" s="28" t="s">
+        <v>47</v>
+      </c>
+      <c r="D17" s="1">
+        <v>1</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="I17" s="8" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>166</v>
+      </c>
+      <c r="C18" s="28" t="s">
+        <v>162</v>
+      </c>
+      <c r="D18" s="1">
+        <v>5</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="G18" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="H18" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="I18" s="10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="C19" s="28" t="s">
+        <v>10</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G19" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="H19" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="I19" s="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="B20" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="C20" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="F20" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="G20" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="H20" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="I20" s="2">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="B21" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="C21" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21" s="2"/>
+      <c r="F21" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="G21" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="H21" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I21" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="B22" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D22" s="2"/>
+      <c r="F22" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="G22" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="H22" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="I22" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="B23" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="C23" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D23" s="2"/>
+      <c r="F23" s="8"/>
+      <c r="G23" s="8"/>
+      <c r="H23" s="8"/>
+      <c r="I23" s="8"/>
+    </row>
+    <row r="24" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="14" t="s">
+        <v>63</v>
+      </c>
+      <c r="B24" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="C24" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D24" s="2"/>
+      <c r="F24" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="G24" s="21"/>
+      <c r="H24" s="21"/>
+      <c r="I24" s="21"/>
+    </row>
+    <row r="25" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="B25" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="C25" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D25" s="2"/>
+      <c r="F25" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="G25" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="H25" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="I25" s="10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="B26" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="C26" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D26" s="2"/>
+      <c r="F26" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="G26" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="H26" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="I26" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="B27" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="C27" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D27" s="2"/>
+      <c r="F27" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="G27" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="H27" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I27" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="B28" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="C28" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D28" s="3"/>
+      <c r="F28" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="G28" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="H28" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="I28" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="25"/>
+      <c r="B29" s="25"/>
+      <c r="C29" s="25"/>
+      <c r="D29" s="25"/>
+      <c r="F29" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="G29" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="H29" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="I29" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="34" t="s">
+        <v>77</v>
+      </c>
+      <c r="B30" s="35"/>
+      <c r="C30" s="35"/>
+      <c r="D30" s="35"/>
+      <c r="F30" s="21"/>
+      <c r="G30" s="21"/>
+      <c r="H30" s="21"/>
+      <c r="I30" s="21"/>
+    </row>
+    <row r="31" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D31" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="F31" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="G31" s="27"/>
+      <c r="H31" s="27"/>
+      <c r="I31" s="27"/>
+    </row>
+    <row r="32" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="B32" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="C32" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D32" s="1">
+        <f>NAE_Structure!B12</f>
+        <v>4.9590959999999997</v>
+      </c>
+      <c r="F32" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="G32" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="H32" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="I32" s="10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="B33" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="C33" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D33" s="2">
+        <f>NAE_Structure!B11</f>
+        <v>3.130296</v>
+      </c>
+      <c r="F33" s="29" t="s">
+        <v>51</v>
+      </c>
+      <c r="G33" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="H33" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="I33" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="B34" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="C34" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="D34" s="2">
+        <f>NAE_Structure!B13*-1</f>
+        <v>-2.8254960000000002</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="B35" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="C35" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D35" s="2">
+        <f>NAE_Structure!B6</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="B36" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="C36" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D36" s="2">
+        <f>NAE_Structure!B6</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37" s="39" t="s">
+        <v>119</v>
+      </c>
+      <c r="B37" s="39" t="s">
+        <v>120</v>
+      </c>
+      <c r="C37" s="45" t="s">
+        <v>10</v>
+      </c>
+      <c r="D37" s="46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A38" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="B38" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="C38" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D38" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="38" t="s">
+        <v>122</v>
+      </c>
+      <c r="B39" s="38" t="s">
+        <v>124</v>
+      </c>
+      <c r="C39" s="43" t="s">
+        <v>10</v>
+      </c>
+      <c r="D39" s="44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A40" s="34"/>
+      <c r="B40" s="34"/>
+      <c r="C40" s="34"/>
+      <c r="D40" s="34"/>
+    </row>
+    <row r="41" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="36" t="s">
+        <v>87</v>
+      </c>
+      <c r="B41" s="37"/>
+      <c r="C41" s="37"/>
+      <c r="D41" s="37"/>
+    </row>
+    <row r="42" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B42" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C42" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D42" s="10" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A43" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="B43" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="C43" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D43" s="1">
+        <v>1.65</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A44" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="B44" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="C44" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="D44" s="2">
+        <v>907.18</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A45" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="B45" s="15" t="s">
+        <v>94</v>
+      </c>
+      <c r="C45" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="D45" s="2">
+        <v>907.18</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A46" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="B46" s="15" t="s">
+        <v>96</v>
+      </c>
+      <c r="C46" s="16" t="s">
+        <v>97</v>
+      </c>
+      <c r="D46" s="2">
+        <v>1027</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A47" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="B47" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="C47" s="16" t="s">
+        <v>100</v>
+      </c>
+      <c r="D47" s="2">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A48" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="B48" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="C48" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D48" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="B49" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="C49" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D49" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="B50" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="C50" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D50" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="39" t="s">
+        <v>107</v>
+      </c>
+      <c r="B51" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="C51" s="41" t="s">
+        <v>10</v>
+      </c>
+      <c r="D51" s="42">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="18" t="s">
+        <v>118</v>
+      </c>
+      <c r="B52" s="48" t="s">
+        <v>125</v>
+      </c>
+      <c r="C52" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D52" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" s="37"/>
+      <c r="B53" s="37"/>
+      <c r="C53" s="37"/>
+      <c r="D53" s="37"/>
+    </row>
+    <row r="66" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B66" s="47"/>
+    </row>
+  </sheetData>
+  <sheetProtection formatColumns="0" selectLockedCells="1"/>
+  <protectedRanges>
+    <protectedRange sqref="D32:D36 I3:I6 I8 D16:D28 I12:I16 I26:I29 I19:I22 D43:D52 I33 D3:D11" name="Range1_1"/>
+    <protectedRange sqref="D12" name="Range1_1_1"/>
+  </protectedRanges>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Removing y2 from hazard curve combiner.
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6727A132-42B0-413D-B539-665E52729C87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AA67EAC-1521-4957-9AA5-EFE4F1656DC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
   <sheets>
-    <sheet name="James_Island_Midbay" sheetId="1" r:id="rId1"/>
-    <sheet name="NAE_Structure" sheetId="2" r:id="rId2"/>
-    <sheet name="NAE_Structure_Inputs" sheetId="3" r:id="rId3"/>
+    <sheet name="NAE_Structure_Inputs" sheetId="3" r:id="rId1"/>
+    <sheet name="James_Island_Midbay" sheetId="1" r:id="rId2"/>
+    <sheet name="NAE_Structure" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="493" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="174">
   <si>
     <t>StormSim Project General Inputs</t>
   </si>
@@ -554,6 +554,12 @@
   </si>
   <si>
     <t>pros_use_aep</t>
+  </si>
+  <si>
+    <t>NAE_Structure</t>
+  </si>
+  <si>
+    <t>C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\CO-OPS_8638660_MSL_m_Tidal_Pred_1_year.csv</t>
   </si>
 </sst>
 </file>
@@ -1294,6 +1300,1059 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9768969-90B5-4E8F-92CE-56AC3208C5A3}">
+  <dimension ref="A1:I66"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="79" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="92.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="171.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="28.42578125" customWidth="1"/>
+    <col min="7" max="7" width="50" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="46.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="F1" s="32" t="s">
+        <v>75</v>
+      </c>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
+    </row>
+    <row r="2" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="I2" s="10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="F3" s="49" t="s">
+        <v>133</v>
+      </c>
+      <c r="G3" s="49" t="s">
+        <v>126</v>
+      </c>
+      <c r="H3" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="I3" s="13">
+        <v>0.33979999999999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" s="49" t="s">
+        <v>134</v>
+      </c>
+      <c r="G4" s="49" t="s">
+        <v>127</v>
+      </c>
+      <c r="H4" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="I4" s="13">
+        <v>0.38219999999999998</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="2">
+        <v>1</v>
+      </c>
+      <c r="F5" s="49" t="s">
+        <v>136</v>
+      </c>
+      <c r="G5" s="49" t="s">
+        <v>128</v>
+      </c>
+      <c r="H5" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="I5" s="13">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="F6" s="49" t="s">
+        <v>135</v>
+      </c>
+      <c r="G6" s="49" t="s">
+        <v>129</v>
+      </c>
+      <c r="H6" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="I6" s="13">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="F7" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="G7" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="H7" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I7" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" s="2">
+        <v>0</v>
+      </c>
+      <c r="F8" s="17" t="s">
+        <v>132</v>
+      </c>
+      <c r="G8" s="18" t="s">
+        <v>130</v>
+      </c>
+      <c r="H8" s="19" t="s">
+        <v>76</v>
+      </c>
+      <c r="I8" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="B9" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="F9" s="33"/>
+      <c r="G9" s="33"/>
+      <c r="H9" s="33"/>
+      <c r="I9" s="33"/>
+    </row>
+    <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>113</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="2">
+        <v>1</v>
+      </c>
+      <c r="F10" s="26" t="s">
+        <v>138</v>
+      </c>
+      <c r="G10" s="27"/>
+      <c r="H10" s="27"/>
+      <c r="I10" s="27"/>
+    </row>
+    <row r="11" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" s="2">
+        <v>1</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="H11" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="I11" s="10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="F12" s="30" t="s">
+        <v>140</v>
+      </c>
+      <c r="G12" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="H12" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="I12" s="2">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="6"/>
+      <c r="B13" s="22"/>
+      <c r="C13" s="23"/>
+      <c r="D13" s="23"/>
+      <c r="F13" s="30" t="s">
+        <v>141</v>
+      </c>
+      <c r="G13" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="H13" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="I13" s="2">
+        <v>0.43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="B14" s="25"/>
+      <c r="C14" s="25"/>
+      <c r="D14" s="25"/>
+      <c r="F14" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="G14" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="H14" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="I14" s="2">
+        <v>0.78</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="F15" s="17" t="s">
+        <v>117</v>
+      </c>
+      <c r="G15" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="H15" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="I15" s="3">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="B16" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" s="2">
+        <v>1</v>
+      </c>
+      <c r="F16" s="27"/>
+      <c r="G16" s="27"/>
+      <c r="H16" s="27"/>
+      <c r="I16" s="27"/>
+    </row>
+    <row r="17" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="C17" s="28" t="s">
+        <v>47</v>
+      </c>
+      <c r="D17" s="1">
+        <v>1</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="I17" s="8" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>166</v>
+      </c>
+      <c r="C18" s="28" t="s">
+        <v>162</v>
+      </c>
+      <c r="D18" s="1">
+        <v>5</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="G18" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="H18" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="I18" s="10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="C19" s="28" t="s">
+        <v>10</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G19" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="H19" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="I19" s="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="B20" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="C20" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="F20" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="G20" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="H20" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="I20" s="2">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="B21" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="C21" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21" s="2"/>
+      <c r="F21" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="G21" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="H21" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I21" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="B22" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D22" s="2"/>
+      <c r="F22" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="G22" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="H22" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="I22" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="B23" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="C23" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D23" s="2"/>
+      <c r="F23" s="8"/>
+      <c r="G23" s="8"/>
+      <c r="H23" s="8"/>
+      <c r="I23" s="8"/>
+    </row>
+    <row r="24" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="14" t="s">
+        <v>63</v>
+      </c>
+      <c r="B24" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="C24" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D24" s="2"/>
+      <c r="F24" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="G24" s="21"/>
+      <c r="H24" s="21"/>
+      <c r="I24" s="21"/>
+    </row>
+    <row r="25" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="B25" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="C25" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D25" s="2"/>
+      <c r="F25" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="G25" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="H25" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="I25" s="10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="B26" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="C26" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D26" s="2"/>
+      <c r="F26" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="G26" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="H26" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="I26" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="B27" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="C27" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D27" s="2"/>
+      <c r="F27" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="G27" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="H27" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I27" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="B28" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="C28" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D28" s="3"/>
+      <c r="F28" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="G28" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="H28" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="I28" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="25"/>
+      <c r="B29" s="25"/>
+      <c r="C29" s="25"/>
+      <c r="D29" s="25"/>
+      <c r="F29" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="G29" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="H29" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="I29" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="34" t="s">
+        <v>77</v>
+      </c>
+      <c r="B30" s="35"/>
+      <c r="C30" s="35"/>
+      <c r="D30" s="35"/>
+      <c r="F30" s="21"/>
+      <c r="G30" s="21"/>
+      <c r="H30" s="21"/>
+      <c r="I30" s="21"/>
+    </row>
+    <row r="31" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D31" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="F31" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="G31" s="27"/>
+      <c r="H31" s="27"/>
+      <c r="I31" s="27"/>
+    </row>
+    <row r="32" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="B32" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="C32" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D32" s="1">
+        <f>NAE_Structure!B12</f>
+        <v>4.9590959999999997</v>
+      </c>
+      <c r="F32" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="G32" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="H32" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="I32" s="10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="B33" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="C33" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D33" s="2">
+        <f>NAE_Structure!B11</f>
+        <v>3.130296</v>
+      </c>
+      <c r="F33" s="29" t="s">
+        <v>51</v>
+      </c>
+      <c r="G33" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="H33" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="I33" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="B34" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="C34" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="D34" s="2">
+        <f>NAE_Structure!B13*-1</f>
+        <v>-2.8254960000000002</v>
+      </c>
+      <c r="F34" s="17" t="s">
+        <v>171</v>
+      </c>
+      <c r="G34" s="18" t="s">
+        <v>170</v>
+      </c>
+      <c r="H34" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="I34" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="B35" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="C35" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D35" s="2">
+        <f>NAE_Structure!B6</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="B36" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="C36" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D36" s="2">
+        <f>NAE_Structure!B6</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37" s="39" t="s">
+        <v>119</v>
+      </c>
+      <c r="B37" s="39" t="s">
+        <v>120</v>
+      </c>
+      <c r="C37" s="45" t="s">
+        <v>10</v>
+      </c>
+      <c r="D37" s="46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A38" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="B38" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="C38" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D38" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="38" t="s">
+        <v>122</v>
+      </c>
+      <c r="B39" s="38" t="s">
+        <v>124</v>
+      </c>
+      <c r="C39" s="43" t="s">
+        <v>10</v>
+      </c>
+      <c r="D39" s="44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A40" s="34"/>
+      <c r="B40" s="34"/>
+      <c r="C40" s="34"/>
+      <c r="D40" s="34"/>
+    </row>
+    <row r="41" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="36" t="s">
+        <v>87</v>
+      </c>
+      <c r="B41" s="37"/>
+      <c r="C41" s="37"/>
+      <c r="D41" s="37"/>
+    </row>
+    <row r="42" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B42" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C42" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D42" s="10" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A43" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="B43" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="C43" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D43" s="1">
+        <v>1.65</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A44" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="B44" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="C44" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="D44" s="2">
+        <v>907.18</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A45" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="B45" s="15" t="s">
+        <v>94</v>
+      </c>
+      <c r="C45" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="D45" s="2">
+        <v>907.18</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A46" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="B46" s="15" t="s">
+        <v>96</v>
+      </c>
+      <c r="C46" s="16" t="s">
+        <v>97</v>
+      </c>
+      <c r="D46" s="2">
+        <v>1027</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A47" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="B47" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="C47" s="16" t="s">
+        <v>100</v>
+      </c>
+      <c r="D47" s="2">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A48" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="B48" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="C48" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D48" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="B49" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="C49" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D49" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="B50" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="C50" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D50" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="39" t="s">
+        <v>107</v>
+      </c>
+      <c r="B51" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="C51" s="41" t="s">
+        <v>10</v>
+      </c>
+      <c r="D51" s="42">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="18" t="s">
+        <v>118</v>
+      </c>
+      <c r="B52" s="48" t="s">
+        <v>125</v>
+      </c>
+      <c r="C52" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D52" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" s="37"/>
+      <c r="B53" s="37"/>
+      <c r="C53" s="37"/>
+      <c r="D53" s="37"/>
+    </row>
+    <row r="66" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B66" s="47"/>
+    </row>
+  </sheetData>
+  <sheetProtection formatColumns="0" selectLockedCells="1"/>
+  <protectedRanges>
+    <protectedRange sqref="D32:D36 I3:I6 I8 D16:D28 I12:I16 I26:I29 I19:I22 D43:D52 I33 D3:D11" name="Range1_1"/>
+    <protectedRange sqref="D12" name="Range1_1_1"/>
+  </protectedRanges>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51D29750-2AFD-4BF7-A911-1DC4ADC0FD7A}">
   <dimension ref="A1:I66"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2343,7 +3402,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF7B9495-7AF2-49CC-975F-069DD3B5C2E2}">
   <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2474,1045 +3533,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9768969-90B5-4E8F-92CE-56AC3208C5A3}">
-  <dimension ref="A1:I66"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="79" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="92.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="171.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="28.42578125" customWidth="1"/>
-    <col min="7" max="7" width="50" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="46.140625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="F1" s="32" t="s">
-        <v>75</v>
-      </c>
-      <c r="G1" s="33"/>
-      <c r="H1" s="33"/>
-      <c r="I1" s="33"/>
-    </row>
-    <row r="2" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="F2" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="G2" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="H2" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="I2" s="10" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="49" t="s">
-        <v>133</v>
-      </c>
-      <c r="G3" s="49" t="s">
-        <v>126</v>
-      </c>
-      <c r="H3" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="I3" s="13">
-        <v>0.33979999999999999</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F4" s="49" t="s">
-        <v>134</v>
-      </c>
-      <c r="G4" s="49" t="s">
-        <v>127</v>
-      </c>
-      <c r="H4" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="I4" s="13">
-        <v>0.38219999999999998</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" s="2">
-        <v>1</v>
-      </c>
-      <c r="F5" s="49" t="s">
-        <v>136</v>
-      </c>
-      <c r="G5" s="49" t="s">
-        <v>128</v>
-      </c>
-      <c r="H5" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="I5" s="13">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="B6" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="F6" s="49" t="s">
-        <v>135</v>
-      </c>
-      <c r="G6" s="49" t="s">
-        <v>129</v>
-      </c>
-      <c r="H6" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="I6" s="13">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="B7" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="C7" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="F7" s="14" t="s">
-        <v>137</v>
-      </c>
-      <c r="G7" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="H7" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="I7" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="B8" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="C8" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D8" s="2">
-        <v>0</v>
-      </c>
-      <c r="F8" s="17" t="s">
-        <v>132</v>
-      </c>
-      <c r="G8" s="18" t="s">
-        <v>130</v>
-      </c>
-      <c r="H8" s="19" t="s">
-        <v>76</v>
-      </c>
-      <c r="I8" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="14" t="s">
-        <v>145</v>
-      </c>
-      <c r="B9" s="15" t="s">
-        <v>146</v>
-      </c>
-      <c r="C9" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="F9" s="33"/>
-      <c r="G9" s="33"/>
-      <c r="H9" s="33"/>
-      <c r="I9" s="33"/>
-    </row>
-    <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="14" t="s">
-        <v>139</v>
-      </c>
-      <c r="B10" s="15" t="s">
-        <v>113</v>
-      </c>
-      <c r="C10" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D10" s="2">
-        <v>1</v>
-      </c>
-      <c r="F10" s="26" t="s">
-        <v>138</v>
-      </c>
-      <c r="G10" s="27"/>
-      <c r="H10" s="27"/>
-      <c r="I10" s="27"/>
-    </row>
-    <row r="11" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="14" t="s">
-        <v>112</v>
-      </c>
-      <c r="B11" s="15" t="s">
-        <v>144</v>
-      </c>
-      <c r="C11" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D11" s="2">
-        <v>1</v>
-      </c>
-      <c r="F11" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="G11" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="H11" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="I11" s="10" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="B12" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="C12" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="F12" s="30" t="s">
-        <v>140</v>
-      </c>
-      <c r="G12" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="H12" s="16" t="s">
-        <v>41</v>
-      </c>
-      <c r="I12" s="2">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="6"/>
-      <c r="B13" s="22"/>
-      <c r="C13" s="23"/>
-      <c r="D13" s="23"/>
-      <c r="F13" s="30" t="s">
-        <v>141</v>
-      </c>
-      <c r="G13" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="H13" s="31" t="s">
-        <v>66</v>
-      </c>
-      <c r="I13" s="2">
-        <v>0.43</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="24" t="s">
-        <v>42</v>
-      </c>
-      <c r="B14" s="25"/>
-      <c r="C14" s="25"/>
-      <c r="D14" s="25"/>
-      <c r="F14" s="14" t="s">
-        <v>116</v>
-      </c>
-      <c r="G14" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="H14" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="I14" s="2">
-        <v>0.78</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B15" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="F15" s="17" t="s">
-        <v>117</v>
-      </c>
-      <c r="G15" s="18" t="s">
-        <v>62</v>
-      </c>
-      <c r="H15" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="I15" s="3">
-        <v>0.13</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="14" t="s">
-        <v>110</v>
-      </c>
-      <c r="B16" s="15" t="s">
-        <v>111</v>
-      </c>
-      <c r="C16" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D16" s="2">
-        <v>1</v>
-      </c>
-      <c r="F16" s="27"/>
-      <c r="G16" s="27"/>
-      <c r="H16" s="27"/>
-      <c r="I16" s="27"/>
-    </row>
-    <row r="17" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="B17" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="C17" s="28" t="s">
-        <v>47</v>
-      </c>
-      <c r="D17" s="1">
-        <v>1</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="G17" s="8"/>
-      <c r="H17" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="I17" s="8" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="11" t="s">
-        <v>165</v>
-      </c>
-      <c r="B18" s="12" t="s">
-        <v>166</v>
-      </c>
-      <c r="C18" s="28" t="s">
-        <v>162</v>
-      </c>
-      <c r="D18" s="1">
-        <v>5</v>
-      </c>
-      <c r="F18" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="G18" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="H18" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="I18" s="10" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="11" t="s">
-        <v>143</v>
-      </c>
-      <c r="B19" s="12" t="s">
-        <v>142</v>
-      </c>
-      <c r="C19" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="F19" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="G19" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="H19" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="I19" s="1">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="B20" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="C20" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="F20" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="G20" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="H20" s="16" t="s">
-        <v>19</v>
-      </c>
-      <c r="I20" s="2">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="B21" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="C21" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D21" s="2"/>
-      <c r="F21" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="G21" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="H21" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="I21" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="B22" s="15" t="s">
-        <v>57</v>
-      </c>
-      <c r="C22" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D22" s="2"/>
-      <c r="F22" s="17" t="s">
-        <v>28</v>
-      </c>
-      <c r="G22" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="H22" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="I22" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="B23" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="C23" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D23" s="2"/>
-      <c r="F23" s="8"/>
-      <c r="G23" s="8"/>
-      <c r="H23" s="8"/>
-      <c r="I23" s="8"/>
-    </row>
-    <row r="24" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="B24" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="C24" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D24" s="2"/>
-      <c r="F24" s="20" t="s">
-        <v>32</v>
-      </c>
-      <c r="G24" s="21"/>
-      <c r="H24" s="21"/>
-      <c r="I24" s="21"/>
-    </row>
-    <row r="25" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="B25" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="C25" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D25" s="2"/>
-      <c r="F25" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="G25" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="H25" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="I25" s="10" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="14" t="s">
-        <v>69</v>
-      </c>
-      <c r="B26" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="C26" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D26" s="2"/>
-      <c r="F26" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="G26" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="H26" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="I26" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="B27" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="C27" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D27" s="2"/>
-      <c r="F27" s="14" t="s">
-        <v>37</v>
-      </c>
-      <c r="G27" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="H27" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="I27" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="17" t="s">
-        <v>73</v>
-      </c>
-      <c r="B28" s="18" t="s">
-        <v>74</v>
-      </c>
-      <c r="C28" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D28" s="3"/>
-      <c r="F28" s="14" t="s">
-        <v>39</v>
-      </c>
-      <c r="G28" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="H28" s="16" t="s">
-        <v>41</v>
-      </c>
-      <c r="I28" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="25"/>
-      <c r="B29" s="25"/>
-      <c r="C29" s="25"/>
-      <c r="D29" s="25"/>
-      <c r="F29" s="17" t="s">
-        <v>43</v>
-      </c>
-      <c r="G29" s="18" t="s">
-        <v>44</v>
-      </c>
-      <c r="H29" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="I29" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="B30" s="35"/>
-      <c r="C30" s="35"/>
-      <c r="D30" s="35"/>
-      <c r="F30" s="21"/>
-      <c r="G30" s="21"/>
-      <c r="H30" s="21"/>
-      <c r="I30" s="21"/>
-    </row>
-    <row r="31" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B31" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C31" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="D31" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="F31" s="26" t="s">
-        <v>48</v>
-      </c>
-      <c r="G31" s="27"/>
-      <c r="H31" s="27"/>
-      <c r="I31" s="27"/>
-    </row>
-    <row r="32" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="B32" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="C32" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="D32" s="1">
-        <f>NAE_Structure!B12</f>
-        <v>4.9590959999999997</v>
-      </c>
-      <c r="F32" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="G32" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="H32" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="I32" s="10" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="B33" s="15" t="s">
-        <v>115</v>
-      </c>
-      <c r="C33" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D33" s="2">
-        <f>NAE_Structure!B11</f>
-        <v>3.130296</v>
-      </c>
-      <c r="F33" s="29" t="s">
-        <v>51</v>
-      </c>
-      <c r="G33" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="H33" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="I33" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" s="14" t="s">
-        <v>81</v>
-      </c>
-      <c r="B34" s="15" t="s">
-        <v>82</v>
-      </c>
-      <c r="C34" s="16" t="s">
-        <v>41</v>
-      </c>
-      <c r="D34" s="2">
-        <f>NAE_Structure!B13*-1</f>
-        <v>-2.8254960000000002</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A35" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="B35" s="15" t="s">
-        <v>84</v>
-      </c>
-      <c r="C35" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D35" s="2">
-        <f>NAE_Structure!B6</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="14" t="s">
-        <v>85</v>
-      </c>
-      <c r="B36" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="C36" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D36" s="2">
-        <f>NAE_Structure!B6</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A37" s="39" t="s">
-        <v>119</v>
-      </c>
-      <c r="B37" s="39" t="s">
-        <v>120</v>
-      </c>
-      <c r="C37" s="45" t="s">
-        <v>10</v>
-      </c>
-      <c r="D37" s="46">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A38" s="14" t="s">
-        <v>121</v>
-      </c>
-      <c r="B38" s="14" t="s">
-        <v>123</v>
-      </c>
-      <c r="C38" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D38" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="38" t="s">
-        <v>122</v>
-      </c>
-      <c r="B39" s="38" t="s">
-        <v>124</v>
-      </c>
-      <c r="C39" s="43" t="s">
-        <v>10</v>
-      </c>
-      <c r="D39" s="44">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A40" s="34"/>
-      <c r="B40" s="34"/>
-      <c r="C40" s="34"/>
-      <c r="D40" s="34"/>
-    </row>
-    <row r="41" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="36" t="s">
-        <v>87</v>
-      </c>
-      <c r="B41" s="37"/>
-      <c r="C41" s="37"/>
-      <c r="D41" s="37"/>
-    </row>
-    <row r="42" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B42" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C42" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="D42" s="10" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A43" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="B43" s="12" t="s">
-        <v>89</v>
-      </c>
-      <c r="C43" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="D43" s="1">
-        <v>1.65</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A44" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="B44" s="15" t="s">
-        <v>91</v>
-      </c>
-      <c r="C44" s="16" t="s">
-        <v>92</v>
-      </c>
-      <c r="D44" s="2">
-        <v>907.18</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A45" s="14" t="s">
-        <v>93</v>
-      </c>
-      <c r="B45" s="15" t="s">
-        <v>94</v>
-      </c>
-      <c r="C45" s="16" t="s">
-        <v>92</v>
-      </c>
-      <c r="D45" s="2">
-        <v>907.18</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A46" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="B46" s="15" t="s">
-        <v>96</v>
-      </c>
-      <c r="C46" s="16" t="s">
-        <v>97</v>
-      </c>
-      <c r="D46" s="2">
-        <v>1027</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A47" s="14" t="s">
-        <v>98</v>
-      </c>
-      <c r="B47" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="C47" s="16" t="s">
-        <v>100</v>
-      </c>
-      <c r="D47" s="2">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A48" s="14" t="s">
-        <v>101</v>
-      </c>
-      <c r="B48" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="C48" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D48" s="2">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="B49" s="15" t="s">
-        <v>104</v>
-      </c>
-      <c r="C49" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D49" s="2">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="14" t="s">
-        <v>105</v>
-      </c>
-      <c r="B50" s="15" t="s">
-        <v>106</v>
-      </c>
-      <c r="C50" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D50" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="39" t="s">
-        <v>107</v>
-      </c>
-      <c r="B51" s="40" t="s">
-        <v>108</v>
-      </c>
-      <c r="C51" s="41" t="s">
-        <v>10</v>
-      </c>
-      <c r="D51" s="42">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="18" t="s">
-        <v>118</v>
-      </c>
-      <c r="B52" s="48" t="s">
-        <v>125</v>
-      </c>
-      <c r="C52" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D52" s="4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="37"/>
-      <c r="B53" s="37"/>
-      <c r="C53" s="37"/>
-      <c r="D53" s="37"/>
-    </row>
-    <row r="66" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B66" s="47"/>
-    </row>
-  </sheetData>
-  <sheetProtection formatColumns="0" selectLockedCells="1"/>
-  <protectedRanges>
-    <protectedRange sqref="D32:D36 I3:I6 I8 D16:D28 I12:I16 I26:I29 I19:I22 D43:D52 I33 D3:D11" name="Range1_1"/>
-    <protectedRange sqref="D12" name="Range1_1_1"/>
-  </protectedRanges>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Adding q limits fix and Dn50_LCBW calcs.
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC4D829D-56C2-45AE-8652-6A7EFFD52701}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82F29518-8B49-4A3F-BDFE-FB60640686B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
@@ -1416,7 +1416,7 @@
         <v>10</v>
       </c>
       <c r="D5" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F5" s="49" t="s">
         <v>136</v>

</xml_diff>

<commit_message>
New output sorting for workflows.
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82F29518-8B49-4A3F-BDFE-FB60640686B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B30E6B2B-471E-42CB-A0B7-F8C6C0DFB384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="177">
   <si>
     <t>StormSim Project General Inputs</t>
   </si>
@@ -560,6 +560,15 @@
   </si>
   <si>
     <t>C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\CO-OPS_8638660_MSL_m_Tidal_Pred_1_year.csv</t>
+  </si>
+  <si>
+    <t>case_name</t>
+  </si>
+  <si>
+    <t>Case Name</t>
+  </si>
+  <si>
+    <t>case_name_0001</t>
   </si>
 </sst>
 </file>
@@ -1301,7 +1310,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51D29750-2AFD-4BF7-A911-1DC4ADC0FD7A}">
-  <dimension ref="A1:I66"/>
+  <dimension ref="A1:I67"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="79" bestFit="1" customWidth="1"/>
@@ -1407,16 +1416,16 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>20</v>
+        <v>174</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>21</v>
+        <v>175</v>
       </c>
       <c r="C5" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="2">
-        <v>3</v>
+      <c r="D5" s="2" t="s">
+        <v>176</v>
       </c>
       <c r="F5" s="49" t="s">
         <v>136</v>
@@ -1433,16 +1442,16 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C6" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>148</v>
+      <c r="D6" s="2">
+        <v>3</v>
       </c>
       <c r="F6" s="49" t="s">
         <v>135</v>
@@ -1459,16 +1468,16 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C7" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>109</v>
+        <v>148</v>
       </c>
       <c r="F7" s="14" t="s">
         <v>137</v>
@@ -1485,16 +1494,16 @@
     </row>
     <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="14" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C8" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D8" s="2">
-        <v>0</v>
+      <c r="D8" s="2" t="s">
+        <v>109</v>
       </c>
       <c r="F8" s="17" t="s">
         <v>132</v>
@@ -1511,16 +1520,16 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>145</v>
+        <v>30</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>146</v>
+        <v>31</v>
       </c>
       <c r="C9" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>168</v>
+      <c r="D9" s="2">
+        <v>0</v>
       </c>
       <c r="F9" s="33"/>
       <c r="G9" s="33"/>
@@ -1529,16 +1538,16 @@
     </row>
     <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="14" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>113</v>
+        <v>146</v>
       </c>
       <c r="C10" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="2">
-        <v>1</v>
+      <c r="D10" s="2" t="s">
+        <v>168</v>
       </c>
       <c r="F10" s="26" t="s">
         <v>138</v>
@@ -1549,10 +1558,10 @@
     </row>
     <row r="11" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="14" t="s">
-        <v>112</v>
+        <v>139</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>144</v>
+        <v>113</v>
       </c>
       <c r="C11" s="16" t="s">
         <v>10</v>
@@ -1573,18 +1582,18 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="B12" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="C12" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>167</v>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="B12" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="C12" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="2">
+        <v>1</v>
       </c>
       <c r="F12" s="30" t="s">
         <v>140</v>
@@ -1599,11 +1608,19 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="6"/>
-      <c r="B13" s="22"/>
-      <c r="C13" s="23"/>
-      <c r="D13" s="23"/>
+    <row r="13" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>167</v>
+      </c>
       <c r="F13" s="30" t="s">
         <v>141</v>
       </c>
@@ -1617,13 +1634,11 @@
         <v>0.43</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="24" t="s">
-        <v>42</v>
-      </c>
-      <c r="B14" s="25"/>
-      <c r="C14" s="25"/>
-      <c r="D14" s="25"/>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="6"/>
+      <c r="B14" s="22"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="23"/>
       <c r="F14" s="14" t="s">
         <v>116</v>
       </c>
@@ -1638,18 +1653,12 @@
       </c>
     </row>
     <row r="15" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B15" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>6</v>
-      </c>
+      <c r="A15" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="B15" s="25"/>
+      <c r="C15" s="25"/>
+      <c r="D15" s="25"/>
       <c r="F15" s="17" t="s">
         <v>117</v>
       </c>
@@ -1663,18 +1672,18 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="14" t="s">
-        <v>110</v>
-      </c>
-      <c r="B16" s="15" t="s">
-        <v>111</v>
-      </c>
-      <c r="C16" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D16" s="2">
-        <v>1</v>
+    <row r="16" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D16" s="10" t="s">
+        <v>6</v>
       </c>
       <c r="F16" s="27"/>
       <c r="G16" s="27"/>
@@ -1682,16 +1691,16 @@
       <c r="I16" s="27"/>
     </row>
     <row r="17" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="B17" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="C17" s="28" t="s">
-        <v>47</v>
-      </c>
-      <c r="D17" s="1">
+      <c r="A17" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="B17" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C17" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D17" s="2">
         <v>1</v>
       </c>
       <c r="F17" s="7" t="s">
@@ -1707,16 +1716,16 @@
     </row>
     <row r="18" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
-        <v>165</v>
+        <v>45</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>166</v>
+        <v>46</v>
       </c>
       <c r="C18" s="28" t="s">
-        <v>162</v>
+        <v>47</v>
       </c>
       <c r="D18" s="1">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>3</v>
@@ -1733,16 +1742,16 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
-        <v>143</v>
+        <v>165</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>142</v>
+        <v>166</v>
       </c>
       <c r="C19" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>147</v>
+        <v>162</v>
+      </c>
+      <c r="D19" s="1">
+        <v>5</v>
       </c>
       <c r="F19" s="11" t="s">
         <v>12</v>
@@ -1758,17 +1767,17 @@
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="B20" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="C20" s="16" t="s">
+      <c r="A20" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="C20" s="28" t="s">
         <v>10</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>169</v>
+        <v>147</v>
       </c>
       <c r="F20" s="14" t="s">
         <v>17</v>
@@ -1785,15 +1794,17 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C21" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D21" s="2"/>
+      <c r="D21" s="2" t="s">
+        <v>169</v>
+      </c>
       <c r="F21" s="14" t="s">
         <v>24</v>
       </c>
@@ -1809,10 +1820,10 @@
     </row>
     <row r="22" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="14" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C22" s="16" t="s">
         <v>10</v>
@@ -1833,10 +1844,10 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C23" s="16" t="s">
         <v>10</v>
@@ -1849,10 +1860,10 @@
     </row>
     <row r="24" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="14" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C24" s="16" t="s">
         <v>10</v>
@@ -1867,10 +1878,10 @@
     </row>
     <row r="25" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="14" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C25" s="16" t="s">
         <v>10</v>
@@ -1891,10 +1902,10 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C26" s="16" t="s">
         <v>10</v>
@@ -1915,10 +1926,10 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C27" s="16" t="s">
         <v>10</v>
@@ -1937,17 +1948,17 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="17" t="s">
-        <v>73</v>
-      </c>
-      <c r="B28" s="18" t="s">
-        <v>74</v>
-      </c>
-      <c r="C28" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D28" s="3"/>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="B28" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="C28" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D28" s="2"/>
       <c r="F28" s="14" t="s">
         <v>39</v>
       </c>
@@ -1962,10 +1973,16 @@
       </c>
     </row>
     <row r="29" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="25"/>
-      <c r="B29" s="25"/>
-      <c r="C29" s="25"/>
-      <c r="D29" s="25"/>
+      <c r="A29" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="B29" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="C29" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D29" s="3"/>
       <c r="F29" s="17" t="s">
         <v>43</v>
       </c>
@@ -1979,31 +1996,23 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="B30" s="35"/>
-      <c r="C30" s="35"/>
-      <c r="D30" s="35"/>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" s="25"/>
+      <c r="B30" s="25"/>
+      <c r="C30" s="25"/>
+      <c r="D30" s="25"/>
       <c r="F30" s="21"/>
       <c r="G30" s="21"/>
       <c r="H30" s="21"/>
       <c r="I30" s="21"/>
     </row>
     <row r="31" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B31" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C31" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="D31" s="10" t="s">
-        <v>78</v>
-      </c>
+      <c r="A31" s="34" t="s">
+        <v>77</v>
+      </c>
+      <c r="B31" s="35"/>
+      <c r="C31" s="35"/>
+      <c r="D31" s="35"/>
       <c r="F31" s="26" t="s">
         <v>48</v>
       </c>
@@ -2012,17 +2021,17 @@
       <c r="I31" s="27"/>
     </row>
     <row r="32" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="B32" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="C32" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="D32" s="1">
-        <v>1.2320122</v>
+      <c r="A32" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B32" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C32" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D32" s="10" t="s">
+        <v>78</v>
       </c>
       <c r="F32" s="9" t="s">
         <v>3</v>
@@ -2038,17 +2047,17 @@
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="B33" s="15" t="s">
-        <v>115</v>
-      </c>
-      <c r="C33" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D33" s="2">
-        <v>1.5243902</v>
+      <c r="A33" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="B33" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="C33" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D33" s="1">
+        <v>1.2320122</v>
       </c>
       <c r="F33" s="29" t="s">
         <v>51</v>
@@ -2065,16 +2074,16 @@
     </row>
     <row r="34" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="14" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>82</v>
+        <v>115</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>41</v>
+        <v>10</v>
       </c>
       <c r="D34" s="2">
-        <v>-1.5969511999999999</v>
+        <v>1.5243902</v>
       </c>
       <c r="F34" s="17" t="s">
         <v>171</v>
@@ -2091,24 +2100,24 @@
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B35" s="15" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C35" s="16" t="s">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="D35" s="2">
-        <v>1.5</v>
+        <v>-1.5969511999999999</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B36" s="15" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C36" s="16" t="s">
         <v>10</v>
@@ -2118,109 +2127,109 @@
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A37" s="39" t="s">
+      <c r="A37" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="B37" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="C37" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D37" s="2">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A38" s="39" t="s">
         <v>119</v>
       </c>
-      <c r="B37" s="39" t="s">
+      <c r="B38" s="39" t="s">
         <v>120</v>
       </c>
-      <c r="C37" s="45" t="s">
-        <v>10</v>
-      </c>
-      <c r="D37" s="46">
+      <c r="C38" s="45" t="s">
+        <v>10</v>
+      </c>
+      <c r="D38" s="46">
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A38" s="14" t="s">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A39" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="B38" s="14" t="s">
+      <c r="B39" s="14" t="s">
         <v>123</v>
       </c>
-      <c r="C38" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D38" s="2">
+      <c r="C39" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D39" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="38" t="s">
+    <row r="40" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="38" t="s">
         <v>122</v>
       </c>
-      <c r="B39" s="38" t="s">
+      <c r="B40" s="38" t="s">
         <v>124</v>
       </c>
-      <c r="C39" s="43" t="s">
-        <v>10</v>
-      </c>
-      <c r="D39" s="44">
+      <c r="C40" s="43" t="s">
+        <v>10</v>
+      </c>
+      <c r="D40" s="44">
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A40" s="34"/>
-      <c r="B40" s="34"/>
-      <c r="C40" s="34"/>
-      <c r="D40" s="34"/>
-    </row>
-    <row r="41" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="36" t="s">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A41" s="34"/>
+      <c r="B41" s="34"/>
+      <c r="C41" s="34"/>
+      <c r="D41" s="34"/>
+    </row>
+    <row r="42" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="36" t="s">
         <v>87</v>
       </c>
-      <c r="B41" s="37"/>
-      <c r="C41" s="37"/>
-      <c r="D41" s="37"/>
-    </row>
-    <row r="42" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="9" t="s">
+      <c r="B42" s="37"/>
+      <c r="C42" s="37"/>
+      <c r="D42" s="37"/>
+    </row>
+    <row r="43" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="B42" s="10" t="s">
+      <c r="B43" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C42" s="10" t="s">
+      <c r="C43" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="D42" s="10" t="s">
+      <c r="D43" s="10" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A43" s="11" t="s">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A44" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="B43" s="12" t="s">
+      <c r="B44" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="C43" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="D43" s="1">
+      <c r="C44" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D44" s="1">
         <v>1.65</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A44" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="B44" s="15" t="s">
-        <v>91</v>
-      </c>
-      <c r="C44" s="16" t="s">
-        <v>92</v>
-      </c>
-      <c r="D44" s="2">
-        <v>500</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B45" s="15" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C45" s="16" t="s">
         <v>92</v>
@@ -2231,52 +2240,52 @@
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B46" s="15" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C46" s="16" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D46" s="2">
-        <v>1027</v>
+        <v>500</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B47" s="15" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C47" s="16" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D47" s="2">
-        <v>0.4</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B48" s="15" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C48" s="16" t="s">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="D48" s="2">
-        <v>20</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B49" s="15" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C49" s="16" t="s">
         <v>10</v>
@@ -2287,62 +2296,76 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="B50" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="C50" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D50" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="14" t="s">
         <v>105</v>
       </c>
-      <c r="B50" s="15" t="s">
+      <c r="B51" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="C50" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D50" s="2">
+      <c r="C51" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D51" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="39" t="s">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" s="39" t="s">
         <v>107</v>
       </c>
-      <c r="B51" s="40" t="s">
+      <c r="B52" s="40" t="s">
         <v>108</v>
       </c>
-      <c r="C51" s="41" t="s">
-        <v>10</v>
-      </c>
-      <c r="D51" s="42">
+      <c r="C52" s="41" t="s">
+        <v>10</v>
+      </c>
+      <c r="D52" s="42">
         <v>2</v>
       </c>
     </row>
-    <row r="52" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="18" t="s">
+    <row r="53" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="18" t="s">
         <v>118</v>
       </c>
-      <c r="B52" s="48" t="s">
+      <c r="B53" s="48" t="s">
         <v>125</v>
       </c>
-      <c r="C52" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D52" s="4">
+      <c r="C53" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D53" s="4">
         <v>2</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="37"/>
-      <c r="B53" s="37"/>
-      <c r="C53" s="37"/>
-      <c r="D53" s="37"/>
-    </row>
-    <row r="66" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B66" s="47"/>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" s="37"/>
+      <c r="B54" s="37"/>
+      <c r="C54" s="37"/>
+      <c r="D54" s="37"/>
+    </row>
+    <row r="67" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B67" s="47"/>
     </row>
   </sheetData>
   <sheetProtection formatColumns="0" selectLockedCells="1"/>
   <protectedRanges>
-    <protectedRange sqref="I3:I6 I8 D16:D28 I12:I16 I26:I29 I19:I22 I33 D3:D11" name="Range1_1"/>
-    <protectedRange sqref="D12" name="Range1_1_1"/>
-    <protectedRange sqref="D32:D36" name="Range1_1_3"/>
-    <protectedRange sqref="D43:D52" name="Range1_1_4"/>
+    <protectedRange sqref="I3:I6 I8 D17:D29 I12:I16 I26:I29 I19:I22 I33 D3:D12" name="Range1_1"/>
+    <protectedRange sqref="D13" name="Range1_1_1"/>
+    <protectedRange sqref="D33:D37" name="Range1_1_3"/>
+    <protectedRange sqref="D44:D53" name="Range1_1_4"/>
   </protectedRanges>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Added new case_name framwork accros workflows
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B30E6B2B-471E-42CB-A0B7-F8C6C0DFB384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{782A8432-6C7B-4434-A51E-AE83797F66C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="178">
   <si>
     <t>StormSim Project General Inputs</t>
   </si>
@@ -568,7 +568,10 @@
     <t>Case Name</t>
   </si>
   <si>
-    <t>case_name_0001</t>
+    <t>case_name_0002</t>
+  </si>
+  <si>
+    <t>TC</t>
   </si>
 </sst>
 </file>
@@ -1503,7 +1506,7 @@
         <v>10</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>109</v>
+        <v>177</v>
       </c>
       <c r="F8" s="17" t="s">
         <v>132</v>

</xml_diff>

<commit_message>
Testing switches. Reverting some changes.
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{782A8432-6C7B-4434-A51E-AE83797F66C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D1AFC7A-67FA-4F83-90D4-1460C085CB5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
@@ -568,10 +568,10 @@
     <t>Case Name</t>
   </si>
   <si>
-    <t>case_name_0002</t>
-  </si>
-  <si>
-    <t>TC</t>
+    <t>James_Island</t>
+  </si>
+  <si>
+    <t>case_1</t>
   </si>
 </sst>
 </file>
@@ -1402,7 +1402,7 @@
         <v>10</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>16</v>
+        <v>176</v>
       </c>
       <c r="F4" s="49" t="s">
         <v>134</v>
@@ -1428,7 +1428,7 @@
         <v>10</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F5" s="49" t="s">
         <v>136</v>
@@ -1506,7 +1506,7 @@
         <v>10</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>177</v>
+        <v>109</v>
       </c>
       <c r="F8" s="17" t="s">
         <v>132</v>

</xml_diff>

<commit_message>
Adding new XC & TC comparison tool for HCs.
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D1AFC7A-67FA-4F83-90D4-1460C085CB5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA557117-FE45-42CC-813C-54851D1649BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
@@ -571,7 +571,7 @@
     <t>James_Island</t>
   </si>
   <si>
-    <t>case_1</t>
+    <t>PROS</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Removing RB workflows from call_uncertainty_engine and Dn50_LCBW bug
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB8203B9-3411-459A-8269-E41770067C8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBFDB968-C1F2-48BF-8A41-B91F5BD970DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
@@ -571,7 +571,7 @@
     <t>James_Island</t>
   </si>
   <si>
-    <t>PROS-Uncert-Outside</t>
+    <t>PROS-latest</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Renamed cast_workflow to workflow.
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBFDB968-C1F2-48BF-8A41-B91F5BD970DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B81CF80B-19ED-4C05-8DD0-DD5289CD77D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="179">
   <si>
     <t>StormSim Project General Inputs</t>
   </si>
@@ -73,9 +73,6 @@
     <t>NA</t>
   </si>
   <si>
-    <t>Midbay_v1</t>
-  </si>
-  <si>
     <t>mcs_nLC</t>
   </si>
   <si>
@@ -572,6 +569,12 @@
   </si>
   <si>
     <t>PROS-latest</t>
+  </si>
+  <si>
+    <t>Midbay_v2</t>
+  </si>
+  <si>
+    <t>workflow</t>
   </si>
 </sst>
 </file>
@@ -1333,7 +1336,7 @@
       <c r="C1" s="6"/>
       <c r="D1" s="6"/>
       <c r="F1" s="32" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G1" s="33"/>
       <c r="H1" s="33"/>
@@ -1376,16 +1379,16 @@
         <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>11</v>
+        <v>177</v>
       </c>
       <c r="F3" s="49" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G3" s="49" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="H3" s="13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I3" s="13">
         <v>0.33979999999999999</v>
@@ -1393,25 +1396,25 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="15" t="s">
-        <v>15</v>
-      </c>
       <c r="C4" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F4" s="49" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G4" s="49" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H4" s="13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I4" s="13">
         <v>0.38219999999999998</v>
@@ -1419,25 +1422,25 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
+        <v>173</v>
+      </c>
+      <c r="B5" s="15" t="s">
         <v>174</v>
       </c>
-      <c r="B5" s="15" t="s">
-        <v>175</v>
-      </c>
       <c r="C5" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F5" s="49" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G5" s="49" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I5" s="13">
         <v>0.3</v>
@@ -1445,10 +1448,10 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="15" t="s">
         <v>20</v>
-      </c>
-      <c r="B6" s="15" t="s">
-        <v>21</v>
       </c>
       <c r="C6" s="16" t="s">
         <v>10</v>
@@ -1457,13 +1460,13 @@
         <v>3</v>
       </c>
       <c r="F6" s="49" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G6" s="49" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="H6" s="13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I6" s="13">
         <v>0.3</v>
@@ -1471,22 +1474,22 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="15" t="s">
-        <v>23</v>
-      </c>
       <c r="C7" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G7" s="15" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H7" s="16" t="s">
         <v>10</v>
@@ -1497,25 +1500,25 @@
     </row>
     <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="15" t="s">
-        <v>27</v>
-      </c>
       <c r="C8" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H8" s="19" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I8" s="3">
         <v>0</v>
@@ -1523,10 +1526,10 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="15" t="s">
         <v>30</v>
-      </c>
-      <c r="B9" s="15" t="s">
-        <v>31</v>
       </c>
       <c r="C9" s="16" t="s">
         <v>10</v>
@@ -1541,19 +1544,19 @@
     </row>
     <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="14" t="s">
+        <v>144</v>
+      </c>
+      <c r="B10" s="15" t="s">
         <v>145</v>
       </c>
-      <c r="B10" s="15" t="s">
-        <v>146</v>
-      </c>
       <c r="C10" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F10" s="26" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G10" s="27"/>
       <c r="H10" s="27"/>
@@ -1561,10 +1564,10 @@
     </row>
     <row r="11" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="14" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C11" s="16" t="s">
         <v>10</v>
@@ -1587,10 +1590,10 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>112</v>
+        <v>178</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C12" s="16" t="s">
         <v>10</v>
@@ -1599,13 +1602,13 @@
         <v>1</v>
       </c>
       <c r="F12" s="30" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G12" s="15" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H12" s="16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I12" s="2">
         <v>0.5</v>
@@ -1613,25 +1616,25 @@
     </row>
     <row r="13" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="B13" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="B13" s="18" t="s">
-        <v>36</v>
-      </c>
       <c r="C13" s="19" t="s">
         <v>10</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F13" s="30" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G13" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="H13" s="31" t="s">
         <v>65</v>
-      </c>
-      <c r="H13" s="31" t="s">
-        <v>66</v>
       </c>
       <c r="I13" s="2">
         <v>0.43</v>
@@ -1643,13 +1646,13 @@
       <c r="C14" s="23"/>
       <c r="D14" s="23"/>
       <c r="F14" s="14" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G14" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="H14" s="16" t="s">
         <v>58</v>
-      </c>
-      <c r="H14" s="16" t="s">
-        <v>59</v>
       </c>
       <c r="I14" s="2">
         <v>0.78</v>
@@ -1657,19 +1660,19 @@
     </row>
     <row r="15" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="24" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B15" s="25"/>
       <c r="C15" s="25"/>
       <c r="D15" s="25"/>
       <c r="F15" s="17" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G15" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H15" s="19" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I15" s="3">
         <v>0.13</v>
@@ -1695,10 +1698,10 @@
     </row>
     <row r="17" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="B17" s="15" t="s">
         <v>110</v>
-      </c>
-      <c r="B17" s="15" t="s">
-        <v>111</v>
       </c>
       <c r="C17" s="16" t="s">
         <v>10</v>
@@ -1719,13 +1722,13 @@
     </row>
     <row r="18" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="B18" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="B18" s="12" t="s">
+      <c r="C18" s="28" t="s">
         <v>46</v>
-      </c>
-      <c r="C18" s="28" t="s">
-        <v>47</v>
       </c>
       <c r="D18" s="1">
         <v>1</v>
@@ -1745,22 +1748,22 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="B19" s="12" t="s">
         <v>165</v>
       </c>
-      <c r="B19" s="12" t="s">
-        <v>166</v>
-      </c>
       <c r="C19" s="28" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D19" s="1">
         <v>5</v>
       </c>
       <c r="F19" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="G19" s="12" t="s">
         <v>12</v>
-      </c>
-      <c r="G19" s="12" t="s">
-        <v>13</v>
       </c>
       <c r="H19" s="13" t="s">
         <v>10</v>
@@ -1771,25 +1774,25 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C20" s="28" t="s">
         <v>10</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F20" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="G20" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="G20" s="15" t="s">
+      <c r="H20" s="16" t="s">
         <v>18</v>
-      </c>
-      <c r="H20" s="16" t="s">
-        <v>19</v>
       </c>
       <c r="I20" s="2">
         <v>50</v>
@@ -1797,22 +1800,22 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="B21" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="B21" s="15" t="s">
-        <v>50</v>
-      </c>
       <c r="C21" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F21" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="G21" s="15" t="s">
         <v>24</v>
-      </c>
-      <c r="G21" s="15" t="s">
-        <v>25</v>
       </c>
       <c r="H21" s="16" t="s">
         <v>10</v>
@@ -1823,20 +1826,20 @@
     </row>
     <row r="22" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="B22" s="15" t="s">
         <v>53</v>
-      </c>
-      <c r="B22" s="15" t="s">
-        <v>54</v>
       </c>
       <c r="C22" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D22" s="2"/>
       <c r="F22" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="G22" s="18" t="s">
         <v>28</v>
-      </c>
-      <c r="G22" s="18" t="s">
-        <v>29</v>
       </c>
       <c r="H22" s="19" t="s">
         <v>10</v>
@@ -1847,10 +1850,10 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="B23" s="15" t="s">
         <v>56</v>
-      </c>
-      <c r="B23" s="15" t="s">
-        <v>57</v>
       </c>
       <c r="C23" s="16" t="s">
         <v>10</v>
@@ -1863,17 +1866,17 @@
     </row>
     <row r="24" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="B24" s="15" t="s">
         <v>60</v>
-      </c>
-      <c r="B24" s="15" t="s">
-        <v>61</v>
       </c>
       <c r="C24" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D24" s="2"/>
       <c r="F24" s="20" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G24" s="21"/>
       <c r="H24" s="21"/>
@@ -1881,10 +1884,10 @@
     </row>
     <row r="25" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="B25" s="15" t="s">
         <v>63</v>
-      </c>
-      <c r="B25" s="15" t="s">
-        <v>64</v>
       </c>
       <c r="C25" s="16" t="s">
         <v>10</v>
@@ -1905,20 +1908,20 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="B26" s="15" t="s">
         <v>67</v>
-      </c>
-      <c r="B26" s="15" t="s">
-        <v>68</v>
       </c>
       <c r="C26" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D26" s="2"/>
       <c r="F26" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="G26" s="12" t="s">
         <v>33</v>
-      </c>
-      <c r="G26" s="12" t="s">
-        <v>34</v>
       </c>
       <c r="H26" s="13" t="s">
         <v>10</v>
@@ -1929,20 +1932,20 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="B27" s="15" t="s">
         <v>69</v>
-      </c>
-      <c r="B27" s="15" t="s">
-        <v>70</v>
       </c>
       <c r="C27" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D27" s="2"/>
       <c r="F27" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="G27" s="15" t="s">
         <v>37</v>
-      </c>
-      <c r="G27" s="15" t="s">
-        <v>38</v>
       </c>
       <c r="H27" s="16" t="s">
         <v>10</v>
@@ -1953,23 +1956,23 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="B28" s="15" t="s">
         <v>71</v>
-      </c>
-      <c r="B28" s="15" t="s">
-        <v>72</v>
       </c>
       <c r="C28" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D28" s="2"/>
       <c r="F28" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="G28" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="G28" s="15" t="s">
+      <c r="H28" s="16" t="s">
         <v>40</v>
-      </c>
-      <c r="H28" s="16" t="s">
-        <v>41</v>
       </c>
       <c r="I28" s="2">
         <v>0</v>
@@ -1977,23 +1980,23 @@
     </row>
     <row r="29" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="B29" s="18" t="s">
         <v>73</v>
-      </c>
-      <c r="B29" s="18" t="s">
-        <v>74</v>
       </c>
       <c r="C29" s="19" t="s">
         <v>10</v>
       </c>
       <c r="D29" s="3"/>
       <c r="F29" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="G29" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="G29" s="18" t="s">
-        <v>44</v>
-      </c>
       <c r="H29" s="19" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I29" s="3">
         <v>1</v>
@@ -2011,13 +2014,13 @@
     </row>
     <row r="31" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="34" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B31" s="35"/>
       <c r="C31" s="35"/>
       <c r="D31" s="35"/>
       <c r="F31" s="26" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G31" s="27"/>
       <c r="H31" s="27"/>
@@ -2034,7 +2037,7 @@
         <v>5</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F32" s="9" t="s">
         <v>3</v>
@@ -2051,10 +2054,10 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="11" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C33" s="13" t="s">
         <v>10</v>
@@ -2063,10 +2066,10 @@
         <v>1.2320122</v>
       </c>
       <c r="F33" s="29" t="s">
+        <v>50</v>
+      </c>
+      <c r="G33" s="12" t="s">
         <v>51</v>
-      </c>
-      <c r="G33" s="12" t="s">
-        <v>52</v>
       </c>
       <c r="H33" s="13" t="s">
         <v>10</v>
@@ -2077,10 +2080,10 @@
     </row>
     <row r="34" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C34" s="16" t="s">
         <v>10</v>
@@ -2089,10 +2092,10 @@
         <v>1.5243902</v>
       </c>
       <c r="F34" s="17" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G34" s="18" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="H34" s="19" t="s">
         <v>10</v>
@@ -2103,13 +2106,13 @@
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="B35" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="B35" s="15" t="s">
-        <v>82</v>
-      </c>
       <c r="C35" s="16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D35" s="2">
         <v>-1.5969511999999999</v>
@@ -2117,10 +2120,10 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="B36" s="15" t="s">
         <v>83</v>
-      </c>
-      <c r="B36" s="15" t="s">
-        <v>84</v>
       </c>
       <c r="C36" s="16" t="s">
         <v>10</v>
@@ -2131,10 +2134,10 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="B37" s="15" t="s">
         <v>85</v>
-      </c>
-      <c r="B37" s="15" t="s">
-        <v>86</v>
       </c>
       <c r="C37" s="16" t="s">
         <v>10</v>
@@ -2145,10 +2148,10 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="39" t="s">
+        <v>118</v>
+      </c>
+      <c r="B38" s="39" t="s">
         <v>119</v>
-      </c>
-      <c r="B38" s="39" t="s">
-        <v>120</v>
       </c>
       <c r="C38" s="45" t="s">
         <v>10</v>
@@ -2159,10 +2162,10 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C39" s="16" t="s">
         <v>10</v>
@@ -2173,10 +2176,10 @@
     </row>
     <row r="40" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="38" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B40" s="38" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C40" s="43" t="s">
         <v>10</v>
@@ -2193,7 +2196,7 @@
     </row>
     <row r="42" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="36" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B42" s="37"/>
       <c r="C42" s="37"/>
@@ -2210,15 +2213,15 @@
         <v>5</v>
       </c>
       <c r="D43" s="10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="B44" s="12" t="s">
         <v>88</v>
-      </c>
-      <c r="B44" s="12" t="s">
-        <v>89</v>
       </c>
       <c r="C44" s="13" t="s">
         <v>10</v>
@@ -2229,13 +2232,13 @@
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="B45" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="B45" s="15" t="s">
+      <c r="C45" s="16" t="s">
         <v>91</v>
-      </c>
-      <c r="C45" s="16" t="s">
-        <v>92</v>
       </c>
       <c r="D45" s="2">
         <v>500</v>
@@ -2243,13 +2246,13 @@
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="B46" s="15" t="s">
         <v>93</v>
       </c>
-      <c r="B46" s="15" t="s">
-        <v>94</v>
-      </c>
       <c r="C46" s="16" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D46" s="2">
         <v>500</v>
@@ -2257,13 +2260,13 @@
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="B47" s="15" t="s">
         <v>95</v>
       </c>
-      <c r="B47" s="15" t="s">
+      <c r="C47" s="16" t="s">
         <v>96</v>
-      </c>
-      <c r="C47" s="16" t="s">
-        <v>97</v>
       </c>
       <c r="D47" s="2">
         <v>1027</v>
@@ -2271,13 +2274,13 @@
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="B48" s="15" t="s">
         <v>98</v>
       </c>
-      <c r="B48" s="15" t="s">
+      <c r="C48" s="16" t="s">
         <v>99</v>
-      </c>
-      <c r="C48" s="16" t="s">
-        <v>100</v>
       </c>
       <c r="D48" s="2">
         <v>0.4</v>
@@ -2285,10 +2288,10 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="B49" s="15" t="s">
         <v>101</v>
-      </c>
-      <c r="B49" s="15" t="s">
-        <v>102</v>
       </c>
       <c r="C49" s="16" t="s">
         <v>10</v>
@@ -2299,10 +2302,10 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="B50" s="15" t="s">
         <v>103</v>
-      </c>
-      <c r="B50" s="15" t="s">
-        <v>104</v>
       </c>
       <c r="C50" s="16" t="s">
         <v>10</v>
@@ -2313,10 +2316,10 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="14" t="s">
+        <v>104</v>
+      </c>
+      <c r="B51" s="15" t="s">
         <v>105</v>
-      </c>
-      <c r="B51" s="15" t="s">
-        <v>106</v>
       </c>
       <c r="C51" s="16" t="s">
         <v>10</v>
@@ -2327,10 +2330,10 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="39" t="s">
+        <v>106</v>
+      </c>
+      <c r="B52" s="40" t="s">
         <v>107</v>
-      </c>
-      <c r="B52" s="40" t="s">
-        <v>108</v>
       </c>
       <c r="C52" s="41" t="s">
         <v>10</v>
@@ -2341,10 +2344,10 @@
     </row>
     <row r="53" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="18" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B53" s="48" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C53" s="19" t="s">
         <v>10</v>
@@ -2397,7 +2400,7 @@
       <c r="C1" s="6"/>
       <c r="D1" s="6"/>
       <c r="F1" s="32" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G1" s="33"/>
       <c r="H1" s="33"/>
@@ -2440,16 +2443,16 @@
         <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F3" s="49" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G3" s="49" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="H3" s="13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I3" s="13">
         <v>0.33979999999999999</v>
@@ -2457,25 +2460,25 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="C4" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="F4" s="49" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G4" s="49" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H4" s="13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I4" s="13">
         <v>0.38219999999999998</v>
@@ -2483,10 +2486,10 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="15" t="s">
         <v>20</v>
-      </c>
-      <c r="B5" s="15" t="s">
-        <v>21</v>
       </c>
       <c r="C5" s="16" t="s">
         <v>10</v>
@@ -2495,13 +2498,13 @@
         <v>1</v>
       </c>
       <c r="F5" s="49" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G5" s="49" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I5" s="13">
         <v>0.3</v>
@@ -2509,25 +2512,25 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="15" t="s">
-        <v>23</v>
-      </c>
       <c r="C6" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F6" s="49" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G6" s="49" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="H6" s="13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I6" s="13">
         <v>0.3</v>
@@ -2535,22 +2538,22 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="15" t="s">
-        <v>27</v>
-      </c>
       <c r="C7" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G7" s="15" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H7" s="16" t="s">
         <v>10</v>
@@ -2561,10 +2564,10 @@
     </row>
     <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="15" t="s">
         <v>30</v>
-      </c>
-      <c r="B8" s="15" t="s">
-        <v>31</v>
       </c>
       <c r="C8" s="16" t="s">
         <v>10</v>
@@ -2573,13 +2576,13 @@
         <v>0</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H8" s="19" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I8" s="3">
         <v>0</v>
@@ -2587,16 +2590,16 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
+        <v>144</v>
+      </c>
+      <c r="B9" s="15" t="s">
         <v>145</v>
       </c>
-      <c r="B9" s="15" t="s">
-        <v>146</v>
-      </c>
       <c r="C9" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F9" s="33"/>
       <c r="G9" s="33"/>
@@ -2605,10 +2608,10 @@
     </row>
     <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="14" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C10" s="16" t="s">
         <v>10</v>
@@ -2617,7 +2620,7 @@
         <v>1</v>
       </c>
       <c r="F10" s="26" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G10" s="27"/>
       <c r="H10" s="27"/>
@@ -2625,10 +2628,10 @@
     </row>
     <row r="11" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="14" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C11" s="16" t="s">
         <v>10</v>
@@ -2651,25 +2654,25 @@
     </row>
     <row r="12" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="B12" s="18" t="s">
-        <v>36</v>
-      </c>
       <c r="C12" s="19" t="s">
         <v>10</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F12" s="30" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G12" s="15" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H12" s="16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I12" s="2">
         <v>0.5</v>
@@ -2681,13 +2684,13 @@
       <c r="C13" s="23"/>
       <c r="D13" s="23"/>
       <c r="F13" s="30" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G13" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="H13" s="31" t="s">
         <v>65</v>
-      </c>
-      <c r="H13" s="31" t="s">
-        <v>66</v>
       </c>
       <c r="I13" s="2">
         <v>0.43</v>
@@ -2695,19 +2698,19 @@
     </row>
     <row r="14" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="24" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B14" s="25"/>
       <c r="C14" s="25"/>
       <c r="D14" s="25"/>
       <c r="F14" s="14" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G14" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="H14" s="16" t="s">
         <v>58</v>
-      </c>
-      <c r="H14" s="16" t="s">
-        <v>59</v>
       </c>
       <c r="I14" s="2">
         <v>0.78</v>
@@ -2727,13 +2730,13 @@
         <v>6</v>
       </c>
       <c r="F15" s="17" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G15" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H15" s="19" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I15" s="3">
         <v>0.13</v>
@@ -2741,10 +2744,10 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="B16" s="15" t="s">
         <v>110</v>
-      </c>
-      <c r="B16" s="15" t="s">
-        <v>111</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>10</v>
@@ -2759,13 +2762,13 @@
     </row>
     <row r="17" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="B17" s="12" t="s">
+      <c r="C17" s="28" t="s">
         <v>46</v>
-      </c>
-      <c r="C17" s="28" t="s">
-        <v>47</v>
       </c>
       <c r="D17" s="1">
         <v>1</v>
@@ -2783,13 +2786,13 @@
     </row>
     <row r="18" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="B18" s="12" t="s">
         <v>165</v>
       </c>
-      <c r="B18" s="12" t="s">
-        <v>166</v>
-      </c>
       <c r="C18" s="28" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D18" s="1">
         <v>5</v>
@@ -2809,22 +2812,22 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C19" s="28" t="s">
         <v>10</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F19" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="G19" s="12" t="s">
         <v>12</v>
-      </c>
-      <c r="G19" s="12" t="s">
-        <v>13</v>
       </c>
       <c r="H19" s="13" t="s">
         <v>10</v>
@@ -2835,25 +2838,25 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="B20" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="B20" s="15" t="s">
-        <v>50</v>
-      </c>
       <c r="C20" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F20" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="G20" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="G20" s="15" t="s">
+      <c r="H20" s="16" t="s">
         <v>18</v>
-      </c>
-      <c r="H20" s="16" t="s">
-        <v>19</v>
       </c>
       <c r="I20" s="2">
         <v>50</v>
@@ -2861,20 +2864,20 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="B21" s="15" t="s">
         <v>53</v>
-      </c>
-      <c r="B21" s="15" t="s">
-        <v>54</v>
       </c>
       <c r="C21" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D21" s="2"/>
       <c r="F21" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="G21" s="15" t="s">
         <v>24</v>
-      </c>
-      <c r="G21" s="15" t="s">
-        <v>25</v>
       </c>
       <c r="H21" s="16" t="s">
         <v>10</v>
@@ -2885,20 +2888,20 @@
     </row>
     <row r="22" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="B22" s="15" t="s">
         <v>56</v>
-      </c>
-      <c r="B22" s="15" t="s">
-        <v>57</v>
       </c>
       <c r="C22" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D22" s="2"/>
       <c r="F22" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="G22" s="18" t="s">
         <v>28</v>
-      </c>
-      <c r="G22" s="18" t="s">
-        <v>29</v>
       </c>
       <c r="H22" s="19" t="s">
         <v>10</v>
@@ -2909,10 +2912,10 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="B23" s="15" t="s">
         <v>60</v>
-      </c>
-      <c r="B23" s="15" t="s">
-        <v>61</v>
       </c>
       <c r="C23" s="16" t="s">
         <v>10</v>
@@ -2925,17 +2928,17 @@
     </row>
     <row r="24" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="B24" s="15" t="s">
         <v>63</v>
-      </c>
-      <c r="B24" s="15" t="s">
-        <v>64</v>
       </c>
       <c r="C24" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D24" s="2"/>
       <c r="F24" s="20" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G24" s="21"/>
       <c r="H24" s="21"/>
@@ -2943,10 +2946,10 @@
     </row>
     <row r="25" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="B25" s="15" t="s">
         <v>67</v>
-      </c>
-      <c r="B25" s="15" t="s">
-        <v>68</v>
       </c>
       <c r="C25" s="16" t="s">
         <v>10</v>
@@ -2967,20 +2970,20 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="B26" s="15" t="s">
         <v>69</v>
-      </c>
-      <c r="B26" s="15" t="s">
-        <v>70</v>
       </c>
       <c r="C26" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D26" s="2"/>
       <c r="F26" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="G26" s="12" t="s">
         <v>33</v>
-      </c>
-      <c r="G26" s="12" t="s">
-        <v>34</v>
       </c>
       <c r="H26" s="13" t="s">
         <v>10</v>
@@ -2991,20 +2994,20 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="B27" s="15" t="s">
         <v>71</v>
-      </c>
-      <c r="B27" s="15" t="s">
-        <v>72</v>
       </c>
       <c r="C27" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D27" s="2"/>
       <c r="F27" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="G27" s="15" t="s">
         <v>37</v>
-      </c>
-      <c r="G27" s="15" t="s">
-        <v>38</v>
       </c>
       <c r="H27" s="16" t="s">
         <v>10</v>
@@ -3015,23 +3018,23 @@
     </row>
     <row r="28" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="B28" s="18" t="s">
         <v>73</v>
-      </c>
-      <c r="B28" s="18" t="s">
-        <v>74</v>
       </c>
       <c r="C28" s="19" t="s">
         <v>10</v>
       </c>
       <c r="D28" s="3"/>
       <c r="F28" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="G28" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="G28" s="15" t="s">
+      <c r="H28" s="16" t="s">
         <v>40</v>
-      </c>
-      <c r="H28" s="16" t="s">
-        <v>41</v>
       </c>
       <c r="I28" s="2">
         <v>0</v>
@@ -3043,13 +3046,13 @@
       <c r="C29" s="25"/>
       <c r="D29" s="25"/>
       <c r="F29" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="G29" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="G29" s="18" t="s">
-        <v>44</v>
-      </c>
       <c r="H29" s="19" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I29" s="3">
         <v>1</v>
@@ -3057,7 +3060,7 @@
     </row>
     <row r="30" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="34" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B30" s="35"/>
       <c r="C30" s="35"/>
@@ -3078,10 +3081,10 @@
         <v>5</v>
       </c>
       <c r="D31" s="10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F31" s="26" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G31" s="27"/>
       <c r="H31" s="27"/>
@@ -3089,10 +3092,10 @@
     </row>
     <row r="32" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="11" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C32" s="13" t="s">
         <v>10</v>
@@ -3116,10 +3119,10 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B33" s="15" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C33" s="16" t="s">
         <v>10</v>
@@ -3129,10 +3132,10 @@
         <v>3.130296</v>
       </c>
       <c r="F33" s="29" t="s">
+        <v>50</v>
+      </c>
+      <c r="G33" s="12" t="s">
         <v>51</v>
-      </c>
-      <c r="G33" s="12" t="s">
-        <v>52</v>
       </c>
       <c r="H33" s="13" t="s">
         <v>10</v>
@@ -3143,23 +3146,23 @@
     </row>
     <row r="34" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="B34" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="B34" s="15" t="s">
-        <v>82</v>
-      </c>
       <c r="C34" s="16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D34" s="2">
         <f>NAE_Structure!B13*-1</f>
         <v>-2.8254960000000002</v>
       </c>
       <c r="F34" s="17" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G34" s="18" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="H34" s="19" t="s">
         <v>10</v>
@@ -3170,10 +3173,10 @@
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="B35" s="15" t="s">
         <v>83</v>
-      </c>
-      <c r="B35" s="15" t="s">
-        <v>84</v>
       </c>
       <c r="C35" s="16" t="s">
         <v>10</v>
@@ -3184,10 +3187,10 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="B36" s="15" t="s">
         <v>85</v>
-      </c>
-      <c r="B36" s="15" t="s">
-        <v>86</v>
       </c>
       <c r="C36" s="16" t="s">
         <v>10</v>
@@ -3198,10 +3201,10 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="39" t="s">
+        <v>118</v>
+      </c>
+      <c r="B37" s="39" t="s">
         <v>119</v>
-      </c>
-      <c r="B37" s="39" t="s">
-        <v>120</v>
       </c>
       <c r="C37" s="45" t="s">
         <v>10</v>
@@ -3212,10 +3215,10 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C38" s="16" t="s">
         <v>10</v>
@@ -3226,10 +3229,10 @@
     </row>
     <row r="39" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="38" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B39" s="38" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C39" s="43" t="s">
         <v>10</v>
@@ -3246,7 +3249,7 @@
     </row>
     <row r="41" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="36" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B41" s="37"/>
       <c r="C41" s="37"/>
@@ -3263,15 +3266,15 @@
         <v>5</v>
       </c>
       <c r="D42" s="10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="B43" s="12" t="s">
         <v>88</v>
-      </c>
-      <c r="B43" s="12" t="s">
-        <v>89</v>
       </c>
       <c r="C43" s="13" t="s">
         <v>10</v>
@@ -3282,13 +3285,13 @@
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="B44" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="B44" s="15" t="s">
+      <c r="C44" s="16" t="s">
         <v>91</v>
-      </c>
-      <c r="C44" s="16" t="s">
-        <v>92</v>
       </c>
       <c r="D44" s="2">
         <v>907.18</v>
@@ -3296,13 +3299,13 @@
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="B45" s="15" t="s">
         <v>93</v>
       </c>
-      <c r="B45" s="15" t="s">
-        <v>94</v>
-      </c>
       <c r="C45" s="16" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D45" s="2">
         <v>907.18</v>
@@ -3310,13 +3313,13 @@
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="B46" s="15" t="s">
         <v>95</v>
       </c>
-      <c r="B46" s="15" t="s">
+      <c r="C46" s="16" t="s">
         <v>96</v>
-      </c>
-      <c r="C46" s="16" t="s">
-        <v>97</v>
       </c>
       <c r="D46" s="2">
         <v>1027</v>
@@ -3324,13 +3327,13 @@
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="B47" s="15" t="s">
         <v>98</v>
       </c>
-      <c r="B47" s="15" t="s">
+      <c r="C47" s="16" t="s">
         <v>99</v>
-      </c>
-      <c r="C47" s="16" t="s">
-        <v>100</v>
       </c>
       <c r="D47" s="2">
         <v>0.4</v>
@@ -3338,10 +3341,10 @@
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="B48" s="15" t="s">
         <v>101</v>
-      </c>
-      <c r="B48" s="15" t="s">
-        <v>102</v>
       </c>
       <c r="C48" s="16" t="s">
         <v>10</v>
@@ -3352,10 +3355,10 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="B49" s="15" t="s">
         <v>103</v>
-      </c>
-      <c r="B49" s="15" t="s">
-        <v>104</v>
       </c>
       <c r="C49" s="16" t="s">
         <v>10</v>
@@ -3366,10 +3369,10 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
+        <v>104</v>
+      </c>
+      <c r="B50" s="15" t="s">
         <v>105</v>
-      </c>
-      <c r="B50" s="15" t="s">
-        <v>106</v>
       </c>
       <c r="C50" s="16" t="s">
         <v>10</v>
@@ -3380,10 +3383,10 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="39" t="s">
+        <v>106</v>
+      </c>
+      <c r="B51" s="40" t="s">
         <v>107</v>
-      </c>
-      <c r="B51" s="40" t="s">
-        <v>108</v>
       </c>
       <c r="C51" s="41" t="s">
         <v>10</v>
@@ -3394,10 +3397,10 @@
     </row>
     <row r="52" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="18" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B52" s="48" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C52" s="19" t="s">
         <v>10</v>
@@ -3437,12 +3440,12 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -3450,40 +3453,40 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>150</v>
+      </c>
+      <c r="B3">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
         <v>151</v>
-      </c>
-      <c r="B3">
-        <v>10</v>
-      </c>
-      <c r="C3" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B4">
         <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B5">
         <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B6">
         <v>3</v>
@@ -3491,7 +3494,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B7">
         <v>1</v>
@@ -3499,58 +3502,58 @@
     </row>
     <row r="8" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B8">
         <f>1.8-1.53</f>
         <v>0.27</v>
       </c>
       <c r="C8" s="50" t="s">
+        <v>158</v>
+      </c>
+      <c r="D8" t="s">
         <v>159</v>
-      </c>
-      <c r="D8" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B11">
         <f>(B3+$B$8)*0.3048</f>
         <v>3.130296</v>
       </c>
       <c r="C11" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B12">
         <f t="shared" ref="B12:B13" si="0">(B4+$B$8)*0.3048</f>
         <v>4.9590959999999997</v>
       </c>
       <c r="C12" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B13">
         <f t="shared" si="0"/>
         <v>2.8254960000000002</v>
       </c>
       <c r="C13" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add StormSim:EVA workflow to StormSim framework. B.E labels for plots.
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B81CF80B-19ED-4C05-8DD0-DD5289CD77D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6B4B73C-B3BF-4953-8375-00C0E6F752E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
@@ -568,13 +568,13 @@
     <t>James_Island</t>
   </si>
   <si>
-    <t>PROS-latest</t>
-  </si>
-  <si>
     <t>Midbay_v2</t>
   </si>
   <si>
     <t>workflow</t>
+  </si>
+  <si>
+    <t>PROS-latest-2</t>
   </si>
 </sst>
 </file>
@@ -1379,7 +1379,7 @@
         <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F3" s="49" t="s">
         <v>132</v>
@@ -1431,7 +1431,7 @@
         <v>10</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="F5" s="49" t="s">
         <v>135</v>
@@ -1590,7 +1590,7 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B12" s="15" t="s">
         <v>143</v>
@@ -1599,7 +1599,7 @@
         <v>10</v>
       </c>
       <c r="D12" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F12" s="30" t="s">
         <v>139</v>

</xml_diff>

<commit_message>
Removing freq limits for HC. Generalizing LCS mean max curve builder.
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27C2439F-E574-4841-B4BC-2FB3F1242F81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4FE039C-692E-4EF6-9FC5-D8D32B9E538A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="1950" windowWidth="29145" windowHeight="8640" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
+    <workbookView xWindow="5190" yWindow="1905" windowWidth="29145" windowHeight="16815" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
   <sheets>
     <sheet name="James_Island_Midbay" sheetId="1" r:id="rId1"/>
@@ -577,7 +577,7 @@
     <t>StormSim workflow to call for project. (1 - StormSim:PROS, 2- StormSim:EVA, 3- StormSim:MCS-LC)</t>
   </si>
   <si>
-    <t>StormSim-LCS-Rubblemound</t>
+    <t>StormSim-PROS</t>
   </si>
 </sst>
 </file>
@@ -1602,7 +1602,7 @@
         <v>10</v>
       </c>
       <c r="D12" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F12" s="30" t="s">
         <v>139</v>

</xml_diff>

<commit_message>
Implementing peaks/timeseries switch accross workflows
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8A7FE69-E863-4A7C-ACFA-6B88AAF10BF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{638ED8CE-F202-422C-8219-B519E938BAFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-285" yWindow="2445" windowWidth="29145" windowHeight="16815" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
+    <workbookView xWindow="2100" yWindow="4065" windowWidth="29145" windowHeight="16815" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
   <sheets>
     <sheet name="James_Island_Midbay" sheetId="1" r:id="rId1"/>
@@ -577,9 +577,6 @@
     <t>StormSim workflow to call for project. (1 - StormSim:PROS, 2- StormSim:EVA, 3- StormSim:MCS-LC)</t>
   </si>
   <si>
-    <t>StormSim-PROS</t>
-  </si>
-  <si>
     <t>Include forcing peaks files as part of the analysis. (0/1)</t>
   </si>
   <si>
@@ -605,6 +602,9 @@
   </si>
   <si>
     <t>create_whp</t>
+  </si>
+  <si>
+    <t>StormSim-MCS-LC</t>
   </si>
 </sst>
 </file>
@@ -1461,7 +1461,7 @@
         <v>10</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="F5" s="49" t="s">
         <v>135</v>
@@ -1539,7 +1539,7 @@
         <v>10</v>
       </c>
       <c r="D8" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F8" s="17" t="s">
         <v>131</v>
@@ -1672,10 +1672,10 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C14" s="16" t="s">
         <v>10</v>
@@ -1701,7 +1701,7 @@
         <v>109</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C15" s="16" t="s">
         <v>10</v>
@@ -1724,10 +1724,10 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>10</v>
@@ -1742,10 +1742,10 @@
     </row>
     <row r="17" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="17" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C17" s="19" t="s">
         <v>10</v>
@@ -1842,10 +1842,10 @@
         <v>1</v>
       </c>
       <c r="F21" s="17" t="s">
+        <v>184</v>
+      </c>
+      <c r="G21" s="18" t="s">
         <v>185</v>
-      </c>
-      <c r="G21" s="18" t="s">
-        <v>186</v>
       </c>
       <c r="H21" s="19" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
Sorting bugs related to peaks/timeseries switch
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{638ED8CE-F202-422C-8219-B519E938BAFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC32CFE8-59EC-4F00-93AC-78096236B513}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2100" yWindow="4065" windowWidth="29145" windowHeight="16815" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
@@ -604,7 +604,7 @@
     <t>create_whp</t>
   </si>
   <si>
-    <t>StormSim-MCS-LC</t>
+    <t>StormSim-PROS-Timeseries</t>
   </si>
 </sst>
 </file>
@@ -1539,7 +1539,7 @@
         <v>10</v>
       </c>
       <c r="D8" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F8" s="17" t="s">
         <v>131</v>

</xml_diff>

<commit_message>
referencing elevations to datum 0
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26227"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC32CFE8-59EC-4F00-93AC-78096236B513}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9487E562-8454-4F8E-909B-831D03E009CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2100" yWindow="4065" windowWidth="29145" windowHeight="16815" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
+    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" activeTab="3" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
   <sheets>
     <sheet name="James_Island_Midbay" sheetId="1" r:id="rId1"/>
     <sheet name="NAE_Structure_Inputs" sheetId="3" r:id="rId2"/>
     <sheet name="NAE_Structure" sheetId="2" r:id="rId3"/>
+    <sheet name="TIming" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="250">
   <si>
     <t>StormSim Project General Inputs</t>
   </si>
@@ -604,13 +605,199 @@
     <t>create_whp</t>
   </si>
   <si>
-    <t>StormSim-PROS-Timeseries</t>
+    <t>Berm Elevation (Negative Below Datum Zero)</t>
+  </si>
+  <si>
+    <t>Crest Elevation/Top of Wall Elevation</t>
+  </si>
+  <si>
+    <t>Mound Toe Elevation (Negative Below Datum Zero)</t>
+  </si>
+  <si>
+    <t>wall_botttom_elevation</t>
+  </si>
+  <si>
+    <t>Bottom of Wall Elevation (Applies to wall type structures)</t>
+  </si>
+  <si>
+    <t>Mound/Berm Seaward Slope</t>
+  </si>
+  <si>
+    <t>Mound Landward Slope</t>
+  </si>
+  <si>
+    <t>[m]</t>
+  </si>
+  <si>
+    <t>[kg]</t>
+  </si>
+  <si>
+    <t>[kg/m^3]</t>
+  </si>
+  <si>
+    <t>[m^3/s/m]</t>
+  </si>
+  <si>
+    <t>[N/m^2]</t>
+  </si>
+  <si>
+    <t>[deg]</t>
+  </si>
+  <si>
+    <t>Wall Seaward Slope (Same Slope Is Assumed For Landward Slope)</t>
+  </si>
+  <si>
+    <t>StormSim-PROS</t>
+  </si>
+  <si>
+    <t>berm_slope</t>
+  </si>
+  <si>
+    <t>Midbay</t>
+  </si>
+  <si>
+    <t>Response Base</t>
+  </si>
+  <si>
+    <t>RB1 + RB3 w WLP &amp; WHP</t>
+  </si>
+  <si>
+    <t>Step #</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set-up Environment </t>
+  </si>
+  <si>
+    <t>CHS Data Formater</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create Project Forcing </t>
+  </si>
+  <si>
+    <t>Create Structure Geometry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Call Uncertainty Engine </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Call Project Forcing Adjsuter </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Call Project Responses </t>
+  </si>
+  <si>
+    <t>Time [s]</t>
+  </si>
+  <si>
+    <t>Total Time</t>
+  </si>
+  <si>
+    <t>(Processed 1031 TC storms + 100 XCs)</t>
+  </si>
+  <si>
+    <t>Time [min]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rubble mound </t>
+  </si>
+  <si>
+    <t>responses</t>
+  </si>
+  <si>
+    <t>SWL</t>
+  </si>
+  <si>
+    <t>Hm0</t>
+  </si>
+  <si>
+    <t>Tp</t>
+  </si>
+  <si>
+    <t>q</t>
+  </si>
+  <si>
+    <t>R2p</t>
+  </si>
+  <si>
+    <t>Dn50</t>
+  </si>
+  <si>
+    <t>P1</t>
+  </si>
+  <si>
+    <t>P2</t>
+  </si>
+  <si>
+    <t>P3</t>
+  </si>
+  <si>
+    <t>Nappe</t>
+  </si>
+  <si>
+    <t>Time Per Dataset (Peak Maxima , Peak WLP, Peak WHP &amp; RB3</t>
+  </si>
+  <si>
+    <t>StormSim Library Stress Testing</t>
+  </si>
+  <si>
+    <t>Computational Kernel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Response Base </t>
+  </si>
+  <si>
+    <t>Workflow</t>
+  </si>
+  <si>
+    <t>PROS</t>
+  </si>
+  <si>
+    <t>Structure Type</t>
+  </si>
+  <si>
+    <t>Rubblemound</t>
+  </si>
+  <si>
+    <t>Use Peaks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Use Timeseries </t>
+  </si>
+  <si>
+    <t>WLP &amp; WHP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rand Tides </t>
+  </si>
+  <si>
+    <t>SLR</t>
+  </si>
+  <si>
+    <t>Depth Limitation</t>
+  </si>
+  <si>
+    <t>Storm Sampling</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>Time Per Response</t>
+  </si>
+  <si>
+    <t>secs</t>
+  </si>
+  <si>
+    <t>Mins</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.000"/>
+  </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -654,7 +841,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -712,6 +899,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -917,7 +1110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1032,6 +1225,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1346,7 +1545,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51D29750-2AFD-4BF7-A911-1DC4ADC0FD7A}">
-  <dimension ref="A1:I70"/>
+  <dimension ref="A1:I72"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52.5703125" customWidth="1"/>
@@ -1418,7 +1617,7 @@
         <v>125</v>
       </c>
       <c r="H3" s="13" t="s">
-        <v>40</v>
+        <v>195</v>
       </c>
       <c r="I3" s="13">
         <v>0.33979999999999999</v>
@@ -1444,7 +1643,7 @@
         <v>126</v>
       </c>
       <c r="H4" s="13" t="s">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="I4" s="13">
         <v>0.38219999999999998</v>
@@ -1461,7 +1660,7 @@
         <v>10</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>188</v>
+        <v>202</v>
       </c>
       <c r="F5" s="49" t="s">
         <v>135</v>
@@ -1470,7 +1669,7 @@
         <v>127</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>40</v>
+        <v>195</v>
       </c>
       <c r="I5" s="13">
         <v>0.3</v>
@@ -1496,7 +1695,7 @@
         <v>128</v>
       </c>
       <c r="H6" s="13" t="s">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="I6" s="13">
         <v>0.3</v>
@@ -1522,7 +1721,7 @@
         <v>130</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>10</v>
+        <v>200</v>
       </c>
       <c r="I7" s="2">
         <v>0</v>
@@ -1638,7 +1837,7 @@
         <v>54</v>
       </c>
       <c r="H12" s="16" t="s">
-        <v>40</v>
+        <v>195</v>
       </c>
       <c r="I12" s="2">
         <v>0.5</v>
@@ -1664,7 +1863,7 @@
         <v>64</v>
       </c>
       <c r="H13" s="31" t="s">
-        <v>65</v>
+        <v>199</v>
       </c>
       <c r="I13" s="2">
         <v>0.43</v>
@@ -1681,7 +1880,7 @@
         <v>10</v>
       </c>
       <c r="D14" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F14" s="14" t="s">
         <v>115</v>
@@ -1690,7 +1889,7 @@
         <v>57</v>
       </c>
       <c r="H14" s="16" t="s">
-        <v>58</v>
+        <v>198</v>
       </c>
       <c r="I14" s="2">
         <v>0.78</v>
@@ -1716,7 +1915,7 @@
         <v>61</v>
       </c>
       <c r="H15" s="19" t="s">
-        <v>40</v>
+        <v>195</v>
       </c>
       <c r="I15" s="3">
         <v>0.13</v>
@@ -1984,7 +2183,7 @@
         <v>39</v>
       </c>
       <c r="H27" s="16" t="s">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="I27" s="2">
         <v>0</v>
@@ -2008,7 +2207,7 @@
         <v>43</v>
       </c>
       <c r="H28" s="19" t="s">
-        <v>40</v>
+        <v>195</v>
       </c>
       <c r="I28" s="3">
         <v>1</v>
@@ -2141,10 +2340,10 @@
         <v>78</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>113</v>
+        <v>189</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>10</v>
+        <v>195</v>
       </c>
       <c r="D36" s="1">
         <v>1.2320122</v>
@@ -2158,7 +2357,7 @@
         <v>114</v>
       </c>
       <c r="C37" s="16" t="s">
-        <v>10</v>
+        <v>195</v>
       </c>
       <c r="D37" s="2">
         <v>1.5243902</v>
@@ -2169,10 +2368,10 @@
         <v>80</v>
       </c>
       <c r="B38" s="15" t="s">
-        <v>81</v>
+        <v>190</v>
       </c>
       <c r="C38" s="16" t="s">
-        <v>40</v>
+        <v>195</v>
       </c>
       <c r="D38" s="2">
         <v>-1.5969511999999999</v>
@@ -2180,24 +2379,24 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
-        <v>82</v>
+        <v>191</v>
       </c>
       <c r="B39" s="15" t="s">
-        <v>83</v>
+        <v>192</v>
       </c>
       <c r="C39" s="16" t="s">
-        <v>10</v>
+        <v>195</v>
       </c>
       <c r="D39" s="2">
-        <v>1.5</v>
+        <v>-0.95799999999999996</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B40" s="15" t="s">
-        <v>85</v>
+        <v>193</v>
       </c>
       <c r="C40" s="16" t="s">
         <v>10</v>
@@ -2207,231 +2406,259 @@
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A41" s="39" t="s">
+      <c r="A41" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="B41" s="15" t="s">
+        <v>194</v>
+      </c>
+      <c r="C41" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D41" s="2">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A42" s="39" t="s">
         <v>118</v>
       </c>
-      <c r="B41" s="39" t="s">
+      <c r="B42" s="39" t="s">
         <v>119</v>
       </c>
-      <c r="C41" s="45" t="s">
-        <v>10</v>
-      </c>
-      <c r="D41" s="46">
+      <c r="C42" s="45" t="s">
+        <v>200</v>
+      </c>
+      <c r="D42" s="46">
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A42" s="14" t="s">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A43" s="14" t="s">
+        <v>203</v>
+      </c>
+      <c r="B43" s="15" t="s">
+        <v>201</v>
+      </c>
+      <c r="C43" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D43" s="2">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A44" s="14" t="s">
         <v>120</v>
       </c>
-      <c r="B42" s="14" t="s">
+      <c r="B44" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="C42" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D42" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="38" t="s">
+      <c r="C44" s="16" t="s">
+        <v>195</v>
+      </c>
+      <c r="D44" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="38" t="s">
         <v>121</v>
       </c>
-      <c r="B43" s="38" t="s">
-        <v>123</v>
-      </c>
-      <c r="C43" s="43" t="s">
-        <v>10</v>
-      </c>
-      <c r="D43" s="44">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A44" s="34"/>
-      <c r="B44" s="34"/>
-      <c r="C44" s="34"/>
-      <c r="D44" s="34"/>
-    </row>
-    <row r="45" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="36" t="s">
+      <c r="B45" s="38" t="s">
+        <v>188</v>
+      </c>
+      <c r="C45" s="43" t="s">
+        <v>195</v>
+      </c>
+      <c r="D45" s="44">
+        <v>-0.82799999999999996</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A46" s="34"/>
+      <c r="B46" s="34"/>
+      <c r="C46" s="34"/>
+      <c r="D46" s="34"/>
+    </row>
+    <row r="47" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="36" t="s">
         <v>86</v>
       </c>
-      <c r="B45" s="37"/>
-      <c r="C45" s="37"/>
-      <c r="D45" s="37"/>
-    </row>
-    <row r="46" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="9" t="s">
+      <c r="B47" s="37"/>
+      <c r="C47" s="37"/>
+      <c r="D47" s="37"/>
+    </row>
+    <row r="48" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="B46" s="10" t="s">
+      <c r="B48" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C46" s="10" t="s">
+      <c r="C48" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="D46" s="10" t="s">
+      <c r="D48" s="10" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A47" s="11" t="s">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="B47" s="12" t="s">
+      <c r="B49" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="C47" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="D47" s="1">
+      <c r="C49" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D49" s="1">
         <v>1.65</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A48" s="14" t="s">
-        <v>89</v>
-      </c>
-      <c r="B48" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="C48" s="16" t="s">
-        <v>91</v>
-      </c>
-      <c r="D48" s="2">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="14" t="s">
-        <v>92</v>
-      </c>
-      <c r="B49" s="15" t="s">
-        <v>93</v>
-      </c>
-      <c r="C49" s="16" t="s">
-        <v>91</v>
-      </c>
-      <c r="D49" s="2">
-        <v>500</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="B50" s="15" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="C50" s="16" t="s">
-        <v>96</v>
+        <v>196</v>
       </c>
       <c r="D50" s="2">
-        <v>1027</v>
+        <v>500</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="14" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="B51" s="15" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="C51" s="16" t="s">
-        <v>99</v>
+        <v>196</v>
       </c>
       <c r="D51" s="2">
-        <v>0.4</v>
+        <v>500</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="14" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="B52" s="15" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="C52" s="16" t="s">
-        <v>10</v>
+        <v>197</v>
       </c>
       <c r="D52" s="2">
-        <v>20</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="14" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="B53" s="15" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="C53" s="16" t="s">
-        <v>10</v>
+        <v>99</v>
       </c>
       <c r="D53" s="2">
-        <v>20</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="B54" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="C54" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D54" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="B55" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="C55" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D55" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" s="14" t="s">
         <v>104</v>
       </c>
-      <c r="B54" s="15" t="s">
+      <c r="B56" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="C54" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D54" s="2">
+      <c r="C56" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D56" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="39" t="s">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" s="39" t="s">
         <v>106</v>
       </c>
-      <c r="B55" s="40" t="s">
+      <c r="B57" s="40" t="s">
         <v>107</v>
       </c>
-      <c r="C55" s="41" t="s">
-        <v>10</v>
-      </c>
-      <c r="D55" s="42">
+      <c r="C57" s="41" t="s">
+        <v>10</v>
+      </c>
+      <c r="D57" s="42">
         <v>2</v>
       </c>
     </row>
-    <row r="56" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="18" t="s">
+    <row r="58" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="B56" s="48" t="s">
+      <c r="B58" s="48" t="s">
         <v>124</v>
       </c>
-      <c r="C56" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D56" s="4">
+      <c r="C58" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D58" s="4">
         <v>2</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="37"/>
-      <c r="B57" s="37"/>
-      <c r="C57" s="37"/>
-      <c r="D57" s="37"/>
-    </row>
-    <row r="70" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B70" s="47"/>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="37"/>
+      <c r="B59" s="37"/>
+      <c r="C59" s="37"/>
+      <c r="D59" s="37"/>
+    </row>
+    <row r="72" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B72" s="47"/>
     </row>
   </sheetData>
   <sheetProtection formatColumns="0" selectLockedCells="1"/>
   <protectedRanges>
     <protectedRange sqref="I3:I6 I8 I12:I16 I25:I28 D15:D17 I32 D21:D32 I19:I20 D3:D6 D8:D13" name="Range1_1"/>
     <protectedRange sqref="D7 D14" name="Range1_1_1"/>
-    <protectedRange sqref="D36:D40" name="Range1_1_3"/>
-    <protectedRange sqref="D47:D56" name="Range1_1_4"/>
+    <protectedRange sqref="D43 D36:D41" name="Range1_1_3"/>
+    <protectedRange sqref="D49:D58" name="Range1_1_4"/>
   </protectedRanges>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -3620,4 +3847,349 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36F05AA9-AA83-414A-9BCA-9A7F3A47A337}">
+  <dimension ref="A1:G38"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19" customWidth="1"/>
+    <col min="6" max="6" width="11.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>204</v>
+      </c>
+      <c r="B1" t="s">
+        <v>205</v>
+      </c>
+      <c r="C1" t="s">
+        <v>206</v>
+      </c>
+      <c r="D1" t="s">
+        <v>219</v>
+      </c>
+      <c r="E1" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>207</v>
+      </c>
+      <c r="B3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s">
+        <v>215</v>
+      </c>
+      <c r="D3" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>0</v>
+      </c>
+      <c r="B4" t="s">
+        <v>208</v>
+      </c>
+      <c r="C4" s="54">
+        <v>0.66720000000000002</v>
+      </c>
+      <c r="D4" s="54">
+        <f>C4/60</f>
+        <v>1.112E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <f>A4+1</f>
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
+        <v>209</v>
+      </c>
+      <c r="C5" s="54">
+        <v>128.0189</v>
+      </c>
+      <c r="D5" s="54">
+        <f>C5/60</f>
+        <v>2.1336483333333334</v>
+      </c>
+      <c r="E5" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <f t="shared" ref="A6:A10" si="0">A5+1</f>
+        <v>2</v>
+      </c>
+      <c r="B6" t="s">
+        <v>210</v>
+      </c>
+      <c r="C6" s="54">
+        <v>1.8109999999999999</v>
+      </c>
+      <c r="D6" s="54">
+        <f t="shared" ref="D6:D11" si="1">C6/60</f>
+        <v>3.0183333333333333E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>211</v>
+      </c>
+      <c r="C7" s="54">
+        <v>0.56489999999999996</v>
+      </c>
+      <c r="D7" s="54">
+        <f t="shared" si="1"/>
+        <v>9.4149999999999998E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
+        <v>212</v>
+      </c>
+      <c r="C8" s="54">
+        <v>1.2150000000000001</v>
+      </c>
+      <c r="D8" s="54">
+        <f t="shared" si="1"/>
+        <v>2.0250000000000001E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="B9" t="s">
+        <v>213</v>
+      </c>
+      <c r="C9" s="54">
+        <v>15.2134</v>
+      </c>
+      <c r="D9" s="54">
+        <f t="shared" si="1"/>
+        <v>0.25355666666666665</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="B10" t="s">
+        <v>214</v>
+      </c>
+      <c r="C10" s="54">
+        <v>648.27599999999995</v>
+      </c>
+      <c r="D10" s="54">
+        <f t="shared" si="1"/>
+        <v>10.804599999999999</v>
+      </c>
+      <c r="E10" s="8">
+        <f>D10/4</f>
+        <v>2.7011499999999997</v>
+      </c>
+      <c r="F10" s="53">
+        <f>E10/7</f>
+        <v>0.3858785714285714</v>
+      </c>
+      <c r="G10" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="51" t="s">
+        <v>216</v>
+      </c>
+      <c r="B11" s="51"/>
+      <c r="C11" s="54">
+        <f>SUM(C4:C10)</f>
+        <v>795.76639999999998</v>
+      </c>
+      <c r="D11" s="54">
+        <f t="shared" si="1"/>
+        <v>13.262773333333334</v>
+      </c>
+      <c r="F11" s="53">
+        <f>F10*60</f>
+        <v>23.152714285714286</v>
+      </c>
+      <c r="G11" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>220</v>
+      </c>
+      <c r="E15" s="8"/>
+      <c r="F15" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="52" t="s">
+        <v>221</v>
+      </c>
+      <c r="E16" s="53"/>
+      <c r="F16" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="52" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="52" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="52" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="52" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="52" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>233</v>
+      </c>
+      <c r="B29" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>239</v>
+      </c>
+      <c r="B30" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>240</v>
+      </c>
+      <c r="B31" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>241</v>
+      </c>
+      <c r="B32" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>245</v>
+      </c>
+      <c r="B33" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>242</v>
+      </c>
+      <c r="B34" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>243</v>
+      </c>
+      <c r="B35" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>244</v>
+      </c>
+      <c r="B36" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>235</v>
+      </c>
+      <c r="B37" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>237</v>
+      </c>
+      <c r="B38" t="s">
+        <v>238</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A11:B11"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fixed several bugs related to data parsing and visualizations. Added new plot outputs for RB
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,15 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9487E562-8454-4F8E-909B-831D03E009CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5836873D-D7CD-4B9A-B51A-D0B9AC399DCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" activeTab="3" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
+    <workbookView xWindow="3645" yWindow="4065" windowWidth="29145" windowHeight="16815" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
   <sheets>
     <sheet name="James_Island_Midbay" sheetId="1" r:id="rId1"/>
-    <sheet name="NAE_Structure_Inputs" sheetId="3" r:id="rId2"/>
-    <sheet name="NAE_Structure" sheetId="2" r:id="rId3"/>
-    <sheet name="TIming" sheetId="4" r:id="rId4"/>
+    <sheet name="TIming" sheetId="4" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="215">
   <si>
     <t>StormSim Project General Inputs</t>
   </si>
@@ -86,9 +84,6 @@
     <t>Structure/Trasnsect ID</t>
   </si>
   <si>
-    <t>A-1</t>
-  </si>
-  <si>
     <t>mcs_nYears</t>
   </si>
   <si>
@@ -110,24 +105,12 @@
     <t>Project output datum. (Still not implemented. Used for plot title currently)</t>
   </si>
   <si>
-    <t>mcs_create_wlp</t>
-  </si>
-  <si>
-    <t>Create Water Level Priority Peaks Dataset (WLP) (0/1)</t>
-  </si>
-  <si>
     <t>storm_sampling</t>
   </si>
   <si>
     <t>Storm sampling scheme to use for project. (XC,TC or CC)</t>
   </si>
   <si>
-    <t>mcs_create_whp</t>
-  </si>
-  <si>
-    <t>Create Wave Height Priority Peaks Dataset (WLP) (0/1)</t>
-  </si>
-  <si>
     <t>swl_slr</t>
   </si>
   <si>
@@ -161,9 +144,6 @@
     <t>Apply Cutoff Correction (0/1)</t>
   </si>
   <si>
-    <t>[m or ft]</t>
-  </si>
-  <si>
     <t>StormSim Project Forcing Data</t>
   </si>
   <si>
@@ -215,9 +195,6 @@
     <t>Overtopping Uncertainty</t>
   </si>
   <si>
-    <t>[m^3/s/m or ft^3/s/ft]</t>
-  </si>
-  <si>
     <t>chs_tc_hm0_peaks</t>
   </si>
   <si>
@@ -236,9 +213,6 @@
     <t>Surface Pressure (p1) Uncertainty' (Floodwalls Only)</t>
   </si>
   <si>
-    <t>[N/m^2 or lbf/ft^2]</t>
-  </si>
-  <si>
     <t>chs_xc_swl_peaks</t>
   </si>
   <si>
@@ -284,21 +258,12 @@
     <t>toe_elevation</t>
   </si>
   <si>
-    <t>Toe Bottom Elevation (Negative Below Datum Zero)</t>
-  </si>
-  <si>
     <t>seaside_slope</t>
   </si>
   <si>
-    <t>Seaside Slope</t>
-  </si>
-  <si>
     <t>leeside_slope</t>
   </si>
   <si>
-    <t>Leeside Slope</t>
-  </si>
-  <si>
     <t>Structure Properties</t>
   </si>
   <si>
@@ -314,9 +279,6 @@
     <t>Seaside Stone Mass</t>
   </si>
   <si>
-    <t>[kg or lb]</t>
-  </si>
-  <si>
     <t>leeside_mass</t>
   </si>
   <si>
@@ -329,9 +291,6 @@
     <t>Water Density</t>
   </si>
   <si>
-    <t>[kg/m^3 or lb/ft^3]</t>
-  </si>
-  <si>
     <t>cem_P</t>
   </si>
   <si>
@@ -371,18 +330,9 @@
     <t>use_timeseries</t>
   </si>
   <si>
-    <t>Include CHS timeseries as part of the analysis. (0/1)</t>
-  </si>
-  <si>
-    <t>cast_workflow</t>
-  </si>
-  <si>
     <t>Apply Depth Limitation To Waves (0/1)</t>
   </si>
   <si>
-    <t xml:space="preserve">Crest Elevation/Wall Height </t>
-  </si>
-  <si>
     <t>Crest Width/Wall Width</t>
   </si>
   <si>
@@ -410,9 +360,6 @@
     <t>Berm Width</t>
   </si>
   <si>
-    <t>Berm Elevation</t>
-  </si>
-  <si>
     <t>Roughness Coefficient, 2 for grass; 1 for concrete, asphalt, or closed blocks; 0.9 for basalt or placed revetment blocks; 0.8 for stepped structure; (rubble mound here! )</t>
   </si>
   <si>
@@ -470,9 +417,6 @@
     <t>chs_bias_file</t>
   </si>
   <si>
-    <t>StormSim workflow to call for project. (1 - StormSim:PROS, 2- StormSim:MCS, 3- StormSim: MCS/CSR, 4- StormSim: EVA (SST + JPM)</t>
-  </si>
-  <si>
     <t>tide_file</t>
   </si>
   <si>
@@ -485,54 +429,9 @@
     <t>NAVD</t>
   </si>
   <si>
-    <t xml:space="preserve">Given </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Structure Type </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Crest Width </t>
-  </si>
-  <si>
-    <t>ft</t>
-  </si>
-  <si>
-    <t>Crest Elevation</t>
-  </si>
-  <si>
-    <t>ft, NAVD88</t>
-  </si>
-  <si>
-    <t>Toe Elevation</t>
-  </si>
-  <si>
-    <t>Side Slope</t>
-  </si>
-  <si>
-    <t>Coverage (RipRap)</t>
-  </si>
-  <si>
-    <t>NAVD88 to MSL</t>
-  </si>
-  <si>
-    <t>Spatially Varying Uncertainty (+/-): 0.298 US_ft</t>
-  </si>
-  <si>
-    <t>How shoud we account for this ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Convert Datums And Units </t>
-  </si>
-  <si>
     <t>m</t>
   </si>
   <si>
-    <t>m, MSL</t>
-  </si>
-  <si>
-    <t>CHSFileDownload_2023-02-23_11-31-35.zip</t>
-  </si>
-  <si>
     <t>chs_sp_depth</t>
   </si>
   <si>
@@ -554,12 +453,6 @@
     <t>pros_use_aep</t>
   </si>
   <si>
-    <t>NAE_Structure</t>
-  </si>
-  <si>
-    <t>C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\CO-OPS_8638660_MSL_m_Tidal_Pred_1_year.csv</t>
-  </si>
-  <si>
     <t>case_name</t>
   </si>
   <si>
@@ -569,9 +462,6 @@
     <t>James_Island</t>
   </si>
   <si>
-    <t>Midbay_v2</t>
-  </si>
-  <si>
     <t>workflow</t>
   </si>
   <si>
@@ -614,9 +504,6 @@
     <t>Mound Toe Elevation (Negative Below Datum Zero)</t>
   </si>
   <si>
-    <t>wall_botttom_elevation</t>
-  </si>
-  <si>
     <t>Bottom of Wall Elevation (Applies to wall type structures)</t>
   </si>
   <si>
@@ -647,9 +534,6 @@
     <t>Wall Seaward Slope (Same Slope Is Assumed For Landward Slope)</t>
   </si>
   <si>
-    <t>StormSim-PROS</t>
-  </si>
-  <si>
     <t>berm_slope</t>
   </si>
   <si>
@@ -789,6 +673,15 @@
   </si>
   <si>
     <t>Mins</t>
+  </si>
+  <si>
+    <t>wall_bottom_elevation</t>
+  </si>
+  <si>
+    <t>Transect_001</t>
+  </si>
+  <si>
+    <t>Alternative_001</t>
   </si>
 </sst>
 </file>
@@ -909,7 +802,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -1106,11 +999,84 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1222,15 +1188,29 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1565,7 +1545,7 @@
       <c r="C1" s="6"/>
       <c r="D1" s="6"/>
       <c r="F1" s="32" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="G1" s="33"/>
       <c r="H1" s="33"/>
@@ -1608,16 +1588,16 @@
         <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>176</v>
+        <v>140</v>
       </c>
       <c r="F3" s="49" t="s">
-        <v>132</v>
+        <v>115</v>
       </c>
       <c r="G3" s="49" t="s">
-        <v>125</v>
+        <v>108</v>
       </c>
       <c r="H3" s="13" t="s">
-        <v>195</v>
+        <v>158</v>
       </c>
       <c r="I3" s="13">
         <v>0.33979999999999999</v>
@@ -1634,13 +1614,13 @@
         <v>10</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>175</v>
+        <v>213</v>
       </c>
       <c r="F4" s="49" t="s">
-        <v>133</v>
+        <v>116</v>
       </c>
       <c r="G4" s="49" t="s">
-        <v>126</v>
+        <v>109</v>
       </c>
       <c r="H4" s="13" t="s">
         <v>10</v>
@@ -1651,25 +1631,25 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>173</v>
+        <v>138</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>174</v>
+        <v>139</v>
       </c>
       <c r="C5" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>202</v>
+        <v>214</v>
       </c>
       <c r="F5" s="49" t="s">
-        <v>135</v>
+        <v>118</v>
       </c>
       <c r="G5" s="49" t="s">
-        <v>127</v>
+        <v>110</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>195</v>
+        <v>158</v>
       </c>
       <c r="I5" s="13">
         <v>0.3</v>
@@ -1677,22 +1657,22 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="15" t="s">
-        <v>22</v>
-      </c>
       <c r="C6" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>147</v>
+        <v>129</v>
       </c>
       <c r="F6" s="49" t="s">
-        <v>134</v>
+        <v>117</v>
       </c>
       <c r="G6" s="49" t="s">
-        <v>128</v>
+        <v>111</v>
       </c>
       <c r="H6" s="13" t="s">
         <v>10</v>
@@ -1703,25 +1683,25 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="C7" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>166</v>
+        <v>133</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>136</v>
+        <v>119</v>
       </c>
       <c r="G7" s="15" t="s">
-        <v>130</v>
+        <v>113</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>200</v>
+        <v>163</v>
       </c>
       <c r="I7" s="2">
         <v>0</v>
@@ -1729,10 +1709,10 @@
     </row>
     <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="14" t="s">
-        <v>177</v>
+        <v>141</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>178</v>
+        <v>142</v>
       </c>
       <c r="C8" s="16" t="s">
         <v>10</v>
@@ -1741,13 +1721,13 @@
         <v>1</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>131</v>
+        <v>114</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>129</v>
+        <v>112</v>
       </c>
       <c r="H8" s="19" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="I8" s="3">
         <v>0</v>
@@ -1755,10 +1735,10 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="15" t="s">
         <v>19</v>
-      </c>
-      <c r="B9" s="15" t="s">
-        <v>20</v>
       </c>
       <c r="C9" s="16" t="s">
         <v>10</v>
@@ -1773,19 +1753,19 @@
     </row>
     <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="14" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C10" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="F10" s="26" t="s">
-        <v>137</v>
+        <v>120</v>
       </c>
       <c r="G10" s="27"/>
       <c r="H10" s="27"/>
@@ -1793,10 +1773,10 @@
     </row>
     <row r="11" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="14" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="C11" s="16" t="s">
         <v>10</v>
@@ -1819,25 +1799,25 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>144</v>
+        <v>126</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>145</v>
+        <v>127</v>
       </c>
       <c r="C12" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>167</v>
+        <v>134</v>
       </c>
       <c r="F12" s="30" t="s">
-        <v>139</v>
+        <v>122</v>
       </c>
       <c r="G12" s="15" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="H12" s="16" t="s">
-        <v>195</v>
+        <v>158</v>
       </c>
       <c r="I12" s="2">
         <v>0.5</v>
@@ -1845,10 +1825,10 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>138</v>
+        <v>121</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>112</v>
+        <v>97</v>
       </c>
       <c r="C13" s="16" t="s">
         <v>10</v>
@@ -1857,13 +1837,13 @@
         <v>1</v>
       </c>
       <c r="F13" s="30" t="s">
-        <v>140</v>
+        <v>123</v>
       </c>
       <c r="G13" s="15" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="H13" s="31" t="s">
-        <v>199</v>
+        <v>162</v>
       </c>
       <c r="I13" s="2">
         <v>0.43</v>
@@ -1871,10 +1851,10 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>181</v>
+        <v>145</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>179</v>
+        <v>143</v>
       </c>
       <c r="C14" s="16" t="s">
         <v>10</v>
@@ -1883,13 +1863,13 @@
         <v>1</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>115</v>
+        <v>99</v>
       </c>
       <c r="G14" s="15" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="H14" s="16" t="s">
-        <v>198</v>
+        <v>161</v>
       </c>
       <c r="I14" s="2">
         <v>0.78</v>
@@ -1897,10 +1877,10 @@
     </row>
     <row r="15" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="14" t="s">
-        <v>109</v>
+        <v>96</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>180</v>
+        <v>144</v>
       </c>
       <c r="C15" s="16" t="s">
         <v>10</v>
@@ -1909,13 +1889,13 @@
         <v>1</v>
       </c>
       <c r="F15" s="17" t="s">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="G15" s="18" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="H15" s="19" t="s">
-        <v>195</v>
+        <v>158</v>
       </c>
       <c r="I15" s="3">
         <v>0.13</v>
@@ -1923,10 +1903,10 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>186</v>
+        <v>150</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>183</v>
+        <v>147</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>10</v>
@@ -1941,10 +1921,10 @@
     </row>
     <row r="17" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="17" t="s">
-        <v>187</v>
+        <v>151</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>182</v>
+        <v>146</v>
       </c>
       <c r="C17" s="19" t="s">
         <v>10</v>
@@ -1983,7 +1963,7 @@
     </row>
     <row r="19" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="24" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B19" s="25"/>
       <c r="C19" s="25"/>
@@ -1998,7 +1978,7 @@
         <v>10</v>
       </c>
       <c r="I19" s="1">
-        <v>9</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2015,13 +1995,13 @@
         <v>6</v>
       </c>
       <c r="F20" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="G20" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="G20" s="15" t="s">
+      <c r="H20" s="16" t="s">
         <v>17</v>
-      </c>
-      <c r="H20" s="16" t="s">
-        <v>18</v>
       </c>
       <c r="I20" s="2">
         <v>50</v>
@@ -2029,22 +2009,22 @@
     </row>
     <row r="21" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="11" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="C21" s="28" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="D21" s="1">
         <v>1</v>
       </c>
       <c r="F21" s="17" t="s">
-        <v>184</v>
+        <v>148</v>
       </c>
       <c r="G21" s="18" t="s">
-        <v>185</v>
+        <v>149</v>
       </c>
       <c r="H21" s="19" t="s">
         <v>10</v>
@@ -2055,13 +2035,13 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>164</v>
+        <v>131</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>165</v>
+        <v>132</v>
       </c>
       <c r="C22" s="28" t="s">
-        <v>161</v>
+        <v>130</v>
       </c>
       <c r="D22" s="1">
         <v>5</v>
@@ -2073,19 +2053,19 @@
     </row>
     <row r="23" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="11" t="s">
-        <v>142</v>
+        <v>125</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>141</v>
+        <v>124</v>
       </c>
       <c r="C23" s="28" t="s">
         <v>10</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>146</v>
+        <v>128</v>
       </c>
       <c r="F23" s="20" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="G23" s="21"/>
       <c r="H23" s="21"/>
@@ -2093,16 +2073,16 @@
     </row>
     <row r="24" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="14" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="C24" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>168</v>
+        <v>135</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>3</v>
@@ -2119,20 +2099,20 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="C25" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D25" s="2"/>
       <c r="F25" s="11" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="G25" s="12" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="H25" s="13" t="s">
         <v>10</v>
@@ -2143,20 +2123,20 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="C26" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D26" s="2"/>
       <c r="F26" s="14" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="G26" s="15" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H26" s="16" t="s">
         <v>10</v>
@@ -2167,20 +2147,20 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="C27" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D27" s="2"/>
       <c r="F27" s="14" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="G27" s="15" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="H27" s="16" t="s">
         <v>10</v>
@@ -2191,23 +2171,23 @@
     </row>
     <row r="28" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="14" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="C28" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D28" s="2"/>
       <c r="F28" s="17" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="G28" s="18" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="H28" s="19" t="s">
-        <v>195</v>
+        <v>158</v>
       </c>
       <c r="I28" s="3">
         <v>1</v>
@@ -2215,10 +2195,10 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="B29" s="15" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="C29" s="16" t="s">
         <v>10</v>
@@ -2231,17 +2211,17 @@
     </row>
     <row r="30" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="14" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="B30" s="15" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="C30" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D30" s="2"/>
       <c r="F30" s="26" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="G30" s="27"/>
       <c r="H30" s="27"/>
@@ -2249,10 +2229,10 @@
     </row>
     <row r="31" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="14" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="C31" s="16" t="s">
         <v>10</v>
@@ -2273,20 +2253,20 @@
     </row>
     <row r="32" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="17" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="B32" s="18" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="C32" s="19" t="s">
         <v>10</v>
       </c>
       <c r="D32" s="3"/>
       <c r="F32" s="29" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="G32" s="12" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H32" s="13" t="s">
         <v>10</v>
@@ -2301,10 +2281,10 @@
       <c r="C33" s="25"/>
       <c r="D33" s="25"/>
       <c r="F33" s="17" t="s">
-        <v>170</v>
+        <v>137</v>
       </c>
       <c r="G33" s="18" t="s">
-        <v>169</v>
+        <v>136</v>
       </c>
       <c r="H33" s="19" t="s">
         <v>10</v>
@@ -2315,7 +2295,7 @@
     </row>
     <row r="34" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="34" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="B34" s="35"/>
       <c r="C34" s="35"/>
@@ -2332,18 +2312,18 @@
         <v>5</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="11" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>189</v>
+        <v>153</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>195</v>
+        <v>158</v>
       </c>
       <c r="D36" s="1">
         <v>1.2320122</v>
@@ -2351,13 +2331,13 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>114</v>
+        <v>98</v>
       </c>
       <c r="C37" s="16" t="s">
-        <v>195</v>
+        <v>158</v>
       </c>
       <c r="D37" s="2">
         <v>1.5243902</v>
@@ -2365,13 +2345,13 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="B38" s="15" t="s">
-        <v>190</v>
+        <v>154</v>
       </c>
       <c r="C38" s="16" t="s">
-        <v>195</v>
+        <v>158</v>
       </c>
       <c r="D38" s="2">
         <v>-1.5969511999999999</v>
@@ -2379,13 +2359,13 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
-        <v>191</v>
+        <v>212</v>
       </c>
       <c r="B39" s="15" t="s">
-        <v>192</v>
+        <v>155</v>
       </c>
       <c r="C39" s="16" t="s">
-        <v>195</v>
+        <v>158</v>
       </c>
       <c r="D39" s="2">
         <v>-0.95799999999999996</v>
@@ -2393,10 +2373,10 @@
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="B40" s="15" t="s">
-        <v>193</v>
+        <v>156</v>
       </c>
       <c r="C40" s="16" t="s">
         <v>10</v>
@@ -2407,10 +2387,10 @@
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="14" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="B41" s="15" t="s">
-        <v>194</v>
+        <v>157</v>
       </c>
       <c r="C41" s="16" t="s">
         <v>10</v>
@@ -2421,13 +2401,13 @@
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="39" t="s">
-        <v>118</v>
+        <v>102</v>
       </c>
       <c r="B42" s="39" t="s">
-        <v>119</v>
+        <v>103</v>
       </c>
       <c r="C42" s="45" t="s">
-        <v>200</v>
+        <v>163</v>
       </c>
       <c r="D42" s="46">
         <v>0</v>
@@ -2435,10 +2415,10 @@
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
-        <v>203</v>
+        <v>165</v>
       </c>
       <c r="B43" s="15" t="s">
-        <v>201</v>
+        <v>164</v>
       </c>
       <c r="C43" s="16" t="s">
         <v>10</v>
@@ -2449,27 +2429,27 @@
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
-        <v>120</v>
+        <v>104</v>
       </c>
       <c r="B44" s="14" t="s">
-        <v>122</v>
+        <v>106</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>195</v>
+        <v>158</v>
       </c>
       <c r="D44" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="38" t="s">
-        <v>121</v>
+        <v>105</v>
       </c>
       <c r="B45" s="38" t="s">
-        <v>188</v>
+        <v>152</v>
       </c>
       <c r="C45" s="43" t="s">
-        <v>195</v>
+        <v>158</v>
       </c>
       <c r="D45" s="44">
         <v>-0.82799999999999996</v>
@@ -2483,7 +2463,7 @@
     </row>
     <row r="47" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="36" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="B47" s="37"/>
       <c r="C47" s="37"/>
@@ -2500,15 +2480,15 @@
         <v>5</v>
       </c>
       <c r="D48" s="10" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="11" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="B49" s="12" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="C49" s="13" t="s">
         <v>10</v>
@@ -2519,13 +2499,13 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="B50" s="15" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="C50" s="16" t="s">
-        <v>196</v>
+        <v>159</v>
       </c>
       <c r="D50" s="2">
         <v>500</v>
@@ -2533,13 +2513,13 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="14" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="B51" s="15" t="s">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="C51" s="16" t="s">
-        <v>196</v>
+        <v>159</v>
       </c>
       <c r="D51" s="2">
         <v>500</v>
@@ -2547,13 +2527,13 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="14" t="s">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="B52" s="15" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="C52" s="16" t="s">
-        <v>197</v>
+        <v>160</v>
       </c>
       <c r="D52" s="2">
         <v>1027</v>
@@ -2561,13 +2541,13 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="14" t="s">
-        <v>97</v>
+        <v>84</v>
       </c>
       <c r="B53" s="15" t="s">
-        <v>98</v>
+        <v>85</v>
       </c>
       <c r="C53" s="16" t="s">
-        <v>99</v>
+        <v>86</v>
       </c>
       <c r="D53" s="2">
         <v>0.4</v>
@@ -2575,10 +2555,10 @@
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="14" t="s">
-        <v>100</v>
+        <v>87</v>
       </c>
       <c r="B54" s="15" t="s">
-        <v>101</v>
+        <v>88</v>
       </c>
       <c r="C54" s="16" t="s">
         <v>10</v>
@@ -2589,10 +2569,10 @@
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
-        <v>102</v>
+        <v>89</v>
       </c>
       <c r="B55" s="15" t="s">
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="C55" s="16" t="s">
         <v>10</v>
@@ -2603,10 +2583,10 @@
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="14" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="B56" s="15" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="C56" s="16" t="s">
         <v>10</v>
@@ -2617,10 +2597,10 @@
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="39" t="s">
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="B57" s="40" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="C57" s="41" t="s">
         <v>10</v>
@@ -2631,10 +2611,10 @@
     </row>
     <row r="58" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="18" t="s">
-        <v>117</v>
+        <v>101</v>
       </c>
       <c r="B58" s="48" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="C58" s="19" t="s">
         <v>10</v>
@@ -2666,1190 +2646,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9768969-90B5-4E8F-92CE-56AC3208C5A3}">
-  <dimension ref="A1:I66"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="79" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="92.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="171.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="28.42578125" customWidth="1"/>
-    <col min="7" max="7" width="50" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="46.140625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="F1" s="32" t="s">
-        <v>74</v>
-      </c>
-      <c r="G1" s="33"/>
-      <c r="H1" s="33"/>
-      <c r="I1" s="33"/>
-    </row>
-    <row r="2" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="F2" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="G2" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="H2" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="I2" s="10" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="F3" s="49" t="s">
-        <v>132</v>
-      </c>
-      <c r="G3" s="49" t="s">
-        <v>125</v>
-      </c>
-      <c r="H3" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="I3" s="13">
-        <v>0.33979999999999999</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F4" s="49" t="s">
-        <v>133</v>
-      </c>
-      <c r="G4" s="49" t="s">
-        <v>126</v>
-      </c>
-      <c r="H4" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="I4" s="13">
-        <v>0.38219999999999998</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" s="2">
-        <v>1</v>
-      </c>
-      <c r="F5" s="49" t="s">
-        <v>135</v>
-      </c>
-      <c r="G5" s="49" t="s">
-        <v>127</v>
-      </c>
-      <c r="H5" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="I5" s="13">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="B6" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="C6" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="F6" s="49" t="s">
-        <v>134</v>
-      </c>
-      <c r="G6" s="49" t="s">
-        <v>128</v>
-      </c>
-      <c r="H6" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="I6" s="13">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="B7" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="C7" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="F7" s="14" t="s">
-        <v>136</v>
-      </c>
-      <c r="G7" s="15" t="s">
-        <v>130</v>
-      </c>
-      <c r="H7" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="I7" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="C8" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D8" s="2">
-        <v>0</v>
-      </c>
-      <c r="F8" s="17" t="s">
-        <v>131</v>
-      </c>
-      <c r="G8" s="18" t="s">
-        <v>129</v>
-      </c>
-      <c r="H8" s="19" t="s">
-        <v>75</v>
-      </c>
-      <c r="I8" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="14" t="s">
-        <v>144</v>
-      </c>
-      <c r="B9" s="15" t="s">
-        <v>145</v>
-      </c>
-      <c r="C9" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="F9" s="33"/>
-      <c r="G9" s="33"/>
-      <c r="H9" s="33"/>
-      <c r="I9" s="33"/>
-    </row>
-    <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="14" t="s">
-        <v>138</v>
-      </c>
-      <c r="B10" s="15" t="s">
-        <v>112</v>
-      </c>
-      <c r="C10" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D10" s="2">
-        <v>1</v>
-      </c>
-      <c r="F10" s="26" t="s">
-        <v>137</v>
-      </c>
-      <c r="G10" s="27"/>
-      <c r="H10" s="27"/>
-      <c r="I10" s="27"/>
-    </row>
-    <row r="11" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="14" t="s">
-        <v>111</v>
-      </c>
-      <c r="B11" s="15" t="s">
-        <v>143</v>
-      </c>
-      <c r="C11" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D11" s="2">
-        <v>1</v>
-      </c>
-      <c r="F11" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="G11" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="H11" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="I11" s="10" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="17" t="s">
-        <v>34</v>
-      </c>
-      <c r="B12" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="C12" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="F12" s="30" t="s">
-        <v>139</v>
-      </c>
-      <c r="G12" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="H12" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="I12" s="2">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="6"/>
-      <c r="B13" s="22"/>
-      <c r="C13" s="23"/>
-      <c r="D13" s="23"/>
-      <c r="F13" s="30" t="s">
-        <v>140</v>
-      </c>
-      <c r="G13" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="H13" s="31" t="s">
-        <v>65</v>
-      </c>
-      <c r="I13" s="2">
-        <v>0.43</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="24" t="s">
-        <v>41</v>
-      </c>
-      <c r="B14" s="25"/>
-      <c r="C14" s="25"/>
-      <c r="D14" s="25"/>
-      <c r="F14" s="14" t="s">
-        <v>115</v>
-      </c>
-      <c r="G14" s="15" t="s">
-        <v>57</v>
-      </c>
-      <c r="H14" s="16" t="s">
-        <v>58</v>
-      </c>
-      <c r="I14" s="2">
-        <v>0.78</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B15" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="F15" s="17" t="s">
-        <v>116</v>
-      </c>
-      <c r="G15" s="18" t="s">
-        <v>61</v>
-      </c>
-      <c r="H15" s="19" t="s">
-        <v>40</v>
-      </c>
-      <c r="I15" s="3">
-        <v>0.13</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="14" t="s">
-        <v>109</v>
-      </c>
-      <c r="B16" s="15" t="s">
-        <v>110</v>
-      </c>
-      <c r="C16" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D16" s="2">
-        <v>1</v>
-      </c>
-      <c r="F16" s="27"/>
-      <c r="G16" s="27"/>
-      <c r="H16" s="27"/>
-      <c r="I16" s="27"/>
-    </row>
-    <row r="17" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="B17" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="C17" s="28" t="s">
-        <v>46</v>
-      </c>
-      <c r="D17" s="1">
-        <v>1</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="G17" s="8"/>
-      <c r="H17" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="I17" s="8" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="11" t="s">
-        <v>164</v>
-      </c>
-      <c r="B18" s="12" t="s">
-        <v>165</v>
-      </c>
-      <c r="C18" s="28" t="s">
-        <v>161</v>
-      </c>
-      <c r="D18" s="1">
-        <v>5</v>
-      </c>
-      <c r="F18" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="G18" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="H18" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="I18" s="10" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="11" t="s">
-        <v>142</v>
-      </c>
-      <c r="B19" s="12" t="s">
-        <v>141</v>
-      </c>
-      <c r="C19" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="F19" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="G19" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="H19" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="I19" s="1">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="14" t="s">
-        <v>48</v>
-      </c>
-      <c r="B20" s="15" t="s">
-        <v>49</v>
-      </c>
-      <c r="C20" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="F20" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G20" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="H20" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="I20" s="2">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="B21" s="15" t="s">
-        <v>53</v>
-      </c>
-      <c r="C21" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D21" s="2"/>
-      <c r="F21" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="G21" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="H21" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="I21" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="14" t="s">
-        <v>55</v>
-      </c>
-      <c r="B22" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="C22" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D22" s="2"/>
-      <c r="F22" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="G22" s="18" t="s">
-        <v>28</v>
-      </c>
-      <c r="H22" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="I22" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="B23" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="C23" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D23" s="2"/>
-      <c r="F23" s="8"/>
-      <c r="G23" s="8"/>
-      <c r="H23" s="8"/>
-      <c r="I23" s="8"/>
-    </row>
-    <row r="24" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="B24" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="C24" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D24" s="2"/>
-      <c r="F24" s="20" t="s">
-        <v>31</v>
-      </c>
-      <c r="G24" s="21"/>
-      <c r="H24" s="21"/>
-      <c r="I24" s="21"/>
-    </row>
-    <row r="25" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="B25" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="C25" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D25" s="2"/>
-      <c r="F25" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="G25" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="H25" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="I25" s="10" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="B26" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="C26" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D26" s="2"/>
-      <c r="F26" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="G26" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="H26" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="I26" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="14" t="s">
-        <v>70</v>
-      </c>
-      <c r="B27" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="C27" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D27" s="2"/>
-      <c r="F27" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="G27" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="H27" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="I27" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="B28" s="18" t="s">
-        <v>73</v>
-      </c>
-      <c r="C28" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D28" s="3"/>
-      <c r="F28" s="14" t="s">
-        <v>38</v>
-      </c>
-      <c r="G28" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="H28" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="I28" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="25"/>
-      <c r="B29" s="25"/>
-      <c r="C29" s="25"/>
-      <c r="D29" s="25"/>
-      <c r="F29" s="17" t="s">
-        <v>42</v>
-      </c>
-      <c r="G29" s="18" t="s">
-        <v>43</v>
-      </c>
-      <c r="H29" s="19" t="s">
-        <v>40</v>
-      </c>
-      <c r="I29" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B30" s="35"/>
-      <c r="C30" s="35"/>
-      <c r="D30" s="35"/>
-      <c r="F30" s="21"/>
-      <c r="G30" s="21"/>
-      <c r="H30" s="21"/>
-      <c r="I30" s="21"/>
-    </row>
-    <row r="31" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B31" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C31" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="D31" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="F31" s="26" t="s">
-        <v>47</v>
-      </c>
-      <c r="G31" s="27"/>
-      <c r="H31" s="27"/>
-      <c r="I31" s="27"/>
-    </row>
-    <row r="32" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="B32" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="C32" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="D32" s="1">
-        <f>NAE_Structure!B12</f>
-        <v>4.9590959999999997</v>
-      </c>
-      <c r="F32" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="G32" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="H32" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="I32" s="10" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="B33" s="15" t="s">
-        <v>114</v>
-      </c>
-      <c r="C33" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D33" s="2">
-        <f>NAE_Structure!B11</f>
-        <v>3.130296</v>
-      </c>
-      <c r="F33" s="29" t="s">
-        <v>50</v>
-      </c>
-      <c r="G33" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="H33" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="I33" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="B34" s="15" t="s">
-        <v>81</v>
-      </c>
-      <c r="C34" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="D34" s="2">
-        <f>NAE_Structure!B13*-1</f>
-        <v>-2.8254960000000002</v>
-      </c>
-      <c r="F34" s="17" t="s">
-        <v>170</v>
-      </c>
-      <c r="G34" s="18" t="s">
-        <v>169</v>
-      </c>
-      <c r="H34" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="I34" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A35" s="14" t="s">
-        <v>82</v>
-      </c>
-      <c r="B35" s="15" t="s">
-        <v>83</v>
-      </c>
-      <c r="C35" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D35" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="14" t="s">
-        <v>84</v>
-      </c>
-      <c r="B36" s="15" t="s">
-        <v>85</v>
-      </c>
-      <c r="C36" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D36" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A37" s="39" t="s">
-        <v>118</v>
-      </c>
-      <c r="B37" s="39" t="s">
-        <v>119</v>
-      </c>
-      <c r="C37" s="45" t="s">
-        <v>10</v>
-      </c>
-      <c r="D37" s="46">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A38" s="14" t="s">
-        <v>120</v>
-      </c>
-      <c r="B38" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="C38" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D38" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="38" t="s">
-        <v>121</v>
-      </c>
-      <c r="B39" s="38" t="s">
-        <v>123</v>
-      </c>
-      <c r="C39" s="43" t="s">
-        <v>10</v>
-      </c>
-      <c r="D39" s="44">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A40" s="34"/>
-      <c r="B40" s="34"/>
-      <c r="C40" s="34"/>
-      <c r="D40" s="34"/>
-    </row>
-    <row r="41" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="36" t="s">
-        <v>86</v>
-      </c>
-      <c r="B41" s="37"/>
-      <c r="C41" s="37"/>
-      <c r="D41" s="37"/>
-    </row>
-    <row r="42" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B42" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C42" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="D42" s="10" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A43" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="B43" s="12" t="s">
-        <v>88</v>
-      </c>
-      <c r="C43" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="D43" s="1">
-        <v>1.65</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A44" s="14" t="s">
-        <v>89</v>
-      </c>
-      <c r="B44" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="C44" s="16" t="s">
-        <v>91</v>
-      </c>
-      <c r="D44" s="2">
-        <v>907.18</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A45" s="14" t="s">
-        <v>92</v>
-      </c>
-      <c r="B45" s="15" t="s">
-        <v>93</v>
-      </c>
-      <c r="C45" s="16" t="s">
-        <v>91</v>
-      </c>
-      <c r="D45" s="2">
-        <v>907.18</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A46" s="14" t="s">
-        <v>94</v>
-      </c>
-      <c r="B46" s="15" t="s">
-        <v>95</v>
-      </c>
-      <c r="C46" s="16" t="s">
-        <v>96</v>
-      </c>
-      <c r="D46" s="2">
-        <v>1027</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A47" s="14" t="s">
-        <v>97</v>
-      </c>
-      <c r="B47" s="15" t="s">
-        <v>98</v>
-      </c>
-      <c r="C47" s="16" t="s">
-        <v>99</v>
-      </c>
-      <c r="D47" s="2">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A48" s="14" t="s">
-        <v>100</v>
-      </c>
-      <c r="B48" s="15" t="s">
-        <v>101</v>
-      </c>
-      <c r="C48" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D48" s="2">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="B49" s="15" t="s">
-        <v>103</v>
-      </c>
-      <c r="C49" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D49" s="2">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="B50" s="15" t="s">
-        <v>105</v>
-      </c>
-      <c r="C50" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D50" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="39" t="s">
-        <v>106</v>
-      </c>
-      <c r="B51" s="40" t="s">
-        <v>107</v>
-      </c>
-      <c r="C51" s="41" t="s">
-        <v>10</v>
-      </c>
-      <c r="D51" s="42">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="18" t="s">
-        <v>117</v>
-      </c>
-      <c r="B52" s="48" t="s">
-        <v>124</v>
-      </c>
-      <c r="C52" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D52" s="4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="37"/>
-      <c r="B53" s="37"/>
-      <c r="C53" s="37"/>
-      <c r="D53" s="37"/>
-    </row>
-    <row r="66" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B66" s="47"/>
-    </row>
-  </sheetData>
-  <sheetProtection formatColumns="0" selectLockedCells="1"/>
-  <protectedRanges>
-    <protectedRange sqref="D32:D36 I3:I6 I8 D16:D28 I12:I16 I26:I29 I19:I22 D43:D52 I33 D3:D11" name="Range1_1"/>
-    <protectedRange sqref="D12" name="Range1_1_1"/>
-  </protectedRanges>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF7B9495-7AF2-49CC-975F-069DD3B5C2E2}">
-  <dimension ref="A1:D13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.140625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>149</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>150</v>
-      </c>
-      <c r="B3">
-        <v>10</v>
-      </c>
-      <c r="C3" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>152</v>
-      </c>
-      <c r="B4">
-        <v>16</v>
-      </c>
-      <c r="C4" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>154</v>
-      </c>
-      <c r="B5">
-        <v>9</v>
-      </c>
-      <c r="C5" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>155</v>
-      </c>
-      <c r="B6">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>156</v>
-      </c>
-      <c r="B7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>157</v>
-      </c>
-      <c r="B8">
-        <f>1.8-1.53</f>
-        <v>0.27</v>
-      </c>
-      <c r="C8" s="50" t="s">
-        <v>158</v>
-      </c>
-      <c r="D8" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>150</v>
-      </c>
-      <c r="B11">
-        <f>(B3+$B$8)*0.3048</f>
-        <v>3.130296</v>
-      </c>
-      <c r="C11" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>152</v>
-      </c>
-      <c r="B12">
-        <f t="shared" ref="B12:B13" si="0">(B4+$B$8)*0.3048</f>
-        <v>4.9590959999999997</v>
-      </c>
-      <c r="C12" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>154</v>
-      </c>
-      <c r="B13">
-        <f t="shared" si="0"/>
-        <v>2.8254960000000002</v>
-      </c>
-      <c r="C13" t="s">
-        <v>162</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36F05AA9-AA83-414A-9BCA-9A7F3A47A337}">
   <dimension ref="A1:G38"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3863,145 +2659,146 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>204</v>
+        <v>166</v>
       </c>
       <c r="B1" t="s">
-        <v>205</v>
+        <v>167</v>
       </c>
       <c r="C1" t="s">
-        <v>206</v>
+        <v>168</v>
       </c>
       <c r="D1" t="s">
-        <v>219</v>
+        <v>181</v>
       </c>
       <c r="E1" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>207</v>
-      </c>
-      <c r="B3" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="54" t="s">
+        <v>169</v>
+      </c>
+      <c r="B3" s="54" t="s">
         <v>4</v>
       </c>
-      <c r="C3" t="s">
-        <v>215</v>
-      </c>
-      <c r="D3" t="s">
-        <v>218</v>
+      <c r="C3" s="54" t="s">
+        <v>177</v>
+      </c>
+      <c r="D3" s="58" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4">
+      <c r="A4" s="55">
         <v>0</v>
       </c>
-      <c r="B4" t="s">
-        <v>208</v>
-      </c>
-      <c r="C4" s="54">
+      <c r="B4" s="55" t="s">
+        <v>170</v>
+      </c>
+      <c r="C4" s="59">
         <v>0.66720000000000002</v>
       </c>
-      <c r="D4" s="54">
+      <c r="D4" s="62">
         <f>C4/60</f>
         <v>1.112E-2</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5">
+      <c r="A5" s="56">
         <f>A4+1</f>
         <v>1</v>
       </c>
-      <c r="B5" t="s">
-        <v>209</v>
-      </c>
-      <c r="C5" s="54">
+      <c r="B5" s="56" t="s">
+        <v>171</v>
+      </c>
+      <c r="C5" s="60">
         <v>128.0189</v>
       </c>
-      <c r="D5" s="54">
+      <c r="D5" s="60">
         <f>C5/60</f>
         <v>2.1336483333333334</v>
       </c>
       <c r="E5" t="s">
-        <v>217</v>
+        <v>179</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6">
+      <c r="A6" s="56">
         <f t="shared" ref="A6:A10" si="0">A5+1</f>
         <v>2</v>
       </c>
-      <c r="B6" t="s">
-        <v>210</v>
-      </c>
-      <c r="C6" s="54">
+      <c r="B6" s="56" t="s">
+        <v>172</v>
+      </c>
+      <c r="C6" s="60">
         <v>1.8109999999999999</v>
       </c>
-      <c r="D6" s="54">
+      <c r="D6" s="60">
         <f t="shared" ref="D6:D11" si="1">C6/60</f>
         <v>3.0183333333333333E-2</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7">
+      <c r="A7" s="56">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="B7" t="s">
-        <v>211</v>
-      </c>
-      <c r="C7" s="54">
+      <c r="B7" s="56" t="s">
+        <v>173</v>
+      </c>
+      <c r="C7" s="60">
         <v>0.56489999999999996</v>
       </c>
-      <c r="D7" s="54">
+      <c r="D7" s="60">
         <f t="shared" si="1"/>
         <v>9.4149999999999998E-3</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8">
+      <c r="A8" s="56">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="B8" t="s">
-        <v>212</v>
-      </c>
-      <c r="C8" s="54">
+      <c r="B8" s="56" t="s">
+        <v>174</v>
+      </c>
+      <c r="C8" s="60">
         <v>1.2150000000000001</v>
       </c>
-      <c r="D8" s="54">
+      <c r="D8" s="60">
         <f t="shared" si="1"/>
         <v>2.0250000000000001E-2</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9">
+      <c r="A9" s="56">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="B9" t="s">
-        <v>213</v>
-      </c>
-      <c r="C9" s="54">
+      <c r="B9" s="56" t="s">
+        <v>175</v>
+      </c>
+      <c r="C9" s="60">
         <v>15.2134</v>
       </c>
-      <c r="D9" s="54">
+      <c r="D9" s="60">
         <f t="shared" si="1"/>
         <v>0.25355666666666665</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10">
+    <row r="10" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="57">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="B10" t="s">
-        <v>214</v>
-      </c>
-      <c r="C10" s="54">
+      <c r="B10" s="57" t="s">
+        <v>176</v>
+      </c>
+      <c r="C10" s="61">
         <v>648.27599999999995</v>
       </c>
-      <c r="D10" s="54">
+      <c r="D10" s="61">
         <f t="shared" si="1"/>
         <v>10.804599999999999</v>
       </c>
@@ -4009,181 +2806,181 @@
         <f>D10/4</f>
         <v>2.7011499999999997</v>
       </c>
-      <c r="F10" s="53">
+      <c r="F10" s="51">
         <f>E10/7</f>
         <v>0.3858785714285714</v>
       </c>
       <c r="G10" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="51" t="s">
-        <v>216</v>
-      </c>
-      <c r="B11" s="51"/>
-      <c r="C11" s="54">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="63" t="s">
+        <v>178</v>
+      </c>
+      <c r="B11" s="64"/>
+      <c r="C11" s="52">
         <f>SUM(C4:C10)</f>
         <v>795.76639999999998</v>
       </c>
-      <c r="D11" s="54">
+      <c r="D11" s="53">
         <f t="shared" si="1"/>
         <v>13.262773333333334</v>
       </c>
-      <c r="F11" s="53">
+      <c r="F11" s="51">
         <f>F10*60</f>
         <v>23.152714285714286</v>
       </c>
       <c r="G11" t="s">
-        <v>248</v>
+        <v>210</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>220</v>
+        <v>182</v>
       </c>
       <c r="E15" s="8"/>
       <c r="F15" t="s">
-        <v>231</v>
+        <v>193</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="52" t="s">
-        <v>221</v>
-      </c>
-      <c r="E16" s="53"/>
+      <c r="A16" s="50" t="s">
+        <v>183</v>
+      </c>
+      <c r="E16" s="51"/>
       <c r="F16" t="s">
-        <v>247</v>
+        <v>209</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="52" t="s">
-        <v>222</v>
+      <c r="A17" s="50" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="52" t="s">
-        <v>223</v>
+      <c r="A18" s="50" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="52" t="s">
-        <v>224</v>
+      <c r="A19" s="50" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="52" t="s">
-        <v>225</v>
+      <c r="A20" s="50" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="52" t="s">
-        <v>226</v>
+      <c r="A21" s="50" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>227</v>
+        <v>189</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>228</v>
+        <v>190</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>229</v>
+        <v>191</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>230</v>
+        <v>192</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>232</v>
+        <v>194</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>233</v>
+        <v>195</v>
       </c>
       <c r="B29" t="s">
-        <v>234</v>
+        <v>196</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>239</v>
+        <v>201</v>
       </c>
       <c r="B30" t="s">
-        <v>246</v>
+        <v>208</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>240</v>
+        <v>202</v>
       </c>
       <c r="B31" t="s">
-        <v>246</v>
+        <v>208</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>241</v>
+        <v>203</v>
       </c>
       <c r="B32" t="s">
-        <v>246</v>
+        <v>208</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>245</v>
+        <v>207</v>
       </c>
       <c r="B33" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>242</v>
+        <v>204</v>
       </c>
       <c r="B34" t="s">
-        <v>246</v>
+        <v>208</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>243</v>
+        <v>205</v>
       </c>
       <c r="B35" t="s">
-        <v>246</v>
+        <v>208</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>244</v>
+        <v>206</v>
       </c>
       <c r="B36" t="s">
-        <v>246</v>
+        <v>208</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>235</v>
+        <v>197</v>
       </c>
       <c r="B37" t="s">
-        <v>236</v>
+        <v>198</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>237</v>
+        <v>199</v>
       </c>
       <c r="B38" t="s">
-        <v>238</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -4191,5 +2988,6 @@
     <mergeCell ref="A11:B11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fixed bug in config parser when more than 1 zip folder was present
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5836873D-D7CD-4B9A-B51A-D0B9AC399DCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93B792C2-D558-4B14-80E7-4EE6B8B019B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3645" yWindow="4065" windowWidth="29145" windowHeight="16815" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
+    <workbookView xWindow="690" yWindow="690" windowWidth="29145" windowHeight="16815" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
   <sheets>
     <sheet name="James_Island_Midbay" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="225">
   <si>
     <t>StormSim Project General Inputs</t>
   </si>
@@ -441,12 +441,6 @@
     <t>[16 84]</t>
   </si>
   <si>
-    <t>C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\CO-OPS_8571421_Bishops_Head_Pred_tide_MSL_m.csv</t>
-  </si>
-  <si>
-    <t>Midbay_CHS_Data.zip</t>
-  </si>
-  <si>
     <t>Use AEP or AEF for hazard curves (1 - AEP, 0-AEF)</t>
   </si>
   <si>
@@ -465,9 +459,6 @@
     <t>workflow</t>
   </si>
   <si>
-    <t>StormSim workflow to call for project. (1 - StormSim:PROS, 2- StormSim:EVA, 3- StormSim:MCS-LC)</t>
-  </si>
-  <si>
     <t>Include forcing peaks files as part of the analysis. (0/1)</t>
   </si>
   <si>
@@ -537,12 +528,6 @@
     <t>berm_slope</t>
   </si>
   <si>
-    <t>Midbay</t>
-  </si>
-  <si>
-    <t>Response Base</t>
-  </si>
-  <si>
     <t>RB1 + RB3 w WLP &amp; WHP</t>
   </si>
   <si>
@@ -585,9 +570,6 @@
     <t xml:space="preserve">Rubble mound </t>
   </si>
   <si>
-    <t>responses</t>
-  </si>
-  <si>
     <t>SWL</t>
   </si>
   <si>
@@ -606,18 +588,6 @@
     <t>Dn50</t>
   </si>
   <si>
-    <t>P1</t>
-  </si>
-  <si>
-    <t>P2</t>
-  </si>
-  <si>
-    <t>P3</t>
-  </si>
-  <si>
-    <t>Nappe</t>
-  </si>
-  <si>
     <t>Time Per Dataset (Peak Maxima , Peak WLP, Peak WHP &amp; RB3</t>
   </si>
   <si>
@@ -681,15 +651,76 @@
     <t>Transect_001</t>
   </si>
   <si>
-    <t>Alternative_001</t>
+    <t>CO-OPS_8571421_Bishops_Head_Pred_tide_MSL_m.csv</t>
+  </si>
+  <si>
+    <t>CHSFileDownload_2023-04-19_11-51-54.zip</t>
+  </si>
+  <si>
+    <t>CHS-NA_TS_SimB_Post0_SP15104_ADCIRC01_Peaks.h5</t>
+  </si>
+  <si>
+    <t>CHS-NA_TS_SimB_Post0_SP15104_ADCIRC01_Timeseries.h5</t>
+  </si>
+  <si>
+    <t>CHS-NA_TS_SimB_Post0_SP2678_STWAVE03_Peaks.h5</t>
+  </si>
+  <si>
+    <t>CHS-NA_TS_SimB_Post0_SP2678_STWAVE03_Timeseries.h5</t>
+  </si>
+  <si>
+    <t>CHS-NA_XH_SimB_Post0_SP15104_ADCIRC01_Peaks.h5</t>
+  </si>
+  <si>
+    <t>CHS-NA_XH_SimB_Post0_SP15104_ADCIRC01_Timeseries.h5</t>
+  </si>
+  <si>
+    <t>CHS-NA_XH_SimB_Post0_SP2678_STWAVE03_Peaks.h5</t>
+  </si>
+  <si>
+    <t>CHS-NA_XH_SimB_Post0_SP2678_STWAVE03_Timeseries.h5</t>
+  </si>
+  <si>
+    <t>StormSim workflow to call for project. (1 - StormSim:PROS, 2- StormSim:EVA, 3- StormSim:LCS)</t>
+  </si>
+  <si>
+    <t>Responses</t>
+  </si>
+  <si>
+    <t>James Island</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peaks Reliability </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seaside Armor damage </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leeside Armor damage </t>
+  </si>
+  <si>
+    <t>Life Cycle Simulation</t>
+  </si>
+  <si>
+    <t>Response Base Simulation</t>
+  </si>
+  <si>
+    <t>Peaks + Timeseries w WLP &amp; WHP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Historical Sampling </t>
+  </si>
+  <si>
+    <t>Alternative_002</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.000000000000000"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -802,7 +833,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="21">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -1072,11 +1103,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1205,6 +1251,10 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1588,7 +1638,7 @@
         <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="F3" s="49" t="s">
         <v>115</v>
@@ -1597,7 +1647,7 @@
         <v>108</v>
       </c>
       <c r="H3" s="13" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="I3" s="13">
         <v>0.33979999999999999</v>
@@ -1614,7 +1664,7 @@
         <v>10</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>213</v>
+        <v>203</v>
       </c>
       <c r="F4" s="49" t="s">
         <v>116</v>
@@ -1631,16 +1681,16 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C5" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>214</v>
+        <v>224</v>
       </c>
       <c r="F5" s="49" t="s">
         <v>118</v>
@@ -1649,7 +1699,7 @@
         <v>110</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="I5" s="13">
         <v>0.3</v>
@@ -1701,7 +1751,7 @@
         <v>113</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="I7" s="2">
         <v>0</v>
@@ -1709,10 +1759,10 @@
     </row>
     <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="14" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>142</v>
+        <v>214</v>
       </c>
       <c r="C8" s="16" t="s">
         <v>10</v>
@@ -1808,7 +1858,7 @@
         <v>10</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>134</v>
+        <v>204</v>
       </c>
       <c r="F12" s="30" t="s">
         <v>122</v>
@@ -1817,7 +1867,7 @@
         <v>48</v>
       </c>
       <c r="H12" s="16" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="I12" s="2">
         <v>0.5</v>
@@ -1843,7 +1893,7 @@
         <v>57</v>
       </c>
       <c r="H13" s="31" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="I13" s="2">
         <v>0.43</v>
@@ -1851,10 +1901,10 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="C14" s="16" t="s">
         <v>10</v>
@@ -1869,7 +1919,7 @@
         <v>51</v>
       </c>
       <c r="H14" s="16" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="I14" s="2">
         <v>0.78</v>
@@ -1880,7 +1930,7 @@
         <v>96</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C15" s="16" t="s">
         <v>10</v>
@@ -1895,7 +1945,7 @@
         <v>54</v>
       </c>
       <c r="H15" s="19" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="I15" s="3">
         <v>0.13</v>
@@ -1903,10 +1953,10 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>10</v>
@@ -1921,10 +1971,10 @@
     </row>
     <row r="17" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="17" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="C17" s="19" t="s">
         <v>10</v>
@@ -2021,16 +2071,16 @@
         <v>1</v>
       </c>
       <c r="F21" s="17" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="G21" s="18" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="H21" s="19" t="s">
         <v>10</v>
       </c>
       <c r="I21" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -2082,7 +2132,7 @@
         <v>10</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>135</v>
+        <v>205</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>3</v>
@@ -2107,7 +2157,9 @@
       <c r="C25" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D25" s="2"/>
+      <c r="D25" s="2" t="s">
+        <v>206</v>
+      </c>
       <c r="F25" s="11" t="s">
         <v>27</v>
       </c>
@@ -2131,7 +2183,9 @@
       <c r="C26" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D26" s="2"/>
+      <c r="D26" s="2" t="s">
+        <v>207</v>
+      </c>
       <c r="F26" s="14" t="s">
         <v>31</v>
       </c>
@@ -2155,7 +2209,9 @@
       <c r="C27" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D27" s="2"/>
+      <c r="D27" s="2" t="s">
+        <v>208</v>
+      </c>
       <c r="F27" s="14" t="s">
         <v>33</v>
       </c>
@@ -2179,7 +2235,9 @@
       <c r="C28" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D28" s="2"/>
+      <c r="D28" s="2" t="s">
+        <v>209</v>
+      </c>
       <c r="F28" s="17" t="s">
         <v>36</v>
       </c>
@@ -2187,7 +2245,7 @@
         <v>37</v>
       </c>
       <c r="H28" s="19" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="I28" s="3">
         <v>1</v>
@@ -2203,7 +2261,9 @@
       <c r="C29" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D29" s="2"/>
+      <c r="D29" s="2" t="s">
+        <v>210</v>
+      </c>
       <c r="F29" s="21"/>
       <c r="G29" s="21"/>
       <c r="H29" s="21"/>
@@ -2219,7 +2279,9 @@
       <c r="C30" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D30" s="2"/>
+      <c r="D30" s="2" t="s">
+        <v>211</v>
+      </c>
       <c r="F30" s="26" t="s">
         <v>41</v>
       </c>
@@ -2237,7 +2299,9 @@
       <c r="C31" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D31" s="2"/>
+      <c r="D31" s="2" t="s">
+        <v>212</v>
+      </c>
       <c r="F31" s="9" t="s">
         <v>3</v>
       </c>
@@ -2261,7 +2325,9 @@
       <c r="C32" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="D32" s="3"/>
+      <c r="D32" s="3" t="s">
+        <v>213</v>
+      </c>
       <c r="F32" s="29" t="s">
         <v>44</v>
       </c>
@@ -2281,10 +2347,10 @@
       <c r="C33" s="25"/>
       <c r="D33" s="25"/>
       <c r="F33" s="17" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="G33" s="18" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="H33" s="19" t="s">
         <v>10</v>
@@ -2320,10 +2386,10 @@
         <v>70</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="D36" s="1">
         <v>1.2320122</v>
@@ -2337,7 +2403,7 @@
         <v>98</v>
       </c>
       <c r="C37" s="16" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="D37" s="2">
         <v>1.5243902</v>
@@ -2348,10 +2414,10 @@
         <v>72</v>
       </c>
       <c r="B38" s="15" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="C38" s="16" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="D38" s="2">
         <v>-1.5969511999999999</v>
@@ -2359,13 +2425,13 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
-        <v>212</v>
+        <v>202</v>
       </c>
       <c r="B39" s="15" t="s">
+        <v>152</v>
+      </c>
+      <c r="C39" s="16" t="s">
         <v>155</v>
-      </c>
-      <c r="C39" s="16" t="s">
-        <v>158</v>
       </c>
       <c r="D39" s="2">
         <v>-0.95799999999999996</v>
@@ -2376,7 +2442,7 @@
         <v>73</v>
       </c>
       <c r="B40" s="15" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="C40" s="16" t="s">
         <v>10</v>
@@ -2390,7 +2456,7 @@
         <v>74</v>
       </c>
       <c r="B41" s="15" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="C41" s="16" t="s">
         <v>10</v>
@@ -2407,7 +2473,7 @@
         <v>103</v>
       </c>
       <c r="C42" s="45" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D42" s="46">
         <v>0</v>
@@ -2415,10 +2481,10 @@
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="B43" s="15" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="C43" s="16" t="s">
         <v>10</v>
@@ -2435,7 +2501,7 @@
         <v>106</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="D44" s="2">
         <v>0</v>
@@ -2446,10 +2512,10 @@
         <v>105</v>
       </c>
       <c r="B45" s="38" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="C45" s="43" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="D45" s="44">
         <v>-0.82799999999999996</v>
@@ -2505,10 +2571,10 @@
         <v>79</v>
       </c>
       <c r="C50" s="16" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="D50" s="2">
-        <v>500</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
@@ -2519,10 +2585,10 @@
         <v>81</v>
       </c>
       <c r="C51" s="16" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="D51" s="2">
-        <v>500</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
@@ -2533,7 +2599,7 @@
         <v>83</v>
       </c>
       <c r="C52" s="16" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="D52" s="2">
         <v>1027</v>
@@ -2629,7 +2695,13 @@
       <c r="C59" s="37"/>
       <c r="D59" s="37"/>
     </row>
-    <row r="72" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C65" s="64"/>
+    </row>
+    <row r="66" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C66" s="63"/>
+    </row>
+    <row r="72" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B72" s="47"/>
     </row>
   </sheetData>
@@ -2647,345 +2719,596 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36F05AA9-AA83-414A-9BCA-9A7F3A47A337}">
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="19" customWidth="1"/>
+    <col min="5" max="5" width="34.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>166</v>
+        <v>216</v>
       </c>
       <c r="B1" t="s">
-        <v>167</v>
+        <v>221</v>
       </c>
       <c r="C1" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="D1" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="E1" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="54" t="s">
-        <v>169</v>
-      </c>
-      <c r="B3" s="54" t="s">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>215</v>
+      </c>
+      <c r="B3" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="50" t="s">
+        <v>177</v>
+      </c>
+      <c r="B4" t="s">
+        <v>185</v>
+      </c>
+      <c r="C4" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="50" t="s">
+        <v>178</v>
+      </c>
+      <c r="B5" t="s">
+        <v>191</v>
+      </c>
+      <c r="C5" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="50" t="s">
+        <v>179</v>
+      </c>
+      <c r="B6" t="s">
+        <v>192</v>
+      </c>
+      <c r="C6" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="B7" t="s">
+        <v>193</v>
+      </c>
+      <c r="C7" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="50" t="s">
+        <v>181</v>
+      </c>
+      <c r="B8" t="s">
+        <v>197</v>
+      </c>
+      <c r="C8" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="50" t="s">
+        <v>182</v>
+      </c>
+      <c r="B9" t="s">
+        <v>194</v>
+      </c>
+      <c r="C9" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>195</v>
+      </c>
+      <c r="C10" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>196</v>
+      </c>
+      <c r="C11" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>187</v>
+      </c>
+      <c r="C12" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>189</v>
+      </c>
+      <c r="C13" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="16" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="54" t="s">
+        <v>164</v>
+      </c>
+      <c r="B16" s="54" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="54" t="s">
-        <v>177</v>
-      </c>
-      <c r="D3" s="58" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="55">
+      <c r="C16" s="54" t="s">
+        <v>172</v>
+      </c>
+      <c r="D16" s="58" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="55">
         <v>0</v>
       </c>
-      <c r="B4" s="55" t="s">
-        <v>170</v>
-      </c>
-      <c r="C4" s="59">
+      <c r="B17" s="55" t="s">
+        <v>165</v>
+      </c>
+      <c r="C17" s="59">
         <v>0.66720000000000002</v>
       </c>
-      <c r="D4" s="62">
-        <f>C4/60</f>
+      <c r="D17" s="62">
+        <f>C17/60</f>
         <v>1.112E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="56">
-        <f>A4+1</f>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="56">
+        <f>A17+1</f>
         <v>1</v>
       </c>
-      <c r="B5" s="56" t="s">
-        <v>171</v>
-      </c>
-      <c r="C5" s="60">
+      <c r="B18" s="56" t="s">
+        <v>166</v>
+      </c>
+      <c r="C18" s="60">
         <v>128.0189</v>
       </c>
-      <c r="D5" s="60">
-        <f>C5/60</f>
+      <c r="D18" s="60">
+        <f>C18/60</f>
         <v>2.1336483333333334</v>
       </c>
-      <c r="E5" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="56">
-        <f t="shared" ref="A6:A10" si="0">A5+1</f>
+      <c r="E18" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="56">
+        <f t="shared" ref="A19:A23" si="0">A18+1</f>
         <v>2</v>
       </c>
-      <c r="B6" s="56" t="s">
-        <v>172</v>
-      </c>
-      <c r="C6" s="60">
+      <c r="B19" s="56" t="s">
+        <v>167</v>
+      </c>
+      <c r="C19" s="60">
         <v>1.8109999999999999</v>
       </c>
-      <c r="D6" s="60">
-        <f t="shared" ref="D6:D11" si="1">C6/60</f>
+      <c r="D19" s="60">
+        <f t="shared" ref="D19:D24" si="1">C19/60</f>
         <v>3.0183333333333333E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="56">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="56">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="B7" s="56" t="s">
-        <v>173</v>
-      </c>
-      <c r="C7" s="60">
+      <c r="B20" s="56" t="s">
+        <v>168</v>
+      </c>
+      <c r="C20" s="60">
         <v>0.56489999999999996</v>
       </c>
-      <c r="D7" s="60">
+      <c r="D20" s="60">
         <f t="shared" si="1"/>
         <v>9.4149999999999998E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="56">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="56">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="B8" s="56" t="s">
-        <v>174</v>
-      </c>
-      <c r="C8" s="60">
+      <c r="B21" s="56" t="s">
+        <v>169</v>
+      </c>
+      <c r="C21" s="60">
         <v>1.2150000000000001</v>
       </c>
-      <c r="D8" s="60">
+      <c r="D21" s="60">
         <f t="shared" si="1"/>
         <v>2.0250000000000001E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="56">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="56">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="B9" s="56" t="s">
-        <v>175</v>
-      </c>
-      <c r="C9" s="60">
+      <c r="B22" s="56" t="s">
+        <v>170</v>
+      </c>
+      <c r="C22" s="60">
         <v>15.2134</v>
       </c>
-      <c r="D9" s="60">
+      <c r="D22" s="60">
         <f t="shared" si="1"/>
         <v>0.25355666666666665</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="57">
+    <row r="23" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="57">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="B10" s="57" t="s">
-        <v>176</v>
-      </c>
-      <c r="C10" s="61">
+      <c r="B23" s="57" t="s">
+        <v>171</v>
+      </c>
+      <c r="C23" s="61">
         <v>648.27599999999995</v>
       </c>
-      <c r="D10" s="61">
+      <c r="D23" s="61">
         <f t="shared" si="1"/>
         <v>10.804599999999999</v>
       </c>
-      <c r="E10" s="8">
-        <f>D10/4</f>
+      <c r="E23" s="8">
+        <f>D23/4</f>
         <v>2.7011499999999997</v>
       </c>
-      <c r="F10" s="51">
-        <f>E10/7</f>
+      <c r="F23" s="51">
+        <f>E23/7</f>
         <v>0.3858785714285714</v>
       </c>
-      <c r="G10" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="63" t="s">
-        <v>178</v>
-      </c>
-      <c r="B11" s="64"/>
-      <c r="C11" s="52">
-        <f>SUM(C4:C10)</f>
+      <c r="G23" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="65" t="s">
+        <v>173</v>
+      </c>
+      <c r="B24" s="66"/>
+      <c r="C24" s="52">
+        <f>SUM(C17:C23)</f>
         <v>795.76639999999998</v>
       </c>
-      <c r="D11" s="53">
+      <c r="D24" s="53">
         <f t="shared" si="1"/>
         <v>13.262773333333334</v>
       </c>
-      <c r="F11" s="51">
-        <f>F10*60</f>
+      <c r="F24" s="51">
+        <f>F23*60</f>
         <v>23.152714285714286</v>
       </c>
-      <c r="G11" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>182</v>
-      </c>
-      <c r="E15" s="8"/>
-      <c r="F15" t="s">
+      <c r="G24" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E28" s="8"/>
+      <c r="F28" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E29" s="51"/>
+      <c r="F29" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>216</v>
+      </c>
+      <c r="B31" t="s">
+        <v>220</v>
+      </c>
+      <c r="C31" t="s">
+        <v>222</v>
+      </c>
+      <c r="D31" t="s">
+        <v>176</v>
+      </c>
+      <c r="E31" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>215</v>
+      </c>
+      <c r="B33" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="50" t="s">
+        <v>217</v>
+      </c>
+      <c r="B34" t="s">
+        <v>185</v>
+      </c>
+      <c r="C34" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="50" t="s">
+        <v>218</v>
+      </c>
+      <c r="B35" t="s">
+        <v>191</v>
+      </c>
+      <c r="C35" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="50" t="s">
+        <v>219</v>
+      </c>
+      <c r="B36" t="s">
+        <v>192</v>
+      </c>
+      <c r="C36" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="B37" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="50" t="s">
-        <v>183</v>
-      </c>
-      <c r="E16" s="51"/>
-      <c r="F16" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="50" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="50" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="50" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="50" t="s">
+      <c r="C37" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" s="50" t="s">
+        <v>181</v>
+      </c>
+      <c r="B38" t="s">
+        <v>197</v>
+      </c>
+      <c r="C38" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B39" t="s">
+        <v>194</v>
+      </c>
+      <c r="C39" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B40" t="s">
+        <v>195</v>
+      </c>
+      <c r="C40" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B41" t="s">
+        <v>196</v>
+      </c>
+      <c r="C41" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B42" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="50" t="s">
+      <c r="C42" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B43" t="s">
         <v>189</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+      <c r="C43" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>195</v>
-      </c>
-      <c r="B29" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>201</v>
-      </c>
-      <c r="B30" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>202</v>
-      </c>
-      <c r="B31" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>203</v>
-      </c>
-      <c r="B32" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>207</v>
-      </c>
-      <c r="B33" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>204</v>
-      </c>
-      <c r="B34" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>205</v>
-      </c>
-      <c r="B35" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>206</v>
-      </c>
-      <c r="B36" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>197</v>
-      </c>
-      <c r="B37" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>199</v>
-      </c>
-      <c r="B38" t="s">
-        <v>200</v>
+    <row r="45" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="46" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="54" t="s">
+        <v>164</v>
+      </c>
+      <c r="B46" s="54" t="s">
+        <v>4</v>
+      </c>
+      <c r="C46" s="54" t="s">
+        <v>172</v>
+      </c>
+      <c r="D46" s="58" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47" s="55">
+        <v>0</v>
+      </c>
+      <c r="B47" s="55" t="s">
+        <v>165</v>
+      </c>
+      <c r="C47" s="59">
+        <v>0.66720000000000002</v>
+      </c>
+      <c r="D47" s="62">
+        <f>C47/60</f>
+        <v>1.112E-2</v>
+      </c>
+      <c r="F47" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48" s="56">
+        <f>A47+1</f>
+        <v>1</v>
+      </c>
+      <c r="B48" s="56" t="s">
+        <v>166</v>
+      </c>
+      <c r="C48" s="60">
+        <v>128.0189</v>
+      </c>
+      <c r="D48" s="60">
+        <f>C48/60</f>
+        <v>2.1336483333333334</v>
+      </c>
+      <c r="E48" t="s">
+        <v>174</v>
+      </c>
+      <c r="F48" t="s">
+        <v>172</v>
+      </c>
+      <c r="G48" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A49" s="56">
+        <f t="shared" ref="A49:A53" si="2">A48+1</f>
+        <v>2</v>
+      </c>
+      <c r="B49" s="56" t="s">
+        <v>167</v>
+      </c>
+      <c r="C49" s="60">
+        <v>77.920665999999997</v>
+      </c>
+      <c r="D49" s="60">
+        <f t="shared" ref="D49:D54" si="3">C49/60</f>
+        <v>1.2986777666666667</v>
+      </c>
+      <c r="F49" s="60">
+        <v>15</v>
+      </c>
+      <c r="G49" s="60">
+        <f t="shared" ref="G49" si="4">F49/60</f>
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A50" s="56">
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="B50" s="56" t="s">
+        <v>168</v>
+      </c>
+      <c r="C50" s="60">
+        <v>0.56489999999999996</v>
+      </c>
+      <c r="D50" s="60">
+        <f t="shared" si="3"/>
+        <v>9.4149999999999998E-3</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A51" s="56">
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="B51" s="56" t="s">
+        <v>169</v>
+      </c>
+      <c r="C51" s="60">
+        <v>2.6115067000000001</v>
+      </c>
+      <c r="D51" s="60">
+        <f t="shared" si="3"/>
+        <v>4.3525111666666665E-2</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A52" s="56">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="B52" s="56" t="s">
+        <v>170</v>
+      </c>
+      <c r="C52" s="60">
+        <v>32.553324799999999</v>
+      </c>
+      <c r="D52" s="60">
+        <f t="shared" si="3"/>
+        <v>0.54255541333333335</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="57">
+        <f t="shared" si="2"/>
+        <v>6</v>
+      </c>
+      <c r="B53" s="57" t="s">
+        <v>171</v>
+      </c>
+      <c r="C53" s="61">
+        <v>197.9727273</v>
+      </c>
+      <c r="D53" s="61">
+        <f t="shared" si="3"/>
+        <v>3.2995454550000001</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="65" t="s">
+        <v>173</v>
+      </c>
+      <c r="B54" s="66"/>
+      <c r="C54" s="52">
+        <f>SUM(C47:C53)</f>
+        <v>440.30922480000004</v>
+      </c>
+      <c r="D54" s="53">
+        <f t="shared" si="3"/>
+        <v>7.3384870800000011</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A11:B11"/>
+  <mergeCells count="2">
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A54:B54"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Fixing bugs found by Jeff
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26501"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93B792C2-D558-4B14-80E7-4EE6B8B019B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{807ECCC6-98B3-4AF9-AAFE-12988EBF70C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="690" yWindow="690" windowWidth="29145" windowHeight="16815" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
   <sheets>
     <sheet name="James_Island_Midbay" sheetId="1" r:id="rId1"/>
@@ -1910,7 +1910,7 @@
         <v>10</v>
       </c>
       <c r="D14" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F14" s="14" t="s">
         <v>99</v>
@@ -1962,7 +1962,7 @@
         <v>10</v>
       </c>
       <c r="D16" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F16" s="27"/>
       <c r="G16" s="27"/>
@@ -1980,7 +1980,7 @@
         <v>10</v>
       </c>
       <c r="D17" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F17" s="7" t="s">
         <v>1</v>

</xml_diff>

<commit_message>
New input file format
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CF6F974-304A-447E-99FF-EAE6185A7F7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA3F0304-26ED-4EB8-84C3-6FD2267592BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="207">
   <si>
     <t>StormSim Project General Inputs</t>
   </si>
@@ -168,75 +168,24 @@
     <t>chs_zip</t>
   </si>
   <si>
-    <t>CHS Zip Folder (Relative Path)</t>
-  </si>
-  <si>
     <t>pros_compute_forcing_HC</t>
   </si>
   <si>
     <t>Compute Hazard for Waves and WL (1 - On, 2 - Off)</t>
   </si>
   <si>
-    <t>chs_tc_swl_peaks</t>
-  </si>
-  <si>
-    <t>ADCIRC TC Peaks</t>
-  </si>
-  <si>
     <t>Dn50 Uncertainty</t>
   </si>
   <si>
-    <t>chs_tc_swl_timeseries</t>
-  </si>
-  <si>
-    <t>ADCIRC TC Timeseries</t>
-  </si>
-  <si>
     <t>Overtopping Uncertainty</t>
   </si>
   <si>
-    <t>chs_tc_hm0_peaks</t>
-  </si>
-  <si>
-    <t>STWAVE TC Peaks</t>
-  </si>
-  <si>
     <t>Runup Uncertainty</t>
   </si>
   <si>
-    <t>chs_tc_hm0_timeseries</t>
-  </si>
-  <si>
-    <t>STWAVE TC Timeseries</t>
-  </si>
-  <si>
     <t>Surface Pressure (p1) Uncertainty' (Floodwalls Only)</t>
   </si>
   <si>
-    <t>chs_xc_swl_peaks</t>
-  </si>
-  <si>
-    <t>ADCIRC XC Peaks</t>
-  </si>
-  <si>
-    <t>chs_xc_swl_timeseries</t>
-  </si>
-  <si>
-    <t>ADCIRC XC Timeseries</t>
-  </si>
-  <si>
-    <t>chs_xc_hm0_peaks</t>
-  </si>
-  <si>
-    <t>STWAVE XC Peaks</t>
-  </si>
-  <si>
-    <t>chs_xc_hm0_timeseries</t>
-  </si>
-  <si>
-    <t>STWAVE XC Timeseries</t>
-  </si>
-  <si>
     <t xml:space="preserve">StormSim Project Forcing Uncertainty </t>
   </si>
   <si>
@@ -654,33 +603,6 @@
     <t>CO-OPS_8571421_Bishops_Head_Pred_tide_MSL_m.csv</t>
   </si>
   <si>
-    <t>CHSFileDownload_2023-04-19_11-51-54.zip</t>
-  </si>
-  <si>
-    <t>CHS-NA_TS_SimB_Post0_SP15104_ADCIRC01_Peaks.h5</t>
-  </si>
-  <si>
-    <t>CHS-NA_TS_SimB_Post0_SP15104_ADCIRC01_Timeseries.h5</t>
-  </si>
-  <si>
-    <t>CHS-NA_TS_SimB_Post0_SP2678_STWAVE03_Peaks.h5</t>
-  </si>
-  <si>
-    <t>CHS-NA_TS_SimB_Post0_SP2678_STWAVE03_Timeseries.h5</t>
-  </si>
-  <si>
-    <t>CHS-NA_XH_SimB_Post0_SP15104_ADCIRC01_Peaks.h5</t>
-  </si>
-  <si>
-    <t>CHS-NA_XH_SimB_Post0_SP15104_ADCIRC01_Timeseries.h5</t>
-  </si>
-  <si>
-    <t>CHS-NA_XH_SimB_Post0_SP2678_STWAVE03_Peaks.h5</t>
-  </si>
-  <si>
-    <t>CHS-NA_XH_SimB_Post0_SP2678_STWAVE03_Timeseries.h5</t>
-  </si>
-  <si>
     <t>StormSim workflow to call for project. (1 - StormSim:PROS, 2- StormSim:EVA, 3- StormSim:LCS)</t>
   </si>
   <si>
@@ -715,6 +637,27 @@
   </si>
   <si>
     <t>TC</t>
+  </si>
+  <si>
+    <t>forcing_type</t>
+  </si>
+  <si>
+    <t>Forcing Data Source (0 - CHS Native Data, 1- Custom Modeling)</t>
+  </si>
+  <si>
+    <t>prob_mass_source</t>
+  </si>
+  <si>
+    <t>Probability Masses (CHS -&gt; MCSim_Inputs folder path, Custom Modeling -&gt; .mat filename with relative path)</t>
+  </si>
+  <si>
+    <t>prob_mass_from_MB_SP2243\prob_mass_from_MB_SP2243.mat</t>
+  </si>
+  <si>
+    <t>CHS Zip Folder or Custom Modeling .mat File (Relative Path)</t>
+  </si>
+  <si>
+    <t>prob_mass_from_MB_SP2243\CHS_Data_from_MB_SP2243.mat</t>
   </si>
 </sst>
 </file>
@@ -1578,7 +1521,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51D29750-2AFD-4BF7-A911-1DC4ADC0FD7A}">
-  <dimension ref="A1:I72"/>
+  <dimension ref="A1:I66"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52.5703125" customWidth="1"/>
@@ -1598,7 +1541,7 @@
       <c r="C1" s="6"/>
       <c r="D1" s="6"/>
       <c r="F1" s="32" t="s">
-        <v>66</v>
+        <v>49</v>
       </c>
       <c r="G1" s="33"/>
       <c r="H1" s="33"/>
@@ -1641,16 +1584,16 @@
         <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="F3" s="49" t="s">
+        <v>98</v>
+      </c>
+      <c r="G3" s="49" t="s">
+        <v>91</v>
+      </c>
+      <c r="H3" s="13" t="s">
         <v>138</v>
-      </c>
-      <c r="F3" s="49" t="s">
-        <v>115</v>
-      </c>
-      <c r="G3" s="49" t="s">
-        <v>108</v>
-      </c>
-      <c r="H3" s="13" t="s">
-        <v>155</v>
       </c>
       <c r="I3" s="13">
         <v>0.33979999999999999</v>
@@ -1667,13 +1610,13 @@
         <v>10</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>203</v>
+        <v>186</v>
       </c>
       <c r="F4" s="49" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="G4" s="49" t="s">
-        <v>109</v>
+        <v>92</v>
       </c>
       <c r="H4" s="13" t="s">
         <v>10</v>
@@ -1684,25 +1627,25 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>136</v>
+        <v>119</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>137</v>
+        <v>120</v>
       </c>
       <c r="C5" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>224</v>
+        <v>198</v>
       </c>
       <c r="F5" s="49" t="s">
-        <v>118</v>
+        <v>101</v>
       </c>
       <c r="G5" s="49" t="s">
-        <v>110</v>
+        <v>93</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>155</v>
+        <v>138</v>
       </c>
       <c r="I5" s="13">
         <v>0.3</v>
@@ -1719,13 +1662,13 @@
         <v>10</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>129</v>
+        <v>112</v>
       </c>
       <c r="F6" s="49" t="s">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="G6" s="49" t="s">
-        <v>111</v>
+        <v>94</v>
       </c>
       <c r="H6" s="13" t="s">
         <v>10</v>
@@ -1745,16 +1688,16 @@
         <v>10</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>133</v>
+        <v>116</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>119</v>
+        <v>102</v>
       </c>
       <c r="G7" s="15" t="s">
-        <v>113</v>
+        <v>96</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>160</v>
+        <v>143</v>
       </c>
       <c r="I7" s="2">
         <v>0</v>
@@ -1762,10 +1705,10 @@
     </row>
     <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="14" t="s">
-        <v>139</v>
+        <v>122</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>214</v>
+        <v>188</v>
       </c>
       <c r="C8" s="16" t="s">
         <v>10</v>
@@ -1774,13 +1717,13 @@
         <v>3</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>112</v>
+        <v>95</v>
       </c>
       <c r="H8" s="19" t="s">
-        <v>67</v>
+        <v>50</v>
       </c>
       <c r="I8" s="3">
         <v>0</v>
@@ -1815,10 +1758,10 @@
         <v>10</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>225</v>
+        <v>199</v>
       </c>
       <c r="F10" s="26" t="s">
-        <v>120</v>
+        <v>103</v>
       </c>
       <c r="G10" s="27"/>
       <c r="H10" s="27"/>
@@ -1852,25 +1795,25 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>126</v>
+        <v>109</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>127</v>
+        <v>110</v>
       </c>
       <c r="C12" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>204</v>
+        <v>187</v>
       </c>
       <c r="F12" s="30" t="s">
-        <v>122</v>
+        <v>105</v>
       </c>
       <c r="G12" s="15" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="H12" s="16" t="s">
-        <v>155</v>
+        <v>138</v>
       </c>
       <c r="I12" s="2">
         <v>0.5</v>
@@ -1878,10 +1821,10 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>121</v>
+        <v>104</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>97</v>
+        <v>80</v>
       </c>
       <c r="C13" s="16" t="s">
         <v>10</v>
@@ -1890,13 +1833,13 @@
         <v>1</v>
       </c>
       <c r="F13" s="30" t="s">
-        <v>123</v>
+        <v>106</v>
       </c>
       <c r="G13" s="15" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="H13" s="31" t="s">
-        <v>159</v>
+        <v>142</v>
       </c>
       <c r="I13" s="2">
         <v>0.43</v>
@@ -1904,10 +1847,10 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>142</v>
+        <v>125</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>140</v>
+        <v>123</v>
       </c>
       <c r="C14" s="16" t="s">
         <v>10</v>
@@ -1916,13 +1859,13 @@
         <v>1</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>99</v>
+        <v>82</v>
       </c>
       <c r="G14" s="15" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="H14" s="16" t="s">
-        <v>158</v>
+        <v>141</v>
       </c>
       <c r="I14" s="2">
         <v>0.78</v>
@@ -1930,10 +1873,10 @@
     </row>
     <row r="15" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="14" t="s">
-        <v>96</v>
+        <v>79</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>141</v>
+        <v>124</v>
       </c>
       <c r="C15" s="16" t="s">
         <v>10</v>
@@ -1942,13 +1885,13 @@
         <v>1</v>
       </c>
       <c r="F15" s="17" t="s">
-        <v>100</v>
+        <v>83</v>
       </c>
       <c r="G15" s="18" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="H15" s="19" t="s">
-        <v>155</v>
+        <v>138</v>
       </c>
       <c r="I15" s="3">
         <v>0.13</v>
@@ -1956,10 +1899,10 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>147</v>
+        <v>130</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>144</v>
+        <v>127</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>10</v>
@@ -1974,10 +1917,10 @@
     </row>
     <row r="17" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="17" t="s">
-        <v>148</v>
+        <v>131</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>143</v>
+        <v>126</v>
       </c>
       <c r="C17" s="19" t="s">
         <v>10</v>
@@ -2062,22 +2005,22 @@
     </row>
     <row r="21" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="11" t="s">
-        <v>38</v>
+        <v>200</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>39</v>
+        <v>201</v>
       </c>
       <c r="C21" s="28" t="s">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="D21" s="1">
         <v>1</v>
       </c>
       <c r="F21" s="17" t="s">
-        <v>145</v>
+        <v>128</v>
       </c>
       <c r="G21" s="18" t="s">
-        <v>146</v>
+        <v>129</v>
       </c>
       <c r="H21" s="19" t="s">
         <v>10</v>
@@ -2088,16 +2031,16 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>131</v>
+        <v>38</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>132</v>
+        <v>39</v>
       </c>
       <c r="C22" s="28" t="s">
-        <v>130</v>
+        <v>40</v>
       </c>
       <c r="D22" s="1">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F22" s="8"/>
       <c r="G22" s="8"/>
@@ -2106,16 +2049,16 @@
     </row>
     <row r="23" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="11" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="C23" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>128</v>
+        <v>113</v>
+      </c>
+      <c r="D23" s="1">
+        <v>5</v>
       </c>
       <c r="F23" s="20" t="s">
         <v>26</v>
@@ -2125,17 +2068,17 @@
       <c r="I23" s="21"/>
     </row>
     <row r="24" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="14" t="s">
-        <v>42</v>
-      </c>
-      <c r="B24" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="C24" s="16" t="s">
+      <c r="A24" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="C24" s="28" t="s">
         <v>10</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>205</v>
+        <v>111</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>3</v>
@@ -2151,17 +2094,17 @@
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="B25" s="15" t="s">
-        <v>47</v>
-      </c>
-      <c r="C25" s="16" t="s">
+      <c r="A25" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>203</v>
+      </c>
+      <c r="C25" s="28" t="s">
         <v>10</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="F25" s="11" t="s">
         <v>27</v>
@@ -2178,16 +2121,16 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>50</v>
+        <v>205</v>
       </c>
       <c r="C26" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F26" s="14" t="s">
         <v>31</v>
@@ -2203,18 +2146,10 @@
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="B27" s="15" t="s">
-        <v>53</v>
-      </c>
-      <c r="C27" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>208</v>
-      </c>
+      <c r="A27" s="25"/>
+      <c r="B27" s="25"/>
+      <c r="C27" s="25"/>
+      <c r="D27" s="25"/>
       <c r="F27" s="14" t="s">
         <v>33</v>
       </c>
@@ -2229,18 +2164,12 @@
       </c>
     </row>
     <row r="28" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="14" t="s">
-        <v>55</v>
-      </c>
-      <c r="B28" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="C28" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>209</v>
-      </c>
+      <c r="A28" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="B28" s="35"/>
+      <c r="C28" s="35"/>
+      <c r="D28" s="35"/>
       <c r="F28" s="17" t="s">
         <v>36</v>
       </c>
@@ -2248,24 +2177,24 @@
         <v>37</v>
       </c>
       <c r="H28" s="19" t="s">
-        <v>155</v>
+        <v>138</v>
       </c>
       <c r="I28" s="3">
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="B29" s="15" t="s">
-        <v>59</v>
-      </c>
-      <c r="C29" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>210</v>
+    <row r="29" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B29" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D29" s="10" t="s">
+        <v>52</v>
       </c>
       <c r="F29" s="21"/>
       <c r="G29" s="21"/>
@@ -2273,17 +2202,17 @@
       <c r="I29" s="21"/>
     </row>
     <row r="30" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="B30" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="C30" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>211</v>
+      <c r="A30" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="B30" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="C30" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="D30" s="1">
+        <v>1.2320122</v>
       </c>
       <c r="F30" s="26" t="s">
         <v>41</v>
@@ -2294,16 +2223,16 @@
     </row>
     <row r="31" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="14" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>63</v>
+        <v>81</v>
       </c>
       <c r="C31" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>212</v>
+        <v>138</v>
+      </c>
+      <c r="D31" s="2">
+        <v>1.5243902</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>3</v>
@@ -2318,24 +2247,24 @@
         <v>6</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="17" t="s">
-        <v>64</v>
-      </c>
-      <c r="B32" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="C32" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D32" s="3" t="s">
-        <v>213</v>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="B32" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="C32" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="D32" s="2">
+        <v>-1.5969511999999999</v>
       </c>
       <c r="F32" s="29" t="s">
+        <v>43</v>
+      </c>
+      <c r="G32" s="12" t="s">
         <v>44</v>
-      </c>
-      <c r="G32" s="12" t="s">
-        <v>45</v>
       </c>
       <c r="H32" s="13" t="s">
         <v>10</v>
@@ -2345,15 +2274,23 @@
       </c>
     </row>
     <row r="33" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="25"/>
-      <c r="B33" s="25"/>
-      <c r="C33" s="25"/>
-      <c r="D33" s="25"/>
+      <c r="A33" s="14" t="s">
+        <v>185</v>
+      </c>
+      <c r="B33" s="15" t="s">
+        <v>135</v>
+      </c>
+      <c r="C33" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="D33" s="2">
+        <v>-0.95799999999999996</v>
+      </c>
       <c r="F33" s="17" t="s">
-        <v>135</v>
+        <v>118</v>
       </c>
       <c r="G33" s="18" t="s">
-        <v>134</v>
+        <v>117</v>
       </c>
       <c r="H33" s="19" t="s">
         <v>10</v>
@@ -2362,358 +2299,280 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="34" t="s">
-        <v>68</v>
-      </c>
-      <c r="B34" s="35"/>
-      <c r="C34" s="35"/>
-      <c r="D34" s="35"/>
-    </row>
-    <row r="35" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B35" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C35" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="D35" s="10" t="s">
-        <v>69</v>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="B34" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="C34" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D34" s="2">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="B35" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="C35" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D35" s="2">
+        <v>1.5</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="B36" s="12" t="s">
-        <v>150</v>
-      </c>
-      <c r="C36" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="D36" s="1">
-        <v>1.2320122</v>
+      <c r="A36" s="39" t="s">
+        <v>85</v>
+      </c>
+      <c r="B36" s="39" t="s">
+        <v>86</v>
+      </c>
+      <c r="C36" s="45" t="s">
+        <v>143</v>
+      </c>
+      <c r="D36" s="46">
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
-        <v>71</v>
+        <v>145</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>98</v>
+        <v>144</v>
       </c>
       <c r="C37" s="16" t="s">
-        <v>155</v>
+        <v>10</v>
       </c>
       <c r="D37" s="2">
-        <v>1.5243902</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
-        <v>72</v>
-      </c>
-      <c r="B38" s="15" t="s">
-        <v>151</v>
+        <v>87</v>
+      </c>
+      <c r="B38" s="14" t="s">
+        <v>89</v>
       </c>
       <c r="C38" s="16" t="s">
-        <v>155</v>
+        <v>138</v>
       </c>
       <c r="D38" s="2">
-        <v>-1.5969511999999999</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A39" s="14" t="s">
-        <v>202</v>
-      </c>
-      <c r="B39" s="15" t="s">
-        <v>152</v>
-      </c>
-      <c r="C39" s="16" t="s">
-        <v>155</v>
-      </c>
-      <c r="D39" s="2">
-        <v>-0.95799999999999996</v>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="38" t="s">
+        <v>88</v>
+      </c>
+      <c r="B39" s="38" t="s">
+        <v>132</v>
+      </c>
+      <c r="C39" s="43" t="s">
+        <v>138</v>
+      </c>
+      <c r="D39" s="44">
+        <v>-0.82799999999999996</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A40" s="14" t="s">
-        <v>73</v>
-      </c>
-      <c r="B40" s="15" t="s">
-        <v>153</v>
-      </c>
-      <c r="C40" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D40" s="2">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A41" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="B41" s="15" t="s">
-        <v>154</v>
-      </c>
-      <c r="C41" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D41" s="2">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A42" s="39" t="s">
-        <v>102</v>
-      </c>
-      <c r="B42" s="39" t="s">
-        <v>103</v>
-      </c>
-      <c r="C42" s="45" t="s">
-        <v>160</v>
-      </c>
-      <c r="D42" s="46">
-        <v>0</v>
+      <c r="A40" s="34"/>
+      <c r="B40" s="34"/>
+      <c r="C40" s="34"/>
+      <c r="D40" s="34"/>
+    </row>
+    <row r="41" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="36" t="s">
+        <v>58</v>
+      </c>
+      <c r="B41" s="37"/>
+      <c r="C41" s="37"/>
+      <c r="D41" s="37"/>
+    </row>
+    <row r="42" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B42" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C42" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D42" s="10" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A43" s="14" t="s">
-        <v>162</v>
-      </c>
-      <c r="B43" s="15" t="s">
-        <v>161</v>
-      </c>
-      <c r="C43" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D43" s="2">
-        <v>1.5</v>
+      <c r="A43" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="B43" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="C43" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D43" s="1">
+        <v>1.65</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="B44" s="14" t="s">
-        <v>106</v>
+        <v>61</v>
+      </c>
+      <c r="B44" s="15" t="s">
+        <v>62</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>155</v>
+        <v>139</v>
       </c>
       <c r="D44" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="38" t="s">
-        <v>105</v>
-      </c>
-      <c r="B45" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="C45" s="43" t="s">
-        <v>155</v>
-      </c>
-      <c r="D45" s="44">
-        <v>-0.82799999999999996</v>
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A45" s="14" t="s">
+        <v>63</v>
+      </c>
+      <c r="B45" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="C45" s="16" t="s">
+        <v>139</v>
+      </c>
+      <c r="D45" s="2">
+        <v>1200</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A46" s="34"/>
-      <c r="B46" s="34"/>
-      <c r="C46" s="34"/>
-      <c r="D46" s="34"/>
-    </row>
-    <row r="47" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="36" t="s">
-        <v>75</v>
-      </c>
-      <c r="B47" s="37"/>
-      <c r="C47" s="37"/>
-      <c r="D47" s="37"/>
-    </row>
-    <row r="48" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B48" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C48" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="D48" s="10" t="s">
+      <c r="A46" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="B46" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="C46" s="16" t="s">
+        <v>140</v>
+      </c>
+      <c r="D46" s="2">
+        <v>1027</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A47" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="B47" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="C47" s="16" t="s">
         <v>69</v>
       </c>
+      <c r="D47" s="2">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A48" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="B48" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="C48" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D48" s="2">
+        <v>20</v>
+      </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="B49" s="12" t="s">
-        <v>77</v>
-      </c>
-      <c r="C49" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="D49" s="1">
-        <v>1.65</v>
+      <c r="A49" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="B49" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="C49" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D49" s="2">
+        <v>20</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B50" s="15" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="C50" s="16" t="s">
-        <v>156</v>
+        <v>10</v>
       </c>
       <c r="D50" s="2">
-        <v>1200</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="B51" s="15" t="s">
-        <v>81</v>
-      </c>
-      <c r="C51" s="16" t="s">
-        <v>156</v>
-      </c>
-      <c r="D51" s="2">
-        <v>1200</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="14" t="s">
-        <v>82</v>
-      </c>
-      <c r="B52" s="15" t="s">
-        <v>83</v>
-      </c>
-      <c r="C52" s="16" t="s">
-        <v>157</v>
-      </c>
-      <c r="D52" s="2">
-        <v>1027</v>
+      <c r="A51" s="39" t="s">
+        <v>76</v>
+      </c>
+      <c r="B51" s="40" t="s">
+        <v>77</v>
+      </c>
+      <c r="C51" s="41" t="s">
+        <v>10</v>
+      </c>
+      <c r="D51" s="42">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="18" t="s">
+        <v>84</v>
+      </c>
+      <c r="B52" s="48" t="s">
+        <v>90</v>
+      </c>
+      <c r="C52" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D52" s="4">
+        <v>2</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="14" t="s">
-        <v>84</v>
-      </c>
-      <c r="B53" s="15" t="s">
-        <v>85</v>
-      </c>
-      <c r="C53" s="16" t="s">
-        <v>86</v>
-      </c>
-      <c r="D53" s="2">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="B54" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="C54" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D54" s="2">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="14" t="s">
-        <v>89</v>
-      </c>
-      <c r="B55" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="C55" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D55" s="2">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="14" t="s">
-        <v>91</v>
-      </c>
-      <c r="B56" s="15" t="s">
-        <v>92</v>
-      </c>
-      <c r="C56" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D56" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="39" t="s">
-        <v>93</v>
-      </c>
-      <c r="B57" s="40" t="s">
-        <v>94</v>
-      </c>
-      <c r="C57" s="41" t="s">
-        <v>10</v>
-      </c>
-      <c r="D57" s="42">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="18" t="s">
-        <v>101</v>
-      </c>
-      <c r="B58" s="48" t="s">
-        <v>107</v>
-      </c>
-      <c r="C58" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D58" s="4">
-        <v>2</v>
-      </c>
+      <c r="A53" s="37"/>
+      <c r="B53" s="37"/>
+      <c r="C53" s="37"/>
+      <c r="D53" s="37"/>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="37"/>
-      <c r="B59" s="37"/>
-      <c r="C59" s="37"/>
-      <c r="D59" s="37"/>
-    </row>
-    <row r="65" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C65" s="64"/>
-    </row>
-    <row r="66" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C66" s="63"/>
-    </row>
-    <row r="72" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B72" s="47"/>
+      <c r="C59" s="64"/>
+    </row>
+    <row r="60" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C60" s="63"/>
+    </row>
+    <row r="66" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B66" s="47"/>
     </row>
   </sheetData>
   <sheetProtection formatColumns="0" selectLockedCells="1"/>
   <protectedRanges>
-    <protectedRange sqref="I3:I6 I8 I12:I16 I25:I28 D15:D17 I32 D21:D32 I19:I20 D3:D6 D8:D13" name="Range1_1"/>
+    <protectedRange sqref="I3:I6 I8 I12:I16 I25:I28 D15:D17 I32 I19:I20 D3:D6 D8:D13 D21:D26" name="Range1_1"/>
     <protectedRange sqref="D7 D14" name="Range1_1_1"/>
-    <protectedRange sqref="D43 D36:D41" name="Range1_1_3"/>
-    <protectedRange sqref="D49:D58" name="Range1_1_4"/>
+    <protectedRange sqref="D37 D30:D35" name="Range1_1_3"/>
+    <protectedRange sqref="D43:D52" name="Range1_1_4"/>
   </protectedRanges>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -2735,140 +2594,140 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>216</v>
+        <v>190</v>
       </c>
       <c r="B1" t="s">
-        <v>221</v>
+        <v>195</v>
       </c>
       <c r="C1" t="s">
-        <v>163</v>
+        <v>146</v>
       </c>
       <c r="D1" t="s">
-        <v>176</v>
+        <v>159</v>
       </c>
       <c r="E1" t="s">
-        <v>95</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>215</v>
+        <v>189</v>
       </c>
       <c r="B3" t="s">
-        <v>184</v>
+        <v>167</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="50" t="s">
-        <v>177</v>
+        <v>160</v>
       </c>
       <c r="B4" t="s">
-        <v>185</v>
+        <v>168</v>
       </c>
       <c r="C4" t="s">
-        <v>186</v>
+        <v>169</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="50" t="s">
-        <v>178</v>
+        <v>161</v>
       </c>
       <c r="B5" t="s">
-        <v>191</v>
+        <v>174</v>
       </c>
       <c r="C5" t="s">
-        <v>198</v>
+        <v>181</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="50" t="s">
-        <v>179</v>
+        <v>162</v>
       </c>
       <c r="B6" t="s">
-        <v>192</v>
+        <v>175</v>
       </c>
       <c r="C6" t="s">
-        <v>198</v>
+        <v>181</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="50" t="s">
-        <v>180</v>
+        <v>163</v>
       </c>
       <c r="B7" t="s">
-        <v>193</v>
+        <v>176</v>
       </c>
       <c r="C7" t="s">
-        <v>198</v>
+        <v>181</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="50" t="s">
-        <v>181</v>
+        <v>164</v>
       </c>
       <c r="B8" t="s">
-        <v>197</v>
+        <v>180</v>
       </c>
       <c r="C8" t="s">
-        <v>95</v>
+        <v>78</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="50" t="s">
-        <v>182</v>
+        <v>165</v>
       </c>
       <c r="B9" t="s">
-        <v>194</v>
+        <v>177</v>
       </c>
       <c r="C9" t="s">
-        <v>198</v>
+        <v>181</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>195</v>
+        <v>178</v>
       </c>
       <c r="C10" t="s">
-        <v>198</v>
+        <v>181</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>196</v>
+        <v>179</v>
       </c>
       <c r="C11" t="s">
-        <v>198</v>
+        <v>181</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>187</v>
+        <v>170</v>
       </c>
       <c r="C12" t="s">
-        <v>188</v>
+        <v>171</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>189</v>
+        <v>172</v>
       </c>
       <c r="C13" t="s">
-        <v>190</v>
+        <v>173</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="16" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="54" t="s">
-        <v>164</v>
+        <v>147</v>
       </c>
       <c r="B16" s="54" t="s">
         <v>4</v>
       </c>
       <c r="C16" s="54" t="s">
-        <v>172</v>
+        <v>155</v>
       </c>
       <c r="D16" s="58" t="s">
-        <v>175</v>
+        <v>158</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -2876,7 +2735,7 @@
         <v>0</v>
       </c>
       <c r="B17" s="55" t="s">
-        <v>165</v>
+        <v>148</v>
       </c>
       <c r="C17" s="59">
         <v>0.66720000000000002</v>
@@ -2892,7 +2751,7 @@
         <v>1</v>
       </c>
       <c r="B18" s="56" t="s">
-        <v>166</v>
+        <v>149</v>
       </c>
       <c r="C18" s="60">
         <v>128.0189</v>
@@ -2902,7 +2761,7 @@
         <v>2.1336483333333334</v>
       </c>
       <c r="E18" t="s">
-        <v>174</v>
+        <v>157</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -2911,7 +2770,7 @@
         <v>2</v>
       </c>
       <c r="B19" s="56" t="s">
-        <v>167</v>
+        <v>150</v>
       </c>
       <c r="C19" s="60">
         <v>1.8109999999999999</v>
@@ -2927,7 +2786,7 @@
         <v>3</v>
       </c>
       <c r="B20" s="56" t="s">
-        <v>168</v>
+        <v>151</v>
       </c>
       <c r="C20" s="60">
         <v>0.56489999999999996</v>
@@ -2943,7 +2802,7 @@
         <v>4</v>
       </c>
       <c r="B21" s="56" t="s">
-        <v>169</v>
+        <v>152</v>
       </c>
       <c r="C21" s="60">
         <v>1.2150000000000001</v>
@@ -2959,7 +2818,7 @@
         <v>5</v>
       </c>
       <c r="B22" s="56" t="s">
-        <v>170</v>
+        <v>153</v>
       </c>
       <c r="C22" s="60">
         <v>15.2134</v>
@@ -2975,7 +2834,7 @@
         <v>6</v>
       </c>
       <c r="B23" s="57" t="s">
-        <v>171</v>
+        <v>154</v>
       </c>
       <c r="C23" s="61">
         <v>648.27599999999995</v>
@@ -2993,12 +2852,12 @@
         <v>0.3858785714285714</v>
       </c>
       <c r="G23" t="s">
-        <v>201</v>
+        <v>184</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="65" t="s">
-        <v>173</v>
+        <v>156</v>
       </c>
       <c r="B24" s="66"/>
       <c r="C24" s="52">
@@ -3014,154 +2873,154 @@
         <v>23.152714285714286</v>
       </c>
       <c r="G24" t="s">
-        <v>200</v>
+        <v>183</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E28" s="8"/>
       <c r="F28" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E29" s="51"/>
       <c r="F29" t="s">
-        <v>199</v>
+        <v>182</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>216</v>
+        <v>190</v>
       </c>
       <c r="B31" t="s">
-        <v>220</v>
+        <v>194</v>
       </c>
       <c r="C31" t="s">
-        <v>222</v>
+        <v>196</v>
       </c>
       <c r="D31" t="s">
-        <v>176</v>
+        <v>159</v>
       </c>
       <c r="E31" t="s">
-        <v>95</v>
+        <v>78</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>215</v>
+        <v>189</v>
       </c>
       <c r="B33" t="s">
-        <v>184</v>
+        <v>167</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="50" t="s">
-        <v>217</v>
+        <v>191</v>
       </c>
       <c r="B34" t="s">
-        <v>185</v>
+        <v>168</v>
       </c>
       <c r="C34" t="s">
-        <v>186</v>
+        <v>169</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="50" t="s">
-        <v>218</v>
+        <v>192</v>
       </c>
       <c r="B35" t="s">
-        <v>191</v>
+        <v>174</v>
       </c>
       <c r="C35" t="s">
-        <v>198</v>
+        <v>181</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="50" t="s">
-        <v>219</v>
+        <v>193</v>
       </c>
       <c r="B36" t="s">
-        <v>192</v>
+        <v>175</v>
       </c>
       <c r="C36" t="s">
-        <v>198</v>
+        <v>181</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="50" t="s">
-        <v>180</v>
+        <v>163</v>
       </c>
       <c r="B37" t="s">
-        <v>193</v>
+        <v>176</v>
       </c>
       <c r="C37" t="s">
-        <v>198</v>
+        <v>181</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="50" t="s">
-        <v>181</v>
+        <v>164</v>
       </c>
       <c r="B38" t="s">
-        <v>197</v>
+        <v>180</v>
       </c>
       <c r="C38" t="s">
-        <v>95</v>
+        <v>78</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
-        <v>194</v>
+        <v>177</v>
       </c>
       <c r="C39" t="s">
-        <v>198</v>
+        <v>181</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
-        <v>195</v>
+        <v>178</v>
       </c>
       <c r="C40" t="s">
-        <v>198</v>
+        <v>181</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
-        <v>196</v>
+        <v>179</v>
       </c>
       <c r="C41" t="s">
-        <v>198</v>
+        <v>181</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B42" t="s">
-        <v>187</v>
+        <v>170</v>
       </c>
       <c r="C42" t="s">
-        <v>188</v>
+        <v>171</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B43" t="s">
-        <v>189</v>
+        <v>172</v>
       </c>
       <c r="C43" t="s">
-        <v>190</v>
+        <v>173</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="46" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="54" t="s">
-        <v>164</v>
+        <v>147</v>
       </c>
       <c r="B46" s="54" t="s">
         <v>4</v>
       </c>
       <c r="C46" s="54" t="s">
-        <v>172</v>
+        <v>155</v>
       </c>
       <c r="D46" s="58" t="s">
-        <v>175</v>
+        <v>158</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
@@ -3169,7 +3028,7 @@
         <v>0</v>
       </c>
       <c r="B47" s="55" t="s">
-        <v>165</v>
+        <v>148</v>
       </c>
       <c r="C47" s="59">
         <v>0.66720000000000002</v>
@@ -3179,7 +3038,7 @@
         <v>1.112E-2</v>
       </c>
       <c r="F47" t="s">
-        <v>223</v>
+        <v>197</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
@@ -3188,7 +3047,7 @@
         <v>1</v>
       </c>
       <c r="B48" s="56" t="s">
-        <v>166</v>
+        <v>149</v>
       </c>
       <c r="C48" s="60">
         <v>128.0189</v>
@@ -3198,13 +3057,13 @@
         <v>2.1336483333333334</v>
       </c>
       <c r="E48" t="s">
-        <v>174</v>
+        <v>157</v>
       </c>
       <c r="F48" t="s">
-        <v>172</v>
+        <v>155</v>
       </c>
       <c r="G48" t="s">
-        <v>175</v>
+        <v>158</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
@@ -3213,7 +3072,7 @@
         <v>2</v>
       </c>
       <c r="B49" s="56" t="s">
-        <v>167</v>
+        <v>150</v>
       </c>
       <c r="C49" s="60">
         <v>77.920665999999997</v>
@@ -3236,7 +3095,7 @@
         <v>3</v>
       </c>
       <c r="B50" s="56" t="s">
-        <v>168</v>
+        <v>151</v>
       </c>
       <c r="C50" s="60">
         <v>0.56489999999999996</v>
@@ -3252,7 +3111,7 @@
         <v>4</v>
       </c>
       <c r="B51" s="56" t="s">
-        <v>169</v>
+        <v>152</v>
       </c>
       <c r="C51" s="60">
         <v>2.6115067000000001</v>
@@ -3268,7 +3127,7 @@
         <v>5</v>
       </c>
       <c r="B52" s="56" t="s">
-        <v>170</v>
+        <v>153</v>
       </c>
       <c r="C52" s="60">
         <v>32.553324799999999</v>
@@ -3284,7 +3143,7 @@
         <v>6</v>
       </c>
       <c r="B53" s="57" t="s">
-        <v>171</v>
+        <v>154</v>
       </c>
       <c r="C53" s="61">
         <v>197.9727273</v>
@@ -3296,7 +3155,7 @@
     </row>
     <row r="54" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="65" t="s">
-        <v>173</v>
+        <v>156</v>
       </c>
       <c r="B54" s="66"/>
       <c r="C54" s="52">

</xml_diff>

<commit_message>
Changing input to be James Island
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA3F0304-26ED-4EB8-84C3-6FD2267592BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EFA5B425-80CD-4624-AAE7-39CFED0A03EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="206">
   <si>
     <t>StormSim Project General Inputs</t>
   </si>
@@ -372,292 +372,289 @@
     <t>Tidal file used to randomly sample tidal values for storm SWL.</t>
   </si>
   <si>
+    <t>NAVD</t>
+  </si>
+  <si>
+    <t>m</t>
+  </si>
+  <si>
+    <t>chs_sp_depth</t>
+  </si>
+  <si>
+    <t>CHS savepoint depth (Will be used if not found in h5)</t>
+  </si>
+  <si>
+    <t>[16 84]</t>
+  </si>
+  <si>
+    <t>Use AEP or AEF for hazard curves (1 - AEP, 0-AEF)</t>
+  </si>
+  <si>
+    <t>pros_use_aep</t>
+  </si>
+  <si>
+    <t>case_name</t>
+  </si>
+  <si>
+    <t>Case Name</t>
+  </si>
+  <si>
+    <t>James_Island</t>
+  </si>
+  <si>
+    <t>workflow</t>
+  </si>
+  <si>
+    <t>Include forcing peaks files as part of the analysis. (0/1)</t>
+  </si>
+  <si>
+    <t>Include forcing timeseries files as part of the analysis. (0/1)</t>
+  </si>
+  <si>
+    <t>use_peaks</t>
+  </si>
+  <si>
+    <t>Create Wave Height Priority Peaks Dataset (WLP) (0/1). (Requires peaks and timeseries files)</t>
+  </si>
+  <si>
+    <t>Create Water Level Priority Peaks Dataset (WLP) (0/1). (Requires peaks and timeseries files)</t>
+  </si>
+  <si>
+    <t>mcs_sampling_mode</t>
+  </si>
+  <si>
+    <t>Sampling method used to pick storms for LCs. (0 - historical, 1 - probabilistic)</t>
+  </si>
+  <si>
+    <t>create_wlp</t>
+  </si>
+  <si>
+    <t>create_whp</t>
+  </si>
+  <si>
+    <t>Berm Elevation (Negative Below Datum Zero)</t>
+  </si>
+  <si>
+    <t>Crest Elevation/Top of Wall Elevation</t>
+  </si>
+  <si>
+    <t>Mound Toe Elevation (Negative Below Datum Zero)</t>
+  </si>
+  <si>
+    <t>Bottom of Wall Elevation (Applies to wall type structures)</t>
+  </si>
+  <si>
+    <t>Mound/Berm Seaward Slope</t>
+  </si>
+  <si>
+    <t>Mound Landward Slope</t>
+  </si>
+  <si>
+    <t>[m]</t>
+  </si>
+  <si>
+    <t>[kg]</t>
+  </si>
+  <si>
+    <t>[kg/m^3]</t>
+  </si>
+  <si>
+    <t>[m^3/s/m]</t>
+  </si>
+  <si>
+    <t>[N/m^2]</t>
+  </si>
+  <si>
+    <t>[deg]</t>
+  </si>
+  <si>
+    <t>Wall Seaward Slope (Same Slope Is Assumed For Landward Slope)</t>
+  </si>
+  <si>
+    <t>berm_slope</t>
+  </si>
+  <si>
+    <t>RB1 + RB3 w WLP &amp; WHP</t>
+  </si>
+  <si>
+    <t>Step #</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set-up Environment </t>
+  </si>
+  <si>
+    <t>CHS Data Formater</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create Project Forcing </t>
+  </si>
+  <si>
+    <t>Create Structure Geometry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Call Uncertainty Engine </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Call Project Forcing Adjsuter </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Call Project Responses </t>
+  </si>
+  <si>
+    <t>Time [s]</t>
+  </si>
+  <si>
+    <t>Total Time</t>
+  </si>
+  <si>
+    <t>(Processed 1031 TC storms + 100 XCs)</t>
+  </si>
+  <si>
+    <t>Time [min]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rubble mound </t>
+  </si>
+  <si>
+    <t>SWL</t>
+  </si>
+  <si>
+    <t>Hm0</t>
+  </si>
+  <si>
+    <t>Tp</t>
+  </si>
+  <si>
+    <t>q</t>
+  </si>
+  <si>
+    <t>R2p</t>
+  </si>
+  <si>
+    <t>Dn50</t>
+  </si>
+  <si>
+    <t>Time Per Dataset (Peak Maxima , Peak WLP, Peak WHP &amp; RB3</t>
+  </si>
+  <si>
+    <t>StormSim Library Stress Testing</t>
+  </si>
+  <si>
+    <t>Computational Kernel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Response Base </t>
+  </si>
+  <si>
+    <t>Workflow</t>
+  </si>
+  <si>
+    <t>PROS</t>
+  </si>
+  <si>
+    <t>Structure Type</t>
+  </si>
+  <si>
+    <t>Rubblemound</t>
+  </si>
+  <si>
+    <t>Use Peaks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Use Timeseries </t>
+  </si>
+  <si>
+    <t>WLP &amp; WHP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rand Tides </t>
+  </si>
+  <si>
+    <t>SLR</t>
+  </si>
+  <si>
+    <t>Depth Limitation</t>
+  </si>
+  <si>
+    <t>Storm Sampling</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>Time Per Response</t>
+  </si>
+  <si>
+    <t>secs</t>
+  </si>
+  <si>
+    <t>Mins</t>
+  </si>
+  <si>
+    <t>wall_bottom_elevation</t>
+  </si>
+  <si>
+    <t>StormSim workflow to call for project. (1 - StormSim:PROS, 2- StormSim:EVA, 3- StormSim:LCS)</t>
+  </si>
+  <si>
+    <t>Responses</t>
+  </si>
+  <si>
+    <t>James Island</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peaks Reliability </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seaside Armor damage </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leeside Armor damage </t>
+  </si>
+  <si>
+    <t>Life Cycle Simulation</t>
+  </si>
+  <si>
+    <t>Response Base Simulation</t>
+  </si>
+  <si>
+    <t>Peaks + Timeseries w WLP &amp; WHP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Historical Sampling </t>
+  </si>
+  <si>
+    <t>Alternative_Feas</t>
+  </si>
+  <si>
+    <t>Sta339_plus2</t>
+  </si>
+  <si>
+    <t>CO-OPS_8571421_Bishops_Head_Pred_tide_MSL_m.csv</t>
+  </si>
+  <si>
     <t>StormSim_Library\CHS\Bias_Correction_Files\NACCS_Comb_BiasUncertainty_perVG_rta.mat</t>
   </si>
   <si>
-    <t>NAVD</t>
-  </si>
-  <si>
-    <t>m</t>
-  </si>
-  <si>
-    <t>chs_sp_depth</t>
-  </si>
-  <si>
-    <t>CHS savepoint depth (Will be used if not found in h5)</t>
-  </si>
-  <si>
-    <t>[16 84]</t>
-  </si>
-  <si>
-    <t>Use AEP or AEF for hazard curves (1 - AEP, 0-AEF)</t>
-  </si>
-  <si>
-    <t>pros_use_aep</t>
-  </si>
-  <si>
-    <t>case_name</t>
-  </si>
-  <si>
-    <t>Case Name</t>
-  </si>
-  <si>
-    <t>James_Island</t>
-  </si>
-  <si>
-    <t>workflow</t>
-  </si>
-  <si>
-    <t>Include forcing peaks files as part of the analysis. (0/1)</t>
-  </si>
-  <si>
-    <t>Include forcing timeseries files as part of the analysis. (0/1)</t>
-  </si>
-  <si>
-    <t>use_peaks</t>
-  </si>
-  <si>
-    <t>Create Wave Height Priority Peaks Dataset (WLP) (0/1). (Requires peaks and timeseries files)</t>
-  </si>
-  <si>
-    <t>Create Water Level Priority Peaks Dataset (WLP) (0/1). (Requires peaks and timeseries files)</t>
-  </si>
-  <si>
-    <t>mcs_sampling_mode</t>
-  </si>
-  <si>
-    <t>Sampling method used to pick storms for LCs. (0 - historical, 1 - probabilistic)</t>
-  </si>
-  <si>
-    <t>create_wlp</t>
-  </si>
-  <si>
-    <t>create_whp</t>
-  </si>
-  <si>
-    <t>Berm Elevation (Negative Below Datum Zero)</t>
-  </si>
-  <si>
-    <t>Crest Elevation/Top of Wall Elevation</t>
-  </si>
-  <si>
-    <t>Mound Toe Elevation (Negative Below Datum Zero)</t>
-  </si>
-  <si>
-    <t>Bottom of Wall Elevation (Applies to wall type structures)</t>
-  </si>
-  <si>
-    <t>Mound/Berm Seaward Slope</t>
-  </si>
-  <si>
-    <t>Mound Landward Slope</t>
-  </si>
-  <si>
-    <t>[m]</t>
-  </si>
-  <si>
-    <t>[kg]</t>
-  </si>
-  <si>
-    <t>[kg/m^3]</t>
-  </si>
-  <si>
-    <t>[m^3/s/m]</t>
-  </si>
-  <si>
-    <t>[N/m^2]</t>
-  </si>
-  <si>
-    <t>[deg]</t>
-  </si>
-  <si>
-    <t>Wall Seaward Slope (Same Slope Is Assumed For Landward Slope)</t>
-  </si>
-  <si>
-    <t>berm_slope</t>
-  </si>
-  <si>
-    <t>RB1 + RB3 w WLP &amp; WHP</t>
-  </si>
-  <si>
-    <t>Step #</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Set-up Environment </t>
-  </si>
-  <si>
-    <t>CHS Data Formater</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Create Project Forcing </t>
-  </si>
-  <si>
-    <t>Create Structure Geometry</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Call Uncertainty Engine </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Call Project Forcing Adjsuter </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Call Project Responses </t>
-  </si>
-  <si>
-    <t>Time [s]</t>
-  </si>
-  <si>
-    <t>Total Time</t>
-  </si>
-  <si>
-    <t>(Processed 1031 TC storms + 100 XCs)</t>
-  </si>
-  <si>
-    <t>Time [min]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rubble mound </t>
-  </si>
-  <si>
-    <t>SWL</t>
-  </si>
-  <si>
-    <t>Hm0</t>
-  </si>
-  <si>
-    <t>Tp</t>
-  </si>
-  <si>
-    <t>q</t>
-  </si>
-  <si>
-    <t>R2p</t>
-  </si>
-  <si>
-    <t>Dn50</t>
-  </si>
-  <si>
-    <t>Time Per Dataset (Peak Maxima , Peak WLP, Peak WHP &amp; RB3</t>
-  </si>
-  <si>
-    <t>StormSim Library Stress Testing</t>
-  </si>
-  <si>
-    <t>Computational Kernel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Response Base </t>
-  </si>
-  <si>
-    <t>Workflow</t>
-  </si>
-  <si>
-    <t>PROS</t>
-  </si>
-  <si>
-    <t>Structure Type</t>
-  </si>
-  <si>
-    <t>Rubblemound</t>
-  </si>
-  <si>
-    <t>Use Peaks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Use Timeseries </t>
-  </si>
-  <si>
-    <t>WLP &amp; WHP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rand Tides </t>
-  </si>
-  <si>
-    <t>SLR</t>
-  </si>
-  <si>
-    <t>Depth Limitation</t>
-  </si>
-  <si>
-    <t>Storm Sampling</t>
-  </si>
-  <si>
-    <t>yes</t>
-  </si>
-  <si>
-    <t>Time Per Response</t>
-  </si>
-  <si>
-    <t>secs</t>
-  </si>
-  <si>
-    <t>Mins</t>
-  </si>
-  <si>
-    <t>wall_bottom_elevation</t>
-  </si>
-  <si>
-    <t>Transect_001</t>
-  </si>
-  <si>
-    <t>CO-OPS_8571421_Bishops_Head_Pred_tide_MSL_m.csv</t>
-  </si>
-  <si>
-    <t>StormSim workflow to call for project. (1 - StormSim:PROS, 2- StormSim:EVA, 3- StormSim:LCS)</t>
-  </si>
-  <si>
-    <t>Responses</t>
-  </si>
-  <si>
-    <t>James Island</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Peaks Reliability </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Seaside Armor damage </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leeside Armor damage </t>
-  </si>
-  <si>
-    <t>Life Cycle Simulation</t>
-  </si>
-  <si>
-    <t>Response Base Simulation</t>
-  </si>
-  <si>
-    <t>Peaks + Timeseries w WLP &amp; WHP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Historical Sampling </t>
-  </si>
-  <si>
-    <t>Alternative_002</t>
-  </si>
-  <si>
-    <t>TC</t>
+    <t>prob_mass_source</t>
+  </si>
+  <si>
+    <t>Probability Masses (CHS -&gt; MCSim_Inputs folder path, Custom Modeling -&gt; .mat filename with relative path)</t>
+  </si>
+  <si>
+    <t>prob_mass_from_MB_SP2243\prob_mass_from_MB_SP2243.mat</t>
   </si>
   <si>
     <t>forcing_type</t>
   </si>
   <si>
-    <t>Forcing Data Source (0 - CHS Native Data, 1- Custom Modeling)</t>
-  </si>
-  <si>
-    <t>prob_mass_source</t>
-  </si>
-  <si>
-    <t>Probability Masses (CHS -&gt; MCSim_Inputs folder path, Custom Modeling -&gt; .mat filename with relative path)</t>
-  </si>
-  <si>
-    <t>prob_mass_from_MB_SP2243\prob_mass_from_MB_SP2243.mat</t>
+    <t>prob_mass_from_MB_SP2243\CHS_Data_from_MB_SP2243.mat</t>
+  </si>
+  <si>
+    <t>Forcing Data Source (0 - CHS/CSTORM, 1- Custom Modeling)</t>
   </si>
   <si>
     <t>CHS Zip Folder or Custom Modeling .mat File (Relative Path)</t>
-  </si>
-  <si>
-    <t>prob_mass_from_MB_SP2243\CHS_Data_from_MB_SP2243.mat</t>
   </si>
 </sst>
 </file>
@@ -1524,8 +1521,8 @@
   <dimension ref="A1:I66"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="52.5703125" customWidth="1"/>
-    <col min="2" max="2" width="162.85546875" customWidth="1"/>
+    <col min="1" max="1" width="24.5703125" customWidth="1"/>
+    <col min="2" max="2" width="100.42578125" customWidth="1"/>
     <col min="3" max="3" width="19.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="171.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="28.42578125" customWidth="1"/>
@@ -1584,7 +1581,7 @@
         <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F3" s="49" t="s">
         <v>98</v>
@@ -1593,7 +1590,7 @@
         <v>91</v>
       </c>
       <c r="H3" s="13" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I3" s="13">
         <v>0.33979999999999999</v>
@@ -1610,7 +1607,7 @@
         <v>10</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>186</v>
+        <v>196</v>
       </c>
       <c r="F4" s="49" t="s">
         <v>99</v>
@@ -1627,16 +1624,16 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="B5" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="B5" s="15" t="s">
-        <v>120</v>
-      </c>
       <c r="C5" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="F5" s="49" t="s">
         <v>101</v>
@@ -1645,7 +1642,7 @@
         <v>93</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I5" s="13">
         <v>0.3</v>
@@ -1662,7 +1659,7 @@
         <v>10</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F6" s="49" t="s">
         <v>100</v>
@@ -1688,7 +1685,7 @@
         <v>10</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F7" s="14" t="s">
         <v>102</v>
@@ -1697,7 +1694,7 @@
         <v>96</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="I7" s="2">
         <v>0</v>
@@ -1705,16 +1702,16 @@
     </row>
     <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="14" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="C8" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F8" s="17" t="s">
         <v>97</v>
@@ -1758,7 +1755,7 @@
         <v>10</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>199</v>
+        <v>78</v>
       </c>
       <c r="F10" s="26" t="s">
         <v>103</v>
@@ -1804,7 +1801,7 @@
         <v>10</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
       <c r="F12" s="30" t="s">
         <v>105</v>
@@ -1813,7 +1810,7 @@
         <v>45</v>
       </c>
       <c r="H12" s="16" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I12" s="2">
         <v>0.5</v>
@@ -1839,7 +1836,7 @@
         <v>48</v>
       </c>
       <c r="H13" s="31" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="I13" s="2">
         <v>0.43</v>
@@ -1847,16 +1844,16 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C14" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D14" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F14" s="14" t="s">
         <v>82</v>
@@ -1865,7 +1862,7 @@
         <v>46</v>
       </c>
       <c r="H14" s="16" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="I14" s="2">
         <v>0.78</v>
@@ -1876,7 +1873,7 @@
         <v>79</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C15" s="16" t="s">
         <v>10</v>
@@ -1891,7 +1888,7 @@
         <v>47</v>
       </c>
       <c r="H15" s="19" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I15" s="3">
         <v>0.13</v>
@@ -1899,16 +1896,16 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D16" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F16" s="27"/>
       <c r="G16" s="27"/>
@@ -1917,16 +1914,16 @@
     </row>
     <row r="17" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="17" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C17" s="19" t="s">
         <v>10</v>
       </c>
       <c r="D17" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F17" s="7" t="s">
         <v>1</v>
@@ -1974,7 +1971,7 @@
         <v>10</v>
       </c>
       <c r="I19" s="1">
-        <v>1000</v>
+        <v>9</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2005,22 +2002,22 @@
     </row>
     <row r="21" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="11" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="C21" s="28" t="s">
         <v>10</v>
       </c>
       <c r="D21" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F21" s="17" t="s">
+        <v>127</v>
+      </c>
+      <c r="G21" s="18" t="s">
         <v>128</v>
-      </c>
-      <c r="G21" s="18" t="s">
-        <v>129</v>
       </c>
       <c r="H21" s="19" t="s">
         <v>10</v>
@@ -2049,16 +2046,16 @@
     </row>
     <row r="23" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="B23" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="B23" s="12" t="s">
-        <v>115</v>
-      </c>
       <c r="C23" s="28" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D23" s="1">
-        <v>5</v>
+        <v>2.42</v>
       </c>
       <c r="F23" s="20" t="s">
         <v>26</v>
@@ -2078,7 +2075,7 @@
         <v>10</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>111</v>
+        <v>198</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>3</v>
@@ -2095,16 +2092,16 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="C25" s="28" t="s">
         <v>10</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="F25" s="11" t="s">
         <v>27</v>
@@ -2130,7 +2127,7 @@
         <v>10</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="F26" s="14" t="s">
         <v>31</v>
@@ -2177,7 +2174,7 @@
         <v>37</v>
       </c>
       <c r="H28" s="19" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I28" s="3">
         <v>1</v>
@@ -2206,13 +2203,13 @@
         <v>53</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D30" s="1">
-        <v>1.2320122</v>
+        <v>3.41</v>
       </c>
       <c r="F30" s="26" t="s">
         <v>41</v>
@@ -2229,10 +2226,10 @@
         <v>81</v>
       </c>
       <c r="C31" s="16" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D31" s="2">
-        <v>1.5243902</v>
+        <v>7.01</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>3</v>
@@ -2252,13 +2249,13 @@
         <v>55</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C32" s="16" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D32" s="2">
-        <v>-1.5969511999999999</v>
+        <v>-2.42</v>
       </c>
       <c r="F32" s="29" t="s">
         <v>43</v>
@@ -2275,22 +2272,22 @@
     </row>
     <row r="33" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="14" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B33" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D33" s="2">
         <v>-0.95799999999999996</v>
       </c>
       <c r="F33" s="17" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G33" s="18" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H33" s="19" t="s">
         <v>10</v>
@@ -2304,13 +2301,13 @@
         <v>56</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C34" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D34" s="2">
-        <v>1.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -2318,7 +2315,7 @@
         <v>57</v>
       </c>
       <c r="B35" s="15" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C35" s="16" t="s">
         <v>10</v>
@@ -2335,7 +2332,7 @@
         <v>86</v>
       </c>
       <c r="C36" s="45" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D36" s="46">
         <v>0</v>
@@ -2343,16 +2340,16 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C37" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D37" s="2">
-        <v>1.5</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
@@ -2363,10 +2360,10 @@
         <v>89</v>
       </c>
       <c r="C38" s="16" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D38" s="2">
-        <v>0</v>
+        <v>3.35</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2374,13 +2371,13 @@
         <v>88</v>
       </c>
       <c r="B39" s="38" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C39" s="43" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D39" s="44">
-        <v>-0.82799999999999996</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
@@ -2433,10 +2430,10 @@
         <v>62</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D44" s="2">
-        <v>1200</v>
+        <v>1134</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
@@ -2447,10 +2444,10 @@
         <v>64</v>
       </c>
       <c r="C45" s="16" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D45" s="2">
-        <v>1200</v>
+        <v>1134</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
@@ -2461,7 +2458,7 @@
         <v>66</v>
       </c>
       <c r="C46" s="16" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D46" s="2">
         <v>1027</v>
@@ -2492,7 +2489,7 @@
         <v>10</v>
       </c>
       <c r="D48" s="2">
-        <v>20</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -2506,7 +2503,7 @@
         <v>10</v>
       </c>
       <c r="D49" s="2">
-        <v>20</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
@@ -2520,7 +2517,7 @@
         <v>10</v>
       </c>
       <c r="D50" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
@@ -2534,10 +2531,10 @@
         <v>10</v>
       </c>
       <c r="D51" s="42">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="18" t="s">
         <v>84</v>
       </c>
@@ -2569,10 +2566,15 @@
   </sheetData>
   <sheetProtection formatColumns="0" selectLockedCells="1"/>
   <protectedRanges>
-    <protectedRange sqref="I3:I6 I8 I12:I16 I25:I28 D15:D17 I32 I19:I20 D3:D6 D8:D13 D21:D26" name="Range1_1"/>
+    <protectedRange sqref="I3:I6 I8 I12:I16 I25:I28 D15:D17 I32 D22:D23 I19:I20 D3:D6 D8:D11 D13" name="Range1_1"/>
     <protectedRange sqref="D7 D14" name="Range1_1_1"/>
     <protectedRange sqref="D37 D30:D35" name="Range1_1_3"/>
     <protectedRange sqref="D43:D52" name="Range1_1_4"/>
+    <protectedRange sqref="D12" name="Range1_1_2"/>
+    <protectedRange sqref="D24" name="Range1_1_6_1"/>
+    <protectedRange sqref="D25" name="Range1_1_5"/>
+    <protectedRange sqref="D21" name="Range1_1_6"/>
+    <protectedRange sqref="D26" name="Range1_1_8"/>
   </protectedRanges>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -2594,16 +2596,16 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B1" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="C1" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E1" t="s">
         <v>78</v>
@@ -2611,62 +2613,62 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="50" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B4" t="s">
+        <v>167</v>
+      </c>
+      <c r="C4" t="s">
         <v>168</v>
-      </c>
-      <c r="C4" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="50" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B5" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C5" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="50" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B6" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="50" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B7" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C7" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="50" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B8" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C8" t="s">
         <v>78</v>
@@ -2674,60 +2676,60 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="50" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C9" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C10" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C11" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
+        <v>169</v>
+      </c>
+      <c r="C12" t="s">
         <v>170</v>
-      </c>
-      <c r="C12" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
+        <v>171</v>
+      </c>
+      <c r="C13" t="s">
         <v>172</v>
-      </c>
-      <c r="C13" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="16" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="54" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B16" s="54" t="s">
         <v>4</v>
       </c>
       <c r="C16" s="54" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D16" s="58" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -2735,7 +2737,7 @@
         <v>0</v>
       </c>
       <c r="B17" s="55" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C17" s="59">
         <v>0.66720000000000002</v>
@@ -2751,7 +2753,7 @@
         <v>1</v>
       </c>
       <c r="B18" s="56" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C18" s="60">
         <v>128.0189</v>
@@ -2761,7 +2763,7 @@
         <v>2.1336483333333334</v>
       </c>
       <c r="E18" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -2770,7 +2772,7 @@
         <v>2</v>
       </c>
       <c r="B19" s="56" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C19" s="60">
         <v>1.8109999999999999</v>
@@ -2786,7 +2788,7 @@
         <v>3</v>
       </c>
       <c r="B20" s="56" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C20" s="60">
         <v>0.56489999999999996</v>
@@ -2802,7 +2804,7 @@
         <v>4</v>
       </c>
       <c r="B21" s="56" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C21" s="60">
         <v>1.2150000000000001</v>
@@ -2818,7 +2820,7 @@
         <v>5</v>
       </c>
       <c r="B22" s="56" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C22" s="60">
         <v>15.2134</v>
@@ -2834,7 +2836,7 @@
         <v>6</v>
       </c>
       <c r="B23" s="57" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C23" s="61">
         <v>648.27599999999995</v>
@@ -2852,12 +2854,12 @@
         <v>0.3858785714285714</v>
       </c>
       <c r="G23" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="65" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B24" s="66"/>
       <c r="C24" s="52">
@@ -2873,33 +2875,33 @@
         <v>23.152714285714286</v>
       </c>
       <c r="G24" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E28" s="8"/>
       <c r="F28" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E29" s="51"/>
       <c r="F29" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B31" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="C31" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="D31" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E31" t="s">
         <v>78</v>
@@ -2907,62 +2909,62 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B33" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="50" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="B34" t="s">
+        <v>167</v>
+      </c>
+      <c r="C34" t="s">
         <v>168</v>
-      </c>
-      <c r="C34" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="50" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="B35" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C35" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="50" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="B36" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C36" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="50" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B37" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C37" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="50" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B38" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C38" t="s">
         <v>78</v>
@@ -2970,57 +2972,57 @@
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C39" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C40" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C41" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B42" t="s">
+        <v>169</v>
+      </c>
+      <c r="C42" t="s">
         <v>170</v>
-      </c>
-      <c r="C42" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B43" t="s">
+        <v>171</v>
+      </c>
+      <c r="C43" t="s">
         <v>172</v>
-      </c>
-      <c r="C43" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="46" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="54" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B46" s="54" t="s">
         <v>4</v>
       </c>
       <c r="C46" s="54" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D46" s="58" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
@@ -3028,7 +3030,7 @@
         <v>0</v>
       </c>
       <c r="B47" s="55" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C47" s="59">
         <v>0.66720000000000002</v>
@@ -3038,7 +3040,7 @@
         <v>1.112E-2</v>
       </c>
       <c r="F47" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
@@ -3047,7 +3049,7 @@
         <v>1</v>
       </c>
       <c r="B48" s="56" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C48" s="60">
         <v>128.0189</v>
@@ -3057,13 +3059,13 @@
         <v>2.1336483333333334</v>
       </c>
       <c r="E48" t="s">
+        <v>156</v>
+      </c>
+      <c r="F48" t="s">
+        <v>154</v>
+      </c>
+      <c r="G48" t="s">
         <v>157</v>
-      </c>
-      <c r="F48" t="s">
-        <v>155</v>
-      </c>
-      <c r="G48" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
@@ -3072,7 +3074,7 @@
         <v>2</v>
       </c>
       <c r="B49" s="56" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C49" s="60">
         <v>77.920665999999997</v>
@@ -3095,7 +3097,7 @@
         <v>3</v>
       </c>
       <c r="B50" s="56" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C50" s="60">
         <v>0.56489999999999996</v>
@@ -3111,7 +3113,7 @@
         <v>4</v>
       </c>
       <c r="B51" s="56" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C51" s="60">
         <v>2.6115067000000001</v>
@@ -3127,7 +3129,7 @@
         <v>5</v>
       </c>
       <c r="B52" s="56" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C52" s="60">
         <v>32.553324799999999</v>
@@ -3143,7 +3145,7 @@
         <v>6</v>
       </c>
       <c r="B53" s="57" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C53" s="61">
         <v>197.9727273</v>
@@ -3155,7 +3157,7 @@
     </row>
     <row r="54" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="65" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B54" s="66"/>
       <c r="C54" s="52">

</xml_diff>

<commit_message>
Implementing StormSim PROS FB1 & FB3 for primary responses.
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EFA5B425-80CD-4624-AAE7-39CFED0A03EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7D4AD6E-6E80-4F4B-A46C-487EC01D644D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
+    <workbookView xWindow="13170" yWindow="1740" windowWidth="15180" windowHeight="18870" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
   <sheets>
     <sheet name="James_Island_Midbay" sheetId="1" r:id="rId1"/>
@@ -594,9 +594,6 @@
     <t>wall_bottom_elevation</t>
   </si>
   <si>
-    <t>StormSim workflow to call for project. (1 - StormSim:PROS, 2- StormSim:EVA, 3- StormSim:LCS)</t>
-  </si>
-  <si>
     <t>Responses</t>
   </si>
   <si>
@@ -655,6 +652,9 @@
   </si>
   <si>
     <t>CHS Zip Folder or Custom Modeling .mat File (Relative Path)</t>
+  </si>
+  <si>
+    <t>StormSim workflow to call for project. (1 - StormSim:PROS Response Base (RB), 2- StormSim:EVA, 3- StormSim:LCS, 4- StormSim: PROS Frequency Base (FB))</t>
   </si>
 </sst>
 </file>
@@ -1522,7 +1522,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.5703125" customWidth="1"/>
-    <col min="2" max="2" width="100.42578125" customWidth="1"/>
+    <col min="2" max="2" width="152" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="171.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="28.42578125" customWidth="1"/>
@@ -1607,7 +1607,7 @@
         <v>10</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F4" s="49" t="s">
         <v>99</v>
@@ -1633,7 +1633,7 @@
         <v>10</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F5" s="49" t="s">
         <v>101</v>
@@ -1705,13 +1705,13 @@
         <v>121</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>185</v>
+        <v>205</v>
       </c>
       <c r="C8" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F8" s="17" t="s">
         <v>97</v>
@@ -1801,7 +1801,7 @@
         <v>10</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F12" s="30" t="s">
         <v>105</v>
@@ -2002,10 +2002,10 @@
     </row>
     <row r="21" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="11" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C21" s="28" t="s">
         <v>10</v>
@@ -2075,7 +2075,7 @@
         <v>10</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>3</v>
@@ -2092,16 +2092,16 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
+        <v>198</v>
+      </c>
+      <c r="B25" s="12" t="s">
         <v>199</v>
       </c>
-      <c r="B25" s="12" t="s">
+      <c r="C25" s="28" t="s">
+        <v>10</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>200</v>
-      </c>
-      <c r="C25" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>201</v>
       </c>
       <c r="F25" s="11" t="s">
         <v>27</v>
@@ -2121,13 +2121,13 @@
         <v>42</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C26" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F26" s="14" t="s">
         <v>31</v>
@@ -2596,10 +2596,10 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C1" t="s">
         <v>145</v>
@@ -2613,7 +2613,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B3" t="s">
         <v>166</v>
@@ -2892,13 +2892,13 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B31" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C31" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D31" t="s">
         <v>158</v>
@@ -2909,7 +2909,7 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B33" t="s">
         <v>166</v>
@@ -2917,7 +2917,7 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="50" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B34" t="s">
         <v>167</v>
@@ -2928,7 +2928,7 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="50" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B35" t="s">
         <v>173</v>
@@ -2939,7 +2939,7 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="50" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B36" t="s">
         <v>174</v>
@@ -3040,7 +3040,7 @@
         <v>1.112E-2</v>
       </c>
       <c r="F47" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Minor bug fix for workflow 4
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26529"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26626"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7D4AD6E-6E80-4F4B-A46C-487EC01D644D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ED4FECB-D599-4B43-813F-CF3C99335CD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="13170" yWindow="1740" windowWidth="15180" windowHeight="18870" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
@@ -624,9 +624,6 @@
     <t>Alternative_Feas</t>
   </si>
   <si>
-    <t>Sta339_plus2</t>
-  </si>
-  <si>
     <t>CO-OPS_8571421_Bishops_Head_Pred_tide_MSL_m.csv</t>
   </si>
   <si>
@@ -655,6 +652,9 @@
   </si>
   <si>
     <t>StormSim workflow to call for project. (1 - StormSim:PROS Response Base (RB), 2- StormSim:EVA, 3- StormSim:LCS, 4- StormSim: PROS Frequency Base (FB))</t>
+  </si>
+  <si>
+    <t>Sta339_plus2_floodwall</t>
   </si>
 </sst>
 </file>
@@ -1607,7 +1607,7 @@
         <v>10</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="F4" s="49" t="s">
         <v>99</v>
@@ -1705,7 +1705,7 @@
         <v>121</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C8" s="16" t="s">
         <v>10</v>
@@ -1737,7 +1737,7 @@
         <v>10</v>
       </c>
       <c r="D9" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F9" s="33"/>
       <c r="G9" s="33"/>
@@ -1801,7 +1801,7 @@
         <v>10</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F12" s="30" t="s">
         <v>105</v>
@@ -2002,10 +2002,10 @@
     </row>
     <row r="21" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="11" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C21" s="28" t="s">
         <v>10</v>
@@ -2075,7 +2075,7 @@
         <v>10</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>3</v>
@@ -2092,16 +2092,16 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="B25" s="12" t="s">
         <v>198</v>
       </c>
-      <c r="B25" s="12" t="s">
+      <c r="C25" s="28" t="s">
+        <v>10</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>199</v>
-      </c>
-      <c r="C25" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>200</v>
       </c>
       <c r="F25" s="11" t="s">
         <v>27</v>
@@ -2121,13 +2121,13 @@
         <v>42</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C26" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F26" s="14" t="s">
         <v>31</v>

</xml_diff>

<commit_message>
Adding new subfolder to store figures.
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ED4FECB-D599-4B43-813F-CF3C99335CD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6A81E34-14B7-4E67-8089-D71FA900AE0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13170" yWindow="1740" windowWidth="15180" windowHeight="18870" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
   <sheets>
     <sheet name="James_Island_Midbay" sheetId="1" r:id="rId1"/>
@@ -1737,7 +1737,7 @@
         <v>10</v>
       </c>
       <c r="D9" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F9" s="33"/>
       <c r="G9" s="33"/>

</xml_diff>

<commit_message>
Fixing Replicates for different workflows
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02E49730-9256-4588-ABB0-81877CB3118F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F258395A-B6AA-4DEB-A369-17E1E238E087}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
+    <workbookView xWindow="11160" yWindow="2010" windowWidth="21555" windowHeight="18870" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
   <sheets>
     <sheet name="James_Island_Midbay" sheetId="1" r:id="rId1"/>
@@ -652,9 +652,6 @@
     <t>StormSim workflow to call for project. (1 - StormSim:PROS Response Base (RB), 2- StormSim:EVA, 3- StormSim:LCS, 4- StormSim: PROS Frequency Base (FB))</t>
   </si>
   <si>
-    <t>Sta339_plus2</t>
-  </si>
-  <si>
     <t>apply_random_tides</t>
   </si>
   <si>
@@ -673,7 +670,10 @@
     <t>SST/JPM old vs SST/JPM New</t>
   </si>
   <si>
-    <t>Current_EVA_Tools_same_switch</t>
+    <t>Validation_Case</t>
+  </si>
+  <si>
+    <t>EVA_Case</t>
   </si>
 </sst>
 </file>
@@ -1626,7 +1626,7 @@
         <v>10</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="F4" s="49" t="s">
         <v>99</v>
@@ -1811,10 +1811,10 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
+        <v>204</v>
+      </c>
+      <c r="B12" s="15" t="s">
         <v>205</v>
-      </c>
-      <c r="B12" s="15" t="s">
-        <v>206</v>
       </c>
       <c r="C12" s="16" t="s">
         <v>10</v>
@@ -1846,7 +1846,7 @@
         <v>10</v>
       </c>
       <c r="D13" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F13" s="30" t="s">
         <v>106</v>
@@ -1872,7 +1872,7 @@
         <v>10</v>
       </c>
       <c r="D14" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F14" s="14" t="s">
         <v>82</v>
@@ -2624,22 +2624,22 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixing typo in parser fopr CHS data
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F258395A-B6AA-4DEB-A369-17E1E238E087}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F458B474-1FD1-4A72-B339-78D13FB1503B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11160" yWindow="2010" windowWidth="21555" windowHeight="18870" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
+    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
   <sheets>
     <sheet name="James_Island_Midbay" sheetId="1" r:id="rId1"/>
@@ -400,9 +400,6 @@
     <t>Case Name</t>
   </si>
   <si>
-    <t>James_Island</t>
-  </si>
-  <si>
     <t>workflow</t>
   </si>
   <si>
@@ -634,15 +631,9 @@
     <t>Probability Masses (CHS -&gt; MCSim_Inputs folder path, Custom Modeling -&gt; .mat filename with relative path)</t>
   </si>
   <si>
-    <t>prob_mass_from_MB_SP2243\prob_mass_from_MB_SP2243.mat</t>
-  </si>
-  <si>
     <t>forcing_type</t>
   </si>
   <si>
-    <t>prob_mass_from_MB_SP2243\CHS_Data_from_MB_SP2243.mat</t>
-  </si>
-  <si>
     <t>Forcing Data Source (0 - CHS/CSTORM, 1- Custom Modeling)</t>
   </si>
   <si>
@@ -674,6 +665,15 @@
   </si>
   <si>
     <t>EVA_Case</t>
+  </si>
+  <si>
+    <t>Midbay_CHS_Data.zip</t>
+  </si>
+  <si>
+    <t>MCSim_Inputs</t>
+  </si>
+  <si>
+    <t>James_Island_CHS</t>
   </si>
 </sst>
 </file>
@@ -1600,7 +1600,7 @@
         <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>120</v>
+        <v>211</v>
       </c>
       <c r="F3" s="49" t="s">
         <v>98</v>
@@ -1609,7 +1609,7 @@
         <v>91</v>
       </c>
       <c r="H3" s="13" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I3" s="13">
         <v>0.33979999999999999</v>
@@ -1626,7 +1626,7 @@
         <v>10</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="F4" s="49" t="s">
         <v>99</v>
@@ -1652,7 +1652,7 @@
         <v>10</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="F5" s="49" t="s">
         <v>101</v>
@@ -1661,7 +1661,7 @@
         <v>93</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I5" s="13">
         <v>0.3</v>
@@ -1713,7 +1713,7 @@
         <v>96</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="I7" s="2">
         <v>0</v>
@@ -1721,10 +1721,10 @@
     </row>
     <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="14" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="C8" s="16" t="s">
         <v>10</v>
@@ -1811,10 +1811,10 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="C12" s="16" t="s">
         <v>10</v>
@@ -1829,7 +1829,7 @@
         <v>45</v>
       </c>
       <c r="H12" s="16" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I12" s="2">
         <v>0.15</v>
@@ -1855,7 +1855,7 @@
         <v>48</v>
       </c>
       <c r="H13" s="31" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="I13" s="2">
         <v>0.43</v>
@@ -1863,10 +1863,10 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C14" s="16" t="s">
         <v>10</v>
@@ -1881,7 +1881,7 @@
         <v>46</v>
       </c>
       <c r="H14" s="16" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="I14" s="2">
         <v>0.78</v>
@@ -1892,7 +1892,7 @@
         <v>79</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C15" s="16" t="s">
         <v>10</v>
@@ -1907,7 +1907,7 @@
         <v>47</v>
       </c>
       <c r="H15" s="19" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I15" s="3">
         <v>0.13</v>
@@ -1915,10 +1915,10 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>10</v>
@@ -1933,10 +1933,10 @@
     </row>
     <row r="17" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="17" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C17" s="19" t="s">
         <v>10</v>
@@ -2021,10 +2021,10 @@
     </row>
     <row r="21" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="11" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="C21" s="28" t="s">
         <v>10</v>
@@ -2033,10 +2033,10 @@
         <v>0</v>
       </c>
       <c r="F21" s="17" t="s">
+        <v>126</v>
+      </c>
+      <c r="G21" s="18" t="s">
         <v>127</v>
-      </c>
-      <c r="G21" s="18" t="s">
-        <v>128</v>
       </c>
       <c r="H21" s="19" t="s">
         <v>10</v>
@@ -2094,7 +2094,7 @@
         <v>10</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>3</v>
@@ -2111,16 +2111,16 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
+        <v>195</v>
+      </c>
+      <c r="B25" s="12" t="s">
         <v>196</v>
       </c>
-      <c r="B25" s="12" t="s">
-        <v>197</v>
-      </c>
       <c r="C25" s="28" t="s">
         <v>10</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>198</v>
+        <v>210</v>
       </c>
       <c r="F25" s="11" t="s">
         <v>27</v>
@@ -2140,13 +2140,13 @@
         <v>42</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="C26" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>200</v>
+        <v>209</v>
       </c>
       <c r="F26" s="14" t="s">
         <v>31</v>
@@ -2172,7 +2172,7 @@
         <v>10</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F27" s="14" t="s">
         <v>33</v>
@@ -2199,7 +2199,7 @@
         <v>37</v>
       </c>
       <c r="H28" s="19" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I28" s="3">
         <v>1</v>
@@ -2242,10 +2242,10 @@
         <v>53</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D31" s="1">
         <v>3.41</v>
@@ -2271,7 +2271,7 @@
         <v>81</v>
       </c>
       <c r="C32" s="16" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D32" s="2">
         <v>7.01</v>
@@ -2294,10 +2294,10 @@
         <v>55</v>
       </c>
       <c r="B33" s="15" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D33" s="2">
         <v>-2.42</v>
@@ -2317,13 +2317,13 @@
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D34" s="2">
         <v>-0.95799999999999996</v>
@@ -2334,7 +2334,7 @@
         <v>56</v>
       </c>
       <c r="B35" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C35" s="16" t="s">
         <v>10</v>
@@ -2348,7 +2348,7 @@
         <v>57</v>
       </c>
       <c r="B36" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C36" s="16" t="s">
         <v>10</v>
@@ -2365,7 +2365,7 @@
         <v>86</v>
       </c>
       <c r="C37" s="45" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D37" s="46">
         <v>0</v>
@@ -2373,10 +2373,10 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B38" s="15" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C38" s="16" t="s">
         <v>10</v>
@@ -2393,7 +2393,7 @@
         <v>89</v>
       </c>
       <c r="C39" s="16" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D39" s="2">
         <v>3.35</v>
@@ -2404,10 +2404,10 @@
         <v>88</v>
       </c>
       <c r="B40" s="38" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C40" s="43" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D40" s="44">
         <v>0.06</v>
@@ -2463,7 +2463,7 @@
         <v>62</v>
       </c>
       <c r="C45" s="16" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D45" s="2">
         <v>1134</v>
@@ -2477,7 +2477,7 @@
         <v>64</v>
       </c>
       <c r="C46" s="16" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D46" s="2">
         <v>1134</v>
@@ -2491,7 +2491,7 @@
         <v>66</v>
       </c>
       <c r="C47" s="16" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D47" s="2">
         <v>1027</v>
@@ -2624,22 +2624,22 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
     </row>
   </sheetData>
@@ -2662,16 +2662,16 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E1" t="s">
         <v>78</v>
@@ -2679,62 +2679,62 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="50" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B4" t="s">
+        <v>166</v>
+      </c>
+      <c r="C4" t="s">
         <v>167</v>
-      </c>
-      <c r="C4" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="50" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B5" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="50" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B6" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C6" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="50" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B7" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C7" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="50" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B8" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C8" t="s">
         <v>78</v>
@@ -2742,60 +2742,60 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="50" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B9" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C10" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C11" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
+        <v>168</v>
+      </c>
+      <c r="C12" t="s">
         <v>169</v>
-      </c>
-      <c r="C12" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
+        <v>170</v>
+      </c>
+      <c r="C13" t="s">
         <v>171</v>
-      </c>
-      <c r="C13" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="16" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="54" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B16" s="54" t="s">
         <v>4</v>
       </c>
       <c r="C16" s="54" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D16" s="58" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -2803,7 +2803,7 @@
         <v>0</v>
       </c>
       <c r="B17" s="55" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C17" s="59">
         <v>0.66720000000000002</v>
@@ -2819,7 +2819,7 @@
         <v>1</v>
       </c>
       <c r="B18" s="56" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C18" s="60">
         <v>128.0189</v>
@@ -2829,7 +2829,7 @@
         <v>2.1336483333333334</v>
       </c>
       <c r="E18" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -2838,7 +2838,7 @@
         <v>2</v>
       </c>
       <c r="B19" s="56" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C19" s="60">
         <v>1.8109999999999999</v>
@@ -2854,7 +2854,7 @@
         <v>3</v>
       </c>
       <c r="B20" s="56" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C20" s="60">
         <v>0.56489999999999996</v>
@@ -2870,7 +2870,7 @@
         <v>4</v>
       </c>
       <c r="B21" s="56" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C21" s="60">
         <v>1.2150000000000001</v>
@@ -2886,7 +2886,7 @@
         <v>5</v>
       </c>
       <c r="B22" s="56" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C22" s="60">
         <v>15.2134</v>
@@ -2902,7 +2902,7 @@
         <v>6</v>
       </c>
       <c r="B23" s="57" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C23" s="61">
         <v>648.27599999999995</v>
@@ -2920,12 +2920,12 @@
         <v>0.3858785714285714</v>
       </c>
       <c r="G23" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="65" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B24" s="66"/>
       <c r="C24" s="52">
@@ -2941,33 +2941,33 @@
         <v>23.152714285714286</v>
       </c>
       <c r="G24" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E28" s="8"/>
       <c r="F28" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E29" s="51"/>
       <c r="F29" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B31" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C31" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D31" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E31" t="s">
         <v>78</v>
@@ -2975,62 +2975,62 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B33" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="50" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B34" t="s">
+        <v>166</v>
+      </c>
+      <c r="C34" t="s">
         <v>167</v>
-      </c>
-      <c r="C34" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="50" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B35" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C35" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="50" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B36" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C36" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="50" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B37" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C37" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="50" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B38" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C38" t="s">
         <v>78</v>
@@ -3038,57 +3038,57 @@
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C39" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C40" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C41" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B42" t="s">
+        <v>168</v>
+      </c>
+      <c r="C42" t="s">
         <v>169</v>
-      </c>
-      <c r="C42" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B43" t="s">
+        <v>170</v>
+      </c>
+      <c r="C43" t="s">
         <v>171</v>
-      </c>
-      <c r="C43" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="46" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="54" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B46" s="54" t="s">
         <v>4</v>
       </c>
       <c r="C46" s="54" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D46" s="58" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
@@ -3096,7 +3096,7 @@
         <v>0</v>
       </c>
       <c r="B47" s="55" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C47" s="59">
         <v>0.66720000000000002</v>
@@ -3106,7 +3106,7 @@
         <v>1.112E-2</v>
       </c>
       <c r="F47" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
@@ -3115,7 +3115,7 @@
         <v>1</v>
       </c>
       <c r="B48" s="56" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C48" s="60">
         <v>128.0189</v>
@@ -3125,13 +3125,13 @@
         <v>2.1336483333333334</v>
       </c>
       <c r="E48" t="s">
+        <v>155</v>
+      </c>
+      <c r="F48" t="s">
+        <v>153</v>
+      </c>
+      <c r="G48" t="s">
         <v>156</v>
-      </c>
-      <c r="F48" t="s">
-        <v>154</v>
-      </c>
-      <c r="G48" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
@@ -3140,7 +3140,7 @@
         <v>2</v>
       </c>
       <c r="B49" s="56" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C49" s="60">
         <v>77.920665999999997</v>
@@ -3163,7 +3163,7 @@
         <v>3</v>
       </c>
       <c r="B50" s="56" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C50" s="60">
         <v>0.56489999999999996</v>
@@ -3179,7 +3179,7 @@
         <v>4</v>
       </c>
       <c r="B51" s="56" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C51" s="60">
         <v>2.6115067000000001</v>
@@ -3195,7 +3195,7 @@
         <v>5</v>
       </c>
       <c r="B52" s="56" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C52" s="60">
         <v>32.553324799999999</v>
@@ -3211,7 +3211,7 @@
         <v>6</v>
       </c>
       <c r="B53" s="57" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C53" s="61">
         <v>197.9727273</v>
@@ -3223,7 +3223,7 @@
     </row>
     <row r="54" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="65" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B54" s="66"/>
       <c r="C54" s="52">

</xml_diff>

<commit_message>
Fixing fucntions to use PM path in input file
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F458B474-1FD1-4A72-B339-78D13FB1503B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4B19983-92C4-4E21-85B2-A65685A41D75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
   <sheets>
     <sheet name="James_Island_Midbay" sheetId="1" r:id="rId1"/>
@@ -667,13 +667,13 @@
     <t>EVA_Case</t>
   </si>
   <si>
-    <t>Midbay_CHS_Data.zip</t>
-  </si>
-  <si>
     <t>MCSim_Inputs</t>
   </si>
   <si>
     <t>James_Island_CHS</t>
+  </si>
+  <si>
+    <t>C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\Midbay_CHS_Data.zip</t>
   </si>
 </sst>
 </file>
@@ -1600,7 +1600,7 @@
         <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F3" s="49" t="s">
         <v>98</v>
@@ -2120,7 +2120,7 @@
         <v>10</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F25" s="11" t="s">
         <v>27</v>
@@ -2146,7 +2146,7 @@
         <v>10</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F26" s="14" t="s">
         <v>31</v>

</xml_diff>

<commit_message>
Changing CHS pathing for loading prob masses
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4B19983-92C4-4E21-85B2-A65685A41D75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F16A4D80-4959-42D3-AB6B-D2C1A817D3DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
@@ -667,13 +667,13 @@
     <t>EVA_Case</t>
   </si>
   <si>
-    <t>MCSim_Inputs</t>
-  </si>
-  <si>
     <t>James_Island_CHS</t>
   </si>
   <si>
     <t>C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\Midbay_CHS_Data.zip</t>
+  </si>
+  <si>
+    <t>MCSim_Inputs\NACCS</t>
   </si>
 </sst>
 </file>
@@ -1600,7 +1600,7 @@
         <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F3" s="49" t="s">
         <v>98</v>
@@ -2120,7 +2120,7 @@
         <v>10</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F25" s="11" t="s">
         <v>27</v>
@@ -2146,7 +2146,7 @@
         <v>10</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F26" s="14" t="s">
         <v>31</v>

</xml_diff>

<commit_message>
Updating new fields in input file
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F16A4D80-4959-42D3-AB6B-D2C1A817D3DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10E4CA27-5B1F-4B40-9FB6-26856F9289E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="228">
   <si>
     <t>StormSim Project General Inputs</t>
   </si>
@@ -661,19 +661,67 @@
     <t>SST/JPM old vs SST/JPM New</t>
   </si>
   <si>
-    <t>Validation_Case</t>
-  </si>
-  <si>
     <t>EVA_Case</t>
   </si>
   <si>
     <t>James_Island_CHS</t>
   </si>
   <si>
-    <t>C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\Midbay_CHS_Data.zip</t>
-  </si>
-  <si>
-    <t>MCSim_Inputs\NACCS</t>
+    <t>prob_mass_from_MB_SP2243\prob_mass_from_MB_SP2243.mat</t>
+  </si>
+  <si>
+    <t>prob_mass_from_MB_SP2243\CHS_Data_from_MB_SP2243.mat</t>
+  </si>
+  <si>
+    <t>Validation_Case_v2</t>
+  </si>
+  <si>
+    <t>pros_dn50_seaside</t>
+  </si>
+  <si>
+    <t>pros_dn50_leeside</t>
+  </si>
+  <si>
+    <t>pros_dn50_lcbw</t>
+  </si>
+  <si>
+    <t>pros_r2p</t>
+  </si>
+  <si>
+    <t>pros_q</t>
+  </si>
+  <si>
+    <t>pros_p1</t>
+  </si>
+  <si>
+    <t>pros_p2_p3</t>
+  </si>
+  <si>
+    <t>pros_nappe</t>
+  </si>
+  <si>
+    <t>Compute Seaward Median Stone Size Response (Momentum Flux)</t>
+  </si>
+  <si>
+    <t>Compute Landward Median Stone Size Response (Van Gent)</t>
+  </si>
+  <si>
+    <t>Compute Seaward Median Stone Size Response (Low Crested Breakwater)</t>
+  </si>
+  <si>
+    <t>Compute Run-up Response (Eurotop)</t>
+  </si>
+  <si>
+    <t>Compute Overtopping Discharge Rate per Unit Width Response (Eurotop)</t>
+  </si>
+  <si>
+    <t>Compute Surface Pressure Response (Goda)</t>
+  </si>
+  <si>
+    <t>Compute P2 &amp; P3 Responses (Goda)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compute Nappe Responses </t>
   </si>
 </sst>
 </file>
@@ -1600,7 +1648,7 @@
         <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F3" s="49" t="s">
         <v>98</v>
@@ -1626,7 +1674,7 @@
         <v>10</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="F4" s="49" t="s">
         <v>99</v>
@@ -1652,7 +1700,7 @@
         <v>10</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F5" s="49" t="s">
         <v>101</v>
@@ -1730,7 +1778,7 @@
         <v>10</v>
       </c>
       <c r="D8" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F8" s="17" t="s">
         <v>97</v>
@@ -1872,7 +1920,7 @@
         <v>10</v>
       </c>
       <c r="D14" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F14" s="14" t="s">
         <v>82</v>
@@ -2120,7 +2168,7 @@
         <v>10</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="F25" s="11" t="s">
         <v>27</v>
@@ -2286,10 +2334,10 @@
         <v>10</v>
       </c>
       <c r="I32" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
         <v>55</v>
       </c>
@@ -2302,16 +2350,16 @@
       <c r="D33" s="2">
         <v>-2.42</v>
       </c>
-      <c r="F33" s="17" t="s">
+      <c r="F33" s="14" t="s">
         <v>117</v>
       </c>
-      <c r="G33" s="18" t="s">
+      <c r="G33" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="H33" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="I33" s="3">
+      <c r="H33" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I33" s="2">
         <v>1</v>
       </c>
     </row>
@@ -2328,6 +2376,18 @@
       <c r="D34" s="2">
         <v>-0.95799999999999996</v>
       </c>
+      <c r="F34" s="14" t="s">
+        <v>212</v>
+      </c>
+      <c r="G34" s="15" t="s">
+        <v>220</v>
+      </c>
+      <c r="H34" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I34" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
@@ -2342,6 +2402,18 @@
       <c r="D35" s="2">
         <v>3</v>
       </c>
+      <c r="F35" s="14" t="s">
+        <v>213</v>
+      </c>
+      <c r="G35" s="15" t="s">
+        <v>221</v>
+      </c>
+      <c r="H35" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I35" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
@@ -2356,6 +2428,18 @@
       <c r="D36" s="2">
         <v>1.5</v>
       </c>
+      <c r="F36" s="14" t="s">
+        <v>214</v>
+      </c>
+      <c r="G36" s="15" t="s">
+        <v>222</v>
+      </c>
+      <c r="H36" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I36" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="39" t="s">
@@ -2370,6 +2454,18 @@
       <c r="D37" s="46">
         <v>0</v>
       </c>
+      <c r="F37" s="14" t="s">
+        <v>215</v>
+      </c>
+      <c r="G37" s="15" t="s">
+        <v>223</v>
+      </c>
+      <c r="H37" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I37" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
@@ -2384,6 +2480,18 @@
       <c r="D38" s="2">
         <v>0.4</v>
       </c>
+      <c r="F38" s="14" t="s">
+        <v>216</v>
+      </c>
+      <c r="G38" s="15" t="s">
+        <v>224</v>
+      </c>
+      <c r="H38" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I38" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
@@ -2398,6 +2506,18 @@
       <c r="D39" s="2">
         <v>3.35</v>
       </c>
+      <c r="F39" s="14" t="s">
+        <v>217</v>
+      </c>
+      <c r="G39" s="15" t="s">
+        <v>225</v>
+      </c>
+      <c r="H39" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I39" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="40" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="38" t="s">
@@ -2412,12 +2532,36 @@
       <c r="D40" s="44">
         <v>0.06</v>
       </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F40" s="14" t="s">
+        <v>218</v>
+      </c>
+      <c r="G40" s="15" t="s">
+        <v>226</v>
+      </c>
+      <c r="H40" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I40" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="34"/>
       <c r="B41" s="34"/>
       <c r="C41" s="34"/>
       <c r="D41" s="34"/>
+      <c r="F41" s="17" t="s">
+        <v>219</v>
+      </c>
+      <c r="G41" s="18" t="s">
+        <v>227</v>
+      </c>
+      <c r="H41" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="I41" s="3">
+        <v>0</v>
+      </c>
     </row>
     <row r="42" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="36" t="s">
@@ -2605,9 +2749,9 @@
     <protectedRange sqref="D44:D53" name="Range1_1_4"/>
     <protectedRange sqref="D12 D27" name="Range1_1_2"/>
     <protectedRange sqref="D24" name="Range1_1_6_1"/>
-    <protectedRange sqref="D25" name="Range1_1_5"/>
     <protectedRange sqref="D21" name="Range1_1_6"/>
-    <protectedRange sqref="D26" name="Range1_1_8"/>
+    <protectedRange sqref="D25" name="Range1_1_5_1"/>
+    <protectedRange sqref="D26" name="Range1_1_8_1"/>
   </protectedRanges>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Addressing issue #61 by astehno
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66D59646-0DE0-45FF-AB5A-D260EB9A4ED5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95DD9B3B-0186-4CA3-87C2-6306424DC701}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15840" yWindow="0" windowWidth="22665" windowHeight="20985" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
+    <workbookView xWindow="3900" yWindow="3900" windowWidth="28800" windowHeight="15345" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
   <sheets>
     <sheet name="James_Island_Midbay" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="233">
   <si>
     <t>StormSim Project General Inputs</t>
   </si>
@@ -190,9 +190,6 @@
     <t xml:space="preserve">StormSim Project Forcing Uncertainty </t>
   </si>
   <si>
-    <t>[s]</t>
-  </si>
-  <si>
     <t>Structure Geometry</t>
   </si>
   <si>
@@ -280,9 +277,6 @@
     <t>use_timeseries</t>
   </si>
   <si>
-    <t>Apply Depth Limitation To Waves (0/1)</t>
-  </si>
-  <si>
     <t>Crest Width/Wall Width</t>
   </si>
   <si>
@@ -361,18 +355,12 @@
     <t>p1_u</t>
   </si>
   <si>
-    <t>CHS Region Bias File</t>
-  </si>
-  <si>
     <t>chs_bias_file</t>
   </si>
   <si>
     <t>tide_file</t>
   </si>
   <si>
-    <t>Tidal file used to randomly sample tidal values for storm SWL.</t>
-  </si>
-  <si>
     <t>NAVD</t>
   </si>
   <si>
@@ -403,21 +391,9 @@
     <t>workflow</t>
   </si>
   <si>
-    <t>Include forcing peaks files as part of the analysis. (0/1)</t>
-  </si>
-  <si>
-    <t>Include forcing timeseries files as part of the analysis. (0/1)</t>
-  </si>
-  <si>
     <t>use_peaks</t>
   </si>
   <si>
-    <t>Create Wave Height Priority Peaks Dataset (WLP) (0/1). (Requires peaks and timeseries files)</t>
-  </si>
-  <si>
-    <t>Create Water Level Priority Peaks Dataset (WLP) (0/1). (Requires peaks and timeseries files)</t>
-  </si>
-  <si>
     <t>mcs_sampling_mode</t>
   </si>
   <si>
@@ -628,9 +604,6 @@
     <t>prob_mass_source</t>
   </si>
   <si>
-    <t>Probability Masses (CHS -&gt; MCSim_Inputs folder path, Custom Modeling -&gt; .mat filename with relative path)</t>
-  </si>
-  <si>
     <t>forcing_type</t>
   </si>
   <si>
@@ -646,9 +619,6 @@
     <t>apply_random_tides</t>
   </si>
   <si>
-    <t>Apply random tide to storm SWL (0/1)</t>
-  </si>
-  <si>
     <t xml:space="preserve">With and without Tides </t>
   </si>
   <si>
@@ -712,9 +682,6 @@
     <t>use_waves_swl</t>
   </si>
   <si>
-    <t>Grab SWL hydrograph from wave model (0/1)</t>
-  </si>
-  <si>
     <t>James_Island</t>
   </si>
   <si>
@@ -728,6 +695,48 @@
   </si>
   <si>
     <t>prob_mass_from_MB_SP2243\CHS_Data_from_MB_SP2243.mat</t>
+  </si>
+  <si>
+    <t>pros_q_vol</t>
+  </si>
+  <si>
+    <t>Compute Overtopping Discharge Volume Unit Width Response (Eurotop) (RB3 Only)</t>
+  </si>
+  <si>
+    <t>lcbw_mass</t>
+  </si>
+  <si>
+    <t>Low Crested Breakwater Seaside Mass</t>
+  </si>
+  <si>
+    <t>Apply random tide to storm SWL (0 - Off / 1 - On)</t>
+  </si>
+  <si>
+    <t>Apply Depth Limitation To Waves  (0 - Off / 1 - On)</t>
+  </si>
+  <si>
+    <t>Include forcing peaks files as part of the analysis.  (0 - Off / 1 - On)</t>
+  </si>
+  <si>
+    <t>Include forcing timeseries files as part of the analysis.  (0 - Off / 1 - On)</t>
+  </si>
+  <si>
+    <t>Grab SWL hydrograph from wave model  (0 - Off / 1 - On)</t>
+  </si>
+  <si>
+    <t>Create Water Level Priority Peaks Dataset (WLP)  (0 - Off / 1 - On). (Requires peaks and timeseries files)</t>
+  </si>
+  <si>
+    <t>Create Wave Height Priority Peaks Dataset (WLP)  (0 - Off / 1 - On). (Requires peaks and timeseries files)</t>
+  </si>
+  <si>
+    <t>CHS Region Bias File (Relative Path)</t>
+  </si>
+  <si>
+    <t>Tidal file used to randomly sample tidal values for storm SWL. (Relative Path)</t>
+  </si>
+  <si>
+    <t>Probability Masses (CHS -&gt; MCSim_Inputs folder relative path, Custom Modeling -&gt; .mat filename with relative path)</t>
   </si>
 </sst>
 </file>
@@ -1591,7 +1600,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51D29750-2AFD-4BF7-A911-1DC4ADC0FD7A}">
-  <dimension ref="A1:I68"/>
+  <dimension ref="A1:I69"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.5703125" customWidth="1"/>
@@ -1599,7 +1608,7 @@
     <col min="3" max="3" width="19.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="171.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="28.42578125" customWidth="1"/>
-    <col min="7" max="7" width="78.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="84.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="46.140625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1654,16 +1663,16 @@
         <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>225</v>
+        <v>214</v>
       </c>
       <c r="F3" s="49" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="G3" s="49" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="H3" s="13" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="I3" s="13">
         <v>0.33979999999999999</v>
@@ -1680,13 +1689,13 @@
         <v>10</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>227</v>
+        <v>216</v>
       </c>
       <c r="F4" s="49" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="G4" s="49" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H4" s="13" t="s">
         <v>10</v>
@@ -1697,25 +1706,25 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C5" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>226</v>
+        <v>215</v>
       </c>
       <c r="F5" s="49" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="G5" s="49" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="I5" s="13">
         <v>0.3</v>
@@ -1732,13 +1741,13 @@
         <v>10</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="F6" s="49" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="G6" s="49" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="H6" s="13" t="s">
         <v>10</v>
@@ -1758,16 +1767,16 @@
         <v>10</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="G7" s="15" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="I7" s="2">
         <v>0</v>
@@ -1775,10 +1784,10 @@
     </row>
     <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="14" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>200</v>
+        <v>191</v>
       </c>
       <c r="C8" s="16" t="s">
         <v>10</v>
@@ -1787,13 +1796,13 @@
         <v>1</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H8" s="19" t="s">
-        <v>50</v>
+        <v>128</v>
       </c>
       <c r="I8" s="3">
         <v>0</v>
@@ -1828,10 +1837,10 @@
         <v>10</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F10" s="26" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="G10" s="27"/>
       <c r="H10" s="27"/>
@@ -1845,7 +1854,7 @@
         <v>25</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>10</v>
+        <v>128</v>
       </c>
       <c r="D11" s="2">
         <v>0</v>
@@ -1865,10 +1874,10 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>201</v>
+        <v>192</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>202</v>
+        <v>223</v>
       </c>
       <c r="C12" s="16" t="s">
         <v>10</v>
@@ -1877,13 +1886,13 @@
         <v>0</v>
       </c>
       <c r="F12" s="30" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="G12" s="15" t="s">
         <v>45</v>
       </c>
       <c r="H12" s="16" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="I12" s="2">
         <v>0.15</v>
@@ -1891,10 +1900,10 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>80</v>
+        <v>224</v>
       </c>
       <c r="C13" s="16" t="s">
         <v>10</v>
@@ -1903,13 +1912,13 @@
         <v>0</v>
       </c>
       <c r="F13" s="30" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="G13" s="15" t="s">
         <v>48</v>
       </c>
       <c r="H13" s="31" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="I13" s="2">
         <v>0.43</v>
@@ -1917,10 +1926,10 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>121</v>
+        <v>225</v>
       </c>
       <c r="C14" s="16" t="s">
         <v>10</v>
@@ -1929,13 +1938,13 @@
         <v>1</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G14" s="15" t="s">
         <v>46</v>
       </c>
       <c r="H14" s="16" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="I14" s="2">
         <v>0.78</v>
@@ -1943,10 +1952,10 @@
     </row>
     <row r="15" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>122</v>
+        <v>226</v>
       </c>
       <c r="C15" s="16" t="s">
         <v>10</v>
@@ -1955,13 +1964,13 @@
         <v>1</v>
       </c>
       <c r="F15" s="17" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G15" s="18" t="s">
         <v>47</v>
       </c>
       <c r="H15" s="19" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="I15" s="3">
         <v>0.13</v>
@@ -1969,10 +1978,10 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>223</v>
+        <v>213</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>10</v>
@@ -1987,10 +1996,10 @@
     </row>
     <row r="17" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="14" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>125</v>
+        <v>228</v>
       </c>
       <c r="C17" s="16" t="s">
         <v>10</v>
@@ -2011,10 +2020,10 @@
     </row>
     <row r="18" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="17" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>124</v>
+        <v>229</v>
       </c>
       <c r="C18" s="19" t="s">
         <v>10</v>
@@ -2087,10 +2096,10 @@
         <v>6</v>
       </c>
       <c r="F21" s="17" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="G21" s="18" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="H21" s="19" t="s">
         <v>10</v>
@@ -2101,10 +2110,10 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>197</v>
+        <v>188</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="C22" s="28" t="s">
         <v>10</v>
@@ -2139,16 +2148,16 @@
     </row>
     <row r="24" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="11" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C24" s="28" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D24" s="1">
-        <v>2.42</v>
+        <v>3.43</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>3</v>
@@ -2165,16 +2174,16 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>107</v>
+        <v>230</v>
       </c>
       <c r="C25" s="28" t="s">
         <v>10</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="F25" s="11" t="s">
         <v>27</v>
@@ -2191,16 +2200,16 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>196</v>
+        <v>232</v>
       </c>
       <c r="C26" s="28" t="s">
         <v>10</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>228</v>
+        <v>217</v>
       </c>
       <c r="F26" s="14" t="s">
         <v>31</v>
@@ -2220,13 +2229,13 @@
         <v>42</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>199</v>
+        <v>190</v>
       </c>
       <c r="C27" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>229</v>
+        <v>218</v>
       </c>
       <c r="F27" s="14" t="s">
         <v>33</v>
@@ -2243,16 +2252,16 @@
     </row>
     <row r="28" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="14" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>110</v>
+        <v>231</v>
       </c>
       <c r="C28" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="F28" s="17" t="s">
         <v>36</v>
@@ -2261,7 +2270,7 @@
         <v>37</v>
       </c>
       <c r="H28" s="19" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="I28" s="3">
         <v>1</v>
@@ -2279,7 +2288,7 @@
     </row>
     <row r="30" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="34" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B30" s="35"/>
       <c r="C30" s="35"/>
@@ -2302,7 +2311,7 @@
         <v>5</v>
       </c>
       <c r="D31" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>3</v>
@@ -2319,13 +2328,13 @@
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="D32" s="1">
         <v>3.41</v>
@@ -2345,22 +2354,22 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B33" s="15" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="D33" s="2">
         <v>7.01</v>
       </c>
       <c r="F33" s="14" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G33" s="15" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="H33" s="16" t="s">
         <v>10</v>
@@ -2371,22 +2380,22 @@
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="D34" s="2">
         <v>-2.42</v>
       </c>
       <c r="F34" s="14" t="s">
-        <v>207</v>
+        <v>197</v>
       </c>
       <c r="G34" s="15" t="s">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="H34" s="16" t="s">
         <v>10</v>
@@ -2397,22 +2406,22 @@
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="B35" s="15" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="C35" s="16" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="D35" s="2">
         <v>-0.95799999999999996</v>
       </c>
       <c r="F35" s="14" t="s">
-        <v>208</v>
+        <v>198</v>
       </c>
       <c r="G35" s="15" t="s">
-        <v>216</v>
+        <v>206</v>
       </c>
       <c r="H35" s="16" t="s">
         <v>10</v>
@@ -2423,10 +2432,10 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B36" s="15" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="C36" s="16" t="s">
         <v>10</v>
@@ -2435,10 +2444,10 @@
         <v>3</v>
       </c>
       <c r="F36" s="14" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="G36" s="15" t="s">
-        <v>217</v>
+        <v>207</v>
       </c>
       <c r="H36" s="16" t="s">
         <v>10</v>
@@ -2449,10 +2458,10 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="C37" s="16" t="s">
         <v>10</v>
@@ -2461,10 +2470,10 @@
         <v>1.5</v>
       </c>
       <c r="F37" s="14" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="G37" s="15" t="s">
-        <v>218</v>
+        <v>208</v>
       </c>
       <c r="H37" s="16" t="s">
         <v>10</v>
@@ -2475,22 +2484,22 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="39" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B38" s="39" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C38" s="45" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="D38" s="46">
         <v>0</v>
       </c>
       <c r="F38" s="14" t="s">
-        <v>211</v>
+        <v>201</v>
       </c>
       <c r="G38" s="15" t="s">
-        <v>219</v>
+        <v>209</v>
       </c>
       <c r="H38" s="16" t="s">
         <v>10</v>
@@ -2501,10 +2510,10 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="B39" s="15" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="C39" s="16" t="s">
         <v>10</v>
@@ -2513,7 +2522,7 @@
         <v>0.4</v>
       </c>
       <c r="F39" s="14" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="G39" s="15" t="s">
         <v>220</v>
@@ -2522,27 +2531,27 @@
         <v>10</v>
       </c>
       <c r="I39" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="B40" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="B40" s="14" t="s">
-        <v>89</v>
-      </c>
       <c r="C40" s="16" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="D40" s="2">
         <v>3.35</v>
       </c>
       <c r="F40" s="14" t="s">
-        <v>213</v>
+        <v>202</v>
       </c>
       <c r="G40" s="15" t="s">
-        <v>221</v>
+        <v>210</v>
       </c>
       <c r="H40" s="16" t="s">
         <v>10</v>
@@ -2553,39 +2562,51 @@
     </row>
     <row r="41" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="38" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B41" s="38" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="C41" s="43" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="D41" s="44">
         <v>0.06</v>
       </c>
-      <c r="F41" s="17" t="s">
-        <v>214</v>
-      </c>
-      <c r="G41" s="18" t="s">
-        <v>222</v>
-      </c>
-      <c r="H41" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="I41" s="3">
+      <c r="F41" s="14" t="s">
+        <v>203</v>
+      </c>
+      <c r="G41" s="15" t="s">
+        <v>211</v>
+      </c>
+      <c r="H41" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I41" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="34"/>
       <c r="B42" s="34"/>
       <c r="C42" s="34"/>
       <c r="D42" s="34"/>
+      <c r="F42" s="17" t="s">
+        <v>204</v>
+      </c>
+      <c r="G42" s="18" t="s">
+        <v>212</v>
+      </c>
+      <c r="H42" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="I42" s="3">
+        <v>0</v>
+      </c>
     </row>
     <row r="43" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="36" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B43" s="37"/>
       <c r="C43" s="37"/>
@@ -2602,15 +2623,15 @@
         <v>5</v>
       </c>
       <c r="D44" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="B45" s="12" t="s">
         <v>59</v>
-      </c>
-      <c r="B45" s="12" t="s">
-        <v>60</v>
       </c>
       <c r="C45" s="13" t="s">
         <v>10</v>
@@ -2621,13 +2642,13 @@
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="B46" s="15" t="s">
         <v>61</v>
       </c>
-      <c r="B46" s="15" t="s">
-        <v>62</v>
-      </c>
       <c r="C46" s="16" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="D46" s="2">
         <v>1134</v>
@@ -2635,13 +2656,13 @@
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="B47" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="B47" s="15" t="s">
-        <v>64</v>
-      </c>
       <c r="C47" s="16" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="D47" s="2">
         <v>1134</v>
@@ -2649,52 +2670,50 @@
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
-        <v>65</v>
+        <v>221</v>
       </c>
       <c r="B48" s="15" t="s">
-        <v>66</v>
+        <v>222</v>
       </c>
       <c r="C48" s="16" t="s">
-        <v>138</v>
-      </c>
-      <c r="D48" s="2">
-        <v>1027</v>
-      </c>
+        <v>129</v>
+      </c>
+      <c r="D48" s="2"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B49" s="15" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C49" s="16" t="s">
-        <v>69</v>
+        <v>130</v>
       </c>
       <c r="D49" s="2">
-        <v>0.4</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B50" s="15" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C50" s="16" t="s">
-        <v>10</v>
+        <v>68</v>
       </c>
       <c r="D50" s="2">
-        <v>1</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="14" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B51" s="15" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C51" s="16" t="s">
         <v>10</v>
@@ -2705,10 +2724,10 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="14" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B52" s="15" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C52" s="16" t="s">
         <v>10</v>
@@ -2718,54 +2737,68 @@
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="39" t="s">
+      <c r="A53" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="B53" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="C53" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D53" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" s="39" t="s">
+        <v>75</v>
+      </c>
+      <c r="B54" s="40" t="s">
         <v>76</v>
       </c>
-      <c r="B53" s="40" t="s">
-        <v>77</v>
-      </c>
-      <c r="C53" s="41" t="s">
-        <v>10</v>
-      </c>
-      <c r="D53" s="42">
+      <c r="C54" s="41" t="s">
+        <v>10</v>
+      </c>
+      <c r="D54" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="18" t="s">
-        <v>84</v>
-      </c>
-      <c r="B54" s="48" t="s">
-        <v>90</v>
-      </c>
-      <c r="C54" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D54" s="4">
+    <row r="55" spans="1:4" ht="60.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="18" t="s">
+        <v>82</v>
+      </c>
+      <c r="B55" s="48" t="s">
+        <v>88</v>
+      </c>
+      <c r="C55" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D55" s="4">
         <v>2</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="37"/>
-      <c r="B55" s="37"/>
-      <c r="C55" s="37"/>
-      <c r="D55" s="37"/>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C61" s="64"/>
-    </row>
-    <row r="62" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C62" s="63"/>
-    </row>
-    <row r="68" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B68" s="47"/>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" s="37"/>
+      <c r="B56" s="37"/>
+      <c r="C56" s="37"/>
+      <c r="D56" s="37"/>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C62" s="64"/>
+    </row>
+    <row r="63" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C63" s="63"/>
+    </row>
+    <row r="69" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B69" s="47"/>
     </row>
   </sheetData>
   <sheetProtection formatColumns="0" selectLockedCells="1"/>
   <protectedRanges>
     <protectedRange sqref="I3:I6 I8 I12:I16 I25:I28 D15:D18 I32 D23 I19:I20 D3:D6 D8:D11 D13" name="Range1_1"/>
     <protectedRange sqref="D7 D14" name="Range1_1_1"/>
-    <protectedRange sqref="D45:D54" name="Range1_1_4"/>
+    <protectedRange sqref="D45:D55" name="Range1_1_4"/>
     <protectedRange sqref="D12 D28" name="Range1_1_2"/>
     <protectedRange sqref="D25" name="Range1_1_6_1"/>
     <protectedRange sqref="D22" name="Range1_1_6"/>
@@ -2789,22 +2822,22 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>203</v>
+        <v>193</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>204</v>
+        <v>194</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>206</v>
+        <v>196</v>
       </c>
     </row>
   </sheetData>
@@ -2827,140 +2860,140 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="B1" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="C1" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="D1" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="E1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="B3" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="50" t="s">
+        <v>150</v>
+      </c>
+      <c r="B4" t="s">
         <v>158</v>
       </c>
-      <c r="B4" t="s">
-        <v>166</v>
-      </c>
       <c r="C4" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="50" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="B5" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="C5" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="50" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="B6" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="C6" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="50" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="B7" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="C7" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="50" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="B8" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="C8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="50" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="B9" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="C9" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="C10" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="C11" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="C12" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="C13" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="16" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="54" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="B16" s="54" t="s">
         <v>4</v>
       </c>
       <c r="C16" s="54" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="D16" s="58" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -2968,7 +3001,7 @@
         <v>0</v>
       </c>
       <c r="B17" s="55" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="C17" s="59">
         <v>0.66720000000000002</v>
@@ -2984,7 +3017,7 @@
         <v>1</v>
       </c>
       <c r="B18" s="56" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="C18" s="60">
         <v>128.0189</v>
@@ -2994,7 +3027,7 @@
         <v>2.1336483333333334</v>
       </c>
       <c r="E18" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -3003,7 +3036,7 @@
         <v>2</v>
       </c>
       <c r="B19" s="56" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="C19" s="60">
         <v>1.8109999999999999</v>
@@ -3019,7 +3052,7 @@
         <v>3</v>
       </c>
       <c r="B20" s="56" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="C20" s="60">
         <v>0.56489999999999996</v>
@@ -3035,7 +3068,7 @@
         <v>4</v>
       </c>
       <c r="B21" s="56" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="C21" s="60">
         <v>1.2150000000000001</v>
@@ -3051,7 +3084,7 @@
         <v>5</v>
       </c>
       <c r="B22" s="56" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="C22" s="60">
         <v>15.2134</v>
@@ -3067,7 +3100,7 @@
         <v>6</v>
       </c>
       <c r="B23" s="57" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="C23" s="61">
         <v>648.27599999999995</v>
@@ -3085,12 +3118,12 @@
         <v>0.3858785714285714</v>
       </c>
       <c r="G23" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="65" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="B24" s="66"/>
       <c r="C24" s="52">
@@ -3106,154 +3139,154 @@
         <v>23.152714285714286</v>
       </c>
       <c r="G24" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E28" s="8"/>
       <c r="F28" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E29" s="51"/>
       <c r="F29" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="B31" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="C31" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="D31" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="E31" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="B33" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="50" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="B34" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="C34" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="50" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="B35" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="C35" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="50" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="B36" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="C36" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="50" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="B37" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="C37" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="50" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="B38" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="C38" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="C39" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="C40" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="C41" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B42" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="C42" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B43" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="C43" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="46" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="54" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="B46" s="54" t="s">
         <v>4</v>
       </c>
       <c r="C46" s="54" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="D46" s="58" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
@@ -3261,7 +3294,7 @@
         <v>0</v>
       </c>
       <c r="B47" s="55" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="C47" s="59">
         <v>0.66720000000000002</v>
@@ -3271,7 +3304,7 @@
         <v>1.112E-2</v>
       </c>
       <c r="F47" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
@@ -3280,7 +3313,7 @@
         <v>1</v>
       </c>
       <c r="B48" s="56" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="C48" s="60">
         <v>128.0189</v>
@@ -3290,13 +3323,13 @@
         <v>2.1336483333333334</v>
       </c>
       <c r="E48" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="F48" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="G48" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
@@ -3305,7 +3338,7 @@
         <v>2</v>
       </c>
       <c r="B49" s="56" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="C49" s="60">
         <v>77.920665999999997</v>
@@ -3328,7 +3361,7 @@
         <v>3</v>
       </c>
       <c r="B50" s="56" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="C50" s="60">
         <v>0.56489999999999996</v>
@@ -3344,7 +3377,7 @@
         <v>4</v>
       </c>
       <c r="B51" s="56" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="C51" s="60">
         <v>2.6115067000000001</v>
@@ -3360,7 +3393,7 @@
         <v>5</v>
       </c>
       <c r="B52" s="56" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="C52" s="60">
         <v>32.553324799999999</v>
@@ -3376,7 +3409,7 @@
         <v>6</v>
       </c>
       <c r="B53" s="57" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="C53" s="61">
         <v>197.9727273</v>
@@ -3388,7 +3421,7 @@
     </row>
     <row r="54" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="65" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="B54" s="66"/>
       <c r="C54" s="52">

</xml_diff>

<commit_message>
Implementing load_project_forcing switch in case user wants to use the same project_forcing for cases
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17F9D841-B9A2-485F-A4B4-8E0367702864}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1460EDF3-7569-446E-A412-720A937FF8C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7245" yWindow="3240" windowWidth="28800" windowHeight="15345" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
+    <workbookView xWindow="570" yWindow="600" windowWidth="28800" windowHeight="15345" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
   <sheets>
     <sheet name="James_Island_Midbay" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="238">
   <si>
     <t>StormSim Project General Inputs</t>
   </si>
@@ -685,9 +685,6 @@
     <t>James_Island</t>
   </si>
   <si>
-    <t>Levee_Case</t>
-  </si>
-  <si>
     <t>SP_2243</t>
   </si>
   <si>
@@ -737,6 +734,24 @@
   </si>
   <si>
     <t>prob_mass_from_MB_SP2243\CHS_Data_from_MB_SP2243.mat</t>
+  </si>
+  <si>
+    <t>Load project_forcing StormSim File From Other case_name Under The Same project_name (0- Sample New Storms/1-Load Previous Storm Suite)</t>
+  </si>
+  <si>
+    <t>Define Reference case_name To Load project_forcing From</t>
+  </si>
+  <si>
+    <t>Levee_Case_2</t>
+  </si>
+  <si>
+    <t>load_project_forcing</t>
+  </si>
+  <si>
+    <t>ref_case_name</t>
+  </si>
+  <si>
+    <t>Levee_Case_5</t>
   </si>
 </sst>
 </file>
@@ -858,7 +873,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="22">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -1143,11 +1158,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1280,6 +1308,17 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1600,7 +1639,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51D29750-2AFD-4BF7-A911-1DC4ADC0FD7A}">
-  <dimension ref="A1:I69"/>
+  <dimension ref="A1:I71"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.5703125" customWidth="1"/>
@@ -1610,6 +1649,7 @@
     <col min="6" max="6" width="28.42578125" customWidth="1"/>
     <col min="7" max="7" width="84.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="46.140625" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1689,7 +1729,7 @@
         <v>10</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F4" s="49" t="s">
         <v>97</v>
@@ -1715,7 +1755,7 @@
         <v>10</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>215</v>
+        <v>237</v>
       </c>
       <c r="F5" s="49" t="s">
         <v>99</v>
@@ -1793,7 +1833,7 @@
         <v>10</v>
       </c>
       <c r="D8" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F8" s="17" t="s">
         <v>95</v>
@@ -1819,7 +1859,7 @@
         <v>10</v>
       </c>
       <c r="D9" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F9" s="33"/>
       <c r="G9" s="33"/>
@@ -1877,7 +1917,7 @@
         <v>192</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C12" s="16" t="s">
         <v>10</v>
@@ -1903,7 +1943,7 @@
         <v>102</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C13" s="16" t="s">
         <v>10</v>
@@ -1929,7 +1969,7 @@
         <v>117</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C14" s="16" t="s">
         <v>10</v>
@@ -1955,7 +1995,7 @@
         <v>78</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C15" s="16" t="s">
         <v>10</v>
@@ -1981,7 +2021,7 @@
         <v>213</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>10</v>
@@ -1999,7 +2039,7 @@
         <v>120</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C17" s="16" t="s">
         <v>10</v>
@@ -2019,16 +2059,16 @@
       </c>
     </row>
     <row r="18" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="17" t="s">
+      <c r="A18" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="B18" s="18" t="s">
-        <v>228</v>
-      </c>
-      <c r="C18" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D18" s="3">
+      <c r="B18" s="15" t="s">
+        <v>227</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18" s="2">
         <v>1</v>
       </c>
       <c r="F18" s="9" t="s">
@@ -2045,30 +2085,44 @@
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="6"/>
-      <c r="B19" s="22"/>
-      <c r="C19" s="23"/>
-      <c r="D19" s="23"/>
-      <c r="F19" s="11" t="s">
+      <c r="A19" s="14" t="s">
+        <v>235</v>
+      </c>
+      <c r="B19" s="15" t="s">
+        <v>232</v>
+      </c>
+      <c r="C19" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D19" s="2">
+        <v>1</v>
+      </c>
+      <c r="F19" s="65" t="s">
         <v>11</v>
       </c>
-      <c r="G19" s="12" t="s">
+      <c r="G19" s="66" t="s">
         <v>12</v>
       </c>
-      <c r="H19" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="I19" s="1">
+      <c r="H19" s="67" t="s">
+        <v>10</v>
+      </c>
+      <c r="I19" s="68">
         <v>9</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="24" t="s">
-        <v>35</v>
-      </c>
-      <c r="B20" s="25"/>
-      <c r="C20" s="25"/>
-      <c r="D20" s="25"/>
+      <c r="A20" s="17" t="s">
+        <v>236</v>
+      </c>
+      <c r="B20" s="18" t="s">
+        <v>233</v>
+      </c>
+      <c r="C20" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>234</v>
+      </c>
       <c r="F20" s="14" t="s">
         <v>15</v>
       </c>
@@ -2082,372 +2136,334 @@
         <v>50</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="9" t="s">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="6"/>
+      <c r="B21" s="22"/>
+      <c r="C21" s="23"/>
+      <c r="D21" s="23"/>
+      <c r="F21" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="G21" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="H21" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I21" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="B22" s="25"/>
+      <c r="C22" s="25"/>
+      <c r="D22" s="25"/>
+    </row>
+    <row r="23" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="B21" s="10" t="s">
+      <c r="B23" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="C23" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="D21" s="10" t="s">
+      <c r="D23" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="F21" s="17" t="s">
-        <v>118</v>
-      </c>
-      <c r="G21" s="18" t="s">
-        <v>119</v>
-      </c>
-      <c r="H21" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="I21" s="3">
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" s="11" t="s">
+        <v>188</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>189</v>
+      </c>
+      <c r="C24" s="28" t="s">
+        <v>10</v>
+      </c>
+      <c r="D24" s="1">
+        <v>0</v>
+      </c>
+      <c r="F24" s="8"/>
+      <c r="G24" s="8"/>
+      <c r="H24" s="8"/>
+      <c r="I24" s="8"/>
+    </row>
+    <row r="25" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C25" s="28" t="s">
+        <v>40</v>
+      </c>
+      <c r="D25" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="11" t="s">
-        <v>188</v>
-      </c>
-      <c r="B22" s="12" t="s">
-        <v>189</v>
-      </c>
-      <c r="C22" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="D22" s="1">
+      <c r="F25" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="G25" s="21"/>
+      <c r="H25" s="21"/>
+      <c r="I25" s="21"/>
+    </row>
+    <row r="26" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="B26" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="C26" s="28" t="s">
+        <v>108</v>
+      </c>
+      <c r="D26" s="1">
+        <v>3.43</v>
+      </c>
+      <c r="F26" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="G26" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="H26" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="I26" s="10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="B27" s="12" t="s">
+        <v>228</v>
+      </c>
+      <c r="C27" s="28" t="s">
+        <v>10</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="F27" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="G27" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="H27" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="I27" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" s="11" t="s">
+        <v>187</v>
+      </c>
+      <c r="B28" s="12" t="s">
+        <v>230</v>
+      </c>
+      <c r="C28" s="28" t="s">
+        <v>10</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="F28" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="G28" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="H28" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I28" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="B29" s="15" t="s">
+        <v>190</v>
+      </c>
+      <c r="C29" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="F29" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="G29" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="H29" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I29" s="2">
         <v>0</v>
       </c>
-      <c r="F22" s="8"/>
-      <c r="G22" s="8"/>
-      <c r="H22" s="8"/>
-      <c r="I22" s="8"/>
-    </row>
-    <row r="23" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="B23" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="C23" s="28" t="s">
-        <v>40</v>
-      </c>
-      <c r="D23" s="1">
+    </row>
+    <row r="30" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="B30" s="15" t="s">
+        <v>229</v>
+      </c>
+      <c r="C30" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="F30" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="G30" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="H30" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="I30" s="3">
         <v>1</v>
       </c>
-      <c r="F23" s="20" t="s">
-        <v>26</v>
-      </c>
-      <c r="G23" s="21"/>
-      <c r="H23" s="21"/>
-      <c r="I23" s="21"/>
-    </row>
-    <row r="24" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="B24" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="C24" s="28" t="s">
-        <v>108</v>
-      </c>
-      <c r="D24" s="1">
-        <v>3.43</v>
-      </c>
-      <c r="F24" s="9" t="s">
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" s="25"/>
+      <c r="B31" s="25"/>
+      <c r="C31" s="25"/>
+      <c r="D31" s="25"/>
+      <c r="F31" s="21"/>
+      <c r="G31" s="21"/>
+      <c r="H31" s="21"/>
+      <c r="I31" s="21"/>
+    </row>
+    <row r="32" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="34" t="s">
+        <v>50</v>
+      </c>
+      <c r="B32" s="35"/>
+      <c r="C32" s="35"/>
+      <c r="D32" s="35"/>
+      <c r="F32" s="26" t="s">
+        <v>41</v>
+      </c>
+      <c r="G32" s="27"/>
+      <c r="H32" s="27"/>
+      <c r="I32" s="27"/>
+    </row>
+    <row r="33" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="G24" s="10" t="s">
+      <c r="B33" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="H24" s="10" t="s">
+      <c r="C33" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="I24" s="10" t="s">
+      <c r="D33" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="F33" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="G33" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="H33" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="I33" s="10" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="B25" s="12" t="s">
-        <v>229</v>
-      </c>
-      <c r="C25" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="F25" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="G25" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="H25" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="I25" s="1">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="B34" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="C34" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="D34" s="1">
+        <v>3.41</v>
+      </c>
+      <c r="F34" s="29" t="s">
+        <v>43</v>
+      </c>
+      <c r="G34" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="H34" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="I34" s="1">
         <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="11" t="s">
-        <v>187</v>
-      </c>
-      <c r="B26" s="12" t="s">
-        <v>231</v>
-      </c>
-      <c r="C26" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="F26" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="G26" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="H26" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="I26" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="14" t="s">
-        <v>42</v>
-      </c>
-      <c r="B27" s="15" t="s">
-        <v>190</v>
-      </c>
-      <c r="C27" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="F27" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="G27" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="H27" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="I27" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="14" t="s">
-        <v>106</v>
-      </c>
-      <c r="B28" s="15" t="s">
-        <v>230</v>
-      </c>
-      <c r="C28" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="F28" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="G28" s="18" t="s">
-        <v>37</v>
-      </c>
-      <c r="H28" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="I28" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="25"/>
-      <c r="B29" s="25"/>
-      <c r="C29" s="25"/>
-      <c r="D29" s="25"/>
-      <c r="F29" s="21"/>
-      <c r="G29" s="21"/>
-      <c r="H29" s="21"/>
-      <c r="I29" s="21"/>
-    </row>
-    <row r="30" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="34" t="s">
-        <v>50</v>
-      </c>
-      <c r="B30" s="35"/>
-      <c r="C30" s="35"/>
-      <c r="D30" s="35"/>
-      <c r="F30" s="26" t="s">
-        <v>41</v>
-      </c>
-      <c r="G30" s="27"/>
-      <c r="H30" s="27"/>
-      <c r="I30" s="27"/>
-    </row>
-    <row r="31" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B31" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C31" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="D31" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="F31" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="G31" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="H31" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="I31" s="10" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="B32" s="12" t="s">
-        <v>123</v>
-      </c>
-      <c r="C32" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="D32" s="1">
-        <v>3.41</v>
-      </c>
-      <c r="F32" s="29" t="s">
-        <v>43</v>
-      </c>
-      <c r="G32" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="H32" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="I32" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="B33" s="15" t="s">
-        <v>79</v>
-      </c>
-      <c r="C33" s="16" t="s">
-        <v>128</v>
-      </c>
-      <c r="D33" s="2">
-        <v>7.01</v>
-      </c>
-      <c r="F33" s="14" t="s">
-        <v>113</v>
-      </c>
-      <c r="G33" s="15" t="s">
-        <v>112</v>
-      </c>
-      <c r="H33" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="I33" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="B34" s="15" t="s">
-        <v>124</v>
-      </c>
-      <c r="C34" s="16" t="s">
-        <v>128</v>
-      </c>
-      <c r="D34" s="2">
-        <v>-2.42</v>
-      </c>
-      <c r="F34" s="14" t="s">
-        <v>197</v>
-      </c>
-      <c r="G34" s="15" t="s">
-        <v>205</v>
-      </c>
-      <c r="H34" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="I34" s="2">
-        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
-        <v>175</v>
+        <v>53</v>
       </c>
       <c r="B35" s="15" t="s">
-        <v>125</v>
+        <v>79</v>
       </c>
       <c r="C35" s="16" t="s">
         <v>128</v>
       </c>
       <c r="D35" s="2">
-        <v>-0.95799999999999996</v>
+        <v>7.01</v>
       </c>
       <c r="F35" s="14" t="s">
-        <v>198</v>
+        <v>113</v>
       </c>
       <c r="G35" s="15" t="s">
-        <v>206</v>
+        <v>112</v>
       </c>
       <c r="H35" s="16" t="s">
         <v>10</v>
       </c>
       <c r="I35" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B36" s="15" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C36" s="16" t="s">
-        <v>10</v>
+        <v>128</v>
       </c>
       <c r="D36" s="2">
-        <v>3</v>
+        <v>-2.42</v>
       </c>
       <c r="F36" s="14" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="G36" s="15" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="H36" s="16" t="s">
         <v>10</v>
@@ -2458,74 +2474,74 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
-        <v>56</v>
+        <v>175</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C37" s="16" t="s">
-        <v>10</v>
+        <v>128</v>
       </c>
       <c r="D37" s="2">
-        <v>1.5</v>
+        <v>-0.95799999999999996</v>
       </c>
       <c r="F37" s="14" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="G37" s="15" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="H37" s="16" t="s">
         <v>10</v>
       </c>
       <c r="I37" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A38" s="39" t="s">
-        <v>83</v>
-      </c>
-      <c r="B38" s="39" t="s">
-        <v>84</v>
-      </c>
-      <c r="C38" s="45" t="s">
-        <v>133</v>
-      </c>
-      <c r="D38" s="46">
+      <c r="A38" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="B38" s="15" t="s">
+        <v>126</v>
+      </c>
+      <c r="C38" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D38" s="2">
+        <v>3</v>
+      </c>
+      <c r="F38" s="14" t="s">
+        <v>199</v>
+      </c>
+      <c r="G38" s="15" t="s">
+        <v>207</v>
+      </c>
+      <c r="H38" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I38" s="2">
         <v>0</v>
-      </c>
-      <c r="F38" s="14" t="s">
-        <v>201</v>
-      </c>
-      <c r="G38" s="15" t="s">
-        <v>209</v>
-      </c>
-      <c r="H38" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="I38" s="2">
-        <v>1</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
-        <v>135</v>
+        <v>56</v>
       </c>
       <c r="B39" s="15" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="C39" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D39" s="2">
-        <v>0.4</v>
+        <v>1.5</v>
       </c>
       <c r="F39" s="14" t="s">
-        <v>218</v>
+        <v>200</v>
       </c>
       <c r="G39" s="15" t="s">
-        <v>219</v>
+        <v>208</v>
       </c>
       <c r="H39" s="16" t="s">
         <v>10</v>
@@ -2535,279 +2551,331 @@
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A40" s="14" t="s">
+      <c r="A40" s="39" t="s">
+        <v>83</v>
+      </c>
+      <c r="B40" s="39" t="s">
+        <v>84</v>
+      </c>
+      <c r="C40" s="45" t="s">
+        <v>133</v>
+      </c>
+      <c r="D40" s="46">
+        <v>0</v>
+      </c>
+      <c r="F40" s="14" t="s">
+        <v>201</v>
+      </c>
+      <c r="G40" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="H40" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I40" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A41" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="B41" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="C41" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D41" s="2">
+        <v>0.4</v>
+      </c>
+      <c r="F41" s="14" t="s">
+        <v>217</v>
+      </c>
+      <c r="G41" s="15" t="s">
+        <v>218</v>
+      </c>
+      <c r="H41" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I41" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A42" s="14" t="s">
         <v>85</v>
       </c>
-      <c r="B40" s="14" t="s">
+      <c r="B42" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="C40" s="16" t="s">
+      <c r="C42" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="D40" s="2">
+      <c r="D42" s="2">
         <v>3.35</v>
       </c>
-      <c r="F40" s="14" t="s">
+      <c r="F42" s="14" t="s">
         <v>202</v>
       </c>
-      <c r="G40" s="15" t="s">
+      <c r="G42" s="15" t="s">
         <v>210</v>
       </c>
-      <c r="H40" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="I40" s="2">
+      <c r="H42" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I42" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="38" t="s">
+    <row r="43" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="38" t="s">
         <v>86</v>
       </c>
-      <c r="B41" s="38" t="s">
+      <c r="B43" s="38" t="s">
         <v>122</v>
       </c>
-      <c r="C41" s="43" t="s">
+      <c r="C43" s="43" t="s">
         <v>128</v>
       </c>
-      <c r="D41" s="44">
+      <c r="D43" s="44">
         <v>0.06</v>
       </c>
-      <c r="F41" s="14" t="s">
+      <c r="F43" s="14" t="s">
         <v>203</v>
       </c>
-      <c r="G41" s="15" t="s">
+      <c r="G43" s="15" t="s">
         <v>211</v>
       </c>
-      <c r="H41" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="I41" s="2">
+      <c r="H43" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I43" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="34"/>
-      <c r="B42" s="34"/>
-      <c r="C42" s="34"/>
-      <c r="D42" s="34"/>
-      <c r="F42" s="17" t="s">
+    <row r="44" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="34"/>
+      <c r="B44" s="34"/>
+      <c r="C44" s="34"/>
+      <c r="D44" s="34"/>
+      <c r="F44" s="17" t="s">
         <v>204</v>
       </c>
-      <c r="G42" s="18" t="s">
+      <c r="G44" s="18" t="s">
         <v>212</v>
       </c>
-      <c r="H42" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="I42" s="3">
+      <c r="H44" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="I44" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="36" t="s">
+    <row r="45" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="36" t="s">
         <v>57</v>
       </c>
-      <c r="B43" s="37"/>
-      <c r="C43" s="37"/>
-      <c r="D43" s="37"/>
-    </row>
-    <row r="44" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="9" t="s">
+      <c r="B45" s="37"/>
+      <c r="C45" s="37"/>
+      <c r="D45" s="37"/>
+    </row>
+    <row r="46" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="B44" s="10" t="s">
+      <c r="B46" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C44" s="10" t="s">
+      <c r="C46" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="D44" s="10" t="s">
+      <c r="D46" s="10" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A45" s="11" t="s">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A47" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="B45" s="12" t="s">
+      <c r="B47" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="C45" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="D45" s="1">
+      <c r="C47" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D47" s="1">
         <v>1.65</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A46" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="B46" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="C46" s="16" t="s">
-        <v>129</v>
-      </c>
-      <c r="D46" s="2">
-        <v>780</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A47" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="B47" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="C47" s="16" t="s">
-        <v>129</v>
-      </c>
-      <c r="D47" s="2">
-        <v>57</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
-        <v>220</v>
+        <v>60</v>
       </c>
       <c r="B48" s="15" t="s">
-        <v>221</v>
+        <v>61</v>
       </c>
       <c r="C48" s="16" t="s">
         <v>129</v>
       </c>
       <c r="D48" s="2">
-        <v>1147</v>
+        <v>780</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B49" s="15" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C49" s="16" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D49" s="2">
-        <v>1027</v>
+        <v>57</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
-        <v>66</v>
+        <v>219</v>
       </c>
       <c r="B50" s="15" t="s">
-        <v>67</v>
+        <v>220</v>
       </c>
       <c r="C50" s="16" t="s">
-        <v>68</v>
+        <v>129</v>
       </c>
       <c r="D50" s="2">
-        <v>0.4</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="14" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="B51" s="15" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="C51" s="16" t="s">
-        <v>10</v>
+        <v>130</v>
       </c>
       <c r="D51" s="2">
-        <v>1</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="14" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B52" s="15" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C52" s="16" t="s">
-        <v>10</v>
+        <v>68</v>
       </c>
       <c r="D52" s="2">
-        <v>1</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="B53" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="C53" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D53" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="B54" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="C54" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D54" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" ht="60.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="B53" s="15" t="s">
+      <c r="B55" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="C53" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D53" s="2">
+      <c r="C55" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D55" s="2">
         <v>17</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="39" t="s">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" s="39" t="s">
         <v>75</v>
       </c>
-      <c r="B54" s="40" t="s">
+      <c r="B56" s="40" t="s">
         <v>76</v>
       </c>
-      <c r="C54" s="41" t="s">
-        <v>10</v>
-      </c>
-      <c r="D54" s="42">
+      <c r="C56" s="41" t="s">
+        <v>10</v>
+      </c>
+      <c r="D56" s="42">
         <v>17</v>
       </c>
     </row>
-    <row r="55" spans="1:4" ht="60.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="18" t="s">
+    <row r="57" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="B55" s="48" t="s">
+      <c r="B57" s="48" t="s">
         <v>88</v>
       </c>
-      <c r="C55" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D55" s="4">
+      <c r="C57" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D57" s="4">
         <v>2</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="37"/>
-      <c r="B56" s="37"/>
-      <c r="C56" s="37"/>
-      <c r="D56" s="37"/>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C62" s="64"/>
-    </row>
-    <row r="63" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C63" s="63"/>
-    </row>
-    <row r="69" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B69" s="47"/>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" s="37"/>
+      <c r="B58" s="37"/>
+      <c r="C58" s="37"/>
+      <c r="D58" s="37"/>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C64" s="64"/>
+    </row>
+    <row r="65" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C65" s="63"/>
+    </row>
+    <row r="71" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B71" s="47"/>
     </row>
   </sheetData>
   <sheetProtection formatColumns="0" selectLockedCells="1"/>
   <protectedRanges>
-    <protectedRange sqref="I3:I6 I8 I12:I16 I25:I28 D15:D18 I32 D23 I19:I20 D3:D6 D8:D11 D13" name="Range1_1"/>
+    <protectedRange sqref="I3:I6 I8 I12:I16 I27:I30 D15:D18 I34 D25 I19:I20 D3:D6 D8:D11 D13" name="Range1_1"/>
     <protectedRange sqref="D7 D14" name="Range1_1_1"/>
-    <protectedRange sqref="D45:D55" name="Range1_1_4"/>
-    <protectedRange sqref="D12 D28" name="Range1_1_2"/>
-    <protectedRange sqref="D25" name="Range1_1_6_1"/>
-    <protectedRange sqref="D22" name="Range1_1_6"/>
-    <protectedRange sqref="D24" name="Range1_1_5"/>
-    <protectedRange sqref="D26" name="Range1_1_5_1_1"/>
-    <protectedRange sqref="D27" name="Range1_1_8_1_1"/>
-    <protectedRange sqref="D39 D32:D37" name="Range1_1_3_1"/>
+    <protectedRange sqref="D47:D57" name="Range1_1_4"/>
+    <protectedRange sqref="D12 D30" name="Range1_1_2"/>
+    <protectedRange sqref="D27" name="Range1_1_6_1"/>
+    <protectedRange sqref="D24" name="Range1_1_6"/>
+    <protectedRange sqref="D26" name="Range1_1_5"/>
+    <protectedRange sqref="D28" name="Range1_1_5_1_1"/>
+    <protectedRange sqref="D29" name="Range1_1_8_1_1"/>
+    <protectedRange sqref="D41 D34:D39" name="Range1_1_3_1"/>
   </protectedRanges>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -3124,10 +3192,10 @@
       </c>
     </row>
     <row r="24" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="65" t="s">
+      <c r="A24" s="69" t="s">
         <v>146</v>
       </c>
-      <c r="B24" s="66"/>
+      <c r="B24" s="70"/>
       <c r="C24" s="52">
         <f>SUM(C17:C23)</f>
         <v>795.76639999999998</v>
@@ -3422,10 +3490,10 @@
       </c>
     </row>
     <row r="54" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="65" t="s">
+      <c r="A54" s="69" t="s">
         <v>146</v>
       </c>
-      <c r="B54" s="66"/>
+      <c r="B54" s="70"/>
       <c r="C54" s="52">
         <f>SUM(C47:C53)</f>
         <v>440.30922480000004</v>

</xml_diff>

<commit_message>
Fixing bugs found through FEMA work
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C47909F1-F930-435F-A158-CC232ABEAF3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E6C7A5D-58C8-4E60-92F3-23DA7B1F9D8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2685" yWindow="5100" windowWidth="28800" windowHeight="15345" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
   <sheets>
     <sheet name="James_Island_Midbay" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="247">
   <si>
     <t>StormSim Project General Inputs</t>
   </si>
@@ -685,9 +685,6 @@
     <t>SP_2243</t>
   </si>
   <si>
-    <t>prob_mass_from_MB_SP2243\prob_mass_from_MB_SP2243.mat</t>
-  </si>
-  <si>
     <t>pros_q_vol</t>
   </si>
   <si>
@@ -730,9 +727,6 @@
     <t>Probability Masses (CHS -&gt; MCSim_Inputs folder relative path, Custom Modeling -&gt; .mat filename with relative path)</t>
   </si>
   <si>
-    <t>prob_mass_from_MB_SP2243\CHS_Data_from_MB_SP2243.mat</t>
-  </si>
-  <si>
     <t>Load project_forcing StormSim File From Other case_name Under The Same project_name (0- Sample New Storms/1-Load Previous Storm Suite)</t>
   </si>
   <si>
@@ -749,6 +743,42 @@
   </si>
   <si>
     <t>Levee_Case_5</t>
+  </si>
+  <si>
+    <t>Midbay_CHS_Data.zip</t>
+  </si>
+  <si>
+    <t>MCSim_Inputs\NACCS</t>
+  </si>
+  <si>
+    <t>outfolder</t>
+  </si>
+  <si>
+    <t>StormSim Project output folder.</t>
+  </si>
+  <si>
+    <t>pros_plot_hc</t>
+  </si>
+  <si>
+    <t>Plot individual responses hazard curves (0 - Off, 1 - On)</t>
+  </si>
+  <si>
+    <t>pros_plot_forcing_hc_w_pot</t>
+  </si>
+  <si>
+    <t>Plot forcing hazard curves with corresponding POT sample (0 - Off, 1 - On)</t>
+  </si>
+  <si>
+    <t>pros_plot_prioty_comp</t>
+  </si>
+  <si>
+    <t>Plot RB1 priority datasets responses comparison (0 - Off, 1 - On)</t>
+  </si>
+  <si>
+    <t>pros_plot_hc_xsec</t>
+  </si>
+  <si>
+    <t>Plot hazard curve cross section plots (0 - Off, 1 - On)</t>
   </si>
 </sst>
 </file>
@@ -1636,7 +1666,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51D29750-2AFD-4BF7-A911-1DC4ADC0FD7A}">
-  <dimension ref="A1:I71"/>
+  <dimension ref="A1:I72"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.5703125" customWidth="1"/>
@@ -1752,7 +1782,7 @@
         <v>10</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="F5" s="49" t="s">
         <v>98</v>
@@ -1769,17 +1799,15 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>20</v>
+        <v>237</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>21</v>
+        <v>238</v>
       </c>
       <c r="C6" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>106</v>
-      </c>
+      <c r="D6" s="2"/>
       <c r="F6" s="49" t="s">
         <v>97</v>
       </c>
@@ -1795,16 +1823,16 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="C7" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F7" s="14" t="s">
         <v>99</v>
@@ -1821,16 +1849,16 @@
     </row>
     <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="14" t="s">
-        <v>115</v>
+        <v>29</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>190</v>
+        <v>30</v>
       </c>
       <c r="C8" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D8" s="2">
-        <v>1</v>
+      <c r="D8" s="2" t="s">
+        <v>110</v>
       </c>
       <c r="F8" s="17" t="s">
         <v>94</v>
@@ -1847,16 +1875,16 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>18</v>
+        <v>115</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>19</v>
+        <v>190</v>
       </c>
       <c r="C9" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D9" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F9" s="33"/>
       <c r="G9" s="33"/>
@@ -1865,16 +1893,16 @@
     </row>
     <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="14" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C10" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>76</v>
+      <c r="D10" s="2">
+        <v>3</v>
       </c>
       <c r="F10" s="26" t="s">
         <v>100</v>
@@ -1885,16 +1913,16 @@
     </row>
     <row r="11" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="14" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>127</v>
-      </c>
-      <c r="D11" s="2">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>76</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>3</v>
@@ -1911,16 +1939,16 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>191</v>
+        <v>24</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>220</v>
+        <v>25</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>10</v>
+        <v>127</v>
       </c>
       <c r="D12" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F12" s="30" t="s">
         <v>102</v>
@@ -1937,16 +1965,16 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>101</v>
+        <v>191</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C13" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D13" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F13" s="30" t="s">
         <v>103</v>
@@ -1963,10 +1991,10 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>116</v>
+        <v>101</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C14" s="16" t="s">
         <v>10</v>
@@ -1989,10 +2017,10 @@
     </row>
     <row r="15" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="14" t="s">
-        <v>77</v>
+        <v>116</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C15" s="16" t="s">
         <v>10</v>
@@ -2015,16 +2043,16 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>212</v>
+        <v>77</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D16" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16" s="27"/>
       <c r="G16" s="27"/>
@@ -2033,16 +2061,16 @@
     </row>
     <row r="17" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="14" t="s">
-        <v>119</v>
+        <v>212</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C17" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D17" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F17" s="7" t="s">
         <v>1</v>
@@ -2057,10 +2085,10 @@
     </row>
     <row r="18" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="14" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C18" s="16" t="s">
         <v>10</v>
@@ -2083,10 +2111,10 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
-        <v>234</v>
+        <v>120</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="C19" s="16" t="s">
         <v>10</v>
@@ -2104,21 +2132,21 @@
         <v>10</v>
       </c>
       <c r="I19" s="68">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="17" t="s">
-        <v>235</v>
-      </c>
-      <c r="B20" s="18" t="s">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="14" t="s">
         <v>232</v>
       </c>
-      <c r="C20" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>233</v>
+      <c r="B20" s="15" t="s">
+        <v>229</v>
+      </c>
+      <c r="C20" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" s="2">
+        <v>1</v>
       </c>
       <c r="F20" s="14" t="s">
         <v>15</v>
@@ -2133,11 +2161,19 @@
         <v>50</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="6"/>
-      <c r="B21" s="22"/>
-      <c r="C21" s="23"/>
-      <c r="D21" s="23"/>
+    <row r="21" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="17" t="s">
+        <v>233</v>
+      </c>
+      <c r="B21" s="18" t="s">
+        <v>230</v>
+      </c>
+      <c r="C21" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>231</v>
+      </c>
       <c r="F21" s="14" t="s">
         <v>117</v>
       </c>
@@ -2151,31 +2187,23 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="24" t="s">
-        <v>35</v>
-      </c>
-      <c r="B22" s="25"/>
-      <c r="C22" s="25"/>
-      <c r="D22" s="25"/>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" s="6"/>
+      <c r="B22" s="22"/>
+      <c r="C22" s="23"/>
+      <c r="D22" s="23"/>
       <c r="F22" s="8"/>
       <c r="G22" s="8"/>
       <c r="H22" s="8"/>
       <c r="I22" s="8"/>
     </row>
     <row r="23" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B23" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="C23" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="D23" s="10" t="s">
-        <v>6</v>
-      </c>
+      <c r="A23" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="B23" s="25"/>
+      <c r="C23" s="25"/>
+      <c r="D23" s="25"/>
       <c r="F23" s="20" t="s">
         <v>26</v>
       </c>
@@ -2184,17 +2212,17 @@
       <c r="I23" s="21"/>
     </row>
     <row r="24" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="11" t="s">
-        <v>187</v>
-      </c>
-      <c r="B24" s="12" t="s">
-        <v>188</v>
-      </c>
-      <c r="C24" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="D24" s="1">
-        <v>0</v>
+      <c r="A24" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C24" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D24" s="10" t="s">
+        <v>6</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>3</v>
@@ -2211,16 +2239,16 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
-        <v>38</v>
+        <v>187</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>39</v>
+        <v>188</v>
       </c>
       <c r="C25" s="28" t="s">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="D25" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F25" s="11" t="s">
         <v>27</v>
@@ -2237,16 +2265,16 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
-        <v>108</v>
+        <v>38</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>109</v>
+        <v>39</v>
       </c>
       <c r="C26" s="28" t="s">
-        <v>107</v>
+        <v>40</v>
       </c>
       <c r="D26" s="1">
-        <v>3.43</v>
+        <v>1</v>
       </c>
       <c r="F26" s="14" t="s">
         <v>31</v>
@@ -2263,16 +2291,16 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="11" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>227</v>
+        <v>109</v>
       </c>
       <c r="C27" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>185</v>
+        <v>107</v>
+      </c>
+      <c r="D27" s="1">
+        <v>3.43</v>
       </c>
       <c r="F27" s="14" t="s">
         <v>33</v>
@@ -2289,16 +2317,16 @@
     </row>
     <row r="28" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
-        <v>186</v>
+        <v>104</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="C28" s="28" t="s">
         <v>10</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>215</v>
+        <v>185</v>
       </c>
       <c r="F28" s="17" t="s">
         <v>36</v>
@@ -2314,17 +2342,17 @@
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="14" t="s">
-        <v>42</v>
-      </c>
-      <c r="B29" s="15" t="s">
-        <v>189</v>
-      </c>
-      <c r="C29" s="16" t="s">
+      <c r="A29" s="11" t="s">
+        <v>186</v>
+      </c>
+      <c r="B29" s="12" t="s">
+        <v>228</v>
+      </c>
+      <c r="C29" s="28" t="s">
         <v>10</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="F29" s="21"/>
       <c r="G29" s="21"/>
@@ -2333,16 +2361,16 @@
     </row>
     <row r="30" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="14" t="s">
-        <v>105</v>
+        <v>42</v>
       </c>
       <c r="B30" s="15" t="s">
-        <v>228</v>
+        <v>189</v>
       </c>
       <c r="C30" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>184</v>
+        <v>235</v>
       </c>
       <c r="F30" s="26" t="s">
         <v>41</v>
@@ -2352,10 +2380,18 @@
       <c r="I30" s="27"/>
     </row>
     <row r="31" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="25"/>
-      <c r="B31" s="25"/>
-      <c r="C31" s="25"/>
-      <c r="D31" s="25"/>
+      <c r="A31" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="B31" s="15" t="s">
+        <v>227</v>
+      </c>
+      <c r="C31" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>184</v>
+      </c>
       <c r="F31" s="9" t="s">
         <v>3</v>
       </c>
@@ -2369,13 +2405,11 @@
         <v>6</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="34" t="s">
-        <v>50</v>
-      </c>
-      <c r="B32" s="35"/>
-      <c r="C32" s="35"/>
-      <c r="D32" s="35"/>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" s="25"/>
+      <c r="B32" s="25"/>
+      <c r="C32" s="25"/>
+      <c r="D32" s="25"/>
       <c r="F32" s="29" t="s">
         <v>43</v>
       </c>
@@ -2390,18 +2424,12 @@
       </c>
     </row>
     <row r="33" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B33" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C33" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="D33" s="10" t="s">
-        <v>6</v>
-      </c>
+      <c r="A33" s="34" t="s">
+        <v>50</v>
+      </c>
+      <c r="B33" s="35"/>
+      <c r="C33" s="35"/>
+      <c r="D33" s="35"/>
       <c r="F33" s="14" t="s">
         <v>112</v>
       </c>
@@ -2415,18 +2443,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="B34" s="12" t="s">
-        <v>122</v>
-      </c>
-      <c r="C34" s="13" t="s">
-        <v>127</v>
-      </c>
-      <c r="D34" s="1">
-        <v>3.41</v>
+    <row r="34" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B34" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C34" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D34" s="10" t="s">
+        <v>6</v>
       </c>
       <c r="F34" s="14" t="s">
         <v>196</v>
@@ -2438,21 +2466,21 @@
         <v>10</v>
       </c>
       <c r="I34" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A35" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="B35" s="15" t="s">
-        <v>78</v>
-      </c>
-      <c r="C35" s="16" t="s">
+      <c r="A35" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="B35" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="C35" s="13" t="s">
         <v>127</v>
       </c>
-      <c r="D35" s="2">
-        <v>7.01</v>
+      <c r="D35" s="1">
+        <v>3.41</v>
       </c>
       <c r="F35" s="14" t="s">
         <v>197</v>
@@ -2464,21 +2492,21 @@
         <v>10</v>
       </c>
       <c r="I35" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B36" s="15" t="s">
-        <v>123</v>
+        <v>78</v>
       </c>
       <c r="C36" s="16" t="s">
         <v>127</v>
       </c>
       <c r="D36" s="2">
-        <v>-2.42</v>
+        <v>7.01</v>
       </c>
       <c r="F36" s="14" t="s">
         <v>198</v>
@@ -2495,16 +2523,16 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
-        <v>174</v>
+        <v>53</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C37" s="16" t="s">
         <v>127</v>
       </c>
       <c r="D37" s="2">
-        <v>-0.95799999999999996</v>
+        <v>-2.42</v>
       </c>
       <c r="F37" s="14" t="s">
         <v>199</v>
@@ -2521,16 +2549,16 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
-        <v>54</v>
+        <v>174</v>
       </c>
       <c r="B38" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C38" s="16" t="s">
-        <v>10</v>
+        <v>127</v>
       </c>
       <c r="D38" s="2">
-        <v>3</v>
+        <v>-0.95799999999999996</v>
       </c>
       <c r="F38" s="14" t="s">
         <v>200</v>
@@ -2547,22 +2575,22 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B39" s="15" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C39" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D39" s="2">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="F39" s="14" t="s">
+        <v>215</v>
+      </c>
+      <c r="G39" s="15" t="s">
         <v>216</v>
-      </c>
-      <c r="G39" s="15" t="s">
-        <v>217</v>
       </c>
       <c r="H39" s="16" t="s">
         <v>10</v>
@@ -2572,17 +2600,17 @@
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A40" s="39" t="s">
-        <v>82</v>
-      </c>
-      <c r="B40" s="39" t="s">
-        <v>83</v>
-      </c>
-      <c r="C40" s="45" t="s">
-        <v>132</v>
-      </c>
-      <c r="D40" s="46">
-        <v>0</v>
+      <c r="A40" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="B40" s="15" t="s">
+        <v>126</v>
+      </c>
+      <c r="C40" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D40" s="2">
+        <v>1.5</v>
       </c>
       <c r="F40" s="14" t="s">
         <v>201</v>
@@ -2598,17 +2626,17 @@
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A41" s="14" t="s">
-        <v>134</v>
-      </c>
-      <c r="B41" s="15" t="s">
-        <v>133</v>
-      </c>
-      <c r="C41" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D41" s="2">
-        <v>0.4</v>
+      <c r="A41" s="39" t="s">
+        <v>82</v>
+      </c>
+      <c r="B41" s="39" t="s">
+        <v>83</v>
+      </c>
+      <c r="C41" s="45" t="s">
+        <v>132</v>
+      </c>
+      <c r="D41" s="46">
+        <v>0</v>
       </c>
       <c r="F41" s="14" t="s">
         <v>202</v>
@@ -2623,178 +2651,226 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="B42" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="C42" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D42" s="2">
+        <v>0.4</v>
+      </c>
+      <c r="F42" s="14" t="s">
+        <v>203</v>
+      </c>
+      <c r="G42" s="15" t="s">
+        <v>211</v>
+      </c>
+      <c r="H42" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I42" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A43" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="B42" s="14" t="s">
+      <c r="B43" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="C42" s="16" t="s">
+      <c r="C43" s="16" t="s">
         <v>127</v>
       </c>
-      <c r="D42" s="2">
+      <c r="D43" s="2">
         <v>3.35</v>
       </c>
-      <c r="F42" s="17" t="s">
-        <v>203</v>
-      </c>
-      <c r="G42" s="18" t="s">
-        <v>211</v>
-      </c>
-      <c r="H42" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="I42" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="38" t="s">
+      <c r="F43" s="14" t="s">
+        <v>239</v>
+      </c>
+      <c r="G43" s="15" t="s">
+        <v>240</v>
+      </c>
+      <c r="H43" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I43" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="38" t="s">
         <v>85</v>
       </c>
-      <c r="B43" s="38" t="s">
+      <c r="B44" s="38" t="s">
         <v>121</v>
       </c>
-      <c r="C43" s="43" t="s">
+      <c r="C44" s="43" t="s">
         <v>127</v>
       </c>
-      <c r="D43" s="44">
+      <c r="D44" s="44">
         <v>0.06</v>
       </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A44" s="34"/>
-      <c r="B44" s="34"/>
-      <c r="C44" s="34"/>
-      <c r="D44" s="34"/>
-    </row>
-    <row r="45" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="36" t="s">
+      <c r="F44" s="14" t="s">
+        <v>241</v>
+      </c>
+      <c r="G44" s="15" t="s">
+        <v>242</v>
+      </c>
+      <c r="H44" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I44" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A45" s="34"/>
+      <c r="B45" s="34"/>
+      <c r="C45" s="34"/>
+      <c r="D45" s="34"/>
+      <c r="F45" s="14" t="s">
+        <v>243</v>
+      </c>
+      <c r="G45" s="15" t="s">
+        <v>244</v>
+      </c>
+      <c r="H45" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I45" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="36" t="s">
         <v>56</v>
       </c>
-      <c r="B45" s="37"/>
-      <c r="C45" s="37"/>
-      <c r="D45" s="37"/>
-    </row>
-    <row r="46" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="9" t="s">
+      <c r="B46" s="37"/>
+      <c r="C46" s="37"/>
+      <c r="D46" s="37"/>
+      <c r="F46" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="G46" s="18" t="s">
+        <v>246</v>
+      </c>
+      <c r="H46" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="I46" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="B46" s="10" t="s">
+      <c r="B47" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C46" s="10" t="s">
+      <c r="C47" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="D46" s="10" t="s">
+      <c r="D47" s="10" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A47" s="11" t="s">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A48" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="B47" s="12" t="s">
+      <c r="B48" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="C47" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="D47" s="1">
+      <c r="C48" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D48" s="1">
         <v>1.65</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A48" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="B48" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="C48" s="16" t="s">
-        <v>128</v>
-      </c>
-      <c r="D48" s="2">
-        <v>780</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B49" s="15" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C49" s="16" t="s">
         <v>128</v>
       </c>
       <c r="D49" s="2">
-        <v>57</v>
+        <v>780</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
-        <v>218</v>
+        <v>61</v>
       </c>
       <c r="B50" s="15" t="s">
-        <v>219</v>
+        <v>62</v>
       </c>
       <c r="C50" s="16" t="s">
         <v>128</v>
       </c>
       <c r="D50" s="2">
-        <v>1147</v>
+        <v>57</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="14" t="s">
-        <v>63</v>
+        <v>217</v>
       </c>
       <c r="B51" s="15" t="s">
-        <v>64</v>
+        <v>218</v>
       </c>
       <c r="C51" s="16" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D51" s="2">
-        <v>1027</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="14" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B52" s="15" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C52" s="16" t="s">
-        <v>67</v>
+        <v>129</v>
       </c>
       <c r="D52" s="2">
-        <v>0.4</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="14" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B53" s="15" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C53" s="16" t="s">
-        <v>10</v>
+        <v>67</v>
       </c>
       <c r="D53" s="2">
-        <v>1</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="14" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B54" s="15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C54" s="16" t="s">
         <v>10</v>
@@ -2805,74 +2881,88 @@
     </row>
     <row r="55" spans="1:4" ht="60.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="B55" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="C55" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D55" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="B55" s="15" t="s">
+      <c r="B56" s="15" t="s">
         <v>73</v>
       </c>
-      <c r="C55" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D55" s="2">
+      <c r="C56" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D56" s="2">
         <v>17</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="39" t="s">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" s="39" t="s">
         <v>74</v>
       </c>
-      <c r="B56" s="40" t="s">
+      <c r="B57" s="40" t="s">
         <v>75</v>
       </c>
-      <c r="C56" s="41" t="s">
-        <v>10</v>
-      </c>
-      <c r="D56" s="42">
+      <c r="C57" s="41" t="s">
+        <v>10</v>
+      </c>
+      <c r="D57" s="42">
         <v>17</v>
       </c>
     </row>
-    <row r="57" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="18" t="s">
+    <row r="58" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="B57" s="48" t="s">
+      <c r="B58" s="48" t="s">
         <v>87</v>
       </c>
-      <c r="C57" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D57" s="4">
+      <c r="C58" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D58" s="4">
         <v>2</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="37"/>
-      <c r="B58" s="37"/>
-      <c r="C58" s="37"/>
-      <c r="D58" s="37"/>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C64" s="64"/>
-    </row>
-    <row r="65" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C65" s="63"/>
-    </row>
-    <row r="71" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B71" s="47"/>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="37"/>
+      <c r="B59" s="37"/>
+      <c r="C59" s="37"/>
+      <c r="D59" s="37"/>
+    </row>
+    <row r="65" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C65" s="64"/>
+    </row>
+    <row r="66" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C66" s="63"/>
+    </row>
+    <row r="72" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B72" s="47"/>
     </row>
   </sheetData>
   <sheetProtection formatColumns="0" selectLockedCells="1"/>
   <protectedRanges>
-    <protectedRange sqref="I3:I6 I8 I12:I16 I25:I28 D15:D18 I32 D25 I19:I20 D3:D6 D8:D11 D13" name="Range1_1"/>
-    <protectedRange sqref="D7 D14" name="Range1_1_1"/>
-    <protectedRange sqref="D47:D57" name="Range1_1_4"/>
-    <protectedRange sqref="D12 D30" name="Range1_1_2"/>
-    <protectedRange sqref="D27" name="Range1_1_6_1"/>
-    <protectedRange sqref="D24" name="Range1_1_6"/>
-    <protectedRange sqref="D26" name="Range1_1_5"/>
-    <protectedRange sqref="D28" name="Range1_1_5_1_1"/>
-    <protectedRange sqref="D29" name="Range1_1_8_1_1"/>
-    <protectedRange sqref="D41 D34:D39" name="Range1_1_3_1"/>
+    <protectedRange sqref="I3:I6 I8 I12:I16 I25:I28 D16:D19 I32 D26 I19:I20 D9:D12 D14 D3:D7" name="Range1_1"/>
+    <protectedRange sqref="D8 D15" name="Range1_1_1"/>
+    <protectedRange sqref="D48:D58" name="Range1_1_4"/>
+    <protectedRange sqref="D13 D31" name="Range1_1_2"/>
+    <protectedRange sqref="D28" name="Range1_1_6_1"/>
+    <protectedRange sqref="D25" name="Range1_1_6"/>
+    <protectedRange sqref="D27" name="Range1_1_5"/>
+    <protectedRange sqref="D29" name="Range1_1_5_1_1"/>
+    <protectedRange sqref="D30" name="Range1_1_8_1_1"/>
+    <protectedRange sqref="D42 D35:D40" name="Range1_1_3_1"/>
   </protectedRanges>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Adding xc bias correction flag
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fagar\OneDrive\Desktop\StormSim-Dev\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\HC_QAQC_NACCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E6C7A5D-58C8-4E60-92F3-23DA7B1F9D8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7938099F-FCCF-4213-9243-72DC3A6868D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="248">
   <si>
     <t>StormSim Project General Inputs</t>
   </si>
@@ -592,12 +592,6 @@
     <t xml:space="preserve">Historical Sampling </t>
   </si>
   <si>
-    <t>CO-OPS_8571421_Bishops_Head_Pred_tide_MSL_m.csv</t>
-  </si>
-  <si>
-    <t>StormSim_Library\CHS\Bias_Correction_Files\NACCS_Comb_BiasUncertainty_perVG_rta.mat</t>
-  </si>
-  <si>
     <t>prob_mass_source</t>
   </si>
   <si>
@@ -779,6 +773,15 @@
   </si>
   <si>
     <t>Plot hazard curve cross section plots (0 - Off, 1 - On)</t>
+  </si>
+  <si>
+    <t>StormSim_PROS_Outputs</t>
+  </si>
+  <si>
+    <t>apply_xc_bias</t>
+  </si>
+  <si>
+    <t>Apply Bias Correction To Extratropical Stomrs  (0 - Off / 1 - On)</t>
   </si>
 </sst>
 </file>
@@ -1370,9 +1373,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1410,7 +1413,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1516,7 +1519,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1658,7 +1661,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1666,7 +1669,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51D29750-2AFD-4BF7-A911-1DC4ADC0FD7A}">
-  <dimension ref="A1:I72"/>
+  <dimension ref="A1:I73"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.5703125" customWidth="1"/>
@@ -1730,7 +1733,7 @@
         <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="F3" s="49" t="s">
         <v>95</v>
@@ -1756,7 +1759,7 @@
         <v>10</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F4" s="49" t="s">
         <v>96</v>
@@ -1782,7 +1785,7 @@
         <v>10</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="F5" s="49" t="s">
         <v>98</v>
@@ -1799,15 +1802,17 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="C6" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="2"/>
+      <c r="D6" s="2" t="s">
+        <v>245</v>
+      </c>
       <c r="F6" s="49" t="s">
         <v>97</v>
       </c>
@@ -1878,7 +1883,7 @@
         <v>115</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C9" s="16" t="s">
         <v>10</v>
@@ -1965,16 +1970,16 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C13" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D13" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F13" s="30" t="s">
         <v>103</v>
@@ -1994,7 +1999,7 @@
         <v>101</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="C14" s="16" t="s">
         <v>10</v>
@@ -2017,16 +2022,16 @@
     </row>
     <row r="15" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="14" t="s">
-        <v>116</v>
+        <v>246</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>221</v>
+        <v>247</v>
       </c>
       <c r="C15" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D15" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F15" s="17" t="s">
         <v>80</v>
@@ -2043,10 +2048,10 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>77</v>
+        <v>116</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>10</v>
@@ -2061,16 +2066,16 @@
     </row>
     <row r="17" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="14" t="s">
-        <v>212</v>
+        <v>77</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="C17" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D17" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F17" s="7" t="s">
         <v>1</v>
@@ -2085,16 +2090,16 @@
     </row>
     <row r="18" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="14" t="s">
-        <v>119</v>
+        <v>210</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C18" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D18" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>3</v>
@@ -2111,16 +2116,16 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="C19" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D19" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F19" s="65" t="s">
         <v>11</v>
@@ -2137,16 +2142,16 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
-        <v>232</v>
+        <v>120</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="C20" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D20" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F20" s="14" t="s">
         <v>15</v>
@@ -2161,18 +2166,18 @@
         <v>50</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="17" t="s">
-        <v>233</v>
-      </c>
-      <c r="B21" s="18" t="s">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="14" t="s">
         <v>230</v>
       </c>
-      <c r="C21" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>231</v>
+      <c r="B21" s="15" t="s">
+        <v>227</v>
+      </c>
+      <c r="C21" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21" s="2">
+        <v>1</v>
       </c>
       <c r="F21" s="14" t="s">
         <v>117</v>
@@ -2187,23 +2192,29 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="6"/>
-      <c r="B22" s="22"/>
-      <c r="C22" s="23"/>
-      <c r="D22" s="23"/>
+    <row r="22" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="17" t="s">
+        <v>231</v>
+      </c>
+      <c r="B22" s="18" t="s">
+        <v>228</v>
+      </c>
+      <c r="C22" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>229</v>
+      </c>
       <c r="F22" s="8"/>
       <c r="G22" s="8"/>
       <c r="H22" s="8"/>
       <c r="I22" s="8"/>
     </row>
     <row r="23" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="24" t="s">
-        <v>35</v>
-      </c>
-      <c r="B23" s="25"/>
-      <c r="C23" s="25"/>
-      <c r="D23" s="25"/>
+      <c r="A23" s="6"/>
+      <c r="B23" s="22"/>
+      <c r="C23" s="23"/>
+      <c r="D23" s="23"/>
       <c r="F23" s="20" t="s">
         <v>26</v>
       </c>
@@ -2212,18 +2223,12 @@
       <c r="I23" s="21"/>
     </row>
     <row r="24" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B24" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="C24" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="D24" s="10" t="s">
-        <v>6</v>
-      </c>
+      <c r="A24" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="B24" s="25"/>
+      <c r="C24" s="25"/>
+      <c r="D24" s="25"/>
       <c r="F24" s="9" t="s">
         <v>3</v>
       </c>
@@ -2237,18 +2242,18 @@
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="11" t="s">
-        <v>187</v>
-      </c>
-      <c r="B25" s="12" t="s">
-        <v>188</v>
-      </c>
-      <c r="C25" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="D25" s="1">
-        <v>0</v>
+    <row r="25" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D25" s="10" t="s">
+        <v>6</v>
       </c>
       <c r="F25" s="11" t="s">
         <v>27</v>
@@ -2265,16 +2270,16 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
-        <v>38</v>
+        <v>185</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>39</v>
+        <v>186</v>
       </c>
       <c r="C26" s="28" t="s">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="D26" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F26" s="14" t="s">
         <v>31</v>
@@ -2291,16 +2296,16 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="11" t="s">
-        <v>108</v>
+        <v>38</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>109</v>
+        <v>39</v>
       </c>
       <c r="C27" s="28" t="s">
-        <v>107</v>
+        <v>40</v>
       </c>
       <c r="D27" s="1">
-        <v>3.43</v>
+        <v>1</v>
       </c>
       <c r="F27" s="14" t="s">
         <v>33</v>
@@ -2317,16 +2322,16 @@
     </row>
     <row r="28" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>226</v>
+        <v>109</v>
       </c>
       <c r="C28" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>185</v>
+        <v>107</v>
+      </c>
+      <c r="D28" s="1">
+        <v>3.43</v>
       </c>
       <c r="F28" s="17" t="s">
         <v>36</v>
@@ -2343,34 +2348,32 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
-        <v>186</v>
+        <v>104</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="C29" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="D29" s="2" t="s">
-        <v>236</v>
-      </c>
+      <c r="D29" s="2"/>
       <c r="F29" s="21"/>
       <c r="G29" s="21"/>
       <c r="H29" s="21"/>
       <c r="I29" s="21"/>
     </row>
     <row r="30" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="14" t="s">
-        <v>42</v>
-      </c>
-      <c r="B30" s="15" t="s">
-        <v>189</v>
-      </c>
-      <c r="C30" s="16" t="s">
+      <c r="A30" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="B30" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="C30" s="28" t="s">
         <v>10</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F30" s="26" t="s">
         <v>41</v>
@@ -2381,16 +2384,16 @@
     </row>
     <row r="31" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="14" t="s">
-        <v>105</v>
+        <v>42</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>227</v>
+        <v>187</v>
       </c>
       <c r="C31" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>184</v>
+        <v>233</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>3</v>
@@ -2406,10 +2409,16 @@
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="25"/>
-      <c r="B32" s="25"/>
-      <c r="C32" s="25"/>
-      <c r="D32" s="25"/>
+      <c r="A32" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="B32" s="15" t="s">
+        <v>225</v>
+      </c>
+      <c r="C32" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D32" s="2"/>
       <c r="F32" s="29" t="s">
         <v>43</v>
       </c>
@@ -2423,13 +2432,11 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="34" t="s">
-        <v>50</v>
-      </c>
-      <c r="B33" s="35"/>
-      <c r="C33" s="35"/>
-      <c r="D33" s="35"/>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" s="25"/>
+      <c r="B33" s="25"/>
+      <c r="C33" s="25"/>
+      <c r="D33" s="25"/>
       <c r="F33" s="14" t="s">
         <v>112</v>
       </c>
@@ -2440,79 +2447,73 @@
         <v>10</v>
       </c>
       <c r="I33" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="9" t="s">
+      <c r="A34" s="34" t="s">
+        <v>50</v>
+      </c>
+      <c r="B34" s="35"/>
+      <c r="C34" s="35"/>
+      <c r="D34" s="35"/>
+      <c r="F34" s="14" t="s">
+        <v>194</v>
+      </c>
+      <c r="G34" s="15" t="s">
+        <v>202</v>
+      </c>
+      <c r="H34" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I34" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="B34" s="10" t="s">
+      <c r="B35" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C34" s="10" t="s">
+      <c r="C35" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="D34" s="10" t="s">
+      <c r="D35" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="F34" s="14" t="s">
+      <c r="F35" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="G35" s="15" t="s">
+        <v>203</v>
+      </c>
+      <c r="H35" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I35" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="B36" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="C36" s="13" t="s">
+        <v>127</v>
+      </c>
+      <c r="D36" s="1">
+        <v>3.41</v>
+      </c>
+      <c r="F36" s="14" t="s">
         <v>196</v>
       </c>
-      <c r="G34" s="15" t="s">
+      <c r="G36" s="15" t="s">
         <v>204</v>
-      </c>
-      <c r="H34" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="I34" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A35" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="B35" s="12" t="s">
-        <v>122</v>
-      </c>
-      <c r="C35" s="13" t="s">
-        <v>127</v>
-      </c>
-      <c r="D35" s="1">
-        <v>3.41</v>
-      </c>
-      <c r="F35" s="14" t="s">
-        <v>197</v>
-      </c>
-      <c r="G35" s="15" t="s">
-        <v>205</v>
-      </c>
-      <c r="H35" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="I35" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="B36" s="15" t="s">
-        <v>78</v>
-      </c>
-      <c r="C36" s="16" t="s">
-        <v>127</v>
-      </c>
-      <c r="D36" s="2">
-        <v>7.01</v>
-      </c>
-      <c r="F36" s="14" t="s">
-        <v>198</v>
-      </c>
-      <c r="G36" s="15" t="s">
-        <v>206</v>
       </c>
       <c r="H36" s="16" t="s">
         <v>10</v>
@@ -2523,100 +2524,100 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>123</v>
+        <v>78</v>
       </c>
       <c r="C37" s="16" t="s">
         <v>127</v>
       </c>
       <c r="D37" s="2">
-        <v>-2.42</v>
+        <v>7.01</v>
       </c>
       <c r="F37" s="14" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="G37" s="15" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="H37" s="16" t="s">
         <v>10</v>
       </c>
       <c r="I37" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
-        <v>174</v>
+        <v>53</v>
       </c>
       <c r="B38" s="15" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C38" s="16" t="s">
         <v>127</v>
       </c>
       <c r="D38" s="2">
-        <v>-0.95799999999999996</v>
+        <v>-2.42</v>
       </c>
       <c r="F38" s="14" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="G38" s="15" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="H38" s="16" t="s">
         <v>10</v>
       </c>
       <c r="I38" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
-        <v>54</v>
+        <v>174</v>
       </c>
       <c r="B39" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C39" s="16" t="s">
-        <v>10</v>
+        <v>127</v>
       </c>
       <c r="D39" s="2">
-        <v>3</v>
+        <v>-0.95799999999999996</v>
       </c>
       <c r="F39" s="14" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="G39" s="15" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="H39" s="16" t="s">
         <v>10</v>
       </c>
       <c r="I39" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B40" s="15" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C40" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D40" s="2">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="F40" s="14" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="G40" s="15" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="H40" s="16" t="s">
         <v>10</v>
@@ -2626,23 +2627,23 @@
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A41" s="39" t="s">
-        <v>82</v>
-      </c>
-      <c r="B41" s="39" t="s">
-        <v>83</v>
-      </c>
-      <c r="C41" s="45" t="s">
-        <v>132</v>
-      </c>
-      <c r="D41" s="46">
-        <v>0</v>
+      <c r="A41" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="B41" s="15" t="s">
+        <v>126</v>
+      </c>
+      <c r="C41" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D41" s="2">
+        <v>1.5</v>
       </c>
       <c r="F41" s="14" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="G41" s="15" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="H41" s="16" t="s">
         <v>10</v>
@@ -2652,23 +2653,23 @@
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A42" s="14" t="s">
-        <v>134</v>
-      </c>
-      <c r="B42" s="15" t="s">
-        <v>133</v>
-      </c>
-      <c r="C42" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D42" s="2">
-        <v>0.4</v>
+      <c r="A42" s="39" t="s">
+        <v>82</v>
+      </c>
+      <c r="B42" s="39" t="s">
+        <v>83</v>
+      </c>
+      <c r="C42" s="45" t="s">
+        <v>132</v>
+      </c>
+      <c r="D42" s="46">
+        <v>0</v>
       </c>
       <c r="F42" s="14" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="G42" s="15" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="H42" s="16" t="s">
         <v>10</v>
@@ -2679,22 +2680,22 @@
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
-        <v>84</v>
-      </c>
-      <c r="B43" s="14" t="s">
-        <v>86</v>
+        <v>134</v>
+      </c>
+      <c r="B43" s="15" t="s">
+        <v>133</v>
       </c>
       <c r="C43" s="16" t="s">
-        <v>127</v>
+        <v>10</v>
       </c>
       <c r="D43" s="2">
-        <v>3.35</v>
+        <v>0.4</v>
       </c>
       <c r="F43" s="14" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="G43" s="15" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="H43" s="16" t="s">
         <v>10</v>
@@ -2703,24 +2704,24 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="38" t="s">
-        <v>85</v>
-      </c>
-      <c r="B44" s="38" t="s">
-        <v>121</v>
-      </c>
-      <c r="C44" s="43" t="s">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A44" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="B44" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="C44" s="16" t="s">
         <v>127</v>
       </c>
-      <c r="D44" s="44">
-        <v>0.06</v>
+      <c r="D44" s="2">
+        <v>3.35</v>
       </c>
       <c r="F44" s="14" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="G44" s="15" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="H44" s="16" t="s">
         <v>10</v>
@@ -2729,162 +2730,162 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A45" s="34"/>
-      <c r="B45" s="34"/>
-      <c r="C45" s="34"/>
-      <c r="D45" s="34"/>
+    <row r="45" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="38" t="s">
+        <v>85</v>
+      </c>
+      <c r="B45" s="38" t="s">
+        <v>121</v>
+      </c>
+      <c r="C45" s="43" t="s">
+        <v>127</v>
+      </c>
+      <c r="D45" s="44">
+        <v>0.06</v>
+      </c>
       <c r="F45" s="14" t="s">
+        <v>241</v>
+      </c>
+      <c r="G45" s="15" t="s">
+        <v>242</v>
+      </c>
+      <c r="H45" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I45" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="34"/>
+      <c r="B46" s="34"/>
+      <c r="C46" s="34"/>
+      <c r="D46" s="34"/>
+      <c r="F46" s="17" t="s">
         <v>243</v>
       </c>
-      <c r="G45" s="15" t="s">
+      <c r="G46" s="18" t="s">
         <v>244</v>
       </c>
-      <c r="H45" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="I45" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="36" t="s">
+      <c r="H46" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="I46" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="36" t="s">
         <v>56</v>
       </c>
-      <c r="B46" s="37"/>
-      <c r="C46" s="37"/>
-      <c r="D46" s="37"/>
-      <c r="F46" s="17" t="s">
-        <v>245</v>
-      </c>
-      <c r="G46" s="18" t="s">
-        <v>246</v>
-      </c>
-      <c r="H46" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="I46" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="9" t="s">
+      <c r="B47" s="37"/>
+      <c r="C47" s="37"/>
+      <c r="D47" s="37"/>
+    </row>
+    <row r="48" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="B47" s="10" t="s">
+      <c r="B48" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C47" s="10" t="s">
+      <c r="C48" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="D47" s="10" t="s">
+      <c r="D48" s="10" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A48" s="11" t="s">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="B48" s="12" t="s">
+      <c r="B49" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="C48" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="D48" s="1">
+      <c r="C49" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D49" s="1">
         <v>1.65</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="B49" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="C49" s="16" t="s">
-        <v>128</v>
-      </c>
-      <c r="D49" s="2">
-        <v>780</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B50" s="15" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C50" s="16" t="s">
         <v>128</v>
       </c>
       <c r="D50" s="2">
-        <v>57</v>
+        <v>780</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="14" t="s">
-        <v>217</v>
+        <v>61</v>
       </c>
       <c r="B51" s="15" t="s">
-        <v>218</v>
+        <v>62</v>
       </c>
       <c r="C51" s="16" t="s">
         <v>128</v>
       </c>
       <c r="D51" s="2">
-        <v>1147</v>
+        <v>57</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="14" t="s">
-        <v>63</v>
+        <v>215</v>
       </c>
       <c r="B52" s="15" t="s">
-        <v>64</v>
+        <v>216</v>
       </c>
       <c r="C52" s="16" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D52" s="2">
-        <v>1027</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="14" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B53" s="15" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C53" s="16" t="s">
-        <v>67</v>
+        <v>129</v>
       </c>
       <c r="D53" s="2">
-        <v>0.4</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="14" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B54" s="15" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C54" s="16" t="s">
-        <v>10</v>
+        <v>67</v>
       </c>
       <c r="D54" s="2">
-        <v>1</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="60.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B55" s="15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C55" s="16" t="s">
         <v>10</v>
@@ -2895,74 +2896,88 @@
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="B56" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="C56" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D56" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="B56" s="15" t="s">
+      <c r="B57" s="15" t="s">
         <v>73</v>
       </c>
-      <c r="C56" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D56" s="2">
+      <c r="C57" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D57" s="2">
         <v>17</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="39" t="s">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" s="39" t="s">
         <v>74</v>
       </c>
-      <c r="B57" s="40" t="s">
+      <c r="B58" s="40" t="s">
         <v>75</v>
       </c>
-      <c r="C57" s="41" t="s">
-        <v>10</v>
-      </c>
-      <c r="D57" s="42">
+      <c r="C58" s="41" t="s">
+        <v>10</v>
+      </c>
+      <c r="D58" s="42">
         <v>17</v>
       </c>
     </row>
-    <row r="58" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="18" t="s">
+    <row r="59" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="B58" s="48" t="s">
+      <c r="B59" s="48" t="s">
         <v>87</v>
       </c>
-      <c r="C58" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D58" s="4">
+      <c r="C59" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D59" s="4">
         <v>2</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="37"/>
-      <c r="B59" s="37"/>
-      <c r="C59" s="37"/>
-      <c r="D59" s="37"/>
-    </row>
-    <row r="65" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C65" s="64"/>
-    </row>
-    <row r="66" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C66" s="63"/>
-    </row>
-    <row r="72" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B72" s="47"/>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" s="37"/>
+      <c r="B60" s="37"/>
+      <c r="C60" s="37"/>
+      <c r="D60" s="37"/>
+    </row>
+    <row r="66" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C66" s="64"/>
+    </row>
+    <row r="67" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C67" s="63"/>
+    </row>
+    <row r="73" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B73" s="47"/>
     </row>
   </sheetData>
   <sheetProtection formatColumns="0" selectLockedCells="1"/>
   <protectedRanges>
-    <protectedRange sqref="I3:I6 I8 I12:I16 I25:I28 D16:D19 I32 D26 I19:I20 D9:D12 D14 D3:D7" name="Range1_1"/>
-    <protectedRange sqref="D8 D15" name="Range1_1_1"/>
-    <protectedRange sqref="D48:D58" name="Range1_1_4"/>
-    <protectedRange sqref="D13 D31" name="Range1_1_2"/>
-    <protectedRange sqref="D28" name="Range1_1_6_1"/>
-    <protectedRange sqref="D25" name="Range1_1_6"/>
-    <protectedRange sqref="D27" name="Range1_1_5"/>
-    <protectedRange sqref="D29" name="Range1_1_5_1_1"/>
-    <protectedRange sqref="D30" name="Range1_1_8_1_1"/>
-    <protectedRange sqref="D42 D35:D40" name="Range1_1_3_1"/>
+    <protectedRange sqref="I3:I6 I8 I12:I16 I25:I28 D17:D20 I32 D27 I19:I20 D9:D12 D14 D3:D7 D15" name="Range1_1"/>
+    <protectedRange sqref="D8 D16" name="Range1_1_1"/>
+    <protectedRange sqref="D49:D59" name="Range1_1_4"/>
+    <protectedRange sqref="D13 D32" name="Range1_1_2"/>
+    <protectedRange sqref="D29" name="Range1_1_6_1"/>
+    <protectedRange sqref="D26" name="Range1_1_6"/>
+    <protectedRange sqref="D28" name="Range1_1_5"/>
+    <protectedRange sqref="D30" name="Range1_1_5_1_1"/>
+    <protectedRange sqref="D31" name="Range1_1_8_1_1"/>
+    <protectedRange sqref="D43 D36:D41" name="Range1_1_3_1"/>
   </protectedRanges>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -2979,22 +2994,22 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updating input file template
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\HC_QAQC_NACCS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Golden_Meadow\Work\6. StormSim Execution\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7938099F-FCCF-4213-9243-72DC3A6868D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{086DBCD6-4B2C-4C51-9968-2CD528D36EF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
+    <workbookView xWindow="180" yWindow="0" windowWidth="28800" windowHeight="14805" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
   <sheets>
     <sheet name="James_Island_Midbay" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="251">
   <si>
     <t>StormSim Project General Inputs</t>
   </si>
@@ -358,9 +358,6 @@
     <t>tide_file</t>
   </si>
   <si>
-    <t>NAVD</t>
-  </si>
-  <si>
     <t>m</t>
   </si>
   <si>
@@ -673,9 +670,6 @@
     <t>use_waves_swl</t>
   </si>
   <si>
-    <t>James_Island</t>
-  </si>
-  <si>
     <t>SP_2243</t>
   </si>
   <si>
@@ -736,15 +730,6 @@
     <t>ref_case_name</t>
   </si>
   <si>
-    <t>Levee_Case_5</t>
-  </si>
-  <si>
-    <t>Midbay_CHS_Data.zip</t>
-  </si>
-  <si>
-    <t>MCSim_Inputs\NACCS</t>
-  </si>
-  <si>
     <t>outfolder</t>
   </si>
   <si>
@@ -782,6 +767,30 @@
   </si>
   <si>
     <t>Apply Bias Correction To Extratropical Stomrs  (0 - Off / 1 - On)</t>
+  </si>
+  <si>
+    <t>CHS_6021_408_base.zip</t>
+  </si>
+  <si>
+    <t>Probability_Masses\CHS-NA</t>
+  </si>
+  <si>
+    <t>Bias_and_Uncertainty\CHS-NA_Comb_BiasUncertainty_perVG_rta.mat</t>
+  </si>
+  <si>
+    <t>TC</t>
+  </si>
+  <si>
+    <t>MSL</t>
+  </si>
+  <si>
+    <t>CHS-LA_Validation</t>
+  </si>
+  <si>
+    <t>Storm_Responses</t>
+  </si>
+  <si>
+    <t>test_001.csv</t>
   </si>
 </sst>
 </file>
@@ -1733,7 +1742,7 @@
         <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>211</v>
+        <v>248</v>
       </c>
       <c r="F3" s="49" t="s">
         <v>95</v>
@@ -1742,7 +1751,7 @@
         <v>88</v>
       </c>
       <c r="H3" s="13" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="I3" s="13">
         <v>0.33979999999999999</v>
@@ -1759,7 +1768,7 @@
         <v>10</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="F4" s="49" t="s">
         <v>96</v>
@@ -1776,16 +1785,16 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="B5" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="B5" s="15" t="s">
-        <v>114</v>
-      </c>
       <c r="C5" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>232</v>
+        <v>249</v>
       </c>
       <c r="F5" s="49" t="s">
         <v>98</v>
@@ -1794,7 +1803,7 @@
         <v>90</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="I5" s="13">
         <v>0.3</v>
@@ -1802,16 +1811,16 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="C6" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="F6" s="49" t="s">
         <v>97</v>
@@ -1837,7 +1846,7 @@
         <v>10</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>106</v>
+        <v>247</v>
       </c>
       <c r="F7" s="14" t="s">
         <v>99</v>
@@ -1846,7 +1855,7 @@
         <v>93</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="I7" s="2">
         <v>0</v>
@@ -1863,7 +1872,7 @@
         <v>10</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F8" s="17" t="s">
         <v>94</v>
@@ -1872,7 +1881,7 @@
         <v>92</v>
       </c>
       <c r="H8" s="19" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="I8" s="3">
         <v>0</v>
@@ -1880,10 +1889,10 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C9" s="16" t="s">
         <v>10</v>
@@ -1927,7 +1936,7 @@
         <v>10</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>76</v>
+        <v>246</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>3</v>
@@ -1950,7 +1959,7 @@
         <v>25</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D12" s="2">
         <v>0</v>
@@ -1962,7 +1971,7 @@
         <v>45</v>
       </c>
       <c r="H12" s="16" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="I12" s="2">
         <v>0.15</v>
@@ -1970,16 +1979,16 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="C13" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D13" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F13" s="30" t="s">
         <v>103</v>
@@ -1988,7 +1997,7 @@
         <v>48</v>
       </c>
       <c r="H13" s="31" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="I13" s="2">
         <v>0.43</v>
@@ -1999,7 +2008,7 @@
         <v>101</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C14" s="16" t="s">
         <v>10</v>
@@ -2014,7 +2023,7 @@
         <v>46</v>
       </c>
       <c r="H14" s="16" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I14" s="2">
         <v>0.78</v>
@@ -2022,10 +2031,10 @@
     </row>
     <row r="15" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="14" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="C15" s="16" t="s">
         <v>10</v>
@@ -2040,7 +2049,7 @@
         <v>47</v>
       </c>
       <c r="H15" s="19" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="I15" s="3">
         <v>0.13</v>
@@ -2048,10 +2057,10 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>10</v>
@@ -2069,13 +2078,13 @@
         <v>77</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="C17" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D17" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F17" s="7" t="s">
         <v>1</v>
@@ -2090,10 +2099,10 @@
     </row>
     <row r="18" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="14" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C18" s="16" t="s">
         <v>10</v>
@@ -2116,10 +2125,10 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C19" s="16" t="s">
         <v>10</v>
@@ -2142,10 +2151,10 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C20" s="16" t="s">
         <v>10</v>
@@ -2168,10 +2177,10 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C21" s="16" t="s">
         <v>10</v>
@@ -2180,10 +2189,10 @@
         <v>1</v>
       </c>
       <c r="F21" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="G21" s="15" t="s">
         <v>117</v>
-      </c>
-      <c r="G21" s="15" t="s">
-        <v>118</v>
       </c>
       <c r="H21" s="16" t="s">
         <v>10</v>
@@ -2194,16 +2203,16 @@
     </row>
     <row r="22" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="17" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="B22" s="18" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C22" s="19" t="s">
         <v>10</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="F22" s="8"/>
       <c r="G22" s="8"/>
@@ -2270,10 +2279,10 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="B26" s="12" t="s">
         <v>185</v>
-      </c>
-      <c r="B26" s="12" t="s">
-        <v>186</v>
       </c>
       <c r="C26" s="28" t="s">
         <v>10</v>
@@ -2322,13 +2331,13 @@
     </row>
     <row r="28" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="B28" s="12" t="s">
         <v>108</v>
       </c>
-      <c r="B28" s="12" t="s">
-        <v>109</v>
-      </c>
       <c r="C28" s="28" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D28" s="1">
         <v>3.43</v>
@@ -2340,7 +2349,7 @@
         <v>37</v>
       </c>
       <c r="H28" s="19" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="I28" s="3">
         <v>1</v>
@@ -2351,12 +2360,14 @@
         <v>104</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C29" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="D29" s="2"/>
+      <c r="D29" s="2" t="s">
+        <v>245</v>
+      </c>
       <c r="F29" s="21"/>
       <c r="G29" s="21"/>
       <c r="H29" s="21"/>
@@ -2364,16 +2375,16 @@
     </row>
     <row r="30" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="11" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C30" s="28" t="s">
         <v>10</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>234</v>
+        <v>244</v>
       </c>
       <c r="F30" s="26" t="s">
         <v>41</v>
@@ -2387,13 +2398,13 @@
         <v>42</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C31" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>233</v>
+        <v>243</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>3</v>
@@ -2413,12 +2424,14 @@
         <v>105</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C32" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D32" s="2"/>
+      <c r="D32" s="2" t="s">
+        <v>250</v>
+      </c>
       <c r="F32" s="29" t="s">
         <v>43</v>
       </c>
@@ -2438,10 +2451,10 @@
       <c r="C33" s="25"/>
       <c r="D33" s="25"/>
       <c r="F33" s="14" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G33" s="15" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H33" s="16" t="s">
         <v>10</v>
@@ -2458,10 +2471,10 @@
       <c r="C34" s="35"/>
       <c r="D34" s="35"/>
       <c r="F34" s="14" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G34" s="15" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="H34" s="16" t="s">
         <v>10</v>
@@ -2484,10 +2497,10 @@
         <v>6</v>
       </c>
       <c r="F35" s="14" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="G35" s="15" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="H35" s="16" t="s">
         <v>10</v>
@@ -2501,19 +2514,19 @@
         <v>51</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D36" s="1">
         <v>3.41</v>
       </c>
       <c r="F36" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G36" s="15" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="H36" s="16" t="s">
         <v>10</v>
@@ -2530,16 +2543,16 @@
         <v>78</v>
       </c>
       <c r="C37" s="16" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D37" s="2">
         <v>7.01</v>
       </c>
       <c r="F37" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G37" s="15" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="H37" s="16" t="s">
         <v>10</v>
@@ -2553,19 +2566,19 @@
         <v>53</v>
       </c>
       <c r="B38" s="15" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C38" s="16" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D38" s="2">
         <v>-2.42</v>
       </c>
       <c r="F38" s="14" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="G38" s="15" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="H38" s="16" t="s">
         <v>10</v>
@@ -2576,22 +2589,22 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B39" s="15" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C39" s="16" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D39" s="2">
         <v>-0.95799999999999996</v>
       </c>
       <c r="F39" s="14" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="G39" s="15" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H39" s="16" t="s">
         <v>10</v>
@@ -2605,7 +2618,7 @@
         <v>54</v>
       </c>
       <c r="B40" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C40" s="16" t="s">
         <v>10</v>
@@ -2614,10 +2627,10 @@
         <v>3</v>
       </c>
       <c r="F40" s="14" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="G40" s="15" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="H40" s="16" t="s">
         <v>10</v>
@@ -2631,7 +2644,7 @@
         <v>55</v>
       </c>
       <c r="B41" s="15" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C41" s="16" t="s">
         <v>10</v>
@@ -2640,10 +2653,10 @@
         <v>1.5</v>
       </c>
       <c r="F41" s="14" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G41" s="15" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="H41" s="16" t="s">
         <v>10</v>
@@ -2660,16 +2673,16 @@
         <v>83</v>
       </c>
       <c r="C42" s="45" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D42" s="46">
         <v>0</v>
       </c>
       <c r="F42" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G42" s="15" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="H42" s="16" t="s">
         <v>10</v>
@@ -2680,10 +2693,10 @@
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B43" s="15" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C43" s="16" t="s">
         <v>10</v>
@@ -2692,10 +2705,10 @@
         <v>0.4</v>
       </c>
       <c r="F43" s="14" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="G43" s="15" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="H43" s="16" t="s">
         <v>10</v>
@@ -2712,22 +2725,22 @@
         <v>86</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D44" s="2">
         <v>3.35</v>
       </c>
       <c r="F44" s="14" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="G44" s="15" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="H44" s="16" t="s">
         <v>10</v>
       </c>
       <c r="I44" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2735,19 +2748,19 @@
         <v>85</v>
       </c>
       <c r="B45" s="38" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C45" s="43" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D45" s="44">
         <v>0.06</v>
       </c>
       <c r="F45" s="14" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="G45" s="15" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="H45" s="16" t="s">
         <v>10</v>
@@ -2762,10 +2775,10 @@
       <c r="C46" s="34"/>
       <c r="D46" s="34"/>
       <c r="F46" s="17" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="G46" s="18" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="H46" s="19" t="s">
         <v>10</v>
@@ -2818,7 +2831,7 @@
         <v>60</v>
       </c>
       <c r="C50" s="16" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D50" s="2">
         <v>780</v>
@@ -2832,7 +2845,7 @@
         <v>62</v>
       </c>
       <c r="C51" s="16" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D51" s="2">
         <v>57</v>
@@ -2840,13 +2853,13 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="14" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B52" s="15" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="C52" s="16" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D52" s="2">
         <v>1147</v>
@@ -2860,7 +2873,7 @@
         <v>64</v>
       </c>
       <c r="C53" s="16" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D53" s="2">
         <v>1027</v>
@@ -2968,7 +2981,7 @@
   </sheetData>
   <sheetProtection formatColumns="0" selectLockedCells="1"/>
   <protectedRanges>
-    <protectedRange sqref="I3:I6 I8 I12:I16 I25:I28 D17:D20 I32 D27 I19:I20 D9:D12 D14 D3:D7 D15" name="Range1_1"/>
+    <protectedRange sqref="I3:I6 I8 I12:I16 I25:I28 D17:D20 I32 D27 I19:I20 D9:D12 D3:D7 D14:D15" name="Range1_1"/>
     <protectedRange sqref="D8 D16" name="Range1_1_1"/>
     <protectedRange sqref="D49:D59" name="Range1_1_4"/>
     <protectedRange sqref="D13 D32" name="Range1_1_2"/>
@@ -2994,22 +3007,22 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -3032,16 +3045,16 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E1" t="s">
         <v>76</v>
@@ -3049,62 +3062,62 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="50" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B4" t="s">
+        <v>156</v>
+      </c>
+      <c r="C4" t="s">
         <v>157</v>
-      </c>
-      <c r="C4" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="50" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="50" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="50" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B7" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C7" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="50" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B8" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C8" t="s">
         <v>76</v>
@@ -3112,60 +3125,60 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="50" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B9" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C9" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C10" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C11" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
+        <v>158</v>
+      </c>
+      <c r="C12" t="s">
         <v>159</v>
-      </c>
-      <c r="C12" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
+        <v>160</v>
+      </c>
+      <c r="C13" t="s">
         <v>161</v>
-      </c>
-      <c r="C13" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="16" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="54" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B16" s="54" t="s">
         <v>4</v>
       </c>
       <c r="C16" s="54" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D16" s="58" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -3173,7 +3186,7 @@
         <v>0</v>
       </c>
       <c r="B17" s="55" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C17" s="59">
         <v>0.66720000000000002</v>
@@ -3189,7 +3202,7 @@
         <v>1</v>
       </c>
       <c r="B18" s="56" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C18" s="60">
         <v>128.0189</v>
@@ -3199,7 +3212,7 @@
         <v>2.1336483333333334</v>
       </c>
       <c r="E18" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -3208,7 +3221,7 @@
         <v>2</v>
       </c>
       <c r="B19" s="56" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C19" s="60">
         <v>1.8109999999999999</v>
@@ -3224,7 +3237,7 @@
         <v>3</v>
       </c>
       <c r="B20" s="56" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C20" s="60">
         <v>0.56489999999999996</v>
@@ -3240,7 +3253,7 @@
         <v>4</v>
       </c>
       <c r="B21" s="56" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C21" s="60">
         <v>1.2150000000000001</v>
@@ -3256,7 +3269,7 @@
         <v>5</v>
       </c>
       <c r="B22" s="56" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C22" s="60">
         <v>15.2134</v>
@@ -3272,7 +3285,7 @@
         <v>6</v>
       </c>
       <c r="B23" s="57" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C23" s="61">
         <v>648.27599999999995</v>
@@ -3290,12 +3303,12 @@
         <v>0.3858785714285714</v>
       </c>
       <c r="G23" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="69" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B24" s="70"/>
       <c r="C24" s="52">
@@ -3311,33 +3324,33 @@
         <v>23.152714285714286</v>
       </c>
       <c r="G24" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E28" s="8"/>
       <c r="F28" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E29" s="51"/>
       <c r="F29" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B31" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C31" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D31" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E31" t="s">
         <v>76</v>
@@ -3345,62 +3358,62 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B33" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="50" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B34" t="s">
+        <v>156</v>
+      </c>
+      <c r="C34" t="s">
         <v>157</v>
-      </c>
-      <c r="C34" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="50" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B35" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C35" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="50" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C36" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="50" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B37" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C37" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="50" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B38" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C38" t="s">
         <v>76</v>
@@ -3408,57 +3421,57 @@
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C39" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C40" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C41" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B42" t="s">
+        <v>158</v>
+      </c>
+      <c r="C42" t="s">
         <v>159</v>
-      </c>
-      <c r="C42" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B43" t="s">
+        <v>160</v>
+      </c>
+      <c r="C43" t="s">
         <v>161</v>
-      </c>
-      <c r="C43" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="46" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="54" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B46" s="54" t="s">
         <v>4</v>
       </c>
       <c r="C46" s="54" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D46" s="58" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
@@ -3466,7 +3479,7 @@
         <v>0</v>
       </c>
       <c r="B47" s="55" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C47" s="59">
         <v>0.66720000000000002</v>
@@ -3476,7 +3489,7 @@
         <v>1.112E-2</v>
       </c>
       <c r="F47" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
@@ -3485,7 +3498,7 @@
         <v>1</v>
       </c>
       <c r="B48" s="56" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C48" s="60">
         <v>128.0189</v>
@@ -3495,13 +3508,13 @@
         <v>2.1336483333333334</v>
       </c>
       <c r="E48" t="s">
+        <v>145</v>
+      </c>
+      <c r="F48" t="s">
+        <v>143</v>
+      </c>
+      <c r="G48" t="s">
         <v>146</v>
-      </c>
-      <c r="F48" t="s">
-        <v>144</v>
-      </c>
-      <c r="G48" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
@@ -3510,7 +3523,7 @@
         <v>2</v>
       </c>
       <c r="B49" s="56" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C49" s="60">
         <v>77.920665999999997</v>
@@ -3533,7 +3546,7 @@
         <v>3</v>
       </c>
       <c r="B50" s="56" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C50" s="60">
         <v>0.56489999999999996</v>
@@ -3549,7 +3562,7 @@
         <v>4</v>
       </c>
       <c r="B51" s="56" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C51" s="60">
         <v>2.6115067000000001</v>
@@ -3565,7 +3578,7 @@
         <v>5</v>
       </c>
       <c r="B52" s="56" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C52" s="60">
         <v>32.553324799999999</v>
@@ -3581,7 +3594,7 @@
         <v>6</v>
       </c>
       <c r="B53" s="57" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C53" s="61">
         <v>197.9727273</v>
@@ -3593,7 +3606,7 @@
     </row>
     <row r="54" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="69" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B54" s="70"/>
       <c r="C54" s="52">

</xml_diff>

<commit_message>
Added flag to control creation of plots (create_plots).
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20408"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Golden_Meadow\Work\6. StormSim Execution\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\StormSim_FEMA_Batch_Processing\StormSim-Library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{086DBCD6-4B2C-4C51-9968-2CD528D36EF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A67D2863-974B-4E4F-B975-BC5AF8DE4D16}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="180" yWindow="0" windowWidth="28800" windowHeight="14805" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
@@ -22,23 +22,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="404" uniqueCount="253">
   <si>
     <t>StormSim Project General Inputs</t>
   </si>
@@ -791,6 +780,12 @@
   </si>
   <si>
     <t>test_001.csv</t>
+  </si>
+  <si>
+    <t>create_plots</t>
+  </si>
+  <si>
+    <t>Generate output visualizations (0 - Off, 1 - On)</t>
   </si>
 </sst>
 </file>
@@ -1382,9 +1377,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1422,7 +1417,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1528,7 +1523,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1670,7 +1665,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1678,7 +1673,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51D29750-2AFD-4BF7-A911-1DC4ADC0FD7A}">
-  <dimension ref="A1:I73"/>
+  <dimension ref="A1:I74"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.5703125" customWidth="1"/>
@@ -2177,16 +2172,16 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
-        <v>228</v>
+        <v>251</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>225</v>
+        <v>252</v>
       </c>
       <c r="C21" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D21" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F21" s="14" t="s">
         <v>116</v>
@@ -2201,18 +2196,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="17" t="s">
-        <v>229</v>
-      </c>
-      <c r="B22" s="18" t="s">
-        <v>226</v>
-      </c>
-      <c r="C22" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>227</v>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" s="14" t="s">
+        <v>228</v>
+      </c>
+      <c r="B22" s="15" t="s">
+        <v>225</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D22" s="2">
+        <v>1</v>
       </c>
       <c r="F22" s="8"/>
       <c r="G22" s="8"/>
@@ -2220,10 +2215,18 @@
       <c r="I22" s="8"/>
     </row>
     <row r="23" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="6"/>
-      <c r="B23" s="22"/>
-      <c r="C23" s="23"/>
-      <c r="D23" s="23"/>
+      <c r="A23" s="17" t="s">
+        <v>229</v>
+      </c>
+      <c r="B23" s="18" t="s">
+        <v>226</v>
+      </c>
+      <c r="C23" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>227</v>
+      </c>
       <c r="F23" s="20" t="s">
         <v>26</v>
       </c>
@@ -2232,12 +2235,10 @@
       <c r="I23" s="21"/>
     </row>
     <row r="24" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="24" t="s">
-        <v>35</v>
-      </c>
-      <c r="B24" s="25"/>
-      <c r="C24" s="25"/>
-      <c r="D24" s="25"/>
+      <c r="A24" s="6"/>
+      <c r="B24" s="22"/>
+      <c r="C24" s="23"/>
+      <c r="D24" s="23"/>
       <c r="F24" s="9" t="s">
         <v>3</v>
       </c>
@@ -2252,18 +2253,12 @@
       </c>
     </row>
     <row r="25" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B25" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="C25" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="D25" s="10" t="s">
-        <v>6</v>
-      </c>
+      <c r="A25" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="B25" s="25"/>
+      <c r="C25" s="25"/>
+      <c r="D25" s="25"/>
       <c r="F25" s="11" t="s">
         <v>27</v>
       </c>
@@ -2277,18 +2272,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="B26" s="12" t="s">
-        <v>185</v>
-      </c>
-      <c r="C26" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="D26" s="1">
-        <v>0</v>
+    <row r="26" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B26" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C26" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D26" s="10" t="s">
+        <v>6</v>
       </c>
       <c r="F26" s="14" t="s">
         <v>31</v>
@@ -2305,16 +2300,16 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="11" t="s">
-        <v>38</v>
+        <v>184</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>39</v>
+        <v>185</v>
       </c>
       <c r="C27" s="28" t="s">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="D27" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F27" s="14" t="s">
         <v>33</v>
@@ -2331,16 +2326,16 @@
     </row>
     <row r="28" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
-        <v>107</v>
+        <v>38</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>108</v>
+        <v>39</v>
       </c>
       <c r="C28" s="28" t="s">
-        <v>106</v>
+        <v>40</v>
       </c>
       <c r="D28" s="1">
-        <v>3.43</v>
+        <v>1</v>
       </c>
       <c r="F28" s="17" t="s">
         <v>36</v>
@@ -2357,16 +2352,16 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>222</v>
+        <v>108</v>
       </c>
       <c r="C29" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>245</v>
+        <v>106</v>
+      </c>
+      <c r="D29" s="1">
+        <v>3.43</v>
       </c>
       <c r="F29" s="21"/>
       <c r="G29" s="21"/>
@@ -2375,16 +2370,16 @@
     </row>
     <row r="30" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="11" t="s">
-        <v>183</v>
+        <v>104</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C30" s="28" t="s">
         <v>10</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="F30" s="26" t="s">
         <v>41</v>
@@ -2394,17 +2389,17 @@
       <c r="I30" s="27"/>
     </row>
     <row r="31" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="14" t="s">
-        <v>42</v>
-      </c>
-      <c r="B31" s="15" t="s">
-        <v>186</v>
-      </c>
-      <c r="C31" s="16" t="s">
+      <c r="A31" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="B31" s="12" t="s">
+        <v>224</v>
+      </c>
+      <c r="C31" s="28" t="s">
         <v>10</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>3</v>
@@ -2421,16 +2416,16 @@
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="14" t="s">
-        <v>105</v>
+        <v>42</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>223</v>
+        <v>186</v>
       </c>
       <c r="C32" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="F32" s="29" t="s">
         <v>43</v>
@@ -2446,10 +2441,18 @@
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="25"/>
-      <c r="B33" s="25"/>
-      <c r="C33" s="25"/>
-      <c r="D33" s="25"/>
+      <c r="A33" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="B33" s="15" t="s">
+        <v>223</v>
+      </c>
+      <c r="C33" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>250</v>
+      </c>
       <c r="F33" s="14" t="s">
         <v>111</v>
       </c>
@@ -2463,13 +2466,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="34" t="s">
-        <v>50</v>
-      </c>
-      <c r="B34" s="35"/>
-      <c r="C34" s="35"/>
-      <c r="D34" s="35"/>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" s="25"/>
+      <c r="B34" s="25"/>
+      <c r="C34" s="25"/>
+      <c r="D34" s="25"/>
       <c r="F34" s="14" t="s">
         <v>193</v>
       </c>
@@ -2484,18 +2485,12 @@
       </c>
     </row>
     <row r="35" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B35" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C35" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="D35" s="10" t="s">
-        <v>6</v>
-      </c>
+      <c r="A35" s="34" t="s">
+        <v>50</v>
+      </c>
+      <c r="B35" s="35"/>
+      <c r="C35" s="35"/>
+      <c r="D35" s="35"/>
       <c r="F35" s="14" t="s">
         <v>194</v>
       </c>
@@ -2509,18 +2504,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="B36" s="12" t="s">
-        <v>121</v>
-      </c>
-      <c r="C36" s="13" t="s">
-        <v>126</v>
-      </c>
-      <c r="D36" s="1">
-        <v>3.41</v>
+    <row r="36" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B36" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C36" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D36" s="10" t="s">
+        <v>6</v>
       </c>
       <c r="F36" s="14" t="s">
         <v>195</v>
@@ -2536,17 +2531,17 @@
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A37" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="B37" s="15" t="s">
-        <v>78</v>
-      </c>
-      <c r="C37" s="16" t="s">
+      <c r="A37" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="B37" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="C37" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="D37" s="2">
-        <v>7.01</v>
+      <c r="D37" s="1">
+        <v>3.41</v>
       </c>
       <c r="F37" s="14" t="s">
         <v>196</v>
@@ -2563,16 +2558,16 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B38" s="15" t="s">
-        <v>122</v>
+        <v>78</v>
       </c>
       <c r="C38" s="16" t="s">
         <v>126</v>
       </c>
       <c r="D38" s="2">
-        <v>-2.42</v>
+        <v>7.01</v>
       </c>
       <c r="F38" s="14" t="s">
         <v>197</v>
@@ -2589,16 +2584,16 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
-        <v>173</v>
+        <v>53</v>
       </c>
       <c r="B39" s="15" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C39" s="16" t="s">
         <v>126</v>
       </c>
       <c r="D39" s="2">
-        <v>-0.95799999999999996</v>
+        <v>-2.42</v>
       </c>
       <c r="F39" s="14" t="s">
         <v>211</v>
@@ -2615,16 +2610,16 @@
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="s">
-        <v>54</v>
+        <v>173</v>
       </c>
       <c r="B40" s="15" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C40" s="16" t="s">
-        <v>10</v>
+        <v>126</v>
       </c>
       <c r="D40" s="2">
-        <v>3</v>
+        <v>-0.95799999999999996</v>
       </c>
       <c r="F40" s="14" t="s">
         <v>198</v>
@@ -2641,16 +2636,16 @@
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B41" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C41" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D41" s="2">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="F41" s="14" t="s">
         <v>199</v>
@@ -2666,17 +2661,17 @@
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A42" s="39" t="s">
-        <v>82</v>
-      </c>
-      <c r="B42" s="39" t="s">
-        <v>83</v>
-      </c>
-      <c r="C42" s="45" t="s">
-        <v>131</v>
-      </c>
-      <c r="D42" s="46">
-        <v>0</v>
+      <c r="A42" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="B42" s="15" t="s">
+        <v>125</v>
+      </c>
+      <c r="C42" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D42" s="2">
+        <v>1.5</v>
       </c>
       <c r="F42" s="14" t="s">
         <v>200</v>
@@ -2692,17 +2687,17 @@
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A43" s="14" t="s">
-        <v>133</v>
-      </c>
-      <c r="B43" s="15" t="s">
-        <v>132</v>
-      </c>
-      <c r="C43" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D43" s="2">
-        <v>0.4</v>
+      <c r="A43" s="39" t="s">
+        <v>82</v>
+      </c>
+      <c r="B43" s="39" t="s">
+        <v>83</v>
+      </c>
+      <c r="C43" s="45" t="s">
+        <v>131</v>
+      </c>
+      <c r="D43" s="46">
+        <v>0</v>
       </c>
       <c r="F43" s="14" t="s">
         <v>232</v>
@@ -2719,16 +2714,16 @@
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
-        <v>84</v>
-      </c>
-      <c r="B44" s="14" t="s">
-        <v>86</v>
+        <v>133</v>
+      </c>
+      <c r="B44" s="15" t="s">
+        <v>132</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>126</v>
+        <v>10</v>
       </c>
       <c r="D44" s="2">
-        <v>3.35</v>
+        <v>0.4</v>
       </c>
       <c r="F44" s="14" t="s">
         <v>234</v>
@@ -2743,18 +2738,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="38" t="s">
-        <v>85</v>
-      </c>
-      <c r="B45" s="38" t="s">
-        <v>120</v>
-      </c>
-      <c r="C45" s="43" t="s">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A45" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="B45" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="C45" s="16" t="s">
         <v>126</v>
       </c>
-      <c r="D45" s="44">
-        <v>0.06</v>
+      <c r="D45" s="2">
+        <v>3.35</v>
       </c>
       <c r="F45" s="14" t="s">
         <v>236</v>
@@ -2770,10 +2765,18 @@
       </c>
     </row>
     <row r="46" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="34"/>
-      <c r="B46" s="34"/>
-      <c r="C46" s="34"/>
-      <c r="D46" s="34"/>
+      <c r="A46" s="38" t="s">
+        <v>85</v>
+      </c>
+      <c r="B46" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="C46" s="43" t="s">
+        <v>126</v>
+      </c>
+      <c r="D46" s="44">
+        <v>0.06</v>
+      </c>
       <c r="F46" s="17" t="s">
         <v>238</v>
       </c>
@@ -2787,132 +2790,124 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="36" t="s">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A47" s="34"/>
+      <c r="B47" s="34"/>
+      <c r="C47" s="34"/>
+      <c r="D47" s="34"/>
+    </row>
+    <row r="48" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="36" t="s">
         <v>56</v>
       </c>
-      <c r="B47" s="37"/>
-      <c r="C47" s="37"/>
-      <c r="D47" s="37"/>
-    </row>
-    <row r="48" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="9" t="s">
+      <c r="B48" s="37"/>
+      <c r="C48" s="37"/>
+      <c r="D48" s="37"/>
+    </row>
+    <row r="49" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="B48" s="10" t="s">
+      <c r="B49" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C48" s="10" t="s">
+      <c r="C49" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="D48" s="10" t="s">
+      <c r="D49" s="10" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="11" t="s">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="B49" s="12" t="s">
+      <c r="B50" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="C49" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="D49" s="1">
+      <c r="C50" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D50" s="1">
         <v>1.65</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="B50" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="C50" s="16" t="s">
-        <v>127</v>
-      </c>
-      <c r="D50" s="2">
-        <v>780</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="14" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B51" s="15" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C51" s="16" t="s">
         <v>127</v>
       </c>
       <c r="D51" s="2">
-        <v>57</v>
+        <v>780</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="14" t="s">
-        <v>213</v>
+        <v>61</v>
       </c>
       <c r="B52" s="15" t="s">
-        <v>214</v>
+        <v>62</v>
       </c>
       <c r="C52" s="16" t="s">
         <v>127</v>
       </c>
       <c r="D52" s="2">
-        <v>1147</v>
+        <v>57</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="14" t="s">
-        <v>63</v>
+        <v>213</v>
       </c>
       <c r="B53" s="15" t="s">
-        <v>64</v>
+        <v>214</v>
       </c>
       <c r="C53" s="16" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D53" s="2">
-        <v>1027</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="14" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B54" s="15" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C54" s="16" t="s">
-        <v>67</v>
+        <v>128</v>
       </c>
       <c r="D54" s="2">
-        <v>0.4</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="60.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B55" s="15" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C55" s="16" t="s">
-        <v>10</v>
+        <v>67</v>
       </c>
       <c r="D55" s="2">
-        <v>1</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="14" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B56" s="15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C56" s="16" t="s">
         <v>10</v>
@@ -2923,74 +2918,88 @@
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="B57" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="C57" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D57" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="B57" s="15" t="s">
+      <c r="B58" s="15" t="s">
         <v>73</v>
       </c>
-      <c r="C57" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D57" s="2">
+      <c r="C58" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D58" s="2">
         <v>17</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="39" t="s">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="39" t="s">
         <v>74</v>
       </c>
-      <c r="B58" s="40" t="s">
+      <c r="B59" s="40" t="s">
         <v>75</v>
       </c>
-      <c r="C58" s="41" t="s">
-        <v>10</v>
-      </c>
-      <c r="D58" s="42">
+      <c r="C59" s="41" t="s">
+        <v>10</v>
+      </c>
+      <c r="D59" s="42">
         <v>17</v>
       </c>
     </row>
-    <row r="59" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="18" t="s">
+    <row r="60" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="B59" s="48" t="s">
+      <c r="B60" s="48" t="s">
         <v>87</v>
       </c>
-      <c r="C59" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D59" s="4">
+      <c r="C60" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D60" s="4">
         <v>2</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="37"/>
-      <c r="B60" s="37"/>
-      <c r="C60" s="37"/>
-      <c r="D60" s="37"/>
-    </row>
-    <row r="66" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C66" s="64"/>
-    </row>
-    <row r="67" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C67" s="63"/>
-    </row>
-    <row r="73" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B73" s="47"/>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" s="37"/>
+      <c r="B61" s="37"/>
+      <c r="C61" s="37"/>
+      <c r="D61" s="37"/>
+    </row>
+    <row r="67" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C67" s="64"/>
+    </row>
+    <row r="68" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C68" s="63"/>
+    </row>
+    <row r="74" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B74" s="47"/>
     </row>
   </sheetData>
   <sheetProtection formatColumns="0" selectLockedCells="1"/>
   <protectedRanges>
-    <protectedRange sqref="I3:I6 I8 I12:I16 I25:I28 D17:D20 I32 D27 I19:I20 D9:D12 D3:D7 D14:D15" name="Range1_1"/>
+    <protectedRange sqref="I3:I6 I8 I12:I16 I25:I28 D17:D20 I32 D28 I19:I20 D9:D12 D3:D7 D14:D15" name="Range1_1"/>
     <protectedRange sqref="D8 D16" name="Range1_1_1"/>
-    <protectedRange sqref="D49:D59" name="Range1_1_4"/>
-    <protectedRange sqref="D13 D32" name="Range1_1_2"/>
-    <protectedRange sqref="D29" name="Range1_1_6_1"/>
-    <protectedRange sqref="D26" name="Range1_1_6"/>
-    <protectedRange sqref="D28" name="Range1_1_5"/>
-    <protectedRange sqref="D30" name="Range1_1_5_1_1"/>
-    <protectedRange sqref="D31" name="Range1_1_8_1_1"/>
-    <protectedRange sqref="D43 D36:D41" name="Range1_1_3_1"/>
+    <protectedRange sqref="D50:D60" name="Range1_1_4"/>
+    <protectedRange sqref="D13 D33" name="Range1_1_2"/>
+    <protectedRange sqref="D30" name="Range1_1_6_1"/>
+    <protectedRange sqref="D27" name="Range1_1_6"/>
+    <protectedRange sqref="D29" name="Range1_1_5"/>
+    <protectedRange sqref="D31" name="Range1_1_5_1_1"/>
+    <protectedRange sqref="D32" name="Range1_1_8_1_1"/>
+    <protectedRange sqref="D44 D37:D42" name="Range1_1_3_1"/>
   </protectedRanges>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Removing hm0 bias correction flag
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\StormSim_Temp_working_dir\StormSim-Library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D4801D3-961A-466D-B1B6-670956E3507B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7CB9FD9-A055-4EA8-BAB3-3DD2CFCFCFB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
+    <workbookView xWindow="13305" yWindow="2535" windowWidth="19410" windowHeight="17385" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
@@ -560,9 +560,6 @@
     <t>Generate output visualizations (0 - Off, 1 - On)</t>
   </si>
   <si>
-    <t>chs_bias_and_uncertainty_source</t>
-  </si>
-  <si>
     <t>CHS_Dependencies\Bias_and_Uncertainty\CHS-GoM</t>
   </si>
   <si>
@@ -630,6 +627,9 @@
   </si>
   <si>
     <t>Roughness Coefficient, 2 for grass; 1 for concrete, asphalt, or closed blocks; 0.9 for basalt or placed revetment blocks; 0.8 for stepped structure; Table 6.2 from EurOtop (2018) (rubble mound )</t>
+  </si>
+  <si>
+    <t>chs_ssl_bias_and_uncertainty_file</t>
   </si>
 </sst>
 </file>
@@ -637,7 +637,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="0.000000000000000"/>
+    <numFmt numFmtId="164" formatCode="0.000000000000000"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -1034,7 +1034,7 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1363,7 +1363,7 @@
   <dimension ref="A1:I76"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.5703125" customWidth="1"/>
+    <col min="1" max="1" width="101.7109375" customWidth="1"/>
     <col min="2" max="2" width="152" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="171.140625" bestFit="1" customWidth="1"/>
@@ -1999,7 +1999,7 @@
     </row>
     <row r="28" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
-        <v>174</v>
+        <v>197</v>
       </c>
       <c r="B28" s="12" t="s">
         <v>150</v>
@@ -2008,7 +2008,7 @@
         <v>10</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F28" s="9" t="s">
         <v>3</v>
@@ -2025,16 +2025,16 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
+        <v>175</v>
+      </c>
+      <c r="B29" s="12" t="s">
         <v>176</v>
       </c>
-      <c r="B29" s="12" t="s">
+      <c r="C29" s="28" t="s">
+        <v>10</v>
+      </c>
+      <c r="D29" s="2" t="s">
         <v>177</v>
-      </c>
-      <c r="C29" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>178</v>
       </c>
       <c r="F29" s="29" t="s">
         <v>43</v>
@@ -2054,13 +2054,13 @@
         <v>117</v>
       </c>
       <c r="B30" s="12" t="s">
+        <v>178</v>
+      </c>
+      <c r="C30" s="28" t="s">
+        <v>10</v>
+      </c>
+      <c r="D30" s="2" t="s">
         <v>179</v>
-      </c>
-      <c r="C30" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>180</v>
       </c>
       <c r="F30" s="14" t="s">
         <v>96</v>
@@ -2086,7 +2086,7 @@
         <v>10</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F31" s="14" t="s">
         <v>123</v>
@@ -2112,7 +2112,7 @@
         <v>10</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F32" s="14" t="s">
         <v>124</v>
@@ -2219,10 +2219,10 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="11" t="s">
+        <v>182</v>
+      </c>
+      <c r="B37" s="12" t="s">
         <v>183</v>
-      </c>
-      <c r="B37" s="12" t="s">
-        <v>184</v>
       </c>
       <c r="C37" s="13" t="s">
         <v>109</v>
@@ -2375,10 +2375,10 @@
     </row>
     <row r="43" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="14" t="s">
+        <v>184</v>
+      </c>
+      <c r="B43" s="15" t="s">
         <v>185</v>
-      </c>
-      <c r="B43" s="15" t="s">
-        <v>186</v>
       </c>
       <c r="C43" s="16" t="s">
         <v>10</v>
@@ -2555,10 +2555,10 @@
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="14" t="s">
+        <v>186</v>
+      </c>
+      <c r="B56" s="15" t="s">
         <v>187</v>
-      </c>
-      <c r="B56" s="15" t="s">
-        <v>188</v>
       </c>
       <c r="C56" s="16" t="s">
         <v>10</v>
@@ -2569,10 +2569,10 @@
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="B57" s="15" t="s">
         <v>189</v>
-      </c>
-      <c r="B57" s="15" t="s">
-        <v>190</v>
       </c>
       <c r="C57" s="16" t="s">
         <v>10</v>
@@ -2586,7 +2586,7 @@
         <v>68</v>
       </c>
       <c r="B58" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C58" s="16" t="s">
         <v>10</v>
@@ -2600,7 +2600,7 @@
         <v>69</v>
       </c>
       <c r="B59" s="15" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C59" s="16" t="s">
         <v>10</v>
@@ -2611,10 +2611,10 @@
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="14" t="s">
+        <v>192</v>
+      </c>
+      <c r="B60" s="15" t="s">
         <v>193</v>
-      </c>
-      <c r="B60" s="15" t="s">
-        <v>194</v>
       </c>
       <c r="C60" s="16" t="s">
         <v>10</v>
@@ -2625,10 +2625,10 @@
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="14" t="s">
+        <v>194</v>
+      </c>
+      <c r="B61" s="15" t="s">
         <v>195</v>
-      </c>
-      <c r="B61" s="15" t="s">
-        <v>196</v>
       </c>
       <c r="C61" s="16" t="s">
         <v>10</v>
@@ -2642,7 +2642,7 @@
         <v>74</v>
       </c>
       <c r="B62" s="42" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C62" s="19" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
Make sure input file is latest
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20408"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\StormSim_Temp_working_dir\StormSim-Library\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\StormSim_Temp_working_dir\StormSim-Library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7CB9FD9-A055-4EA8-BAB3-3DD2CFCFCFB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE8ED2B5-17C7-439F-8E87-07625219DA71}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13305" yWindow="2535" windowWidth="19410" windowHeight="17385" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
@@ -25,10 +25,10 @@
         <xcalcf:feature name="microsoft.com:RD"/>
         <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="194">
   <si>
     <t>StormSim Project General Inputs</t>
   </si>
@@ -242,12 +242,6 @@
     <t>[Figure VI-5-11 CEM]</t>
   </si>
   <si>
-    <t>seaside_init_S</t>
-  </si>
-  <si>
-    <t>leeside_init_S</t>
-  </si>
-  <si>
     <t>use_timeseries</t>
   </si>
   <si>
@@ -606,12 +600,6 @@
   </si>
   <si>
     <t>StormSim:PROS Design Leeside Limit Damage State (Estimate stone size)</t>
-  </si>
-  <si>
-    <t>StormSim: LCS-CSR Seaside Zero Damage Level S_Ss (Damage initiation)</t>
-  </si>
-  <si>
-    <t>StormSim: LCS-CSR Leeside Zero Damage Level S_Ls (Damage initiation)</t>
   </si>
   <si>
     <t>seaside_S_uls</t>
@@ -1064,9 +1052,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1104,7 +1092,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1210,7 +1198,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1352,7 +1340,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1360,20 +1348,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51D29750-2AFD-4BF7-A911-1DC4ADC0FD7A}">
-  <dimension ref="A1:I76"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I74"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="101.7109375" customWidth="1"/>
+    <col min="1" max="1" width="101.6640625" customWidth="1"/>
     <col min="2" max="2" width="152" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="171.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="28.42578125" customWidth="1"/>
-    <col min="7" max="7" width="84.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="46.140625" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="171.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="28.44140625" customWidth="1"/>
+    <col min="7" max="7" width="84.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="46.109375" customWidth="1"/>
+    <col min="9" max="9" width="13.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -1387,7 +1375,7 @@
       <c r="H1" s="33"/>
       <c r="I1" s="33"/>
     </row>
-    <row r="2" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="s">
         <v>3</v>
       </c>
@@ -1413,7 +1401,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="11" t="s">
         <v>8</v>
       </c>
@@ -1424,22 +1412,22 @@
         <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F3" s="43" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G3" s="43" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H3" s="13" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="I3" s="13">
         <v>0.33979999999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="14" t="s">
         <v>13</v>
       </c>
@@ -1450,13 +1438,13 @@
         <v>10</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F4" s="43" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G4" s="43" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="H4" s="13" t="s">
         <v>10</v>
@@ -1465,50 +1453,50 @@
         <v>0.38219999999999998</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="14" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C5" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="F5" s="43" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="G5" s="43" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="I5" s="13">
         <v>0.3</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="14" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C6" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="F6" s="43" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="G6" s="43" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="H6" s="13" t="s">
         <v>10</v>
@@ -1517,7 +1505,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="14" t="s">
         <v>20</v>
       </c>
@@ -1528,14 +1516,14 @@
         <v>10</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="F7" s="33"/>
       <c r="G7" s="33"/>
       <c r="H7" s="33"/>
       <c r="I7" s="33"/>
     </row>
-    <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="14" t="s">
         <v>29</v>
       </c>
@@ -1546,21 +1534,21 @@
         <v>10</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="F8" s="26" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="G8" s="27"/>
       <c r="H8" s="27"/>
       <c r="I8" s="27"/>
     </row>
-    <row r="9" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="14" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C9" s="16" t="s">
         <v>10</v>
@@ -1581,7 +1569,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="14" t="s">
         <v>18</v>
       </c>
@@ -1595,19 +1583,19 @@
         <v>3</v>
       </c>
       <c r="F10" s="30" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="G10" s="15" t="s">
         <v>45</v>
       </c>
       <c r="H10" s="16" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="I10" s="2">
         <v>0.15</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="14" t="s">
         <v>22</v>
       </c>
@@ -1618,22 +1606,22 @@
         <v>10</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="F11" s="30" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="G11" s="15" t="s">
         <v>48</v>
       </c>
       <c r="H11" s="31" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="I11" s="2">
         <v>0.43</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="14" t="s">
         <v>24</v>
       </c>
@@ -1641,30 +1629,30 @@
         <v>25</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D12" s="2">
         <v>0</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G12" s="15" t="s">
         <v>46</v>
       </c>
       <c r="H12" s="16" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="I12" s="2">
         <v>0.78</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="14" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C13" s="16" t="s">
         <v>10</v>
@@ -1673,24 +1661,24 @@
         <v>1</v>
       </c>
       <c r="F13" s="17" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G13" s="18" t="s">
         <v>47</v>
       </c>
       <c r="H13" s="19" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="I13" s="3">
         <v>0.13</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="14" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C14" s="16" t="s">
         <v>10</v>
@@ -1703,12 +1691,12 @@
       <c r="H14" s="27"/>
       <c r="I14" s="27"/>
     </row>
-    <row r="15" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="14" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C15" s="16" t="s">
         <v>10</v>
@@ -1727,12 +1715,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="14" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>10</v>
@@ -1753,12 +1741,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="14" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C17" s="16" t="s">
         <v>10</v>
@@ -1779,12 +1767,12 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="14" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C18" s="16" t="s">
         <v>10</v>
@@ -1805,12 +1793,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="14" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C19" s="16" t="s">
         <v>10</v>
@@ -1823,12 +1811,12 @@
       <c r="H19" s="8"/>
       <c r="I19" s="8"/>
     </row>
-    <row r="20" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="14" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C20" s="16" t="s">
         <v>10</v>
@@ -1843,18 +1831,18 @@
       <c r="H20" s="21"/>
       <c r="I20" s="21"/>
     </row>
-    <row r="21" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="17" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C21" s="19" t="s">
         <v>10</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>3</v>
@@ -1869,7 +1857,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="6"/>
       <c r="B22" s="22"/>
       <c r="C22" s="23"/>
@@ -1887,7 +1875,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="24" t="s">
         <v>35</v>
       </c>
@@ -1907,7 +1895,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="9" t="s">
         <v>3</v>
       </c>
@@ -1933,12 +1921,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="11" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C25" s="28" t="s">
         <v>10</v>
@@ -1953,13 +1941,13 @@
         <v>37</v>
       </c>
       <c r="H25" s="19" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="I25" s="3">
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="11" t="s">
         <v>38</v>
       </c>
@@ -1977,15 +1965,15 @@
       <c r="H26" s="21"/>
       <c r="I26" s="21"/>
     </row>
-    <row r="27" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="11" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C27" s="28" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D27" s="1">
         <v>3.43</v>
@@ -1997,18 +1985,18 @@
       <c r="H27" s="27"/>
       <c r="I27" s="27"/>
     </row>
-    <row r="28" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="11" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C28" s="28" t="s">
         <v>10</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="F28" s="9" t="s">
         <v>3</v>
@@ -2023,18 +2011,18 @@
         <v>6</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" s="11" t="s">
+        <v>173</v>
+      </c>
+      <c r="B29" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="C29" s="28" t="s">
+        <v>10</v>
+      </c>
+      <c r="D29" s="2" t="s">
         <v>175</v>
-      </c>
-      <c r="B29" s="12" t="s">
-        <v>176</v>
-      </c>
-      <c r="C29" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>177</v>
       </c>
       <c r="F29" s="29" t="s">
         <v>43</v>
@@ -2049,24 +2037,24 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30" s="11" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C30" s="28" t="s">
         <v>10</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="F30" s="14" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="G30" s="15" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H30" s="16" t="s">
         <v>10</v>
@@ -2075,24 +2063,24 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" s="14" t="s">
         <v>42</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C31" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="F31" s="14" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="G31" s="15" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H31" s="16" t="s">
         <v>10</v>
@@ -2101,24 +2089,24 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" s="14" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C32" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="F32" s="14" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G32" s="15" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="H32" s="16" t="s">
         <v>10</v>
@@ -2127,16 +2115,16 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" s="25"/>
       <c r="B33" s="25"/>
       <c r="C33" s="25"/>
       <c r="D33" s="25"/>
       <c r="F33" s="14" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G33" s="15" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="H33" s="16" t="s">
         <v>10</v>
@@ -2145,7 +2133,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="34" t="s">
         <v>50</v>
       </c>
@@ -2153,10 +2141,10 @@
       <c r="C34" s="35"/>
       <c r="D34" s="35"/>
       <c r="F34" s="14" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="G34" s="15" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="H34" s="16" t="s">
         <v>10</v>
@@ -2165,7 +2153,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="9" t="s">
         <v>3</v>
       </c>
@@ -2179,10 +2167,10 @@
         <v>6</v>
       </c>
       <c r="F35" s="14" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="G35" s="15" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H35" s="16" t="s">
         <v>10</v>
@@ -2191,24 +2179,24 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36" s="11" t="s">
         <v>51</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D36" s="1">
         <v>3.41</v>
       </c>
       <c r="F36" s="14" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="G36" s="15" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="H36" s="16" t="s">
         <v>10</v>
@@ -2217,24 +2205,24 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37" s="11" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D37" s="1">
         <v>1.0668</v>
       </c>
       <c r="F37" s="14" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="G37" s="15" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="H37" s="16" t="s">
         <v>10</v>
@@ -2243,24 +2231,24 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" s="14" t="s">
         <v>52</v>
       </c>
       <c r="B38" s="15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C38" s="16" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D38" s="2">
         <v>7.01</v>
       </c>
       <c r="F38" s="14" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="G38" s="15" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="H38" s="16" t="s">
         <v>10</v>
@@ -2269,24 +2257,24 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39" s="14" t="s">
         <v>53</v>
       </c>
       <c r="B39" s="15" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C39" s="16" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D39" s="2">
         <v>-2.42</v>
       </c>
       <c r="F39" s="14" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="G39" s="15" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="H39" s="16" t="s">
         <v>10</v>
@@ -2295,24 +2283,24 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40" s="14" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B40" s="15" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C40" s="16" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D40" s="2">
         <v>-0.95799999999999996</v>
       </c>
       <c r="F40" s="14" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="G40" s="15" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="H40" s="16" t="s">
         <v>10</v>
@@ -2321,12 +2309,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A41" s="14" t="s">
         <v>54</v>
       </c>
       <c r="B41" s="15" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C41" s="16" t="s">
         <v>10</v>
@@ -2335,10 +2323,10 @@
         <v>3</v>
       </c>
       <c r="F41" s="14" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="G41" s="15" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="H41" s="16" t="s">
         <v>10</v>
@@ -2347,12 +2335,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A42" s="14" t="s">
         <v>55</v>
       </c>
       <c r="B42" s="15" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C42" s="16" t="s">
         <v>10</v>
@@ -2361,10 +2349,10 @@
         <v>1.5</v>
       </c>
       <c r="F42" s="14" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="G42" s="15" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="H42" s="16" t="s">
         <v>10</v>
@@ -2373,12 +2361,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A43" s="14" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B43" s="15" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C43" s="16" t="s">
         <v>10</v>
@@ -2387,10 +2375,10 @@
         <v>0</v>
       </c>
       <c r="F43" s="17" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="G43" s="18" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="H43" s="19" t="s">
         <v>10</v>
@@ -2399,12 +2387,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A44" s="14" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B44" s="15" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C44" s="16" t="s">
         <v>10</v>
@@ -2413,41 +2401,41 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A45" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="B45" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="B45" s="14" t="s">
-        <v>77</v>
-      </c>
       <c r="C45" s="16" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D45" s="2">
         <v>3.35</v>
       </c>
     </row>
-    <row r="46" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A46" s="38" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B46" s="38" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C46" s="39" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D46" s="40">
         <v>0.06</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A47" s="34"/>
       <c r="B47" s="34"/>
       <c r="C47" s="34"/>
       <c r="D47" s="34"/>
     </row>
-    <row r="48" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A48" s="36" t="s">
         <v>56</v>
       </c>
@@ -2455,7 +2443,7 @@
       <c r="C48" s="37"/>
       <c r="D48" s="37"/>
     </row>
-    <row r="49" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A49" s="9" t="s">
         <v>3</v>
       </c>
@@ -2469,7 +2457,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" s="11" t="s">
         <v>57</v>
       </c>
@@ -2483,7 +2471,7 @@
         <v>1.65</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" s="14" t="s">
         <v>59</v>
       </c>
@@ -2491,13 +2479,13 @@
         <v>60</v>
       </c>
       <c r="C51" s="16" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D51" s="2">
         <v>780</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" s="14" t="s">
         <v>61</v>
       </c>
@@ -2505,27 +2493,27 @@
         <v>62</v>
       </c>
       <c r="C52" s="16" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D52" s="2">
         <v>57</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53" s="14" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B53" s="15" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C53" s="16" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D53" s="2">
         <v>1147</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54" s="14" t="s">
         <v>63</v>
       </c>
@@ -2533,13 +2521,13 @@
         <v>64</v>
       </c>
       <c r="C54" s="16" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D54" s="2">
         <v>1027</v>
       </c>
     </row>
-    <row r="55" spans="1:4" ht="60.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" ht="60.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="14" t="s">
         <v>65</v>
       </c>
@@ -2553,12 +2541,12 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A56" s="14" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B56" s="15" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C56" s="16" t="s">
         <v>10</v>
@@ -2567,12 +2555,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A57" s="14" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B57" s="15" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C57" s="16" t="s">
         <v>10</v>
@@ -2581,23 +2569,23 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A58" s="14" t="s">
-        <v>68</v>
+        <v>188</v>
       </c>
       <c r="B58" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="C58" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D58" s="2">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A59" s="14" t="s">
         <v>190</v>
-      </c>
-      <c r="C58" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D58" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="14" t="s">
-        <v>69</v>
       </c>
       <c r="B59" s="15" t="s">
         <v>191</v>
@@ -2606,72 +2594,45 @@
         <v>10</v>
       </c>
       <c r="D59" s="2">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A60" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="B60" s="42" t="s">
+        <v>192</v>
+      </c>
+      <c r="C60" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D60" s="4">
         <v>2</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="14" t="s">
-        <v>192</v>
-      </c>
-      <c r="B60" s="15" t="s">
-        <v>193</v>
-      </c>
-      <c r="C60" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D60" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="14" t="s">
-        <v>194</v>
-      </c>
-      <c r="B61" s="15" t="s">
-        <v>195</v>
-      </c>
-      <c r="C61" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D61" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" ht="88.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="18" t="s">
-        <v>74</v>
-      </c>
-      <c r="B62" s="42" t="s">
-        <v>196</v>
-      </c>
-      <c r="C62" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D62" s="4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A63" s="37"/>
-      <c r="B63" s="37"/>
-      <c r="C63" s="37"/>
-      <c r="D63" s="37"/>
-    </row>
-    <row r="69" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C69" s="45"/>
-    </row>
-    <row r="70" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C70" s="44"/>
-    </row>
-    <row r="76" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B76" s="41"/>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A61" s="37"/>
+      <c r="B61" s="37"/>
+      <c r="C61" s="37"/>
+      <c r="D61" s="37"/>
+    </row>
+    <row r="62" spans="1:4" ht="88.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="67" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="C67" s="45"/>
+    </row>
+    <row r="68" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C68" s="44"/>
+    </row>
+    <row r="74" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B74" s="41"/>
     </row>
   </sheetData>
   <sheetProtection formatColumns="0" selectLockedCells="1"/>
   <protectedRanges>
     <protectedRange sqref="I3:I6 D14 I10:I14 I22:I25 I29 D16:D18 I17:I18 D9:D12 D3:D7" name="Range1_1"/>
     <protectedRange sqref="D8 D15" name="Range1_1_1"/>
-    <protectedRange sqref="D50:D55 D62" name="Range1_1_4"/>
+    <protectedRange sqref="D50:D55 D60" name="Range1_1_4"/>
     <protectedRange sqref="D13" name="Range1_1_2"/>
     <protectedRange sqref="D44 D36 D38:D42" name="Range1_1_3_1"/>
     <protectedRange sqref="D26" name="Range1_1_3"/>
@@ -2683,7 +2644,7 @@
     <protectedRange sqref="D31" name="Range1_1_8_1_1_1"/>
     <protectedRange sqref="D37" name="Range1_1_3_1_1"/>
     <protectedRange sqref="D43" name="Range1_1_3_1_2"/>
-    <protectedRange sqref="D56:D60" name="Range1_1_4_1"/>
+    <protectedRange sqref="D56:D58" name="Range1_1_4_1"/>
   </protectedRanges>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Removing lcbw mass input field.
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\StormSim_Temp_working_dir\StormSim-Library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3639BA2-1F4B-4395-89F4-9262DCFFA587}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D38E776E-79C1-47F8-924C-338709367ACC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="19485" windowHeight="17385" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="28395" windowHeight="17385" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="192">
   <si>
     <t>StormSim Project General Inputs</t>
   </si>
@@ -456,12 +456,6 @@
   </si>
   <si>
     <t>Compute Overtopping Discharge Volume Unit Width Response (Eurotop) (RB3 Only)</t>
-  </si>
-  <si>
-    <t>lcbw_mass</t>
-  </si>
-  <si>
-    <t>Low Crested Breakwater Seaside Mass</t>
   </si>
   <si>
     <t>Apply random tide to storm SWL (0 - Off / 1 - On)</t>
@@ -1348,7 +1342,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51D29750-2AFD-4BF7-A911-1DC4ADC0FD7A}">
-  <dimension ref="A1:I74"/>
+  <dimension ref="A1:I73"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="101.7109375" customWidth="1"/>
@@ -1412,7 +1406,7 @@
         <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="F3" s="43" t="s">
         <v>80</v>
@@ -1464,7 +1458,7 @@
         <v>10</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="F5" s="43" t="s">
         <v>83</v>
@@ -1481,16 +1475,16 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C6" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="F6" s="43" t="s">
         <v>82</v>
@@ -1516,7 +1510,7 @@
         <v>10</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="F7" s="33"/>
       <c r="G7" s="33"/>
@@ -1606,7 +1600,7 @@
         <v>10</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="F11" s="30" t="s">
         <v>87</v>
@@ -1652,7 +1646,7 @@
         <v>120</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C13" s="16" t="s">
         <v>10</v>
@@ -1678,7 +1672,7 @@
         <v>85</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C14" s="16" t="s">
         <v>10</v>
@@ -1696,7 +1690,7 @@
         <v>98</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C15" s="16" t="s">
         <v>10</v>
@@ -1720,7 +1714,7 @@
         <v>68</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>10</v>
@@ -1746,7 +1740,7 @@
         <v>99</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C17" s="16" t="s">
         <v>10</v>
@@ -1772,7 +1766,7 @@
         <v>100</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C18" s="16" t="s">
         <v>10</v>
@@ -1795,10 +1789,10 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C19" s="16" t="s">
         <v>10</v>
@@ -1813,10 +1807,10 @@
     </row>
     <row r="20" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="14" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C20" s="16" t="s">
         <v>10</v>
@@ -1833,16 +1827,16 @@
     </row>
     <row r="21" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="17" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C21" s="19" t="s">
         <v>10</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>3</v>
@@ -1987,16 +1981,16 @@
     </row>
     <row r="28" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C28" s="28" t="s">
         <v>10</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="F28" s="9" t="s">
         <v>3</v>
@@ -2013,16 +2007,16 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="B29" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="C29" s="28" t="s">
+        <v>10</v>
+      </c>
+      <c r="D29" s="2" t="s">
         <v>173</v>
-      </c>
-      <c r="B29" s="12" t="s">
-        <v>174</v>
-      </c>
-      <c r="C29" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>175</v>
       </c>
       <c r="F29" s="29" t="s">
         <v>43</v>
@@ -2042,13 +2036,13 @@
         <v>115</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C30" s="28" t="s">
         <v>10</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="F30" s="14" t="s">
         <v>94</v>
@@ -2074,7 +2068,7 @@
         <v>10</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F31" s="14" t="s">
         <v>121</v>
@@ -2094,13 +2088,13 @@
         <v>88</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C32" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="F32" s="14" t="s">
         <v>122</v>
@@ -2207,10 +2201,10 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="11" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C37" s="13" t="s">
         <v>107</v>
@@ -2297,10 +2291,10 @@
         <v>-0.95799999999999996</v>
       </c>
       <c r="F40" s="14" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="G40" s="15" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="H40" s="16" t="s">
         <v>10</v>
@@ -2323,10 +2317,10 @@
         <v>3</v>
       </c>
       <c r="F41" s="14" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="G41" s="15" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="H41" s="16" t="s">
         <v>10</v>
@@ -2349,10 +2343,10 @@
         <v>1.5</v>
       </c>
       <c r="F42" s="14" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="G42" s="15" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="H42" s="16" t="s">
         <v>10</v>
@@ -2363,10 +2357,10 @@
     </row>
     <row r="43" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="14" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B43" s="15" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C43" s="16" t="s">
         <v>10</v>
@@ -2375,10 +2369,10 @@
         <v>0</v>
       </c>
       <c r="F43" s="17" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="G43" s="18" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="H43" s="19" t="s">
         <v>10</v>
@@ -2501,44 +2495,44 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="14" t="s">
-        <v>140</v>
+        <v>63</v>
       </c>
       <c r="B53" s="15" t="s">
-        <v>141</v>
+        <v>64</v>
       </c>
       <c r="C53" s="16" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D53" s="2">
-        <v>1147</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="14" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B54" s="15" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C54" s="16" t="s">
-        <v>109</v>
+        <v>67</v>
       </c>
       <c r="D54" s="2">
-        <v>1027</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="60.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
-        <v>65</v>
+        <v>182</v>
       </c>
       <c r="B55" s="15" t="s">
-        <v>66</v>
+        <v>183</v>
       </c>
       <c r="C55" s="16" t="s">
-        <v>67</v>
+        <v>10</v>
       </c>
       <c r="D55" s="2">
-        <v>0.4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
@@ -2566,7 +2560,7 @@
         <v>10</v>
       </c>
       <c r="D57" s="2">
-        <v>1</v>
+        <v>15</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
@@ -2583,56 +2577,42 @@
         <v>15</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="14" t="s">
+    <row r="59" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="B59" s="42" t="s">
         <v>190</v>
       </c>
-      <c r="B59" s="15" t="s">
-        <v>191</v>
-      </c>
-      <c r="C59" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D59" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="18" t="s">
-        <v>72</v>
-      </c>
-      <c r="B60" s="42" t="s">
-        <v>192</v>
-      </c>
-      <c r="C60" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D60" s="4">
+      <c r="C59" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D59" s="4">
         <v>2</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="37"/>
-      <c r="B61" s="37"/>
-      <c r="C61" s="37"/>
-      <c r="D61" s="37"/>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" s="37"/>
+      <c r="B60" s="37"/>
+      <c r="C60" s="37"/>
+      <c r="D60" s="37"/>
     </row>
     <row r="62" spans="1:4" ht="88.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="67" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C67" s="45"/>
-    </row>
-    <row r="68" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C68" s="44"/>
-    </row>
-    <row r="74" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B74" s="41"/>
+    <row r="66" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C66" s="45"/>
+    </row>
+    <row r="67" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C67" s="44"/>
+    </row>
+    <row r="73" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B73" s="41"/>
     </row>
   </sheetData>
   <sheetProtection formatColumns="0" selectLockedCells="1"/>
   <protectedRanges>
     <protectedRange sqref="I3:I6 D14 I10:I14 I22:I25 I29 D16:D18 I17:I18 D9:D12 D3:D7" name="Range1_1"/>
     <protectedRange sqref="D8 D15" name="Range1_1_1"/>
-    <protectedRange sqref="D50:D55 D60" name="Range1_1_4"/>
+    <protectedRange sqref="D59 D50:D54" name="Range1_1_4"/>
     <protectedRange sqref="D13" name="Range1_1_2"/>
     <protectedRange sqref="D44 D36 D38:D42" name="Range1_1_3_1"/>
     <protectedRange sqref="D26" name="Range1_1_3"/>
@@ -2644,7 +2624,7 @@
     <protectedRange sqref="D31" name="Range1_1_8_1_1_1"/>
     <protectedRange sqref="D37" name="Range1_1_3_1_1"/>
     <protectedRange sqref="D43" name="Range1_1_3_1_2"/>
-    <protectedRange sqref="D56:D58" name="Range1_1_4_1"/>
+    <protectedRange sqref="D55:D57" name="Range1_1_4_1"/>
   </protectedRanges>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Changing response computation switches from pros_r2p to compute_r2p.
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\StormSim_Temp_working_dir\StormSim-Library\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\0_StormSim_Development\StormSim-Library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71564579-E648-4868-9155-3FB6BBDBBC78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85290D33-0448-4D16-A8BE-04CF93CFA637}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="28395" windowHeight="17385" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="193">
   <si>
     <t>StormSim Project General Inputs</t>
   </si>
@@ -395,36 +395,9 @@
     <t>CHS Zip Folder or Custom Modeling .mat File (Relative Path)</t>
   </si>
   <si>
-    <t>StormSim workflow to call for project. (1 - StormSim:PROS Response Base (RB), 2- StormSim:EVA, 3- StormSim:LCS, 4- StormSim: PROS Frequency Base (FB))</t>
-  </si>
-  <si>
     <t>apply_random_tides</t>
   </si>
   <si>
-    <t>pros_dn50_seaside</t>
-  </si>
-  <si>
-    <t>pros_dn50_leeside</t>
-  </si>
-  <si>
-    <t>pros_dn50_lcbw</t>
-  </si>
-  <si>
-    <t>pros_r2p</t>
-  </si>
-  <si>
-    <t>pros_q</t>
-  </si>
-  <si>
-    <t>pros_p1</t>
-  </si>
-  <si>
-    <t>pros_p2_p3</t>
-  </si>
-  <si>
-    <t>pros_nappe</t>
-  </si>
-  <si>
     <t>Compute Seaward Median Stone Size Response (Momentum Flux)</t>
   </si>
   <si>
@@ -452,9 +425,6 @@
     <t>SP_2243</t>
   </si>
   <si>
-    <t>pros_q_vol</t>
-  </si>
-  <si>
     <t>Compute Overtopping Discharge Volume Unit Width Response (Eurotop) (RB3 Only)</t>
   </si>
   <si>
@@ -612,15 +582,45 @@
   </si>
   <si>
     <t>chs_ssl_bias_and_uncertainty_file</t>
+  </si>
+  <si>
+    <t>StormSim workflow to call for project. (1 - StormSim:PROS , 3- StormSim:LCS, 4- StormSim: PROS Frequency Base (FB))</t>
+  </si>
+  <si>
+    <t>Structure Responses</t>
+  </si>
+  <si>
+    <t>compute_dn50_seaside</t>
+  </si>
+  <si>
+    <t>compute_dn50_leeside</t>
+  </si>
+  <si>
+    <t>compute_dn50_lcbw</t>
+  </si>
+  <si>
+    <t>compute_r2p</t>
+  </si>
+  <si>
+    <t>compute_q</t>
+  </si>
+  <si>
+    <t>compute_q_vol</t>
+  </si>
+  <si>
+    <t>compute_p1</t>
+  </si>
+  <si>
+    <t>compute_p2_p3</t>
+  </si>
+  <si>
+    <t>compute_nappe</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.000000000000000"/>
-  </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -657,7 +657,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -718,8 +718,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00FFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="15">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -888,21 +894,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -919,7 +910,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1004,20 +995,13 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1028,12 +1012,19 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF00FFFF"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1342,7 +1333,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51D29750-2AFD-4BF7-A911-1DC4ADC0FD7A}">
-  <dimension ref="A1:I73"/>
+  <dimension ref="A1:I72"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="101.7109375" customWidth="1"/>
@@ -1406,12 +1397,12 @@
         <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="F3" s="43" t="s">
+        <v>156</v>
+      </c>
+      <c r="F3" s="42" t="s">
         <v>80</v>
       </c>
-      <c r="G3" s="43" t="s">
+      <c r="G3" s="42" t="s">
         <v>76</v>
       </c>
       <c r="H3" s="13" t="s">
@@ -1432,12 +1423,12 @@
         <v>10</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="F4" s="43" t="s">
+        <v>128</v>
+      </c>
+      <c r="F4" s="42" t="s">
         <v>81</v>
       </c>
-      <c r="G4" s="43" t="s">
+      <c r="G4" s="42" t="s">
         <v>77</v>
       </c>
       <c r="H4" s="13" t="s">
@@ -1458,12 +1449,12 @@
         <v>10</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="F5" s="43" t="s">
+        <v>157</v>
+      </c>
+      <c r="F5" s="42" t="s">
         <v>83</v>
       </c>
-      <c r="G5" s="43" t="s">
+      <c r="G5" s="42" t="s">
         <v>78</v>
       </c>
       <c r="H5" s="13" t="s">
@@ -1475,21 +1466,21 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="B6" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="B6" s="15" t="s">
-        <v>154</v>
-      </c>
-      <c r="C6" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="F6" s="43" t="s">
+      <c r="F6" s="42" t="s">
         <v>82</v>
       </c>
-      <c r="G6" s="43" t="s">
+      <c r="G6" s="42" t="s">
         <v>79</v>
       </c>
       <c r="H6" s="13" t="s">
@@ -1510,7 +1501,7 @@
         <v>10</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="F7" s="33"/>
       <c r="G7" s="33"/>
@@ -1542,7 +1533,7 @@
         <v>97</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>119</v>
+        <v>182</v>
       </c>
       <c r="C9" s="16" t="s">
         <v>10</v>
@@ -1600,7 +1591,7 @@
         <v>10</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="F11" s="30" t="s">
         <v>87</v>
@@ -1643,10 +1634,10 @@
     </row>
     <row r="13" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="14" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="C13" s="16" t="s">
         <v>10</v>
@@ -1672,7 +1663,7 @@
         <v>85</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C14" s="16" t="s">
         <v>10</v>
@@ -1690,7 +1681,7 @@
         <v>98</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="C15" s="16" t="s">
         <v>10</v>
@@ -1714,7 +1705,7 @@
         <v>68</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>10</v>
@@ -1740,7 +1731,7 @@
         <v>99</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C17" s="16" t="s">
         <v>10</v>
@@ -1748,16 +1739,16 @@
       <c r="D17" s="2">
         <v>0</v>
       </c>
-      <c r="F17" s="46" t="s">
+      <c r="F17" s="43" t="s">
         <v>11</v>
       </c>
-      <c r="G17" s="47" t="s">
+      <c r="G17" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="H17" s="48" t="s">
-        <v>10</v>
-      </c>
-      <c r="I17" s="49">
+      <c r="H17" s="45" t="s">
+        <v>10</v>
+      </c>
+      <c r="I17" s="46">
         <v>1000</v>
       </c>
     </row>
@@ -1766,7 +1757,7 @@
         <v>100</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="C18" s="16" t="s">
         <v>10</v>
@@ -1789,10 +1780,10 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="C19" s="16" t="s">
         <v>10</v>
@@ -1807,10 +1798,10 @@
     </row>
     <row r="20" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="14" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="C20" s="16" t="s">
         <v>10</v>
@@ -1827,16 +1818,16 @@
     </row>
     <row r="21" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="17" t="s">
-        <v>152</v>
+        <v>142</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="C21" s="19" t="s">
         <v>10</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>3</v>
@@ -1981,16 +1972,16 @@
     </row>
     <row r="28" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="C28" s="28" t="s">
         <v>10</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="F28" s="9" t="s">
         <v>3</v>
@@ -2007,16 +1998,16 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="C29" s="28" t="s">
         <v>10</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="F29" s="29" t="s">
         <v>43</v>
@@ -2036,13 +2027,13 @@
         <v>115</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="C30" s="28" t="s">
         <v>10</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="F30" s="14" t="s">
         <v>94</v>
@@ -2068,19 +2059,19 @@
         <v>10</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
       <c r="F31" s="14" t="s">
-        <v>121</v>
+        <v>145</v>
       </c>
       <c r="G31" s="15" t="s">
-        <v>129</v>
+        <v>146</v>
       </c>
       <c r="H31" s="16" t="s">
         <v>10</v>
       </c>
       <c r="I31" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -2088,19 +2079,19 @@
         <v>88</v>
       </c>
       <c r="B32" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="C32" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="F32" s="14" t="s">
         <v>147</v>
       </c>
-      <c r="C32" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="F32" s="14" t="s">
-        <v>122</v>
-      </c>
       <c r="G32" s="15" t="s">
-        <v>130</v>
+        <v>148</v>
       </c>
       <c r="H32" s="16" t="s">
         <v>10</v>
@@ -2115,10 +2106,10 @@
       <c r="C33" s="25"/>
       <c r="D33" s="25"/>
       <c r="F33" s="14" t="s">
-        <v>123</v>
+        <v>149</v>
       </c>
       <c r="G33" s="15" t="s">
-        <v>131</v>
+        <v>150</v>
       </c>
       <c r="H33" s="16" t="s">
         <v>10</v>
@@ -2134,16 +2125,16 @@
       <c r="B34" s="35"/>
       <c r="C34" s="35"/>
       <c r="D34" s="35"/>
-      <c r="F34" s="14" t="s">
-        <v>124</v>
-      </c>
-      <c r="G34" s="15" t="s">
-        <v>132</v>
-      </c>
-      <c r="H34" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="I34" s="2">
+      <c r="F34" s="17" t="s">
+        <v>151</v>
+      </c>
+      <c r="G34" s="18" t="s">
+        <v>152</v>
+      </c>
+      <c r="H34" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="I34" s="3">
         <v>0</v>
       </c>
     </row>
@@ -2160,18 +2151,6 @@
       <c r="D35" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="F35" s="14" t="s">
-        <v>125</v>
-      </c>
-      <c r="G35" s="15" t="s">
-        <v>133</v>
-      </c>
-      <c r="H35" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="I35" s="2">
-        <v>0</v>
-      </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="11" t="s">
@@ -2186,43 +2165,19 @@
       <c r="D36" s="1">
         <v>3.41</v>
       </c>
-      <c r="F36" s="14" t="s">
-        <v>138</v>
-      </c>
-      <c r="G36" s="15" t="s">
-        <v>139</v>
-      </c>
-      <c r="H36" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="I36" s="2">
-        <v>0</v>
-      </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="11" t="s">
-        <v>178</v>
+        <v>168</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="C37" s="13" t="s">
         <v>107</v>
       </c>
       <c r="D37" s="1">
         <v>1.0668</v>
-      </c>
-      <c r="F37" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="G37" s="15" t="s">
-        <v>134</v>
-      </c>
-      <c r="H37" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="I37" s="2">
-        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
@@ -2238,18 +2193,6 @@
       <c r="D38" s="2">
         <v>7.01</v>
       </c>
-      <c r="F38" s="14" t="s">
-        <v>127</v>
-      </c>
-      <c r="G38" s="15" t="s">
-        <v>135</v>
-      </c>
-      <c r="H38" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="I38" s="2">
-        <v>0</v>
-      </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
@@ -2264,18 +2207,6 @@
       <c r="D39" s="2">
         <v>-2.42</v>
       </c>
-      <c r="F39" s="14" t="s">
-        <v>128</v>
-      </c>
-      <c r="G39" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="H39" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="I39" s="2">
-        <v>0</v>
-      </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="s">
@@ -2290,18 +2221,6 @@
       <c r="D40" s="2">
         <v>-0.95799999999999996</v>
       </c>
-      <c r="F40" s="14" t="s">
-        <v>155</v>
-      </c>
-      <c r="G40" s="15" t="s">
-        <v>156</v>
-      </c>
-      <c r="H40" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="I40" s="2">
-        <v>1</v>
-      </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="14" t="s">
@@ -2316,18 +2235,6 @@
       <c r="D41" s="2">
         <v>3</v>
       </c>
-      <c r="F41" s="14" t="s">
-        <v>157</v>
-      </c>
-      <c r="G41" s="15" t="s">
-        <v>158</v>
-      </c>
-      <c r="H41" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="I41" s="2">
-        <v>0</v>
-      </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="14" t="s">
@@ -2342,42 +2249,18 @@
       <c r="D42" s="2">
         <v>1.5</v>
       </c>
-      <c r="F42" s="14" t="s">
-        <v>159</v>
-      </c>
-      <c r="G42" s="15" t="s">
-        <v>160</v>
-      </c>
-      <c r="H42" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="I42" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="B43" s="15" t="s">
-        <v>181</v>
+        <v>171</v>
       </c>
       <c r="C43" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D43" s="2">
-        <v>0</v>
-      </c>
-      <c r="F43" s="17" t="s">
-        <v>161</v>
-      </c>
-      <c r="G43" s="18" t="s">
-        <v>162</v>
-      </c>
-      <c r="H43" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="I43" s="3">
         <v>0</v>
       </c>
     </row>
@@ -2523,10 +2406,10 @@
     </row>
     <row r="55" spans="1:4" ht="60.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
-        <v>182</v>
+        <v>172</v>
       </c>
       <c r="B55" s="15" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="C55" s="16" t="s">
         <v>10</v>
@@ -2537,10 +2420,10 @@
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="14" t="s">
-        <v>184</v>
+        <v>174</v>
       </c>
       <c r="B56" s="15" t="s">
-        <v>185</v>
+        <v>175</v>
       </c>
       <c r="C56" s="16" t="s">
         <v>10</v>
@@ -2551,10 +2434,10 @@
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="14" t="s">
-        <v>186</v>
+        <v>176</v>
       </c>
       <c r="B57" s="15" t="s">
-        <v>187</v>
+        <v>177</v>
       </c>
       <c r="C57" s="16" t="s">
         <v>10</v>
@@ -2565,10 +2448,10 @@
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="14" t="s">
-        <v>188</v>
+        <v>178</v>
       </c>
       <c r="B58" s="15" t="s">
-        <v>189</v>
+        <v>179</v>
       </c>
       <c r="C58" s="16" t="s">
         <v>10</v>
@@ -2581,8 +2464,8 @@
       <c r="A59" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="B59" s="42" t="s">
-        <v>190</v>
+      <c r="B59" s="41" t="s">
+        <v>180</v>
       </c>
       <c r="C59" s="19" t="s">
         <v>10</v>
@@ -2597,15 +2480,159 @@
       <c r="C60" s="37"/>
       <c r="D60" s="37"/>
     </row>
-    <row r="62" spans="1:4" ht="88.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="66" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C66" s="45"/>
-    </row>
-    <row r="67" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C67" s="44"/>
-    </row>
-    <row r="73" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B73" s="41"/>
+    <row r="61" spans="1:4" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="47" t="s">
+        <v>183</v>
+      </c>
+      <c r="B61" s="48"/>
+      <c r="C61" s="48"/>
+      <c r="D61" s="48"/>
+    </row>
+    <row r="62" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B62" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C62" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D62" s="10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63" s="43" t="s">
+        <v>184</v>
+      </c>
+      <c r="B63" s="44" t="s">
+        <v>120</v>
+      </c>
+      <c r="C63" s="45" t="s">
+        <v>10</v>
+      </c>
+      <c r="D63" s="46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64" s="14" t="s">
+        <v>185</v>
+      </c>
+      <c r="B64" s="15" t="s">
+        <v>121</v>
+      </c>
+      <c r="C64" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D64" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65" s="14" t="s">
+        <v>186</v>
+      </c>
+      <c r="B65" s="15" t="s">
+        <v>122</v>
+      </c>
+      <c r="C65" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D65" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66" s="14" t="s">
+        <v>187</v>
+      </c>
+      <c r="B66" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="C66" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D66" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="B67" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="C67" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D67" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68" s="14" t="s">
+        <v>189</v>
+      </c>
+      <c r="B68" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="C68" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D68" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="B69" s="15" t="s">
+        <v>125</v>
+      </c>
+      <c r="C69" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D69" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="B70" s="15" t="s">
+        <v>126</v>
+      </c>
+      <c r="C70" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D70" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="17" t="s">
+        <v>192</v>
+      </c>
+      <c r="B71" s="18" t="s">
+        <v>127</v>
+      </c>
+      <c r="C71" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D71" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72" s="48"/>
+      <c r="B72" s="48"/>
+      <c r="C72" s="48"/>
+      <c r="D72" s="48"/>
     </row>
   </sheetData>
   <sheetProtection formatColumns="0" selectLockedCells="1"/>

</xml_diff>

<commit_message>
Adding damaging depth and elevation responses.
</commit_message>
<xml_diff>
--- a/StormSim_Inputs.xlsx
+++ b/StormSim_Inputs.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\0_StormSim_Task\StormSim-Library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CF759CD-2E39-478C-945A-B1F5FCC39D7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED4F07E9-A631-43EB-9225-F55FEA3F9520}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCE98FF7-F0BD-48B7-BD15-98C25A65ECBE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="199">
   <si>
     <t>StormSim Project General Inputs</t>
   </si>
@@ -353,12 +353,6 @@
     <t>Bottom of Wall Elevation (Applies to wall type structures)</t>
   </si>
   <si>
-    <t>Mound/Berm Seaward Slope</t>
-  </si>
-  <si>
-    <t>Mound Landward Slope</t>
-  </si>
-  <si>
     <t>[m]</t>
   </si>
   <si>
@@ -615,6 +609,30 @@
   </si>
   <si>
     <t>..\CHS_Dependencies\Bias_and_Uncertainty\CHS-GoM\CHS-GoM_Comb_BiasUncertainty_perVG_rta.mat</t>
+  </si>
+  <si>
+    <t>compute_damaging_depth</t>
+  </si>
+  <si>
+    <t>Comput Damaging Depth Response</t>
+  </si>
+  <si>
+    <t>Mound/Berm Seaward Slope (cota)</t>
+  </si>
+  <si>
+    <t>Mound Landward Slope (cota)</t>
+  </si>
+  <si>
+    <t>compute_damaging_depth_Ks</t>
+  </si>
+  <si>
+    <t>Shielding Parameter To Use For Damaging Depths</t>
+  </si>
+  <si>
+    <t>compute_damaging_depth_slope</t>
+  </si>
+  <si>
+    <t>Bottom Slope To Use For Damaging Dpeths (tanb)</t>
   </si>
 </sst>
 </file>
@@ -1333,7 +1351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51D29750-2AFD-4BF7-A911-1DC4ADC0FD7A}">
-  <dimension ref="A1:I72"/>
+  <dimension ref="A1:I75"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="101.7109375" customWidth="1"/>
@@ -1397,7 +1415,7 @@
         <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="F3" s="42" t="s">
         <v>80</v>
@@ -1406,7 +1424,7 @@
         <v>76</v>
       </c>
       <c r="H3" s="13" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="I3" s="13">
         <v>0.33979999999999999</v>
@@ -1423,7 +1441,7 @@
         <v>10</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="F4" s="42" t="s">
         <v>81</v>
@@ -1449,7 +1467,7 @@
         <v>10</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="F5" s="42" t="s">
         <v>83</v>
@@ -1458,7 +1476,7 @@
         <v>78</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="I5" s="13">
         <v>0.3</v>
@@ -1466,16 +1484,16 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C6" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="F6" s="42" t="s">
         <v>82</v>
@@ -1501,7 +1519,7 @@
         <v>10</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="F7" s="33"/>
       <c r="G7" s="33"/>
@@ -1533,7 +1551,7 @@
         <v>97</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C9" s="16" t="s">
         <v>10</v>
@@ -1574,7 +1592,7 @@
         <v>45</v>
       </c>
       <c r="H10" s="16" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="I10" s="2">
         <v>0.15</v>
@@ -1591,7 +1609,7 @@
         <v>10</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="F11" s="30" t="s">
         <v>87</v>
@@ -1600,7 +1618,7 @@
         <v>48</v>
       </c>
       <c r="H11" s="31" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="I11" s="2">
         <v>0.43</v>
@@ -1614,7 +1632,7 @@
         <v>25</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D12" s="2">
         <v>0</v>
@@ -1626,7 +1644,7 @@
         <v>46</v>
       </c>
       <c r="H12" s="16" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="I12" s="2">
         <v>0.78</v>
@@ -1634,10 +1652,10 @@
     </row>
     <row r="13" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="14" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C13" s="16" t="s">
         <v>10</v>
@@ -1652,7 +1670,7 @@
         <v>47</v>
       </c>
       <c r="H13" s="19" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="I13" s="3">
         <v>0.13</v>
@@ -1663,7 +1681,7 @@
         <v>85</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C14" s="16" t="s">
         <v>10</v>
@@ -1681,7 +1699,7 @@
         <v>98</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C15" s="16" t="s">
         <v>10</v>
@@ -1705,7 +1723,7 @@
         <v>68</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>10</v>
@@ -1731,7 +1749,7 @@
         <v>99</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C17" s="16" t="s">
         <v>10</v>
@@ -1757,7 +1775,7 @@
         <v>100</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C18" s="16" t="s">
         <v>10</v>
@@ -1780,10 +1798,10 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C19" s="16" t="s">
         <v>10</v>
@@ -1798,10 +1816,10 @@
     </row>
     <row r="20" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="14" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C20" s="16" t="s">
         <v>10</v>
@@ -1818,16 +1836,16 @@
     </row>
     <row r="21" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="17" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C21" s="19" t="s">
         <v>10</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>3</v>
@@ -1908,10 +1926,10 @@
     </row>
     <row r="25" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="11" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C25" s="28" t="s">
         <v>10</v>
@@ -1926,7 +1944,7 @@
         <v>37</v>
       </c>
       <c r="H25" s="19" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="I25" s="3">
         <v>1</v>
@@ -1972,16 +1990,16 @@
     </row>
     <row r="28" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C28" s="28" t="s">
         <v>10</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="F28" s="9" t="s">
         <v>3</v>
@@ -1998,16 +2016,16 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C29" s="28" t="s">
         <v>10</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F29" s="29" t="s">
         <v>43</v>
@@ -2024,16 +2042,16 @@
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="11" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C30" s="28" t="s">
         <v>10</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F30" s="14" t="s">
         <v>94</v>
@@ -2053,19 +2071,19 @@
         <v>42</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C31" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="F31" s="14" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="G31" s="15" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="H31" s="16" t="s">
         <v>10</v>
@@ -2079,19 +2097,19 @@
         <v>88</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C32" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="F32" s="14" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G32" s="15" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="H32" s="16" t="s">
         <v>10</v>
@@ -2106,10 +2124,10 @@
       <c r="C33" s="25"/>
       <c r="D33" s="25"/>
       <c r="F33" s="14" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G33" s="15" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="H33" s="16" t="s">
         <v>10</v>
@@ -2126,10 +2144,10 @@
       <c r="C34" s="35"/>
       <c r="D34" s="35"/>
       <c r="F34" s="17" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="G34" s="18" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="H34" s="19" t="s">
         <v>10</v>
@@ -2160,7 +2178,7 @@
         <v>102</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D36" s="1">
         <v>3.41</v>
@@ -2174,7 +2192,7 @@
         <v>69</v>
       </c>
       <c r="C37" s="16" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D37" s="2">
         <v>7.01</v>
@@ -2188,7 +2206,7 @@
         <v>103</v>
       </c>
       <c r="C38" s="16" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D38" s="2">
         <v>-2.42</v>
@@ -2196,13 +2214,13 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B39" s="15" t="s">
         <v>104</v>
       </c>
       <c r="C39" s="16" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D39" s="2">
         <v>-0.95799999999999996</v>
@@ -2213,7 +2231,7 @@
         <v>54</v>
       </c>
       <c r="B40" s="15" t="s">
-        <v>105</v>
+        <v>193</v>
       </c>
       <c r="C40" s="16" t="s">
         <v>10</v>
@@ -2227,7 +2245,7 @@
         <v>55</v>
       </c>
       <c r="B41" s="15" t="s">
-        <v>106</v>
+        <v>194</v>
       </c>
       <c r="C41" s="16" t="s">
         <v>10</v>
@@ -2238,10 +2256,10 @@
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="14" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B42" s="15" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C42" s="16" t="s">
         <v>10</v>
@@ -2252,10 +2270,10 @@
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B43" s="15" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C43" s="16" t="s">
         <v>10</v>
@@ -2272,7 +2290,7 @@
         <v>75</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D44" s="2">
         <v>3.35</v>
@@ -2286,7 +2304,7 @@
         <v>101</v>
       </c>
       <c r="C45" s="39" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D45" s="40">
         <v>0.06</v>
@@ -2342,7 +2360,7 @@
         <v>60</v>
       </c>
       <c r="C50" s="16" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D50" s="2">
         <v>780</v>
@@ -2350,13 +2368,13 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="14" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B51" s="12" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C51" s="16" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D51" s="2">
         <v>780</v>
@@ -2370,7 +2388,7 @@
         <v>62</v>
       </c>
       <c r="C52" s="16" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D52" s="2">
         <v>57</v>
@@ -2384,7 +2402,7 @@
         <v>64</v>
       </c>
       <c r="C53" s="16" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D53" s="2">
         <v>1027</v>
@@ -2406,10 +2424,10 @@
     </row>
     <row r="55" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B55" s="15" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C55" s="16" t="s">
         <v>10</v>
@@ -2420,10 +2438,10 @@
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="14" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B56" s="15" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C56" s="16" t="s">
         <v>10</v>
@@ -2434,10 +2452,10 @@
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="14" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B57" s="15" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C57" s="16" t="s">
         <v>10</v>
@@ -2448,10 +2466,10 @@
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="14" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B58" s="15" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C58" s="16" t="s">
         <v>10</v>
@@ -2465,7 +2483,7 @@
         <v>72</v>
       </c>
       <c r="B59" s="41" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C59" s="19" t="s">
         <v>10</v>
@@ -2482,7 +2500,7 @@
     </row>
     <row r="61" spans="1:4" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A61" s="47" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B61" s="48"/>
       <c r="C61" s="48"/>
@@ -2504,10 +2522,10 @@
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="43" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B63" s="44" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C63" s="45" t="s">
         <v>10</v>
@@ -2518,10 +2536,10 @@
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="14" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B64" s="15" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C64" s="16" t="s">
         <v>10</v>
@@ -2532,10 +2550,10 @@
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="14" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B65" s="15" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C65" s="16" t="s">
         <v>10</v>
@@ -2546,10 +2564,10 @@
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="14" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B66" s="15" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C66" s="16" t="s">
         <v>10</v>
@@ -2560,10 +2578,10 @@
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="14" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B67" s="15" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C67" s="16" t="s">
         <v>10</v>
@@ -2574,10 +2592,10 @@
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="14" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B68" s="15" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C68" s="16" t="s">
         <v>10</v>
@@ -2588,51 +2606,93 @@
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="14" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
       <c r="B69" s="15" t="s">
-        <v>125</v>
+        <v>192</v>
       </c>
       <c r="C69" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D69" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="14" t="s">
-        <v>179</v>
+        <v>195</v>
       </c>
       <c r="B70" s="15" t="s">
-        <v>126</v>
+        <v>196</v>
       </c>
       <c r="C70" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D70" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71" s="14" t="s">
+        <v>197</v>
+      </c>
+      <c r="B71" s="15" t="s">
+        <v>198</v>
+      </c>
+      <c r="C71" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D71" s="2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="B72" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="C72" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D72" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="17" t="s">
-        <v>180</v>
-      </c>
-      <c r="B71" s="18" t="s">
-        <v>127</v>
-      </c>
-      <c r="C71" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D71" s="3">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="B73" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="C73" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D73" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72" s="48"/>
-      <c r="B72" s="48"/>
-      <c r="C72" s="48"/>
-      <c r="D72" s="48"/>
+    <row r="74" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A74" s="17" t="s">
+        <v>178</v>
+      </c>
+      <c r="B74" s="18" t="s">
+        <v>125</v>
+      </c>
+      <c r="C74" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D74" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75" s="48"/>
+      <c r="B75" s="48"/>
+      <c r="C75" s="48"/>
+      <c r="D75" s="48"/>
     </row>
   </sheetData>
   <sheetProtection formatColumns="0" selectLockedCells="1"/>

</xml_diff>